<commit_message>
data updates for 4.0.5
</commit_message>
<xml_diff>
--- a/InputData/elec/CSC/Capacity Supply Curve.xlsx
+++ b/InputData/elec/CSC/Capacity Supply Curve.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\elec\CSC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\US\Models\eps-us\InputData\elec\CSC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6367CB4D-9140-4286-9A37-2062052CD2A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D47818FD-27FB-4FD4-968C-58E44B45BDB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{F87DB1D1-DC21-4EA7-B1DF-998EE56837F8}"/>
+    <workbookView xWindow="3720" yWindow="3720" windowWidth="43200" windowHeight="17085" xr2:uid="{F87DB1D1-DC21-4EA7-B1DF-998EE56837F8}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -214,9 +214,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -306,307 +307,307 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="101"/>
                 <c:pt idx="0">
-                  <c:v>0.25</c:v>
+                  <c:v>500</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.5</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.75</c:v>
+                  <c:v>1500</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1</c:v>
+                  <c:v>2000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1.25</c:v>
+                  <c:v>2500</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.5</c:v>
+                  <c:v>3000</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1.75</c:v>
+                  <c:v>3500</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>2</c:v>
+                  <c:v>4000</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>2.25</c:v>
+                  <c:v>4500</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>2.5</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>2.75</c:v>
+                  <c:v>5500</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>3</c:v>
+                  <c:v>6000</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>3.25</c:v>
+                  <c:v>6500</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>3.5</c:v>
+                  <c:v>7000</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>3.75</c:v>
+                  <c:v>7500</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>4</c:v>
+                  <c:v>8000</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>4.25</c:v>
+                  <c:v>8500</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>4.5</c:v>
+                  <c:v>9000</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>4.75</c:v>
+                  <c:v>9500</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>5</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>5.25</c:v>
+                  <c:v>10500</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>5.5</c:v>
+                  <c:v>11000</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>5.75</c:v>
+                  <c:v>11500</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>6</c:v>
+                  <c:v>12000</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>6.25</c:v>
+                  <c:v>12500</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>6.5</c:v>
+                  <c:v>13000</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>6.75</c:v>
+                  <c:v>13500</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>7</c:v>
+                  <c:v>14000</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>7.25</c:v>
+                  <c:v>14500</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>7.5</c:v>
+                  <c:v>15000</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>7.75</c:v>
+                  <c:v>15500</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>8</c:v>
+                  <c:v>16000</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>8.25</c:v>
+                  <c:v>16500</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>8.5</c:v>
+                  <c:v>17000</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>8.75</c:v>
+                  <c:v>17500</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>9</c:v>
+                  <c:v>18000</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>9.25</c:v>
+                  <c:v>18500</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>9.5</c:v>
+                  <c:v>19000</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>9.75</c:v>
+                  <c:v>19500</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>10</c:v>
+                  <c:v>20000</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>10.25</c:v>
+                  <c:v>20500</c:v>
                 </c:pt>
                 <c:pt idx="41">
-                  <c:v>10.5</c:v>
+                  <c:v>21000</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>10.75</c:v>
+                  <c:v>21500</c:v>
                 </c:pt>
                 <c:pt idx="43">
-                  <c:v>11</c:v>
+                  <c:v>22000</c:v>
                 </c:pt>
                 <c:pt idx="44">
-                  <c:v>11.25</c:v>
+                  <c:v>22500</c:v>
                 </c:pt>
                 <c:pt idx="45">
-                  <c:v>11.5</c:v>
+                  <c:v>23000</c:v>
                 </c:pt>
                 <c:pt idx="46">
-                  <c:v>11.75</c:v>
+                  <c:v>23500</c:v>
                 </c:pt>
                 <c:pt idx="47">
-                  <c:v>12</c:v>
+                  <c:v>24000</c:v>
                 </c:pt>
                 <c:pt idx="48">
-                  <c:v>12.25</c:v>
+                  <c:v>24500</c:v>
                 </c:pt>
                 <c:pt idx="49">
-                  <c:v>12.5</c:v>
+                  <c:v>25000</c:v>
                 </c:pt>
                 <c:pt idx="50">
-                  <c:v>12.75</c:v>
+                  <c:v>25500</c:v>
                 </c:pt>
                 <c:pt idx="51">
-                  <c:v>13</c:v>
+                  <c:v>26000</c:v>
                 </c:pt>
                 <c:pt idx="52">
-                  <c:v>13.25</c:v>
+                  <c:v>26500</c:v>
                 </c:pt>
                 <c:pt idx="53">
-                  <c:v>13.5</c:v>
+                  <c:v>27000</c:v>
                 </c:pt>
                 <c:pt idx="54">
-                  <c:v>13.75</c:v>
+                  <c:v>27500</c:v>
                 </c:pt>
                 <c:pt idx="55">
-                  <c:v>14</c:v>
+                  <c:v>28000</c:v>
                 </c:pt>
                 <c:pt idx="56">
-                  <c:v>14.25</c:v>
+                  <c:v>28500</c:v>
                 </c:pt>
                 <c:pt idx="57">
-                  <c:v>14.5</c:v>
+                  <c:v>29000</c:v>
                 </c:pt>
                 <c:pt idx="58">
-                  <c:v>14.75</c:v>
+                  <c:v>29500</c:v>
                 </c:pt>
                 <c:pt idx="59">
-                  <c:v>15</c:v>
+                  <c:v>30000</c:v>
                 </c:pt>
                 <c:pt idx="60">
-                  <c:v>15.25</c:v>
+                  <c:v>30500</c:v>
                 </c:pt>
                 <c:pt idx="61">
-                  <c:v>15.5</c:v>
+                  <c:v>31000</c:v>
                 </c:pt>
                 <c:pt idx="62">
-                  <c:v>15.75</c:v>
+                  <c:v>31500</c:v>
                 </c:pt>
                 <c:pt idx="63">
-                  <c:v>16</c:v>
+                  <c:v>32000</c:v>
                 </c:pt>
                 <c:pt idx="64">
-                  <c:v>16.25</c:v>
+                  <c:v>32500</c:v>
                 </c:pt>
                 <c:pt idx="65">
-                  <c:v>16.5</c:v>
+                  <c:v>33000</c:v>
                 </c:pt>
                 <c:pt idx="66">
-                  <c:v>16.75</c:v>
+                  <c:v>33500</c:v>
                 </c:pt>
                 <c:pt idx="67">
-                  <c:v>17</c:v>
+                  <c:v>34000</c:v>
                 </c:pt>
                 <c:pt idx="68">
-                  <c:v>17.25</c:v>
+                  <c:v>34500</c:v>
                 </c:pt>
                 <c:pt idx="69">
-                  <c:v>17.5</c:v>
+                  <c:v>35000</c:v>
                 </c:pt>
                 <c:pt idx="70">
-                  <c:v>17.75</c:v>
+                  <c:v>35500</c:v>
                 </c:pt>
                 <c:pt idx="71">
-                  <c:v>18</c:v>
+                  <c:v>36000</c:v>
                 </c:pt>
                 <c:pt idx="72">
-                  <c:v>18.25</c:v>
+                  <c:v>36500</c:v>
                 </c:pt>
                 <c:pt idx="73">
-                  <c:v>18.5</c:v>
+                  <c:v>37000</c:v>
                 </c:pt>
                 <c:pt idx="74">
-                  <c:v>18.75</c:v>
+                  <c:v>37500</c:v>
                 </c:pt>
                 <c:pt idx="75">
-                  <c:v>19</c:v>
+                  <c:v>38000</c:v>
                 </c:pt>
                 <c:pt idx="76">
-                  <c:v>19.25</c:v>
+                  <c:v>38500</c:v>
                 </c:pt>
                 <c:pt idx="77">
-                  <c:v>19.5</c:v>
+                  <c:v>39000</c:v>
                 </c:pt>
                 <c:pt idx="78">
-                  <c:v>19.75</c:v>
+                  <c:v>39500</c:v>
                 </c:pt>
                 <c:pt idx="79">
-                  <c:v>20</c:v>
+                  <c:v>40000</c:v>
                 </c:pt>
                 <c:pt idx="80">
-                  <c:v>20.25</c:v>
+                  <c:v>40500</c:v>
                 </c:pt>
                 <c:pt idx="81">
-                  <c:v>20.5</c:v>
+                  <c:v>41000</c:v>
                 </c:pt>
                 <c:pt idx="82">
-                  <c:v>20.75</c:v>
+                  <c:v>41500</c:v>
                 </c:pt>
                 <c:pt idx="83">
-                  <c:v>21</c:v>
+                  <c:v>42000</c:v>
                 </c:pt>
                 <c:pt idx="84">
-                  <c:v>21.25</c:v>
+                  <c:v>42500</c:v>
                 </c:pt>
                 <c:pt idx="85">
-                  <c:v>21.5</c:v>
+                  <c:v>43000</c:v>
                 </c:pt>
                 <c:pt idx="86">
-                  <c:v>21.75</c:v>
+                  <c:v>43500</c:v>
                 </c:pt>
                 <c:pt idx="87">
-                  <c:v>22</c:v>
+                  <c:v>44000</c:v>
                 </c:pt>
                 <c:pt idx="88">
-                  <c:v>22.25</c:v>
+                  <c:v>44500</c:v>
                 </c:pt>
                 <c:pt idx="89">
-                  <c:v>22.5</c:v>
+                  <c:v>45000</c:v>
                 </c:pt>
                 <c:pt idx="90">
-                  <c:v>22.75</c:v>
+                  <c:v>45500</c:v>
                 </c:pt>
                 <c:pt idx="91">
-                  <c:v>23</c:v>
+                  <c:v>46000</c:v>
                 </c:pt>
                 <c:pt idx="92">
-                  <c:v>23.25</c:v>
+                  <c:v>46500</c:v>
                 </c:pt>
                 <c:pt idx="93">
-                  <c:v>23.5</c:v>
+                  <c:v>47000</c:v>
                 </c:pt>
                 <c:pt idx="94">
-                  <c:v>23.75</c:v>
+                  <c:v>47500</c:v>
                 </c:pt>
                 <c:pt idx="95">
-                  <c:v>24</c:v>
+                  <c:v>48000</c:v>
                 </c:pt>
                 <c:pt idx="96">
-                  <c:v>24.25</c:v>
+                  <c:v>48500</c:v>
                 </c:pt>
                 <c:pt idx="97">
-                  <c:v>24.5</c:v>
+                  <c:v>49000</c:v>
                 </c:pt>
                 <c:pt idx="98">
-                  <c:v>24.75</c:v>
+                  <c:v>49500</c:v>
                 </c:pt>
                 <c:pt idx="99">
-                  <c:v>25</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="100">
-                  <c:v>25.25</c:v>
+                  <c:v>50500</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -618,307 +619,307 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="101"/>
                 <c:pt idx="0">
-                  <c:v>1.1302755611730664E-6</c:v>
+                  <c:v>4.0187703366778572E-7</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>9.041918329455445E-6</c:v>
+                  <c:v>3.2149861218577768E-6</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>3.0513853137847935E-5</c:v>
+                  <c:v>1.0850301995346534E-5</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>7.2317035876470759E-5</c:v>
+                  <c:v>2.571795964551593E-5</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1.4120526808655831E-4</c:v>
+                  <c:v>5.0226285691895579E-5</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>2.4390236156555944E-4</c:v>
+                  <c:v>8.6780443051764905E-5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>3.8708568873771498E-4</c:v>
+                  <c:v>1.3778069003070326E-4</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>5.7736617667798751E-4</c:v>
+                  <c:v>2.0562025564793696E-4</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>8.2126483012147367E-4</c:v>
+                  <c:v>2.926828338786713E-4</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1.1251859013301779E-3</c:v>
+                  <c:v>4.0133970053291554E-4</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1.4953868620252581E-3</c:v>
+                  <c:v>5.3394645769462839E-4</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>1.9379453743239433E-3</c:v>
+                  <c:v>6.9283941201358503E-4</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>2.4587235032284965E-3</c:v>
+                  <c:v>8.8033159466762703E-4</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>3.0633294620639323E-3</c:v>
+                  <c:v>1.0987084324921848E-3</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>3.7570772335819985E-3</c:v>
+                  <c:v>1.3502230815962135E-3</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>4.5449444623392177E-3</c:v>
+                  <c:v>1.6370914367420941E-3</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>5.4315290673835337E-3</c:v>
+                  <c:v>1.9614868318508726E-3</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>6.4210050770837218E-3</c:v>
+                  <c:v>2.325534449188732E-3</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>7.5170782388275237E-3</c:v>
+                  <c:v>2.7313054570853477E-3</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>8.7229420039149769E-3</c:v>
+                  <c:v>3.1808108984106021E-3</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>1.0041234530816401E-2</c:v>
+                  <c:v>3.6759953544767184E-3</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>1.1473997386527171E-2</c:v>
+                  <c:v>4.2187304115184395E-3</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>1.3022636654488842E-2</c:v>
+                  <c:v>4.8108079594126937E-3</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>1.4687887176925568E-2</c:v>
+                  <c:v>5.4539333548070607E-3</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>1.6469780667991457E-2</c:v>
+                  <c:v>6.149718483310862E-3</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>1.8367618430465693E-2</c:v>
+                  <c:v>6.899674757832674E-3</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>2.0379949391649221E-2</c:v>
+                  <c:v>7.7052060925004657E-3</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>2.2504554142594765E-2</c:v>
+                  <c:v>8.5676018938412868E-3</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>2.4738435618083782E-2</c:v>
+                  <c:v>9.4880301129990352E-3</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>2.7077816992397724E-2</c:v>
+                  <c:v>1.0467530404697972E-2</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>2.951814728782165E-2</c:v>
+                  <c:v>1.1507007440385136E-2</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>3.2054115099261718E-2</c:v>
+                  <c:v>1.2607224424474078E-2</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>3.467967073008181E-2</c:v>
+                  <c:v>1.3768796863832604E-2</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>3.7388056912446274E-2</c:v>
+                  <c:v>1.4992186641577837E-2</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>4.0171848151733677E-2</c:v>
+                  <c:v>1.6277696446830824E-2</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>4.3022998591062303E-2</c:v>
+                  <c:v>1.7625464612310682E-2</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>4.5932898141179429E-2</c:v>
+                  <c:v>1.9035460411488268E-2</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>4.8892436465861083E-2</c:v>
+                  <c:v>2.0507479866443433E-2</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>5.1892074256846804E-2</c:v>
+                  <c:v>2.2041142116558832E-2</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>5.4921921078778663E-2</c:v>
+                  <c:v>2.3635886396712456E-2</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>5.7971818917411488E-2</c:v>
+                  <c:v>2.5290969671690554E-2</c:v>
                 </c:pt>
                 <c:pt idx="41">
-                  <c:v>6.1031430427395852E-2</c:v>
+                  <c:v>2.7005464971113717E-2</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>6.4090330753079128E-2</c:v>
+                  <c:v>2.8778260466251364E-2</c:v>
                 </c:pt>
                 <c:pt idx="43">
-                  <c:v>6.7138101690766061E-2</c:v>
+                  <c:v>3.0608059326685061E-2</c:v>
                 </c:pt>
                 <c:pt idx="44">
-                  <c:v>7.0164426877205852E-2</c:v>
+                  <c:v>3.249338039087727E-2</c:v>
                 </c:pt>
                 <c:pt idx="45">
-                  <c:v>7.3159186629829842E-2</c:v>
+                  <c:v>3.4432559680315195E-2</c:v>
                 </c:pt>
                 <c:pt idx="46">
-                  <c:v>7.6112551032035736E-2</c:v>
+                  <c:v>3.6423752782045189E-2</c:v>
                 </c:pt>
                 <c:pt idx="47">
-                  <c:v>7.9015069853569708E-2</c:v>
+                  <c:v>3.8464938119114063E-2</c:v>
                 </c:pt>
                 <c:pt idx="48">
-                  <c:v>8.1857757923041286E-2</c:v>
+                  <c:v>4.055392112271447E-2</c:v>
                 </c:pt>
                 <c:pt idx="49">
-                  <c:v>8.4632174627258694E-2</c:v>
+                  <c:v>4.2688339313730859E-2</c:v>
                 </c:pt>
                 <c:pt idx="50">
-                  <c:v>8.7330496299984461E-2</c:v>
+                  <c:v>4.4865668294935525E-2</c:v>
                 </c:pt>
                 <c:pt idx="51">
-                  <c:v>8.9945580379575493E-2</c:v>
+                  <c:v>4.7083228648343023E-2</c:v>
                 </c:pt>
                 <c:pt idx="52">
-                  <c:v>9.2471020358609296E-2</c:v>
+                  <c:v>4.9338193725244575E-2</c:v>
                 </c:pt>
                 <c:pt idx="53">
-                  <c:v>9.4901190715968961E-2</c:v>
+                  <c:v>5.1627598309274762E-2</c:v>
                 </c:pt>
                 <c:pt idx="54">
-                  <c:v>9.7231281209145953E-2</c:v>
+                  <c:v>5.3948348125570124E-2</c:v>
                 </c:pt>
                 <c:pt idx="55">
-                  <c:v>9.9457320107219804E-2</c:v>
+                  <c:v>5.629723016173821E-2</c:v>
                 </c:pt>
                 <c:pt idx="56">
-                  <c:v>0.10157618615802415</c:v>
+                  <c:v>5.8670923759033294E-2</c:v>
                 </c:pt>
                 <c:pt idx="57">
-                  <c:v>0.1035856093009499</c:v>
+                  <c:v>6.1066012424913607E-2</c:v>
                 </c:pt>
                 <c:pt idx="58">
-                  <c:v>0.10548416035397182</c:v>
+                  <c:v>6.3478996311107899E-2</c:v>
                 </c:pt>
                 <c:pt idx="59">
-                  <c:v>0.10727123011408218</c:v>
+                  <c:v>6.5906305294534395E-2</c:v>
                 </c:pt>
                 <c:pt idx="60">
-                  <c:v>0.10894699850878881</c:v>
+                  <c:v>6.8344312591966452E-2</c:v>
                 </c:pt>
                 <c:pt idx="61">
-                  <c:v>0.11051239461744319</c:v>
+                  <c:v>7.0789348833315488E-2</c:v>
                 </c:pt>
                 <c:pt idx="62">
-                  <c:v>0.11196904854019522</c:v>
+                  <c:v>7.3237716512875015E-2</c:v>
                 </c:pt>
                 <c:pt idx="63">
-                  <c:v>0.11331923622529684</c:v>
+                  <c:v>7.5685704732924589E-2</c:v>
                 </c:pt>
                 <c:pt idx="64">
-                  <c:v>0.11456581846910648</c:v>
+                  <c:v>7.8129604149794987E-2</c:v>
                 </c:pt>
                 <c:pt idx="65">
-                  <c:v>0.11571217537522674</c:v>
+                  <c:v>8.0565722028919276E-2</c:v>
                 </c:pt>
                 <c:pt idx="66">
-                  <c:v>0.11676213759849677</c:v>
+                  <c:v>8.2990397312597802E-2</c:v>
                 </c:pt>
                 <c:pt idx="67">
-                  <c:v>0.11771991570586685</c:v>
+                  <c:v>8.5400015602243903E-2</c:v>
                 </c:pt>
                 <c:pt idx="68">
-                  <c:v>0.11859002896034841</c:v>
+                  <c:v>8.7791023955795813E-2</c:v>
                 </c:pt>
                 <c:pt idx="69">
-                  <c:v>0.11937723477809242</c:v>
+                  <c:v>9.015994540081855E-2</c:v>
                 </c:pt>
                 <c:pt idx="70">
-                  <c:v>0.12008646002494117</c:v>
+                  <c:v>9.2503393064599676E-2</c:v>
                 </c:pt>
                 <c:pt idx="71">
-                  <c:v>0.12072273521104175</c:v>
+                  <c:v>9.4818083824283653E-2</c:v>
                 </c:pt>
                 <c:pt idx="72">
-                  <c:v>0.12129113251445571</c:v>
+                  <c:v>9.7100851382792161E-2</c:v>
                 </c:pt>
                 <c:pt idx="73">
-                  <c:v>0.12179670842176366</c:v>
+                  <c:v>9.9348658679935559E-2</c:v>
                 </c:pt>
                 <c:pt idx="74">
-                  <c:v>0.12224445162033554</c:v>
+                  <c:v>0.10155860955271043</c:v>
                 </c:pt>
                 <c:pt idx="75">
-                  <c:v>0.12263923661819812</c:v>
+                  <c:v>0.10372795956427108</c:v>
                 </c:pt>
                 <c:pt idx="76">
-                  <c:v>0.12298578340816241</c:v>
+                  <c:v>0.10585412592740542</c:v>
                 </c:pt>
                 <c:pt idx="77">
-                  <c:v>0.12328862333768843</c:v>
+                  <c:v>0.10793469645549059</c:v>
                 </c:pt>
                 <c:pt idx="78">
-                  <c:v>0.12355207119904957</c:v>
+                  <c:v>0.10996743748177233</c:v>
                 </c:pt>
                 <c:pt idx="79">
-                  <c:v>0.12378020341934777</c:v>
+                  <c:v>0.11195030069632968</c:v>
                 </c:pt>
                 <c:pt idx="80">
-                  <c:v>0.1239768421098045</c:v>
+                  <c:v>0.11388142885916275</c:v>
                 </c:pt>
                 <c:pt idx="81">
-                  <c:v>0.12414554463077215</c:v>
+                  <c:v>0.11575916035737591</c:v>
                 </c:pt>
                 <c:pt idx="82">
-                  <c:v>0.12428959824458628</c:v>
+                  <c:v>0.11758203258431722</c:v>
                 </c:pt>
                 <c:pt idx="83">
-                  <c:v>0.12441201936347031</c:v>
+                  <c:v>0.11934878412866376</c:v>
                 </c:pt>
                 <c:pt idx="84">
-                  <c:v>0.12451555685425303</c:v>
+                  <c:v>0.12105835577169748</c:v>
                 </c:pt>
                 <c:pt idx="85">
-                  <c:v>0.12460269883504811</c:v>
+                  <c:v>0.12270989030127519</c:v>
                 </c:pt>
                 <c:pt idx="86">
-                  <c:v>0.12467568239008178</c:v>
+                  <c:v>0.12430273116113988</c:v>
                 </c:pt>
                 <c:pt idx="87">
-                  <c:v>0.12473650563587114</c:v>
+                  <c:v>0.12583641996413128</c:v>
                 </c:pt>
                 <c:pt idx="88">
-                  <c:v>0.12478694159291652</c:v>
+                  <c:v>0.12731069290740946</c:v>
                 </c:pt>
                 <c:pt idx="89">
-                  <c:v>0.12482855334969299</c:v>
+                  <c:v>0.12872547613689861</c:v>
                 </c:pt>
                 <c:pt idx="90">
-                  <c:v>0.12486271004758752</c:v>
+                  <c:v>0.1300808801166794</c:v>
                 </c:pt>
                 <c:pt idx="91">
-                  <c:v>0.12489060326408261</c:v>
+                  <c:v>0.13137719306690807</c:v>
                 </c:pt>
                 <c:pt idx="92">
-                  <c:v>0.12491326342455751</c:v>
+                  <c:v>0.13261487354093182</c:v>
                 </c:pt>
                 <c:pt idx="93">
-                  <c:v>0.12493157592833935</c:v>
+                  <c:v>0.13379454221852241</c:v>
                 </c:pt>
                 <c:pt idx="94">
-                  <c:v>0.12494629673008874</c:v>
+                  <c:v>0.1349169729974935</c:v>
                 </c:pt>
                 <c:pt idx="95">
-                  <c:v>0.12495806717151219</c:v>
+                  <c:v>0.1359830834703562</c:v>
                 </c:pt>
                 <c:pt idx="96">
-                  <c:v>0.12496742790932699</c:v>
+                  <c:v>0.13699392487605058</c:v>
                 </c:pt>
                 <c:pt idx="97">
-                  <c:v>0.1249748318322462</c:v>
+                  <c:v>0.13795067161915198</c:v>
                 </c:pt>
                 <c:pt idx="98">
-                  <c:v>0.12498065590169766</c:v>
+                  <c:v>0.13885461045027209</c:v>
                 </c:pt>
                 <c:pt idx="99">
-                  <c:v>0.12498521188753921</c:v>
+                  <c:v>0.13970712940166313</c:v>
                 </c:pt>
                 <c:pt idx="100">
-                  <c:v>0.1249887560009456</c:v>
+                  <c:v>0.14050970657130474</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1204,124 +1205,124 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.25</c:v>
+                  <c:v>750</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.5</c:v>
+                  <c:v>1500</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.75</c:v>
+                  <c:v>2250</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1</c:v>
+                  <c:v>3000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.25</c:v>
+                  <c:v>3750</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1.5</c:v>
+                  <c:v>4500</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1.75</c:v>
+                  <c:v>5250</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>2</c:v>
+                  <c:v>6000</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>2.25</c:v>
+                  <c:v>6750</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>2.5</c:v>
+                  <c:v>7500</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>2.75</c:v>
+                  <c:v>8250</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>3</c:v>
+                  <c:v>9000</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>3.25</c:v>
+                  <c:v>9750</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>3.5</c:v>
+                  <c:v>10500</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>3.75</c:v>
+                  <c:v>11250</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>4</c:v>
+                  <c:v>12000</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>4.25</c:v>
+                  <c:v>12750</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>4.5</c:v>
+                  <c:v>13500</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>4.75</c:v>
+                  <c:v>14250</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>5</c:v>
+                  <c:v>15000</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>5.25</c:v>
+                  <c:v>15750</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>5.5</c:v>
+                  <c:v>16500</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>5.75</c:v>
+                  <c:v>17250</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>6</c:v>
+                  <c:v>18000</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>6.25</c:v>
+                  <c:v>18750</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>6.5</c:v>
+                  <c:v>19500</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>6.75</c:v>
+                  <c:v>20250</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>7</c:v>
+                  <c:v>21000</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>7.25</c:v>
+                  <c:v>21750</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>7.5</c:v>
+                  <c:v>22500</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>7.75</c:v>
+                  <c:v>23250</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>8</c:v>
+                  <c:v>24000</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>8.25</c:v>
+                  <c:v>24750</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>8.5</c:v>
+                  <c:v>25500</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>8.75</c:v>
+                  <c:v>26250</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>9</c:v>
+                  <c:v>27000</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>9.25</c:v>
+                  <c:v>27750</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>9.5</c:v>
+                  <c:v>28500</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>9.75</c:v>
+                  <c:v>29250</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>10</c:v>
+                  <c:v>30000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1336,124 +1337,124 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.1302755611730664E-6</c:v>
+                  <c:v>1.3563306734076795E-6</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>9.041918329455445E-6</c:v>
+                  <c:v>1.0850301995346534E-5</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>3.0513853137847935E-5</c:v>
+                  <c:v>3.6616623765417522E-5</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>7.2317035876470759E-5</c:v>
+                  <c:v>8.6780443051764905E-5</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.4120526808655831E-4</c:v>
+                  <c:v>1.6944632170386997E-4</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>2.4390236156555944E-4</c:v>
+                  <c:v>2.926828338786713E-4</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>3.8708568873771498E-4</c:v>
+                  <c:v>4.6450282648525794E-4</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>5.7736617667798751E-4</c:v>
+                  <c:v>6.9283941201358503E-4</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>8.2126483012147367E-4</c:v>
+                  <c:v>9.8551779614576844E-4</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1.1251859013301779E-3</c:v>
+                  <c:v>1.3502230815962135E-3</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>1.4953868620252581E-3</c:v>
+                  <c:v>1.7944642344303095E-3</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>1.9379453743239433E-3</c:v>
+                  <c:v>2.325534449188732E-3</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>2.4587235032284965E-3</c:v>
+                  <c:v>2.9504682038741957E-3</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>3.0633294620639323E-3</c:v>
+                  <c:v>3.6759953544767184E-3</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>3.7570772335819985E-3</c:v>
+                  <c:v>4.5084926802983977E-3</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>4.5449444623392177E-3</c:v>
+                  <c:v>5.4539333548070607E-3</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>5.4315290673835337E-3</c:v>
+                  <c:v>6.5178348808602399E-3</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>6.4210050770837218E-3</c:v>
+                  <c:v>7.7052060925004657E-3</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>7.5170782388275237E-3</c:v>
+                  <c:v>9.0204938865930274E-3</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>8.7229420039149769E-3</c:v>
+                  <c:v>1.0467530404697972E-2</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>1.0041234530816401E-2</c:v>
+                  <c:v>1.2049481436979681E-2</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>1.1473997386527171E-2</c:v>
+                  <c:v>1.3768796863832604E-2</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>1.3022636654488842E-2</c:v>
+                  <c:v>1.5627163985386609E-2</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>1.4687887176925568E-2</c:v>
+                  <c:v>1.7625464612310682E-2</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>1.6469780667991457E-2</c:v>
+                  <c:v>1.9763736801589746E-2</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>1.8367618430465693E-2</c:v>
+                  <c:v>2.2041142116558832E-2</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>2.0379949391649221E-2</c:v>
+                  <c:v>2.4455939269979066E-2</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>2.2504554142594765E-2</c:v>
+                  <c:v>2.7005464971113717E-2</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>2.4738435618083782E-2</c:v>
+                  <c:v>2.9686122741700537E-2</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>2.7077816992397724E-2</c:v>
+                  <c:v>3.249338039087727E-2</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>2.951814728782165E-2</c:v>
+                  <c:v>3.5421776745385977E-2</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>3.2054115099261718E-2</c:v>
+                  <c:v>3.8464938119114063E-2</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>3.467967073008181E-2</c:v>
+                  <c:v>4.1615604876098174E-2</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>3.7388056912446274E-2</c:v>
+                  <c:v>4.4865668294935525E-2</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>4.0171848151733677E-2</c:v>
+                  <c:v>4.820621778208041E-2</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>4.3022998591062303E-2</c:v>
+                  <c:v>5.1627598309274762E-2</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>4.5932898141179429E-2</c:v>
+                  <c:v>5.5119477769415316E-2</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>4.8892436465861083E-2</c:v>
+                  <c:v>5.8670923759033294E-2</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>5.1892074256846804E-2</c:v>
+                  <c:v>6.2270489108216164E-2</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>5.4921921078778663E-2</c:v>
+                  <c:v>6.5906305294534395E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1739,124 +1740,124 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.25</c:v>
+                  <c:v>750</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.5</c:v>
+                  <c:v>1500</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.75</c:v>
+                  <c:v>2250</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1</c:v>
+                  <c:v>3000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.25</c:v>
+                  <c:v>3750</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1.5</c:v>
+                  <c:v>4500</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1.75</c:v>
+                  <c:v>5250</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>2</c:v>
+                  <c:v>6000</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>2.25</c:v>
+                  <c:v>6750</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>2.5</c:v>
+                  <c:v>7500</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>2.75</c:v>
+                  <c:v>8250</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>3</c:v>
+                  <c:v>9000</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>3.25</c:v>
+                  <c:v>9750</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>3.5</c:v>
+                  <c:v>10500</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>3.75</c:v>
+                  <c:v>11250</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>4</c:v>
+                  <c:v>12000</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>4.25</c:v>
+                  <c:v>12750</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>4.5</c:v>
+                  <c:v>13500</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>4.75</c:v>
+                  <c:v>14250</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>5</c:v>
+                  <c:v>15000</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>5.25</c:v>
+                  <c:v>15750</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>5.5</c:v>
+                  <c:v>16500</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>5.75</c:v>
+                  <c:v>17250</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>6</c:v>
+                  <c:v>18000</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>6.25</c:v>
+                  <c:v>18750</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>6.5</c:v>
+                  <c:v>19500</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>6.75</c:v>
+                  <c:v>20250</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>7</c:v>
+                  <c:v>21000</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>7.25</c:v>
+                  <c:v>21750</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>7.5</c:v>
+                  <c:v>22500</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>7.75</c:v>
+                  <c:v>23250</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>8</c:v>
+                  <c:v>24000</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>8.25</c:v>
+                  <c:v>24750</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>8.5</c:v>
+                  <c:v>25500</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>8.75</c:v>
+                  <c:v>26250</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>9</c:v>
+                  <c:v>27000</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>9.25</c:v>
+                  <c:v>27750</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>9.5</c:v>
+                  <c:v>28500</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>9.75</c:v>
+                  <c:v>29250</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>10</c:v>
+                  <c:v>30000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1871,124 +1872,124 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.1302755611730664E-6</c:v>
+                  <c:v>1.3563306734076795E-6</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>9.041918329455445E-6</c:v>
+                  <c:v>1.0850301995346534E-5</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>3.0513853137847935E-5</c:v>
+                  <c:v>3.6616623765417522E-5</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>7.2317035876470759E-5</c:v>
+                  <c:v>8.6780443051764905E-5</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.4120526808655831E-4</c:v>
+                  <c:v>1.6944632170386997E-4</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>2.4390236156555944E-4</c:v>
+                  <c:v>2.926828338786713E-4</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>3.8708568873771498E-4</c:v>
+                  <c:v>4.6450282648525794E-4</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>5.7736617667798751E-4</c:v>
+                  <c:v>6.9283941201358503E-4</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>8.2126483012147367E-4</c:v>
+                  <c:v>9.8551779614576844E-4</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1.1251859013301779E-3</c:v>
+                  <c:v>1.3502230815962135E-3</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>1.4953868620252581E-3</c:v>
+                  <c:v>1.7944642344303095E-3</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>1.9379453743239433E-3</c:v>
+                  <c:v>2.325534449188732E-3</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>2.4587235032284965E-3</c:v>
+                  <c:v>2.9504682038741957E-3</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>3.0633294620639323E-3</c:v>
+                  <c:v>3.6759953544767184E-3</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>3.7570772335819985E-3</c:v>
+                  <c:v>4.5084926802983977E-3</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>4.5449444623392177E-3</c:v>
+                  <c:v>5.4539333548070607E-3</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>5.4315290673835337E-3</c:v>
+                  <c:v>6.5178348808602399E-3</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>6.4210050770837218E-3</c:v>
+                  <c:v>7.7052060925004657E-3</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>7.5170782388275237E-3</c:v>
+                  <c:v>9.0204938865930274E-3</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>8.7229420039149769E-3</c:v>
+                  <c:v>1.0467530404697972E-2</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>1.0041234530816401E-2</c:v>
+                  <c:v>1.2049481436979681E-2</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>1.1473997386527171E-2</c:v>
+                  <c:v>1.3768796863832604E-2</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>1.3022636654488842E-2</c:v>
+                  <c:v>1.5627163985386609E-2</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>1.4687887176925568E-2</c:v>
+                  <c:v>1.7625464612310682E-2</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>1.6469780667991457E-2</c:v>
+                  <c:v>1.9763736801589746E-2</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>1.8367618430465693E-2</c:v>
+                  <c:v>2.2041142116558832E-2</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>2.0379949391649221E-2</c:v>
+                  <c:v>2.4455939269979066E-2</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>2.2504554142594765E-2</c:v>
+                  <c:v>2.7005464971113717E-2</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>2.4738435618083782E-2</c:v>
+                  <c:v>2.9686122741700537E-2</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>2.7077816992397724E-2</c:v>
+                  <c:v>3.249338039087727E-2</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>2.951814728782165E-2</c:v>
+                  <c:v>3.5421776745385977E-2</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>3.2054115099261718E-2</c:v>
+                  <c:v>3.8464938119114063E-2</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>3.467967073008181E-2</c:v>
+                  <c:v>4.1615604876098174E-2</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>3.7388056912446274E-2</c:v>
+                  <c:v>4.4865668294935525E-2</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>4.0171848151733677E-2</c:v>
+                  <c:v>4.820621778208041E-2</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>4.3022998591062303E-2</c:v>
+                  <c:v>5.1627598309274762E-2</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>4.5932898141179429E-2</c:v>
+                  <c:v>5.5119477769415316E-2</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>4.8892436465861083E-2</c:v>
+                  <c:v>5.8670923759033294E-2</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>5.1892074256846804E-2</c:v>
+                  <c:v>6.2270489108216164E-2</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>5.4921921078778663E-2</c:v>
+                  <c:v>6.5906305294534395E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4340,7 +4341,7 @@
         <v>37</v>
       </c>
       <c r="B15">
-        <v>0.125</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -4372,7 +4373,7 @@
         <v>39</v>
       </c>
       <c r="B19">
-        <v>20</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -4387,1011 +4388,1009 @@
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B24">
         <f t="shared" ref="B24:B87" si="0">(1-EXP(-((C24/$B$19-($B$18-0.5))/$B$16)^$B$17))*$B$15</f>
-        <v>1.1302755611730664E-6</v>
+        <v>4.0187703366778572E-7</v>
       </c>
       <c r="C24">
-        <f>C23+0.25</f>
-        <v>0.25</v>
+        <v>500</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B25">
         <f t="shared" si="0"/>
-        <v>9.041918329455445E-6</v>
+        <v>3.2149861218577768E-6</v>
       </c>
       <c r="C25">
-        <f t="shared" ref="C25:C88" si="1">C24+0.25</f>
-        <v>0.5</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B26">
         <f t="shared" si="0"/>
-        <v>3.0513853137847935E-5</v>
+        <v>1.0850301995346534E-5</v>
       </c>
       <c r="C26">
-        <f t="shared" si="1"/>
-        <v>0.75</v>
+        <f>C25+500</f>
+        <v>1500</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B27">
         <f t="shared" si="0"/>
-        <v>7.2317035876470759E-5</v>
+        <v>2.571795964551593E-5</v>
       </c>
       <c r="C27">
-        <f t="shared" si="1"/>
-        <v>1</v>
+        <f t="shared" ref="C27:C90" si="1">C26+500</f>
+        <v>2000</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B28">
         <f t="shared" si="0"/>
-        <v>1.4120526808655831E-4</v>
+        <v>5.0226285691895579E-5</v>
       </c>
       <c r="C28">
         <f t="shared" si="1"/>
-        <v>1.25</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B29">
         <f t="shared" si="0"/>
-        <v>2.4390236156555944E-4</v>
+        <v>8.6780443051764905E-5</v>
       </c>
       <c r="C29">
         <f t="shared" si="1"/>
-        <v>1.5</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B30">
         <f t="shared" si="0"/>
-        <v>3.8708568873771498E-4</v>
+        <v>1.3778069003070326E-4</v>
       </c>
       <c r="C30">
         <f t="shared" si="1"/>
-        <v>1.75</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B31">
         <f t="shared" si="0"/>
-        <v>5.7736617667798751E-4</v>
+        <v>2.0562025564793696E-4</v>
       </c>
       <c r="C31">
         <f t="shared" si="1"/>
-        <v>2</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B32">
         <f t="shared" si="0"/>
-        <v>8.2126483012147367E-4</v>
+        <v>2.926828338786713E-4</v>
       </c>
       <c r="C32">
         <f t="shared" si="1"/>
-        <v>2.25</v>
+        <v>4500</v>
       </c>
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B33">
         <f t="shared" si="0"/>
-        <v>1.1251859013301779E-3</v>
+        <v>4.0133970053291554E-4</v>
       </c>
       <c r="C33">
         <f t="shared" si="1"/>
-        <v>2.5</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="34" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B34">
         <f t="shared" si="0"/>
-        <v>1.4953868620252581E-3</v>
+        <v>5.3394645769462839E-4</v>
       </c>
       <c r="C34">
         <f t="shared" si="1"/>
-        <v>2.75</v>
+        <v>5500</v>
       </c>
     </row>
     <row r="35" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B35">
         <f t="shared" si="0"/>
-        <v>1.9379453743239433E-3</v>
+        <v>6.9283941201358503E-4</v>
       </c>
       <c r="C35">
         <f t="shared" si="1"/>
-        <v>3</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="36" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B36">
         <f t="shared" si="0"/>
-        <v>2.4587235032284965E-3</v>
+        <v>8.8033159466762703E-4</v>
       </c>
       <c r="C36">
         <f t="shared" si="1"/>
-        <v>3.25</v>
+        <v>6500</v>
       </c>
     </row>
     <row r="37" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B37">
         <f t="shared" si="0"/>
-        <v>3.0633294620639323E-3</v>
+        <v>1.0987084324921848E-3</v>
       </c>
       <c r="C37">
         <f t="shared" si="1"/>
-        <v>3.5</v>
+        <v>7000</v>
       </c>
     </row>
     <row r="38" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B38">
         <f t="shared" si="0"/>
-        <v>3.7570772335819985E-3</v>
+        <v>1.3502230815962135E-3</v>
       </c>
       <c r="C38">
         <f t="shared" si="1"/>
-        <v>3.75</v>
+        <v>7500</v>
       </c>
     </row>
     <row r="39" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B39">
         <f t="shared" si="0"/>
-        <v>4.5449444623392177E-3</v>
+        <v>1.6370914367420941E-3</v>
       </c>
       <c r="C39">
         <f t="shared" si="1"/>
-        <v>4</v>
+        <v>8000</v>
       </c>
     </row>
     <row r="40" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B40">
         <f t="shared" si="0"/>
-        <v>5.4315290673835337E-3</v>
+        <v>1.9614868318508726E-3</v>
       </c>
       <c r="C40">
         <f t="shared" si="1"/>
-        <v>4.25</v>
+        <v>8500</v>
       </c>
     </row>
     <row r="41" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B41">
         <f t="shared" si="0"/>
-        <v>6.4210050770837218E-3</v>
+        <v>2.325534449188732E-3</v>
       </c>
       <c r="C41">
         <f t="shared" si="1"/>
-        <v>4.5</v>
+        <v>9000</v>
       </c>
     </row>
     <row r="42" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B42">
         <f t="shared" si="0"/>
-        <v>7.5170782388275237E-3</v>
+        <v>2.7313054570853477E-3</v>
       </c>
       <c r="C42">
         <f t="shared" si="1"/>
-        <v>4.75</v>
+        <v>9500</v>
       </c>
     </row>
     <row r="43" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B43">
         <f t="shared" si="0"/>
-        <v>8.7229420039149769E-3</v>
+        <v>3.1808108984106021E-3</v>
       </c>
       <c r="C43">
         <f t="shared" si="1"/>
-        <v>5</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="44" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B44">
         <f t="shared" si="0"/>
-        <v>1.0041234530816401E-2</v>
+        <v>3.6759953544767184E-3</v>
       </c>
       <c r="C44">
         <f t="shared" si="1"/>
-        <v>5.25</v>
+        <v>10500</v>
       </c>
     </row>
     <row r="45" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B45">
         <f t="shared" si="0"/>
-        <v>1.1473997386527171E-2</v>
+        <v>4.2187304115184395E-3</v>
       </c>
       <c r="C45">
         <f t="shared" si="1"/>
-        <v>5.5</v>
+        <v>11000</v>
       </c>
     </row>
     <row r="46" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B46">
         <f t="shared" si="0"/>
-        <v>1.3022636654488842E-2</v>
+        <v>4.8108079594126937E-3</v>
       </c>
       <c r="C46">
         <f t="shared" si="1"/>
-        <v>5.75</v>
+        <v>11500</v>
       </c>
     </row>
     <row r="47" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B47">
         <f t="shared" si="0"/>
-        <v>1.4687887176925568E-2</v>
+        <v>5.4539333548070607E-3</v>
       </c>
       <c r="C47">
         <f t="shared" si="1"/>
-        <v>6</v>
+        <v>12000</v>
       </c>
     </row>
     <row r="48" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B48">
         <f t="shared" si="0"/>
-        <v>1.6469780667991457E-2</v>
+        <v>6.149718483310862E-3</v>
       </c>
       <c r="C48">
         <f t="shared" si="1"/>
-        <v>6.25</v>
+        <v>12500</v>
       </c>
     </row>
     <row r="49" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B49">
         <f t="shared" si="0"/>
-        <v>1.8367618430465693E-2</v>
+        <v>6.899674757832674E-3</v>
       </c>
       <c r="C49">
         <f t="shared" si="1"/>
-        <v>6.5</v>
+        <v>13000</v>
       </c>
     </row>
     <row r="50" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B50">
         <f t="shared" si="0"/>
-        <v>2.0379949391649221E-2</v>
+        <v>7.7052060925004657E-3</v>
       </c>
       <c r="C50">
         <f t="shared" si="1"/>
-        <v>6.75</v>
+        <v>13500</v>
       </c>
     </row>
     <row r="51" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B51">
         <f t="shared" si="0"/>
-        <v>2.2504554142594765E-2</v>
+        <v>8.5676018938412868E-3</v>
       </c>
       <c r="C51">
         <f t="shared" si="1"/>
-        <v>7</v>
+        <v>14000</v>
       </c>
     </row>
     <row r="52" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B52">
         <f t="shared" si="0"/>
-        <v>2.4738435618083782E-2</v>
+        <v>9.4880301129990352E-3</v>
       </c>
       <c r="C52">
         <f t="shared" si="1"/>
-        <v>7.25</v>
+        <v>14500</v>
       </c>
     </row>
     <row r="53" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B53">
         <f t="shared" si="0"/>
-        <v>2.7077816992397724E-2</v>
+        <v>1.0467530404697972E-2</v>
       </c>
       <c r="C53">
         <f t="shared" si="1"/>
-        <v>7.5</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="54" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B54">
         <f t="shared" si="0"/>
-        <v>2.951814728782165E-2</v>
+        <v>1.1507007440385136E-2</v>
       </c>
       <c r="C54">
         <f t="shared" si="1"/>
-        <v>7.75</v>
+        <v>15500</v>
       </c>
     </row>
     <row r="55" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B55">
         <f t="shared" si="0"/>
-        <v>3.2054115099261718E-2</v>
+        <v>1.2607224424474078E-2</v>
       </c>
       <c r="C55">
         <f t="shared" si="1"/>
-        <v>8</v>
+        <v>16000</v>
       </c>
     </row>
     <row r="56" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B56">
         <f t="shared" si="0"/>
-        <v>3.467967073008181E-2</v>
+        <v>1.3768796863832604E-2</v>
       </c>
       <c r="C56">
         <f t="shared" si="1"/>
-        <v>8.25</v>
+        <v>16500</v>
       </c>
     </row>
     <row r="57" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B57">
         <f t="shared" si="0"/>
-        <v>3.7388056912446274E-2</v>
+        <v>1.4992186641577837E-2</v>
       </c>
       <c r="C57">
         <f t="shared" si="1"/>
-        <v>8.5</v>
+        <v>17000</v>
       </c>
     </row>
     <row r="58" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B58">
         <f t="shared" si="0"/>
-        <v>4.0171848151733677E-2</v>
+        <v>1.6277696446830824E-2</v>
       </c>
       <c r="C58">
         <f t="shared" si="1"/>
-        <v>8.75</v>
+        <v>17500</v>
       </c>
     </row>
     <row r="59" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B59">
         <f t="shared" si="0"/>
-        <v>4.3022998591062303E-2</v>
+        <v>1.7625464612310682E-2</v>
       </c>
       <c r="C59">
         <f t="shared" si="1"/>
-        <v>9</v>
+        <v>18000</v>
       </c>
     </row>
     <row r="60" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B60">
         <f t="shared" si="0"/>
-        <v>4.5932898141179429E-2</v>
+        <v>1.9035460411488268E-2</v>
       </c>
       <c r="C60">
         <f t="shared" si="1"/>
-        <v>9.25</v>
+        <v>18500</v>
       </c>
     </row>
     <row r="61" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B61">
         <f t="shared" si="0"/>
-        <v>4.8892436465861083E-2</v>
+        <v>2.0507479866443433E-2</v>
       </c>
       <c r="C61">
         <f t="shared" si="1"/>
-        <v>9.5</v>
+        <v>19000</v>
       </c>
     </row>
     <row r="62" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B62">
         <f t="shared" si="0"/>
-        <v>5.1892074256846804E-2</v>
+        <v>2.2041142116558832E-2</v>
       </c>
       <c r="C62">
         <f t="shared" si="1"/>
-        <v>9.75</v>
+        <v>19500</v>
       </c>
     </row>
     <row r="63" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B63">
         <f t="shared" si="0"/>
-        <v>5.4921921078778663E-2</v>
+        <v>2.3635886396712456E-2</v>
       </c>
       <c r="C63">
         <f t="shared" si="1"/>
-        <v>10</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="64" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B64">
         <f t="shared" si="0"/>
-        <v>5.7971818917411488E-2</v>
+        <v>2.5290969671690554E-2</v>
       </c>
       <c r="C64">
         <f t="shared" si="1"/>
-        <v>10.25</v>
+        <v>20500</v>
       </c>
     </row>
     <row r="65" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B65">
         <f t="shared" si="0"/>
-        <v>6.1031430427395852E-2</v>
+        <v>2.7005464971113717E-2</v>
       </c>
       <c r="C65">
         <f t="shared" si="1"/>
-        <v>10.5</v>
+        <v>21000</v>
       </c>
     </row>
     <row r="66" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B66">
         <f t="shared" si="0"/>
-        <v>6.4090330753079128E-2</v>
+        <v>2.8778260466251364E-2</v>
       </c>
       <c r="C66">
         <f t="shared" si="1"/>
-        <v>10.75</v>
+        <v>21500</v>
       </c>
     </row>
     <row r="67" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B67">
         <f t="shared" si="0"/>
-        <v>6.7138101690766061E-2</v>
+        <v>3.0608059326685061E-2</v>
       </c>
       <c r="C67">
         <f t="shared" si="1"/>
-        <v>11</v>
+        <v>22000</v>
       </c>
     </row>
     <row r="68" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B68">
         <f t="shared" si="0"/>
-        <v>7.0164426877205852E-2</v>
+        <v>3.249338039087727E-2</v>
       </c>
       <c r="C68">
         <f t="shared" si="1"/>
-        <v>11.25</v>
+        <v>22500</v>
       </c>
     </row>
     <row r="69" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B69">
         <f t="shared" si="0"/>
-        <v>7.3159186629829842E-2</v>
+        <v>3.4432559680315195E-2</v>
       </c>
       <c r="C69">
         <f t="shared" si="1"/>
-        <v>11.5</v>
+        <v>23000</v>
       </c>
     </row>
     <row r="70" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B70">
         <f t="shared" si="0"/>
-        <v>7.6112551032035736E-2</v>
+        <v>3.6423752782045189E-2</v>
       </c>
       <c r="C70">
         <f t="shared" si="1"/>
-        <v>11.75</v>
+        <v>23500</v>
       </c>
     </row>
     <row r="71" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B71">
         <f t="shared" si="0"/>
-        <v>7.9015069853569708E-2</v>
+        <v>3.8464938119114063E-2</v>
       </c>
       <c r="C71">
         <f t="shared" si="1"/>
-        <v>12</v>
+        <v>24000</v>
       </c>
     </row>
     <row r="72" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B72">
         <f t="shared" si="0"/>
-        <v>8.1857757923041286E-2</v>
+        <v>4.055392112271447E-2</v>
       </c>
       <c r="C72">
         <f t="shared" si="1"/>
-        <v>12.25</v>
+        <v>24500</v>
       </c>
     </row>
     <row r="73" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B73">
         <f t="shared" si="0"/>
-        <v>8.4632174627258694E-2</v>
+        <v>4.2688339313730859E-2</v>
       </c>
       <c r="C73">
         <f t="shared" si="1"/>
-        <v>12.5</v>
+        <v>25000</v>
       </c>
     </row>
     <row r="74" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B74">
         <f t="shared" si="0"/>
-        <v>8.7330496299984461E-2</v>
+        <v>4.4865668294935525E-2</v>
       </c>
       <c r="C74">
         <f t="shared" si="1"/>
-        <v>12.75</v>
+        <v>25500</v>
       </c>
     </row>
     <row r="75" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B75">
         <f t="shared" si="0"/>
-        <v>8.9945580379575493E-2</v>
+        <v>4.7083228648343023E-2</v>
       </c>
       <c r="C75">
         <f t="shared" si="1"/>
-        <v>13</v>
+        <v>26000</v>
       </c>
     </row>
     <row r="76" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B76">
         <f t="shared" si="0"/>
-        <v>9.2471020358609296E-2</v>
+        <v>4.9338193725244575E-2</v>
       </c>
       <c r="C76">
         <f t="shared" si="1"/>
-        <v>13.25</v>
+        <v>26500</v>
       </c>
     </row>
     <row r="77" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B77">
         <f t="shared" si="0"/>
-        <v>9.4901190715968961E-2</v>
+        <v>5.1627598309274762E-2</v>
       </c>
       <c r="C77">
         <f t="shared" si="1"/>
-        <v>13.5</v>
+        <v>27000</v>
       </c>
     </row>
     <row r="78" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B78">
         <f t="shared" si="0"/>
-        <v>9.7231281209145953E-2</v>
+        <v>5.3948348125570124E-2</v>
       </c>
       <c r="C78">
         <f t="shared" si="1"/>
-        <v>13.75</v>
+        <v>27500</v>
       </c>
     </row>
     <row r="79" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B79">
         <f t="shared" si="0"/>
-        <v>9.9457320107219804E-2</v>
+        <v>5.629723016173821E-2</v>
       </c>
       <c r="C79">
         <f t="shared" si="1"/>
-        <v>14</v>
+        <v>28000</v>
       </c>
     </row>
     <row r="80" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B80">
         <f t="shared" si="0"/>
-        <v>0.10157618615802415</v>
+        <v>5.8670923759033294E-2</v>
       </c>
       <c r="C80">
         <f t="shared" si="1"/>
-        <v>14.25</v>
+        <v>28500</v>
       </c>
     </row>
     <row r="81" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B81">
         <f t="shared" si="0"/>
-        <v>0.1035856093009499</v>
+        <v>6.1066012424913607E-2</v>
       </c>
       <c r="C81">
         <f t="shared" si="1"/>
-        <v>14.5</v>
+        <v>29000</v>
       </c>
     </row>
     <row r="82" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B82">
         <f t="shared" si="0"/>
-        <v>0.10548416035397182</v>
+        <v>6.3478996311107899E-2</v>
       </c>
       <c r="C82">
         <f t="shared" si="1"/>
-        <v>14.75</v>
+        <v>29500</v>
       </c>
     </row>
     <row r="83" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B83">
         <f t="shared" si="0"/>
-        <v>0.10727123011408218</v>
+        <v>6.5906305294534395E-2</v>
       </c>
       <c r="C83">
         <f t="shared" si="1"/>
-        <v>15</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="84" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B84">
         <f t="shared" si="0"/>
-        <v>0.10894699850878881</v>
+        <v>6.8344312591966452E-2</v>
       </c>
       <c r="C84">
         <f t="shared" si="1"/>
-        <v>15.25</v>
+        <v>30500</v>
       </c>
     </row>
     <row r="85" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B85">
         <f t="shared" si="0"/>
-        <v>0.11051239461744319</v>
+        <v>7.0789348833315488E-2</v>
       </c>
       <c r="C85">
         <f t="shared" si="1"/>
-        <v>15.5</v>
+        <v>31000</v>
       </c>
     </row>
     <row r="86" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B86">
         <f t="shared" si="0"/>
-        <v>0.11196904854019522</v>
+        <v>7.3237716512875015E-2</v>
       </c>
       <c r="C86">
         <f t="shared" si="1"/>
-        <v>15.75</v>
+        <v>31500</v>
       </c>
     </row>
     <row r="87" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B87">
         <f t="shared" si="0"/>
-        <v>0.11331923622529684</v>
+        <v>7.5685704732924589E-2</v>
       </c>
       <c r="C87">
         <f t="shared" si="1"/>
-        <v>16</v>
+        <v>32000</v>
       </c>
     </row>
     <row r="88" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B88">
         <f t="shared" ref="B88:B124" si="2">(1-EXP(-((C88/$B$19-($B$18-0.5))/$B$16)^$B$17))*$B$15</f>
-        <v>0.11456581846910648</v>
+        <v>7.8129604149794987E-2</v>
       </c>
       <c r="C88">
         <f t="shared" si="1"/>
-        <v>16.25</v>
+        <v>32500</v>
       </c>
     </row>
     <row r="89" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B89">
         <f t="shared" si="2"/>
-        <v>0.11571217537522674</v>
+        <v>8.0565722028919276E-2</v>
       </c>
       <c r="C89">
-        <f t="shared" ref="C89:C124" si="3">C88+0.25</f>
-        <v>16.5</v>
+        <f t="shared" si="1"/>
+        <v>33000</v>
       </c>
     </row>
     <row r="90" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B90">
         <f t="shared" si="2"/>
-        <v>0.11676213759849677</v>
+        <v>8.2990397312597802E-2</v>
       </c>
       <c r="C90">
-        <f t="shared" si="3"/>
-        <v>16.75</v>
+        <f t="shared" si="1"/>
+        <v>33500</v>
       </c>
     </row>
     <row r="91" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B91">
         <f t="shared" si="2"/>
-        <v>0.11771991570586685</v>
+        <v>8.5400015602243903E-2</v>
       </c>
       <c r="C91">
-        <f t="shared" si="3"/>
-        <v>17</v>
+        <f t="shared" ref="C91:C124" si="3">C90+500</f>
+        <v>34000</v>
       </c>
     </row>
     <row r="92" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B92">
         <f t="shared" si="2"/>
-        <v>0.11859002896034841</v>
+        <v>8.7791023955795813E-2</v>
       </c>
       <c r="C92">
         <f t="shared" si="3"/>
-        <v>17.25</v>
+        <v>34500</v>
       </c>
     </row>
     <row r="93" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B93">
         <f t="shared" si="2"/>
-        <v>0.11937723477809242</v>
+        <v>9.015994540081855E-2</v>
       </c>
       <c r="C93">
         <f t="shared" si="3"/>
-        <v>17.5</v>
+        <v>35000</v>
       </c>
     </row>
     <row r="94" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B94">
         <f t="shared" si="2"/>
-        <v>0.12008646002494117</v>
+        <v>9.2503393064599676E-2</v>
       </c>
       <c r="C94">
         <f t="shared" si="3"/>
-        <v>17.75</v>
+        <v>35500</v>
       </c>
     </row>
     <row r="95" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B95">
         <f t="shared" si="2"/>
-        <v>0.12072273521104175</v>
+        <v>9.4818083824283653E-2</v>
       </c>
       <c r="C95">
         <f t="shared" si="3"/>
-        <v>18</v>
+        <v>36000</v>
       </c>
     </row>
     <row r="96" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B96">
         <f t="shared" si="2"/>
-        <v>0.12129113251445571</v>
+        <v>9.7100851382792161E-2</v>
       </c>
       <c r="C96">
         <f t="shared" si="3"/>
-        <v>18.25</v>
+        <v>36500</v>
       </c>
     </row>
     <row r="97" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B97">
         <f t="shared" si="2"/>
-        <v>0.12179670842176366</v>
+        <v>9.9348658679935559E-2</v>
       </c>
       <c r="C97">
         <f t="shared" si="3"/>
-        <v>18.5</v>
+        <v>37000</v>
       </c>
     </row>
     <row r="98" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B98">
         <f t="shared" si="2"/>
-        <v>0.12224445162033554</v>
+        <v>0.10155860955271043</v>
       </c>
       <c r="C98">
         <f t="shared" si="3"/>
-        <v>18.75</v>
+        <v>37500</v>
       </c>
     </row>
     <row r="99" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B99">
         <f t="shared" si="2"/>
-        <v>0.12263923661819812</v>
+        <v>0.10372795956427108</v>
       </c>
       <c r="C99">
         <f t="shared" si="3"/>
-        <v>19</v>
+        <v>38000</v>
       </c>
     </row>
     <row r="100" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B100">
         <f t="shared" si="2"/>
-        <v>0.12298578340816241</v>
+        <v>0.10585412592740542</v>
       </c>
       <c r="C100">
         <f t="shared" si="3"/>
-        <v>19.25</v>
+        <v>38500</v>
       </c>
     </row>
     <row r="101" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B101">
         <f t="shared" si="2"/>
-        <v>0.12328862333768843</v>
+        <v>0.10793469645549059</v>
       </c>
       <c r="C101">
         <f t="shared" si="3"/>
-        <v>19.5</v>
+        <v>39000</v>
       </c>
     </row>
     <row r="102" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B102">
         <f t="shared" si="2"/>
-        <v>0.12355207119904957</v>
+        <v>0.10996743748177233</v>
       </c>
       <c r="C102">
         <f t="shared" si="3"/>
-        <v>19.75</v>
+        <v>39500</v>
       </c>
     </row>
     <row r="103" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B103">
         <f t="shared" si="2"/>
-        <v>0.12378020341934777</v>
+        <v>0.11195030069632968</v>
       </c>
       <c r="C103">
         <f t="shared" si="3"/>
-        <v>20</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="104" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B104">
         <f t="shared" si="2"/>
-        <v>0.1239768421098045</v>
+        <v>0.11388142885916275</v>
       </c>
       <c r="C104">
         <f t="shared" si="3"/>
-        <v>20.25</v>
+        <v>40500</v>
       </c>
     </row>
     <row r="105" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B105">
         <f t="shared" si="2"/>
-        <v>0.12414554463077215</v>
+        <v>0.11575916035737591</v>
       </c>
       <c r="C105">
         <f t="shared" si="3"/>
-        <v>20.5</v>
+        <v>41000</v>
       </c>
     </row>
     <row r="106" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B106">
         <f t="shared" si="2"/>
-        <v>0.12428959824458628</v>
+        <v>0.11758203258431722</v>
       </c>
       <c r="C106">
         <f t="shared" si="3"/>
-        <v>20.75</v>
+        <v>41500</v>
       </c>
     </row>
     <row r="107" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B107">
         <f t="shared" si="2"/>
-        <v>0.12441201936347031</v>
+        <v>0.11934878412866376</v>
       </c>
       <c r="C107">
         <f t="shared" si="3"/>
-        <v>21</v>
+        <v>42000</v>
       </c>
     </row>
     <row r="108" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B108">
         <f t="shared" si="2"/>
-        <v>0.12451555685425303</v>
+        <v>0.12105835577169748</v>
       </c>
       <c r="C108">
         <f t="shared" si="3"/>
-        <v>21.25</v>
+        <v>42500</v>
       </c>
     </row>
     <row r="109" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B109">
         <f t="shared" si="2"/>
-        <v>0.12460269883504811</v>
+        <v>0.12270989030127519</v>
       </c>
       <c r="C109">
         <f t="shared" si="3"/>
-        <v>21.5</v>
+        <v>43000</v>
       </c>
     </row>
     <row r="110" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B110">
         <f t="shared" si="2"/>
-        <v>0.12467568239008178</v>
+        <v>0.12430273116113988</v>
       </c>
       <c r="C110">
         <f t="shared" si="3"/>
-        <v>21.75</v>
+        <v>43500</v>
       </c>
     </row>
     <row r="111" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B111">
         <f t="shared" si="2"/>
-        <v>0.12473650563587114</v>
+        <v>0.12583641996413128</v>
       </c>
       <c r="C111">
         <f t="shared" si="3"/>
-        <v>22</v>
+        <v>44000</v>
       </c>
     </row>
     <row r="112" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B112">
         <f t="shared" si="2"/>
-        <v>0.12478694159291652</v>
+        <v>0.12731069290740946</v>
       </c>
       <c r="C112">
         <f t="shared" si="3"/>
-        <v>22.25</v>
+        <v>44500</v>
       </c>
     </row>
     <row r="113" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B113">
         <f t="shared" si="2"/>
-        <v>0.12482855334969299</v>
+        <v>0.12872547613689861</v>
       </c>
       <c r="C113">
         <f t="shared" si="3"/>
-        <v>22.5</v>
+        <v>45000</v>
       </c>
     </row>
     <row r="114" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B114">
         <f t="shared" si="2"/>
-        <v>0.12486271004758752</v>
+        <v>0.1300808801166794</v>
       </c>
       <c r="C114">
         <f t="shared" si="3"/>
-        <v>22.75</v>
+        <v>45500</v>
       </c>
     </row>
     <row r="115" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B115">
         <f t="shared" si="2"/>
-        <v>0.12489060326408261</v>
+        <v>0.13137719306690807</v>
       </c>
       <c r="C115">
         <f t="shared" si="3"/>
-        <v>23</v>
+        <v>46000</v>
       </c>
     </row>
     <row r="116" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B116">
         <f t="shared" si="2"/>
-        <v>0.12491326342455751</v>
+        <v>0.13261487354093182</v>
       </c>
       <c r="C116">
         <f t="shared" si="3"/>
-        <v>23.25</v>
+        <v>46500</v>
       </c>
     </row>
     <row r="117" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B117">
         <f t="shared" si="2"/>
-        <v>0.12493157592833935</v>
+        <v>0.13379454221852241</v>
       </c>
       <c r="C117">
         <f t="shared" si="3"/>
-        <v>23.5</v>
+        <v>47000</v>
       </c>
     </row>
     <row r="118" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B118">
         <f t="shared" si="2"/>
-        <v>0.12494629673008874</v>
+        <v>0.1349169729974935</v>
       </c>
       <c r="C118">
         <f t="shared" si="3"/>
-        <v>23.75</v>
+        <v>47500</v>
       </c>
     </row>
     <row r="119" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B119">
         <f t="shared" si="2"/>
-        <v>0.12495806717151219</v>
+        <v>0.1359830834703562</v>
       </c>
       <c r="C119">
         <f t="shared" si="3"/>
-        <v>24</v>
+        <v>48000</v>
       </c>
     </row>
     <row r="120" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B120">
         <f t="shared" si="2"/>
-        <v>0.12496742790932699</v>
+        <v>0.13699392487605058</v>
       </c>
       <c r="C120">
         <f t="shared" si="3"/>
-        <v>24.25</v>
+        <v>48500</v>
       </c>
     </row>
     <row r="121" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B121">
         <f t="shared" si="2"/>
-        <v>0.1249748318322462</v>
+        <v>0.13795067161915198</v>
       </c>
       <c r="C121">
         <f t="shared" si="3"/>
-        <v>24.5</v>
+        <v>49000</v>
       </c>
     </row>
     <row r="122" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B122">
         <f t="shared" si="2"/>
-        <v>0.12498065590169766</v>
+        <v>0.13885461045027209</v>
       </c>
       <c r="C122">
         <f t="shared" si="3"/>
-        <v>24.75</v>
+        <v>49500</v>
       </c>
     </row>
     <row r="123" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B123">
         <f t="shared" si="2"/>
-        <v>0.12498521188753921</v>
+        <v>0.13970712940166313</v>
       </c>
       <c r="C123">
         <f t="shared" si="3"/>
-        <v>25</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="124" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B124">
         <f t="shared" si="2"/>
-        <v>0.1249887560009456</v>
+        <v>0.14050970657130474</v>
       </c>
       <c r="C124">
         <f t="shared" si="3"/>
-        <v>25.25</v>
+        <v>50500</v>
       </c>
     </row>
   </sheetData>
@@ -5422,331 +5421,331 @@
       </c>
       <c r="C1">
         <f>(1-EXP(-((C2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>1.1302755611730664E-6</v>
+        <v>1.3563306734076795E-6</v>
       </c>
       <c r="D1">
         <f>(1-EXP(-((D2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>9.041918329455445E-6</v>
+        <v>1.0850301995346534E-5</v>
       </c>
       <c r="E1">
         <f>(1-EXP(-((E2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>3.0513853137847935E-5</v>
+        <v>3.6616623765417522E-5</v>
       </c>
       <c r="F1">
         <f>(1-EXP(-((F2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>7.2317035876470759E-5</v>
+        <v>8.6780443051764905E-5</v>
       </c>
       <c r="G1">
         <f>(1-EXP(-((G2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>1.4120526808655831E-4</v>
+        <v>1.6944632170386997E-4</v>
       </c>
       <c r="H1">
         <f>(1-EXP(-((H2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>2.4390236156555944E-4</v>
+        <v>2.926828338786713E-4</v>
       </c>
       <c r="I1">
         <f>(1-EXP(-((I2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>3.8708568873771498E-4</v>
+        <v>4.6450282648525794E-4</v>
       </c>
       <c r="J1">
         <f>(1-EXP(-((J2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>5.7736617667798751E-4</v>
+        <v>6.9283941201358503E-4</v>
       </c>
       <c r="K1">
         <f>(1-EXP(-((K2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>8.2126483012147367E-4</v>
+        <v>9.8551779614576844E-4</v>
       </c>
       <c r="L1">
         <f>(1-EXP(-((L2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>1.1251859013301779E-3</v>
+        <v>1.3502230815962135E-3</v>
       </c>
       <c r="M1">
         <f>(1-EXP(-((M2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>1.4953868620252581E-3</v>
+        <v>1.7944642344303095E-3</v>
       </c>
       <c r="N1">
         <f>(1-EXP(-((N2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>1.9379453743239433E-3</v>
+        <v>2.325534449188732E-3</v>
       </c>
       <c r="O1">
         <f>(1-EXP(-((O2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>2.4587235032284965E-3</v>
+        <v>2.9504682038741957E-3</v>
       </c>
       <c r="P1">
         <f>(1-EXP(-((P2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>3.0633294620639323E-3</v>
+        <v>3.6759953544767184E-3</v>
       </c>
       <c r="Q1">
         <f>(1-EXP(-((Q2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>3.7570772335819985E-3</v>
+        <v>4.5084926802983977E-3</v>
       </c>
       <c r="R1">
         <f>(1-EXP(-((R2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>4.5449444623392177E-3</v>
+        <v>5.4539333548070607E-3</v>
       </c>
       <c r="S1">
         <f>(1-EXP(-((S2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>5.4315290673835337E-3</v>
+        <v>6.5178348808602399E-3</v>
       </c>
       <c r="T1">
         <f>(1-EXP(-((T2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>6.4210050770837218E-3</v>
+        <v>7.7052060925004657E-3</v>
       </c>
       <c r="U1">
         <f>(1-EXP(-((U2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>7.5170782388275237E-3</v>
+        <v>9.0204938865930274E-3</v>
       </c>
       <c r="V1">
         <f>(1-EXP(-((V2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>8.7229420039149769E-3</v>
+        <v>1.0467530404697972E-2</v>
       </c>
       <c r="W1">
         <f>(1-EXP(-((W2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>1.0041234530816401E-2</v>
+        <v>1.2049481436979681E-2</v>
       </c>
       <c r="X1">
         <f>(1-EXP(-((X2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>1.1473997386527171E-2</v>
+        <v>1.3768796863832604E-2</v>
       </c>
       <c r="Y1">
         <f>(1-EXP(-((Y2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>1.3022636654488842E-2</v>
+        <v>1.5627163985386609E-2</v>
       </c>
       <c r="Z1">
         <f>(1-EXP(-((Z2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>1.4687887176925568E-2</v>
+        <v>1.7625464612310682E-2</v>
       </c>
       <c r="AA1">
         <f>(1-EXP(-((AA2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>1.6469780667991457E-2</v>
+        <v>1.9763736801589746E-2</v>
       </c>
       <c r="AB1">
         <f>(1-EXP(-((AB2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>1.8367618430465693E-2</v>
+        <v>2.2041142116558832E-2</v>
       </c>
       <c r="AC1">
         <f>(1-EXP(-((AC2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>2.0379949391649221E-2</v>
+        <v>2.4455939269979066E-2</v>
       </c>
       <c r="AD1">
         <f>(1-EXP(-((AD2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>2.2504554142594765E-2</v>
+        <v>2.7005464971113717E-2</v>
       </c>
       <c r="AE1">
         <f>(1-EXP(-((AE2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>2.4738435618083782E-2</v>
+        <v>2.9686122741700537E-2</v>
       </c>
       <c r="AF1">
         <f>(1-EXP(-((AF2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>2.7077816992397724E-2</v>
+        <v>3.249338039087727E-2</v>
       </c>
       <c r="AG1">
         <f>(1-EXP(-((AG2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>2.951814728782165E-2</v>
+        <v>3.5421776745385977E-2</v>
       </c>
       <c r="AH1">
         <f>(1-EXP(-((AH2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>3.2054115099261718E-2</v>
+        <v>3.8464938119114063E-2</v>
       </c>
       <c r="AI1">
         <f>(1-EXP(-((AI2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>3.467967073008181E-2</v>
+        <v>4.1615604876098174E-2</v>
       </c>
       <c r="AJ1">
         <f>(1-EXP(-((AJ2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>3.7388056912446274E-2</v>
+        <v>4.4865668294935525E-2</v>
       </c>
       <c r="AK1">
         <f>(1-EXP(-((AK2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>4.0171848151733677E-2</v>
+        <v>4.820621778208041E-2</v>
       </c>
       <c r="AL1">
         <f>(1-EXP(-((AL2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>4.3022998591062303E-2</v>
+        <v>5.1627598309274762E-2</v>
       </c>
       <c r="AM1">
         <f>(1-EXP(-((AM2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>4.5932898141179429E-2</v>
+        <v>5.5119477769415316E-2</v>
       </c>
       <c r="AN1">
         <f>(1-EXP(-((AN2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>4.8892436465861083E-2</v>
+        <v>5.8670923759033294E-2</v>
       </c>
       <c r="AO1">
         <f>(1-EXP(-((AO2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>5.1892074256846804E-2</v>
+        <v>6.2270489108216164E-2</v>
       </c>
       <c r="AP1">
         <f>(1-EXP(-((AP2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>5.4921921078778663E-2</v>
+        <v>6.5906305294534395E-2</v>
       </c>
       <c r="AQ1">
         <f>(1-EXP(-((AQ2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>5.7971818917411488E-2</v>
+        <v>6.9566182700893778E-2</v>
       </c>
       <c r="AR1">
         <f>(1-EXP(-((AR2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>6.1031430427395852E-2</v>
+        <v>7.3237716512875015E-2</v>
       </c>
       <c r="AS1">
         <f>(1-EXP(-((AS2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>6.4090330753079128E-2</v>
+        <v>7.6908396903694956E-2</v>
       </c>
       <c r="AT1">
         <f>(1-EXP(-((AT2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>6.7138101690766061E-2</v>
+        <v>8.0565722028919276E-2</v>
       </c>
       <c r="AU1">
         <f>(1-EXP(-((AU2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>7.0164426877205852E-2</v>
+        <v>8.4197312252647025E-2</v>
       </c>
       <c r="AV1">
         <f>(1-EXP(-((AV2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>7.3159186629829842E-2</v>
+        <v>8.7791023955795813E-2</v>
       </c>
       <c r="AW1">
         <f>(1-EXP(-((AW2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>7.6112551032035736E-2</v>
+        <v>9.1335061238442886E-2</v>
       </c>
       <c r="AX1">
         <f>(1-EXP(-((AX2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>7.9015069853569708E-2</v>
+        <v>9.4818083824283653E-2</v>
       </c>
       <c r="AY1">
         <f>(1-EXP(-((AY2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>8.1857757923041286E-2</v>
+        <v>9.8229309507649534E-2</v>
       </c>
       <c r="AZ1">
         <f>(1-EXP(-((AZ2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>8.4632174627258694E-2</v>
+        <v>0.10155860955271043</v>
       </c>
       <c r="BA1">
         <f>(1-EXP(-((BA2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>8.7330496299984461E-2</v>
+        <v>0.10479659555998135</v>
       </c>
       <c r="BB1">
         <f>(1-EXP(-((BB2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>8.9945580379575493E-2</v>
+        <v>0.10793469645549059</v>
       </c>
       <c r="BC1">
         <f>(1-EXP(-((BC2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>9.2471020358609296E-2</v>
+        <v>0.11096522443033115</v>
       </c>
       <c r="BD1">
         <f>(1-EXP(-((BD2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>9.4901190715968961E-2</v>
+        <v>0.11388142885916275</v>
       </c>
       <c r="BE1">
         <f>(1-EXP(-((BE2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>9.7231281209145953E-2</v>
+        <v>0.11667753745097514</v>
       </c>
       <c r="BF1">
         <f>(1-EXP(-((BF2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>9.9457320107219804E-2</v>
+        <v>0.11934878412866376</v>
       </c>
       <c r="BG1">
         <f>(1-EXP(-((BG2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.10157618615802415</v>
+        <v>0.12189142338962897</v>
       </c>
       <c r="BH1">
         <f>(1-EXP(-((BH2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.1035856093009499</v>
+        <v>0.12430273116113988</v>
       </c>
       <c r="BI1">
         <f>(1-EXP(-((BI2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.10548416035397182</v>
+        <v>0.12658099242476617</v>
       </c>
       <c r="BJ1">
         <f>(1-EXP(-((BJ2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.10727123011408218</v>
+        <v>0.12872547613689861</v>
       </c>
       <c r="BK1">
         <f>(1-EXP(-((BK2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.10894699850878881</v>
+        <v>0.13073639821054656</v>
       </c>
       <c r="BL1">
         <f>(1-EXP(-((BL2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.11051239461744319</v>
+        <v>0.13261487354093182</v>
       </c>
       <c r="BM1">
         <f>(1-EXP(-((BM2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.11196904854019522</v>
+        <v>0.13436285824823427</v>
       </c>
       <c r="BN1">
         <f>(1-EXP(-((BN2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.11331923622529684</v>
+        <v>0.1359830834703562</v>
       </c>
       <c r="BO1">
         <f>(1-EXP(-((BO2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.11456581846910648</v>
+        <v>0.13747898216292775</v>
       </c>
       <c r="BP1">
         <f>(1-EXP(-((BP2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.11571217537522674</v>
+        <v>0.13885461045027209</v>
       </c>
       <c r="BQ1">
         <f>(1-EXP(-((BQ2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.11676213759849677</v>
+        <v>0.14011456511819612</v>
       </c>
       <c r="BR1">
         <f>(1-EXP(-((BR2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.11771991570586685</v>
+        <v>0.14126389884704021</v>
       </c>
       <c r="BS1">
         <f>(1-EXP(-((BS2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.11859002896034841</v>
+        <v>0.1423080347524181</v>
       </c>
       <c r="BT1">
         <f>(1-EXP(-((BT2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.11937723477809242</v>
+        <v>0.14325268173371089</v>
       </c>
       <c r="BU1">
         <f>(1-EXP(-((BU2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.12008646002494117</v>
+        <v>0.14410375202992939</v>
       </c>
       <c r="BV1">
         <f>(1-EXP(-((BV2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.12072273521104175</v>
+        <v>0.1448672822532501</v>
       </c>
       <c r="BW1">
         <f>(1-EXP(-((BW2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.12129113251445571</v>
+        <v>0.14554935901734684</v>
       </c>
       <c r="BX1">
         <f>(1-EXP(-((BX2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.12179670842176366</v>
+        <v>0.14615605010611638</v>
       </c>
       <c r="BY1">
         <f>(1-EXP(-((BY2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.12224445162033554</v>
+        <v>0.14669334194440264</v>
       </c>
       <c r="BZ1">
         <f>(1-EXP(-((BZ2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.12263923661819812</v>
+        <v>0.14716708394183772</v>
       </c>
       <c r="CA1">
         <f>(1-EXP(-((CA2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.12298578340816241</v>
+        <v>0.14758294008979489</v>
       </c>
       <c r="CB1">
         <f>(1-EXP(-((CB2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.12328862333768843</v>
+        <v>0.1479463480052261</v>
       </c>
       <c r="CC1">
         <f>(1-EXP(-((CC2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.12355207119904957</v>
+        <v>0.14826248543885948</v>
       </c>
       <c r="CD1">
         <f>(1-EXP(-((CD2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.12378020341934777</v>
+        <v>0.14853624410321731</v>
       </c>
       <c r="CE1">
         <f>(1-EXP(-((CE2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.125</v>
+        <v>0.1487722105317654</v>
       </c>
       <c r="CF1">
         <f>(1-EXP(-((CF2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.125</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="2" spans="1:84" x14ac:dyDescent="0.25">
@@ -5757,330 +5756,331 @@
         <v>0</v>
       </c>
       <c r="C2">
-        <f>B2+0.25</f>
-        <v>0.25</v>
+        <f>B2+750</f>
+        <v>750</v>
       </c>
       <c r="D2">
-        <f t="shared" ref="D2:AI2" si="0">C2+0.25</f>
-        <v>0.5</v>
+        <f t="shared" ref="D2:BO2" si="0">C2+750</f>
+        <v>1500</v>
       </c>
       <c r="E2">
         <f t="shared" si="0"/>
-        <v>0.75</v>
+        <v>2250</v>
       </c>
       <c r="F2">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>3000</v>
       </c>
       <c r="G2">
         <f t="shared" si="0"/>
-        <v>1.25</v>
+        <v>3750</v>
       </c>
       <c r="H2">
         <f t="shared" si="0"/>
-        <v>1.5</v>
+        <v>4500</v>
       </c>
       <c r="I2">
         <f t="shared" si="0"/>
-        <v>1.75</v>
+        <v>5250</v>
       </c>
       <c r="J2">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>6000</v>
       </c>
       <c r="K2">
         <f t="shared" si="0"/>
-        <v>2.25</v>
+        <v>6750</v>
       </c>
       <c r="L2">
         <f t="shared" si="0"/>
-        <v>2.5</v>
+        <v>7500</v>
       </c>
       <c r="M2">
         <f t="shared" si="0"/>
-        <v>2.75</v>
+        <v>8250</v>
       </c>
       <c r="N2">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>9000</v>
       </c>
       <c r="O2">
         <f t="shared" si="0"/>
-        <v>3.25</v>
+        <v>9750</v>
       </c>
       <c r="P2">
         <f t="shared" si="0"/>
-        <v>3.5</v>
+        <v>10500</v>
       </c>
       <c r="Q2">
         <f t="shared" si="0"/>
-        <v>3.75</v>
+        <v>11250</v>
       </c>
       <c r="R2">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>12000</v>
       </c>
       <c r="S2">
         <f t="shared" si="0"/>
-        <v>4.25</v>
+        <v>12750</v>
       </c>
       <c r="T2">
         <f t="shared" si="0"/>
-        <v>4.5</v>
+        <v>13500</v>
       </c>
       <c r="U2">
         <f t="shared" si="0"/>
-        <v>4.75</v>
+        <v>14250</v>
       </c>
       <c r="V2">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>15000</v>
       </c>
       <c r="W2">
         <f t="shared" si="0"/>
-        <v>5.25</v>
+        <v>15750</v>
       </c>
       <c r="X2">
         <f t="shared" si="0"/>
-        <v>5.5</v>
+        <v>16500</v>
       </c>
       <c r="Y2">
         <f t="shared" si="0"/>
-        <v>5.75</v>
+        <v>17250</v>
       </c>
       <c r="Z2">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>18000</v>
       </c>
       <c r="AA2">
         <f t="shared" si="0"/>
-        <v>6.25</v>
+        <v>18750</v>
       </c>
       <c r="AB2">
         <f t="shared" si="0"/>
-        <v>6.5</v>
+        <v>19500</v>
       </c>
       <c r="AC2">
         <f t="shared" si="0"/>
-        <v>6.75</v>
+        <v>20250</v>
       </c>
       <c r="AD2">
         <f t="shared" si="0"/>
-        <v>7</v>
+        <v>21000</v>
       </c>
       <c r="AE2">
         <f t="shared" si="0"/>
-        <v>7.25</v>
+        <v>21750</v>
       </c>
       <c r="AF2">
         <f t="shared" si="0"/>
-        <v>7.5</v>
+        <v>22500</v>
       </c>
       <c r="AG2">
         <f t="shared" si="0"/>
-        <v>7.75</v>
+        <v>23250</v>
       </c>
       <c r="AH2">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>24000</v>
       </c>
       <c r="AI2">
         <f t="shared" si="0"/>
-        <v>8.25</v>
+        <v>24750</v>
       </c>
       <c r="AJ2">
-        <f>AI2+0.25</f>
-        <v>8.5</v>
+        <f t="shared" si="0"/>
+        <v>25500</v>
       </c>
       <c r="AK2">
-        <f t="shared" ref="AK2:AO2" si="1">AJ2+0.25</f>
-        <v>8.75</v>
+        <f t="shared" si="0"/>
+        <v>26250</v>
       </c>
       <c r="AL2">
+        <f t="shared" si="0"/>
+        <v>27000</v>
+      </c>
+      <c r="AM2">
+        <f t="shared" si="0"/>
+        <v>27750</v>
+      </c>
+      <c r="AN2">
+        <f t="shared" si="0"/>
+        <v>28500</v>
+      </c>
+      <c r="AO2">
+        <f t="shared" si="0"/>
+        <v>29250</v>
+      </c>
+      <c r="AP2">
+        <f t="shared" si="0"/>
+        <v>30000</v>
+      </c>
+      <c r="AQ2">
+        <f t="shared" si="0"/>
+        <v>30750</v>
+      </c>
+      <c r="AR2">
+        <f t="shared" si="0"/>
+        <v>31500</v>
+      </c>
+      <c r="AS2">
+        <f t="shared" si="0"/>
+        <v>32250</v>
+      </c>
+      <c r="AT2">
+        <f t="shared" si="0"/>
+        <v>33000</v>
+      </c>
+      <c r="AU2">
+        <f t="shared" si="0"/>
+        <v>33750</v>
+      </c>
+      <c r="AV2">
+        <f t="shared" si="0"/>
+        <v>34500</v>
+      </c>
+      <c r="AW2">
+        <f t="shared" si="0"/>
+        <v>35250</v>
+      </c>
+      <c r="AX2">
+        <f t="shared" si="0"/>
+        <v>36000</v>
+      </c>
+      <c r="AY2">
+        <f t="shared" si="0"/>
+        <v>36750</v>
+      </c>
+      <c r="AZ2">
+        <f t="shared" si="0"/>
+        <v>37500</v>
+      </c>
+      <c r="BA2">
+        <f t="shared" si="0"/>
+        <v>38250</v>
+      </c>
+      <c r="BB2">
+        <f t="shared" si="0"/>
+        <v>39000</v>
+      </c>
+      <c r="BC2">
+        <f t="shared" si="0"/>
+        <v>39750</v>
+      </c>
+      <c r="BD2">
+        <f t="shared" si="0"/>
+        <v>40500</v>
+      </c>
+      <c r="BE2">
+        <f t="shared" si="0"/>
+        <v>41250</v>
+      </c>
+      <c r="BF2">
+        <f t="shared" si="0"/>
+        <v>42000</v>
+      </c>
+      <c r="BG2">
+        <f t="shared" si="0"/>
+        <v>42750</v>
+      </c>
+      <c r="BH2">
+        <f t="shared" si="0"/>
+        <v>43500</v>
+      </c>
+      <c r="BI2">
+        <f t="shared" si="0"/>
+        <v>44250</v>
+      </c>
+      <c r="BJ2">
+        <f t="shared" si="0"/>
+        <v>45000</v>
+      </c>
+      <c r="BK2">
+        <f t="shared" si="0"/>
+        <v>45750</v>
+      </c>
+      <c r="BL2">
+        <f t="shared" si="0"/>
+        <v>46500</v>
+      </c>
+      <c r="BM2">
+        <f t="shared" si="0"/>
+        <v>47250</v>
+      </c>
+      <c r="BN2">
+        <f t="shared" si="0"/>
+        <v>48000</v>
+      </c>
+      <c r="BO2">
+        <f t="shared" si="0"/>
+        <v>48750</v>
+      </c>
+      <c r="BP2">
+        <f t="shared" ref="BP2:CE2" si="1">BO2+750</f>
+        <v>49500</v>
+      </c>
+      <c r="BQ2">
         <f t="shared" si="1"/>
-        <v>9</v>
-      </c>
-      <c r="AM2">
+        <v>50250</v>
+      </c>
+      <c r="BR2">
         <f t="shared" si="1"/>
-        <v>9.25</v>
-      </c>
-      <c r="AN2">
+        <v>51000</v>
+      </c>
+      <c r="BS2">
         <f t="shared" si="1"/>
-        <v>9.5</v>
-      </c>
-      <c r="AO2">
+        <v>51750</v>
+      </c>
+      <c r="BT2">
         <f t="shared" si="1"/>
-        <v>9.75</v>
-      </c>
-      <c r="AP2">
-        <f>AO2+0.25</f>
-        <v>10</v>
-      </c>
-      <c r="AQ2">
-        <f t="shared" ref="AQ2:BJ2" si="2">AP2+0.25</f>
-        <v>10.25</v>
-      </c>
-      <c r="AR2">
-        <f t="shared" si="2"/>
-        <v>10.5</v>
-      </c>
-      <c r="AS2">
-        <f t="shared" si="2"/>
-        <v>10.75</v>
-      </c>
-      <c r="AT2">
-        <f t="shared" si="2"/>
-        <v>11</v>
-      </c>
-      <c r="AU2">
-        <f t="shared" si="2"/>
-        <v>11.25</v>
-      </c>
-      <c r="AV2">
-        <f t="shared" si="2"/>
-        <v>11.5</v>
-      </c>
-      <c r="AW2">
-        <f t="shared" si="2"/>
-        <v>11.75</v>
-      </c>
-      <c r="AX2">
-        <f t="shared" si="2"/>
-        <v>12</v>
-      </c>
-      <c r="AY2">
-        <f t="shared" si="2"/>
-        <v>12.25</v>
-      </c>
-      <c r="AZ2">
-        <f t="shared" si="2"/>
-        <v>12.5</v>
-      </c>
-      <c r="BA2">
-        <f t="shared" si="2"/>
-        <v>12.75</v>
-      </c>
-      <c r="BB2">
-        <f t="shared" si="2"/>
-        <v>13</v>
-      </c>
-      <c r="BC2">
-        <f t="shared" si="2"/>
-        <v>13.25</v>
-      </c>
-      <c r="BD2">
-        <f t="shared" si="2"/>
-        <v>13.5</v>
-      </c>
-      <c r="BE2">
-        <f t="shared" si="2"/>
-        <v>13.75</v>
-      </c>
-      <c r="BF2">
-        <f t="shared" si="2"/>
-        <v>14</v>
-      </c>
-      <c r="BG2">
-        <f t="shared" si="2"/>
-        <v>14.25</v>
-      </c>
-      <c r="BH2">
-        <f t="shared" si="2"/>
-        <v>14.5</v>
-      </c>
-      <c r="BI2">
-        <f t="shared" si="2"/>
-        <v>14.75</v>
-      </c>
-      <c r="BJ2">
-        <f t="shared" si="2"/>
-        <v>15</v>
-      </c>
-      <c r="BK2">
-        <f t="shared" ref="BK2" si="3">BJ2+0.25</f>
-        <v>15.25</v>
-      </c>
-      <c r="BL2">
-        <f t="shared" ref="BL2" si="4">BK2+0.25</f>
-        <v>15.5</v>
-      </c>
-      <c r="BM2">
-        <f t="shared" ref="BM2" si="5">BL2+0.25</f>
-        <v>15.75</v>
-      </c>
-      <c r="BN2">
-        <f t="shared" ref="BN2" si="6">BM2+0.25</f>
-        <v>16</v>
-      </c>
-      <c r="BO2">
-        <f t="shared" ref="BO2" si="7">BN2+0.25</f>
-        <v>16.25</v>
-      </c>
-      <c r="BP2">
-        <f t="shared" ref="BP2" si="8">BO2+0.25</f>
-        <v>16.5</v>
-      </c>
-      <c r="BQ2">
-        <f t="shared" ref="BQ2" si="9">BP2+0.25</f>
-        <v>16.75</v>
-      </c>
-      <c r="BR2">
-        <f t="shared" ref="BR2" si="10">BQ2+0.25</f>
-        <v>17</v>
-      </c>
-      <c r="BS2">
-        <f t="shared" ref="BS2" si="11">BR2+0.25</f>
-        <v>17.25</v>
-      </c>
-      <c r="BT2">
-        <f t="shared" ref="BT2" si="12">BS2+0.25</f>
-        <v>17.5</v>
+        <v>52500</v>
       </c>
       <c r="BU2">
-        <f t="shared" ref="BU2" si="13">BT2+0.25</f>
-        <v>17.75</v>
+        <f t="shared" si="1"/>
+        <v>53250</v>
       </c>
       <c r="BV2">
-        <f t="shared" ref="BV2" si="14">BU2+0.25</f>
-        <v>18</v>
+        <f t="shared" si="1"/>
+        <v>54000</v>
       </c>
       <c r="BW2">
-        <f t="shared" ref="BW2" si="15">BV2+0.25</f>
-        <v>18.25</v>
+        <f t="shared" si="1"/>
+        <v>54750</v>
       </c>
       <c r="BX2">
-        <f t="shared" ref="BX2" si="16">BW2+0.25</f>
-        <v>18.5</v>
+        <f t="shared" si="1"/>
+        <v>55500</v>
       </c>
       <c r="BY2">
-        <f t="shared" ref="BY2" si="17">BX2+0.25</f>
-        <v>18.75</v>
+        <f t="shared" si="1"/>
+        <v>56250</v>
       </c>
       <c r="BZ2">
-        <f t="shared" ref="BZ2" si="18">BY2+0.25</f>
-        <v>19</v>
+        <f t="shared" si="1"/>
+        <v>57000</v>
       </c>
       <c r="CA2">
-        <f t="shared" ref="CA2" si="19">BZ2+0.25</f>
-        <v>19.25</v>
+        <f t="shared" si="1"/>
+        <v>57750</v>
       </c>
       <c r="CB2">
-        <f t="shared" ref="CB2" si="20">CA2+0.25</f>
-        <v>19.5</v>
+        <f t="shared" si="1"/>
+        <v>58500</v>
       </c>
       <c r="CC2">
-        <f t="shared" ref="CC2" si="21">CB2+0.25</f>
-        <v>19.75</v>
+        <f t="shared" si="1"/>
+        <v>59250</v>
       </c>
       <c r="CD2">
-        <f t="shared" ref="CD2" si="22">CC2+0.25</f>
-        <v>20</v>
+        <f t="shared" si="1"/>
+        <v>60000</v>
       </c>
       <c r="CE2">
-        <v>1000</v>
-      </c>
-      <c r="CF2">
-        <v>10000</v>
+        <f t="shared" si="1"/>
+        <v>60750</v>
+      </c>
+      <c r="CF2" s="2">
+        <v>1000000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Interim electricity calibration edits
</commit_message>
<xml_diff>
--- a/InputData/elec/CSC/Capacity Supply Curve.xlsx
+++ b/InputData/elec/CSC/Capacity Supply Curve.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\US\Models\eps-us\InputData\elec\CSC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\elec\CSC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D47818FD-27FB-4FD4-968C-58E44B45BDB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C208883-69A2-4C97-8CB4-4A540A7A8C47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3720" yWindow="3720" windowWidth="43200" windowHeight="17085" xr2:uid="{F87DB1D1-DC21-4EA7-B1DF-998EE56837F8}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{F87DB1D1-DC21-4EA7-B1DF-998EE56837F8}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -619,307 +619,307 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="101"/>
                 <c:pt idx="0">
-                  <c:v>4.0187703366778572E-7</c:v>
+                  <c:v>3.3489752805648809E-7</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3.2149861218577768E-6</c:v>
+                  <c:v>2.6791551015481474E-6</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.0850301995346534E-5</c:v>
+                  <c:v>9.041918329455445E-6</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2.571795964551593E-5</c:v>
+                  <c:v>2.1431633037929942E-5</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>5.0226285691895579E-5</c:v>
+                  <c:v>4.1855238076579648E-5</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>8.6780443051764905E-5</c:v>
+                  <c:v>7.2317035876470759E-5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1.3778069003070326E-4</c:v>
+                  <c:v>1.1481724169225271E-4</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>2.0562025564793696E-4</c:v>
+                  <c:v>1.7135021303994746E-4</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>2.926828338786713E-4</c:v>
+                  <c:v>2.4390236156555944E-4</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>4.0133970053291554E-4</c:v>
+                  <c:v>3.3444975044409631E-4</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>5.3394645769462839E-4</c:v>
+                  <c:v>4.4495538141219038E-4</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>6.9283941201358503E-4</c:v>
+                  <c:v>5.7736617667798751E-4</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>8.8033159466762703E-4</c:v>
+                  <c:v>7.336096622230226E-4</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>1.0987084324921848E-3</c:v>
+                  <c:v>9.1559036041015396E-4</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>1.3502230815962135E-3</c:v>
+                  <c:v>1.1251859013301779E-3</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>1.6370914367420941E-3</c:v>
+                  <c:v>1.3642428639517451E-3</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>1.9614868318508726E-3</c:v>
+                  <c:v>1.6345723598757272E-3</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>2.325534449188732E-3</c:v>
+                  <c:v>1.9379453743239433E-3</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>2.7313054570853477E-3</c:v>
+                  <c:v>2.2760878809044566E-3</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>3.1808108984106021E-3</c:v>
+                  <c:v>2.6506757486755017E-3</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>3.6759953544767184E-3</c:v>
+                  <c:v>3.0633294620639323E-3</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>4.2187304115184395E-3</c:v>
+                  <c:v>3.5156086762653666E-3</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>4.8108079594126937E-3</c:v>
+                  <c:v>4.0090066328439117E-3</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>5.4539333548070607E-3</c:v>
+                  <c:v>4.5449444623392177E-3</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>6.149718483310862E-3</c:v>
+                  <c:v>5.1247654027590517E-3</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>6.899674757832674E-3</c:v>
+                  <c:v>5.7497289648605621E-3</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>7.7052060925004657E-3</c:v>
+                  <c:v>6.4210050770837218E-3</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>8.5676018938412868E-3</c:v>
+                  <c:v>7.139668244867739E-3</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>9.4880301129990352E-3</c:v>
+                  <c:v>7.9066917608325293E-3</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>1.0467530404697972E-2</c:v>
+                  <c:v>8.7229420039149769E-3</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>1.1507007440385136E-2</c:v>
+                  <c:v>9.5891728669876136E-3</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>1.2607224424474078E-2</c:v>
+                  <c:v>1.0506020353728399E-2</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>1.3768796863832604E-2</c:v>
+                  <c:v>1.1473997386527171E-2</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>1.4992186641577837E-2</c:v>
+                  <c:v>1.2493488867981531E-2</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>1.6277696446830824E-2</c:v>
+                  <c:v>1.3564747039025687E-2</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>1.7625464612310682E-2</c:v>
+                  <c:v>1.4687887176925568E-2</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>1.9035460411488268E-2</c:v>
+                  <c:v>1.5862883676240225E-2</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>2.0507479866443433E-2</c:v>
+                  <c:v>1.7089566555369529E-2</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>2.2041142116558832E-2</c:v>
+                  <c:v>1.8367618430465693E-2</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>2.3635886396712456E-2</c:v>
+                  <c:v>1.9696571997260381E-2</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>2.5290969671690554E-2</c:v>
+                  <c:v>2.1075808059742129E-2</c:v>
                 </c:pt>
                 <c:pt idx="41">
-                  <c:v>2.7005464971113717E-2</c:v>
+                  <c:v>2.2504554142594765E-2</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>2.8778260466251364E-2</c:v>
+                  <c:v>2.3981883721876138E-2</c:v>
                 </c:pt>
                 <c:pt idx="43">
-                  <c:v>3.0608059326685061E-2</c:v>
+                  <c:v>2.5506716105570884E-2</c:v>
                 </c:pt>
                 <c:pt idx="44">
-                  <c:v>3.249338039087727E-2</c:v>
+                  <c:v>2.7077816992397724E-2</c:v>
                 </c:pt>
                 <c:pt idx="45">
-                  <c:v>3.4432559680315195E-2</c:v>
+                  <c:v>2.8693799733595995E-2</c:v>
                 </c:pt>
                 <c:pt idx="46">
-                  <c:v>3.6423752782045189E-2</c:v>
+                  <c:v>3.035312731837099E-2</c:v>
                 </c:pt>
                 <c:pt idx="47">
-                  <c:v>3.8464938119114063E-2</c:v>
+                  <c:v>3.2054115099261718E-2</c:v>
                 </c:pt>
                 <c:pt idx="48">
-                  <c:v>4.055392112271447E-2</c:v>
+                  <c:v>3.3794934268928725E-2</c:v>
                 </c:pt>
                 <c:pt idx="49">
-                  <c:v>4.2688339313730859E-2</c:v>
+                  <c:v>3.5573616094775717E-2</c:v>
                 </c:pt>
                 <c:pt idx="50">
-                  <c:v>4.4865668294935525E-2</c:v>
+                  <c:v>3.7388056912446274E-2</c:v>
                 </c:pt>
                 <c:pt idx="51">
-                  <c:v>4.7083228648343023E-2</c:v>
+                  <c:v>3.9236023873619186E-2</c:v>
                 </c:pt>
                 <c:pt idx="52">
-                  <c:v>4.9338193725244575E-2</c:v>
+                  <c:v>4.1115161437703815E-2</c:v>
                 </c:pt>
                 <c:pt idx="53">
-                  <c:v>5.1627598309274762E-2</c:v>
+                  <c:v>4.3022998591062303E-2</c:v>
                 </c:pt>
                 <c:pt idx="54">
-                  <c:v>5.3948348125570124E-2</c:v>
+                  <c:v>4.495695677130844E-2</c:v>
                 </c:pt>
                 <c:pt idx="55">
-                  <c:v>5.629723016173821E-2</c:v>
+                  <c:v>4.6914358468115175E-2</c:v>
                 </c:pt>
                 <c:pt idx="56">
-                  <c:v>5.8670923759033294E-2</c:v>
+                  <c:v>4.8892436465861083E-2</c:v>
                 </c:pt>
                 <c:pt idx="57">
-                  <c:v>6.1066012424913607E-2</c:v>
+                  <c:v>5.0888343687428006E-2</c:v>
                 </c:pt>
                 <c:pt idx="58">
-                  <c:v>6.3478996311107899E-2</c:v>
+                  <c:v>5.2899163592589921E-2</c:v>
                 </c:pt>
                 <c:pt idx="59">
-                  <c:v>6.5906305294534395E-2</c:v>
+                  <c:v>5.4921921078778663E-2</c:v>
                 </c:pt>
                 <c:pt idx="60">
-                  <c:v>6.8344312591966452E-2</c:v>
+                  <c:v>5.6953593826638713E-2</c:v>
                 </c:pt>
                 <c:pt idx="61">
-                  <c:v>7.0789348833315488E-2</c:v>
+                  <c:v>5.8991124027762909E-2</c:v>
                 </c:pt>
                 <c:pt idx="62">
-                  <c:v>7.3237716512875015E-2</c:v>
+                  <c:v>6.1031430427395852E-2</c:v>
                 </c:pt>
                 <c:pt idx="63">
-                  <c:v>7.5685704732924589E-2</c:v>
+                  <c:v>6.3071420610770493E-2</c:v>
                 </c:pt>
                 <c:pt idx="64">
-                  <c:v>7.8129604149794987E-2</c:v>
+                  <c:v>6.5108003458162492E-2</c:v>
                 </c:pt>
                 <c:pt idx="65">
-                  <c:v>8.0565722028919276E-2</c:v>
+                  <c:v>6.7138101690766061E-2</c:v>
                 </c:pt>
                 <c:pt idx="66">
-                  <c:v>8.2990397312597802E-2</c:v>
+                  <c:v>6.915866442716484E-2</c:v>
                 </c:pt>
                 <c:pt idx="67">
-                  <c:v>8.5400015602243903E-2</c:v>
+                  <c:v>7.1166679668536584E-2</c:v>
                 </c:pt>
                 <c:pt idx="68">
-                  <c:v>8.7791023955795813E-2</c:v>
+                  <c:v>7.3159186629829842E-2</c:v>
                 </c:pt>
                 <c:pt idx="69">
-                  <c:v>9.015994540081855E-2</c:v>
+                  <c:v>7.5133287834015461E-2</c:v>
                 </c:pt>
                 <c:pt idx="70">
-                  <c:v>9.2503393064599676E-2</c:v>
+                  <c:v>7.7086160887166397E-2</c:v>
                 </c:pt>
                 <c:pt idx="71">
-                  <c:v>9.4818083824283653E-2</c:v>
+                  <c:v>7.9015069853569708E-2</c:v>
                 </c:pt>
                 <c:pt idx="72">
-                  <c:v>9.7100851382792161E-2</c:v>
+                  <c:v>8.0917376152326803E-2</c:v>
                 </c:pt>
                 <c:pt idx="73">
-                  <c:v>9.9348658679935559E-2</c:v>
+                  <c:v>8.2790548899946304E-2</c:v>
                 </c:pt>
                 <c:pt idx="74">
-                  <c:v>0.10155860955271043</c:v>
+                  <c:v>8.4632174627258694E-2</c:v>
                 </c:pt>
                 <c:pt idx="75">
-                  <c:v>0.10372795956427108</c:v>
+                  <c:v>8.643996630355924E-2</c:v>
                 </c:pt>
                 <c:pt idx="76">
-                  <c:v>0.10585412592740542</c:v>
+                  <c:v>8.8211771606171191E-2</c:v>
                 </c:pt>
                 <c:pt idx="77">
-                  <c:v>0.10793469645549059</c:v>
+                  <c:v>8.9945580379575493E-2</c:v>
                 </c:pt>
                 <c:pt idx="78">
-                  <c:v>0.10996743748177233</c:v>
+                  <c:v>9.1639531234810279E-2</c:v>
                 </c:pt>
                 <c:pt idx="79">
-                  <c:v>0.11195030069632968</c:v>
+                  <c:v>9.32919172469414E-2</c:v>
                 </c:pt>
                 <c:pt idx="80">
-                  <c:v>0.11388142885916275</c:v>
+                  <c:v>9.4901190715968961E-2</c:v>
                 </c:pt>
                 <c:pt idx="81">
-                  <c:v>0.11575916035737591</c:v>
+                  <c:v>9.6465966964479927E-2</c:v>
                 </c:pt>
                 <c:pt idx="82">
-                  <c:v>0.11758203258431722</c:v>
+                  <c:v>9.7985027153597692E-2</c:v>
                 </c:pt>
                 <c:pt idx="83">
-                  <c:v>0.11934878412866376</c:v>
+                  <c:v>9.9457320107219804E-2</c:v>
                 </c:pt>
                 <c:pt idx="84">
-                  <c:v>0.12105835577169748</c:v>
+                  <c:v>0.10088196314308123</c:v>
                 </c:pt>
                 <c:pt idx="85">
-                  <c:v>0.12270989030127519</c:v>
+                  <c:v>0.10225824191772932</c:v>
                 </c:pt>
                 <c:pt idx="86">
-                  <c:v>0.12430273116113988</c:v>
+                  <c:v>0.1035856093009499</c:v>
                 </c:pt>
                 <c:pt idx="87">
-                  <c:v>0.12583641996413128</c:v>
+                  <c:v>0.10486368330344273</c:v>
                 </c:pt>
                 <c:pt idx="88">
-                  <c:v>0.12731069290740946</c:v>
+                  <c:v>0.10609224408950788</c:v>
                 </c:pt>
                 <c:pt idx="89">
-                  <c:v>0.12872547613689861</c:v>
+                  <c:v>0.10727123011408218</c:v>
                 </c:pt>
                 <c:pt idx="90">
-                  <c:v>0.1300808801166794</c:v>
+                  <c:v>0.10840073343056618</c:v>
                 </c:pt>
                 <c:pt idx="91">
-                  <c:v>0.13137719306690807</c:v>
+                  <c:v>0.10948099422242338</c:v>
                 </c:pt>
                 <c:pt idx="92">
-                  <c:v>0.13261487354093182</c:v>
+                  <c:v>0.11051239461744319</c:v>
                 </c:pt>
                 <c:pt idx="93">
-                  <c:v>0.13379454221852241</c:v>
+                  <c:v>0.11149545184876868</c:v>
                 </c:pt>
                 <c:pt idx="94">
-                  <c:v>0.1349169729974935</c:v>
+                  <c:v>0.11243081083124459</c:v>
                 </c:pt>
                 <c:pt idx="95">
-                  <c:v>0.1359830834703562</c:v>
+                  <c:v>0.11331923622529684</c:v>
                 </c:pt>
                 <c:pt idx="96">
-                  <c:v>0.13699392487605058</c:v>
+                  <c:v>0.11416160406337549</c:v>
                 </c:pt>
                 <c:pt idx="97">
-                  <c:v>0.13795067161915198</c:v>
+                  <c:v>0.11495889301595999</c:v>
                 </c:pt>
                 <c:pt idx="98">
-                  <c:v>0.13885461045027209</c:v>
+                  <c:v>0.11571217537522674</c:v>
                 </c:pt>
                 <c:pt idx="99">
-                  <c:v>0.13970712940166313</c:v>
+                  <c:v>0.11642260783471928</c:v>
                 </c:pt>
                 <c:pt idx="100">
-                  <c:v>0.14050970657130474</c:v>
+                  <c:v>0.11709142214275396</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1076,6 +1076,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1083,7 +1084,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1337,124 +1337,124 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.3563306734076795E-6</c:v>
+                  <c:v>1.1302755611730664E-6</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.0850301995346534E-5</c:v>
+                  <c:v>9.041918329455445E-6</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>3.6616623765417522E-5</c:v>
+                  <c:v>3.0513853137847935E-5</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>8.6780443051764905E-5</c:v>
+                  <c:v>7.2317035876470759E-5</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.6944632170386997E-4</c:v>
+                  <c:v>1.4120526808655831E-4</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>2.926828338786713E-4</c:v>
+                  <c:v>2.4390236156555944E-4</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>4.6450282648525794E-4</c:v>
+                  <c:v>3.8708568873771498E-4</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>6.9283941201358503E-4</c:v>
+                  <c:v>5.7736617667798751E-4</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>9.8551779614576844E-4</c:v>
+                  <c:v>8.2126483012147367E-4</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1.3502230815962135E-3</c:v>
+                  <c:v>1.1251859013301779E-3</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>1.7944642344303095E-3</c:v>
+                  <c:v>1.4953868620252581E-3</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>2.325534449188732E-3</c:v>
+                  <c:v>1.9379453743239433E-3</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>2.9504682038741957E-3</c:v>
+                  <c:v>2.4587235032284965E-3</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>3.6759953544767184E-3</c:v>
+                  <c:v>3.0633294620639323E-3</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>4.5084926802983977E-3</c:v>
+                  <c:v>3.7570772335819985E-3</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>5.4539333548070607E-3</c:v>
+                  <c:v>4.5449444623392177E-3</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>6.5178348808602399E-3</c:v>
+                  <c:v>5.4315290673835337E-3</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>7.7052060925004657E-3</c:v>
+                  <c:v>6.4210050770837218E-3</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>9.0204938865930274E-3</c:v>
+                  <c:v>7.5170782388275237E-3</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>1.0467530404697972E-2</c:v>
+                  <c:v>8.7229420039149769E-3</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>1.2049481436979681E-2</c:v>
+                  <c:v>1.0041234530816401E-2</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>1.3768796863832604E-2</c:v>
+                  <c:v>1.1473997386527171E-2</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>1.5627163985386609E-2</c:v>
+                  <c:v>1.3022636654488842E-2</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>1.7625464612310682E-2</c:v>
+                  <c:v>1.4687887176925568E-2</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>1.9763736801589746E-2</c:v>
+                  <c:v>1.6469780667991457E-2</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>2.2041142116558832E-2</c:v>
+                  <c:v>1.8367618430465693E-2</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>2.4455939269979066E-2</c:v>
+                  <c:v>2.0379949391649221E-2</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>2.7005464971113717E-2</c:v>
+                  <c:v>2.2504554142594765E-2</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>2.9686122741700537E-2</c:v>
+                  <c:v>2.4738435618083782E-2</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>3.249338039087727E-2</c:v>
+                  <c:v>2.7077816992397724E-2</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>3.5421776745385977E-2</c:v>
+                  <c:v>2.951814728782165E-2</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>3.8464938119114063E-2</c:v>
+                  <c:v>3.2054115099261718E-2</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>4.1615604876098174E-2</c:v>
+                  <c:v>3.467967073008181E-2</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>4.4865668294935525E-2</c:v>
+                  <c:v>3.7388056912446274E-2</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>4.820621778208041E-2</c:v>
+                  <c:v>4.0171848151733677E-2</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>5.1627598309274762E-2</c:v>
+                  <c:v>4.3022998591062303E-2</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>5.5119477769415316E-2</c:v>
+                  <c:v>4.5932898141179429E-2</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>5.8670923759033294E-2</c:v>
+                  <c:v>4.8892436465861083E-2</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>6.2270489108216164E-2</c:v>
+                  <c:v>5.1892074256846804E-2</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>6.5906305294534395E-2</c:v>
+                  <c:v>5.4921921078778663E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1611,6 +1611,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1618,7 +1619,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1872,124 +1872,124 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.3563306734076795E-6</c:v>
+                  <c:v>1.1302755611730664E-6</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.0850301995346534E-5</c:v>
+                  <c:v>9.041918329455445E-6</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>3.6616623765417522E-5</c:v>
+                  <c:v>3.0513853137847935E-5</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>8.6780443051764905E-5</c:v>
+                  <c:v>7.2317035876470759E-5</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.6944632170386997E-4</c:v>
+                  <c:v>1.4120526808655831E-4</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>2.926828338786713E-4</c:v>
+                  <c:v>2.4390236156555944E-4</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>4.6450282648525794E-4</c:v>
+                  <c:v>3.8708568873771498E-4</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>6.9283941201358503E-4</c:v>
+                  <c:v>5.7736617667798751E-4</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>9.8551779614576844E-4</c:v>
+                  <c:v>8.2126483012147367E-4</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1.3502230815962135E-3</c:v>
+                  <c:v>1.1251859013301779E-3</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>1.7944642344303095E-3</c:v>
+                  <c:v>1.4953868620252581E-3</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>2.325534449188732E-3</c:v>
+                  <c:v>1.9379453743239433E-3</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>2.9504682038741957E-3</c:v>
+                  <c:v>2.4587235032284965E-3</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>3.6759953544767184E-3</c:v>
+                  <c:v>3.0633294620639323E-3</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>4.5084926802983977E-3</c:v>
+                  <c:v>3.7570772335819985E-3</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>5.4539333548070607E-3</c:v>
+                  <c:v>4.5449444623392177E-3</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>6.5178348808602399E-3</c:v>
+                  <c:v>5.4315290673835337E-3</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>7.7052060925004657E-3</c:v>
+                  <c:v>6.4210050770837218E-3</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>9.0204938865930274E-3</c:v>
+                  <c:v>7.5170782388275237E-3</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>1.0467530404697972E-2</c:v>
+                  <c:v>8.7229420039149769E-3</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>1.2049481436979681E-2</c:v>
+                  <c:v>1.0041234530816401E-2</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>1.3768796863832604E-2</c:v>
+                  <c:v>1.1473997386527171E-2</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>1.5627163985386609E-2</c:v>
+                  <c:v>1.3022636654488842E-2</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>1.7625464612310682E-2</c:v>
+                  <c:v>1.4687887176925568E-2</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>1.9763736801589746E-2</c:v>
+                  <c:v>1.6469780667991457E-2</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>2.2041142116558832E-2</c:v>
+                  <c:v>1.8367618430465693E-2</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>2.4455939269979066E-2</c:v>
+                  <c:v>2.0379949391649221E-2</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>2.7005464971113717E-2</c:v>
+                  <c:v>2.2504554142594765E-2</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>2.9686122741700537E-2</c:v>
+                  <c:v>2.4738435618083782E-2</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>3.249338039087727E-2</c:v>
+                  <c:v>2.7077816992397724E-2</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>3.5421776745385977E-2</c:v>
+                  <c:v>2.951814728782165E-2</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>3.8464938119114063E-2</c:v>
+                  <c:v>3.2054115099261718E-2</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>4.1615604876098174E-2</c:v>
+                  <c:v>3.467967073008181E-2</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>4.4865668294935525E-2</c:v>
+                  <c:v>3.7388056912446274E-2</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>4.820621778208041E-2</c:v>
+                  <c:v>4.0171848151733677E-2</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>5.1627598309274762E-2</c:v>
+                  <c:v>4.3022998591062303E-2</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>5.5119477769415316E-2</c:v>
+                  <c:v>4.5932898141179429E-2</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>5.8670923759033294E-2</c:v>
+                  <c:v>4.8892436465861083E-2</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>6.2270489108216164E-2</c:v>
+                  <c:v>5.1892074256846804E-2</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>6.5906305294534395E-2</c:v>
+                  <c:v>5.4921921078778663E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2146,6 +2146,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -2153,7 +2154,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -4274,28 +4274,28 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D3D2DEE-686E-48A0-AC3D-0F54DEA5D0EC}">
   <dimension ref="A1:C124"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="88.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="88.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
@@ -4303,48 +4303,48 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" s="1"/>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>37</v>
       </c>
       <c r="B15">
-        <v>0.15</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.125</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>35</v>
       </c>
@@ -4352,7 +4352,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>36</v>
       </c>
@@ -4360,7 +4360,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>38</v>
       </c>
@@ -4368,7 +4368,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>39</v>
       </c>
@@ -4376,7 +4376,7 @@
         <v>60000</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B23">
         <f>(1-EXP(-((C23/$B$19-($B$18-0.5))/$B$16)^$B$17))*$B$15</f>
         <v>0</v>
@@ -4385,1008 +4385,1008 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B24">
         <f t="shared" ref="B24:B87" si="0">(1-EXP(-((C24/$B$19-($B$18-0.5))/$B$16)^$B$17))*$B$15</f>
-        <v>4.0187703366778572E-7</v>
+        <v>3.3489752805648809E-7</v>
       </c>
       <c r="C24">
         <v>500</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B25">
         <f t="shared" si="0"/>
-        <v>3.2149861218577768E-6</v>
+        <v>2.6791551015481474E-6</v>
       </c>
       <c r="C25">
         <v>1000</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B26">
         <f t="shared" si="0"/>
-        <v>1.0850301995346534E-5</v>
+        <v>9.041918329455445E-6</v>
       </c>
       <c r="C26">
         <f>C25+500</f>
         <v>1500</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B27">
         <f t="shared" si="0"/>
-        <v>2.571795964551593E-5</v>
+        <v>2.1431633037929942E-5</v>
       </c>
       <c r="C27">
         <f t="shared" ref="C27:C90" si="1">C26+500</f>
         <v>2000</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B28">
         <f t="shared" si="0"/>
-        <v>5.0226285691895579E-5</v>
+        <v>4.1855238076579648E-5</v>
       </c>
       <c r="C28">
         <f t="shared" si="1"/>
         <v>2500</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B29">
         <f t="shared" si="0"/>
-        <v>8.6780443051764905E-5</v>
+        <v>7.2317035876470759E-5</v>
       </c>
       <c r="C29">
         <f t="shared" si="1"/>
         <v>3000</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B30">
         <f t="shared" si="0"/>
-        <v>1.3778069003070326E-4</v>
+        <v>1.1481724169225271E-4</v>
       </c>
       <c r="C30">
         <f t="shared" si="1"/>
         <v>3500</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B31">
         <f t="shared" si="0"/>
-        <v>2.0562025564793696E-4</v>
+        <v>1.7135021303994746E-4</v>
       </c>
       <c r="C31">
         <f t="shared" si="1"/>
         <v>4000</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B32">
         <f t="shared" si="0"/>
-        <v>2.926828338786713E-4</v>
+        <v>2.4390236156555944E-4</v>
       </c>
       <c r="C32">
         <f t="shared" si="1"/>
         <v>4500</v>
       </c>
     </row>
-    <row r="33" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B33">
         <f t="shared" si="0"/>
-        <v>4.0133970053291554E-4</v>
+        <v>3.3444975044409631E-4</v>
       </c>
       <c r="C33">
         <f t="shared" si="1"/>
         <v>5000</v>
       </c>
     </row>
-    <row r="34" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B34">
         <f t="shared" si="0"/>
-        <v>5.3394645769462839E-4</v>
+        <v>4.4495538141219038E-4</v>
       </c>
       <c r="C34">
         <f t="shared" si="1"/>
         <v>5500</v>
       </c>
     </row>
-    <row r="35" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B35">
         <f t="shared" si="0"/>
-        <v>6.9283941201358503E-4</v>
+        <v>5.7736617667798751E-4</v>
       </c>
       <c r="C35">
         <f t="shared" si="1"/>
         <v>6000</v>
       </c>
     </row>
-    <row r="36" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B36">
         <f t="shared" si="0"/>
-        <v>8.8033159466762703E-4</v>
+        <v>7.336096622230226E-4</v>
       </c>
       <c r="C36">
         <f t="shared" si="1"/>
         <v>6500</v>
       </c>
     </row>
-    <row r="37" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B37">
         <f t="shared" si="0"/>
-        <v>1.0987084324921848E-3</v>
+        <v>9.1559036041015396E-4</v>
       </c>
       <c r="C37">
         <f t="shared" si="1"/>
         <v>7000</v>
       </c>
     </row>
-    <row r="38" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B38">
         <f t="shared" si="0"/>
-        <v>1.3502230815962135E-3</v>
+        <v>1.1251859013301779E-3</v>
       </c>
       <c r="C38">
         <f t="shared" si="1"/>
         <v>7500</v>
       </c>
     </row>
-    <row r="39" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B39">
         <f t="shared" si="0"/>
-        <v>1.6370914367420941E-3</v>
+        <v>1.3642428639517451E-3</v>
       </c>
       <c r="C39">
         <f t="shared" si="1"/>
         <v>8000</v>
       </c>
     </row>
-    <row r="40" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B40">
         <f t="shared" si="0"/>
-        <v>1.9614868318508726E-3</v>
+        <v>1.6345723598757272E-3</v>
       </c>
       <c r="C40">
         <f t="shared" si="1"/>
         <v>8500</v>
       </c>
     </row>
-    <row r="41" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B41">
         <f t="shared" si="0"/>
-        <v>2.325534449188732E-3</v>
+        <v>1.9379453743239433E-3</v>
       </c>
       <c r="C41">
         <f t="shared" si="1"/>
         <v>9000</v>
       </c>
     </row>
-    <row r="42" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B42">
         <f t="shared" si="0"/>
-        <v>2.7313054570853477E-3</v>
+        <v>2.2760878809044566E-3</v>
       </c>
       <c r="C42">
         <f t="shared" si="1"/>
         <v>9500</v>
       </c>
     </row>
-    <row r="43" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B43">
         <f t="shared" si="0"/>
-        <v>3.1808108984106021E-3</v>
+        <v>2.6506757486755017E-3</v>
       </c>
       <c r="C43">
         <f t="shared" si="1"/>
         <v>10000</v>
       </c>
     </row>
-    <row r="44" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B44">
         <f t="shared" si="0"/>
-        <v>3.6759953544767184E-3</v>
+        <v>3.0633294620639323E-3</v>
       </c>
       <c r="C44">
         <f t="shared" si="1"/>
         <v>10500</v>
       </c>
     </row>
-    <row r="45" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B45">
         <f t="shared" si="0"/>
-        <v>4.2187304115184395E-3</v>
+        <v>3.5156086762653666E-3</v>
       </c>
       <c r="C45">
         <f t="shared" si="1"/>
         <v>11000</v>
       </c>
     </row>
-    <row r="46" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B46">
         <f t="shared" si="0"/>
-        <v>4.8108079594126937E-3</v>
+        <v>4.0090066328439117E-3</v>
       </c>
       <c r="C46">
         <f t="shared" si="1"/>
         <v>11500</v>
       </c>
     </row>
-    <row r="47" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B47">
         <f t="shared" si="0"/>
-        <v>5.4539333548070607E-3</v>
+        <v>4.5449444623392177E-3</v>
       </c>
       <c r="C47">
         <f t="shared" si="1"/>
         <v>12000</v>
       </c>
     </row>
-    <row r="48" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B48">
         <f t="shared" si="0"/>
-        <v>6.149718483310862E-3</v>
+        <v>5.1247654027590517E-3</v>
       </c>
       <c r="C48">
         <f t="shared" si="1"/>
         <v>12500</v>
       </c>
     </row>
-    <row r="49" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B49">
         <f t="shared" si="0"/>
-        <v>6.899674757832674E-3</v>
+        <v>5.7497289648605621E-3</v>
       </c>
       <c r="C49">
         <f t="shared" si="1"/>
         <v>13000</v>
       </c>
     </row>
-    <row r="50" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B50">
         <f t="shared" si="0"/>
-        <v>7.7052060925004657E-3</v>
+        <v>6.4210050770837218E-3</v>
       </c>
       <c r="C50">
         <f t="shared" si="1"/>
         <v>13500</v>
       </c>
     </row>
-    <row r="51" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B51">
         <f t="shared" si="0"/>
-        <v>8.5676018938412868E-3</v>
+        <v>7.139668244867739E-3</v>
       </c>
       <c r="C51">
         <f t="shared" si="1"/>
         <v>14000</v>
       </c>
     </row>
-    <row r="52" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B52">
         <f t="shared" si="0"/>
-        <v>9.4880301129990352E-3</v>
+        <v>7.9066917608325293E-3</v>
       </c>
       <c r="C52">
         <f t="shared" si="1"/>
         <v>14500</v>
       </c>
     </row>
-    <row r="53" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B53">
         <f t="shared" si="0"/>
-        <v>1.0467530404697972E-2</v>
+        <v>8.7229420039149769E-3</v>
       </c>
       <c r="C53">
         <f t="shared" si="1"/>
         <v>15000</v>
       </c>
     </row>
-    <row r="54" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B54">
         <f t="shared" si="0"/>
-        <v>1.1507007440385136E-2</v>
+        <v>9.5891728669876136E-3</v>
       </c>
       <c r="C54">
         <f t="shared" si="1"/>
         <v>15500</v>
       </c>
     </row>
-    <row r="55" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B55">
         <f t="shared" si="0"/>
-        <v>1.2607224424474078E-2</v>
+        <v>1.0506020353728399E-2</v>
       </c>
       <c r="C55">
         <f t="shared" si="1"/>
         <v>16000</v>
       </c>
     </row>
-    <row r="56" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B56">
         <f t="shared" si="0"/>
-        <v>1.3768796863832604E-2</v>
+        <v>1.1473997386527171E-2</v>
       </c>
       <c r="C56">
         <f t="shared" si="1"/>
         <v>16500</v>
       </c>
     </row>
-    <row r="57" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B57">
         <f t="shared" si="0"/>
-        <v>1.4992186641577837E-2</v>
+        <v>1.2493488867981531E-2</v>
       </c>
       <c r="C57">
         <f t="shared" si="1"/>
         <v>17000</v>
       </c>
     </row>
-    <row r="58" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B58">
         <f t="shared" si="0"/>
-        <v>1.6277696446830824E-2</v>
+        <v>1.3564747039025687E-2</v>
       </c>
       <c r="C58">
         <f t="shared" si="1"/>
         <v>17500</v>
       </c>
     </row>
-    <row r="59" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B59">
         <f t="shared" si="0"/>
-        <v>1.7625464612310682E-2</v>
+        <v>1.4687887176925568E-2</v>
       </c>
       <c r="C59">
         <f t="shared" si="1"/>
         <v>18000</v>
       </c>
     </row>
-    <row r="60" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B60">
         <f t="shared" si="0"/>
-        <v>1.9035460411488268E-2</v>
+        <v>1.5862883676240225E-2</v>
       </c>
       <c r="C60">
         <f t="shared" si="1"/>
         <v>18500</v>
       </c>
     </row>
-    <row r="61" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B61">
         <f t="shared" si="0"/>
-        <v>2.0507479866443433E-2</v>
+        <v>1.7089566555369529E-2</v>
       </c>
       <c r="C61">
         <f t="shared" si="1"/>
         <v>19000</v>
       </c>
     </row>
-    <row r="62" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B62">
         <f t="shared" si="0"/>
-        <v>2.2041142116558832E-2</v>
+        <v>1.8367618430465693E-2</v>
       </c>
       <c r="C62">
         <f t="shared" si="1"/>
         <v>19500</v>
       </c>
     </row>
-    <row r="63" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B63">
         <f t="shared" si="0"/>
-        <v>2.3635886396712456E-2</v>
+        <v>1.9696571997260381E-2</v>
       </c>
       <c r="C63">
         <f t="shared" si="1"/>
         <v>20000</v>
       </c>
     </row>
-    <row r="64" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B64">
         <f t="shared" si="0"/>
-        <v>2.5290969671690554E-2</v>
+        <v>2.1075808059742129E-2</v>
       </c>
       <c r="C64">
         <f t="shared" si="1"/>
         <v>20500</v>
       </c>
     </row>
-    <row r="65" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B65">
         <f t="shared" si="0"/>
-        <v>2.7005464971113717E-2</v>
+        <v>2.2504554142594765E-2</v>
       </c>
       <c r="C65">
         <f t="shared" si="1"/>
         <v>21000</v>
       </c>
     </row>
-    <row r="66" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B66">
         <f t="shared" si="0"/>
-        <v>2.8778260466251364E-2</v>
+        <v>2.3981883721876138E-2</v>
       </c>
       <c r="C66">
         <f t="shared" si="1"/>
         <v>21500</v>
       </c>
     </row>
-    <row r="67" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B67">
         <f t="shared" si="0"/>
-        <v>3.0608059326685061E-2</v>
+        <v>2.5506716105570884E-2</v>
       </c>
       <c r="C67">
         <f t="shared" si="1"/>
         <v>22000</v>
       </c>
     </row>
-    <row r="68" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B68">
         <f t="shared" si="0"/>
-        <v>3.249338039087727E-2</v>
+        <v>2.7077816992397724E-2</v>
       </c>
       <c r="C68">
         <f t="shared" si="1"/>
         <v>22500</v>
       </c>
     </row>
-    <row r="69" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B69">
         <f t="shared" si="0"/>
-        <v>3.4432559680315195E-2</v>
+        <v>2.8693799733595995E-2</v>
       </c>
       <c r="C69">
         <f t="shared" si="1"/>
         <v>23000</v>
       </c>
     </row>
-    <row r="70" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B70">
         <f t="shared" si="0"/>
-        <v>3.6423752782045189E-2</v>
+        <v>3.035312731837099E-2</v>
       </c>
       <c r="C70">
         <f t="shared" si="1"/>
         <v>23500</v>
       </c>
     </row>
-    <row r="71" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B71">
         <f t="shared" si="0"/>
-        <v>3.8464938119114063E-2</v>
+        <v>3.2054115099261718E-2</v>
       </c>
       <c r="C71">
         <f t="shared" si="1"/>
         <v>24000</v>
       </c>
     </row>
-    <row r="72" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B72">
         <f t="shared" si="0"/>
-        <v>4.055392112271447E-2</v>
+        <v>3.3794934268928725E-2</v>
       </c>
       <c r="C72">
         <f t="shared" si="1"/>
         <v>24500</v>
       </c>
     </row>
-    <row r="73" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="73" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B73">
         <f t="shared" si="0"/>
-        <v>4.2688339313730859E-2</v>
+        <v>3.5573616094775717E-2</v>
       </c>
       <c r="C73">
         <f t="shared" si="1"/>
         <v>25000</v>
       </c>
     </row>
-    <row r="74" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="74" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B74">
         <f t="shared" si="0"/>
-        <v>4.4865668294935525E-2</v>
+        <v>3.7388056912446274E-2</v>
       </c>
       <c r="C74">
         <f t="shared" si="1"/>
         <v>25500</v>
       </c>
     </row>
-    <row r="75" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="75" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B75">
         <f t="shared" si="0"/>
-        <v>4.7083228648343023E-2</v>
+        <v>3.9236023873619186E-2</v>
       </c>
       <c r="C75">
         <f t="shared" si="1"/>
         <v>26000</v>
       </c>
     </row>
-    <row r="76" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="76" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B76">
         <f t="shared" si="0"/>
-        <v>4.9338193725244575E-2</v>
+        <v>4.1115161437703815E-2</v>
       </c>
       <c r="C76">
         <f t="shared" si="1"/>
         <v>26500</v>
       </c>
     </row>
-    <row r="77" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="77" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B77">
         <f t="shared" si="0"/>
-        <v>5.1627598309274762E-2</v>
+        <v>4.3022998591062303E-2</v>
       </c>
       <c r="C77">
         <f t="shared" si="1"/>
         <v>27000</v>
       </c>
     </row>
-    <row r="78" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="78" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B78">
         <f t="shared" si="0"/>
-        <v>5.3948348125570124E-2</v>
+        <v>4.495695677130844E-2</v>
       </c>
       <c r="C78">
         <f t="shared" si="1"/>
         <v>27500</v>
       </c>
     </row>
-    <row r="79" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="79" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B79">
         <f t="shared" si="0"/>
-        <v>5.629723016173821E-2</v>
+        <v>4.6914358468115175E-2</v>
       </c>
       <c r="C79">
         <f t="shared" si="1"/>
         <v>28000</v>
       </c>
     </row>
-    <row r="80" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="80" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B80">
         <f t="shared" si="0"/>
-        <v>5.8670923759033294E-2</v>
+        <v>4.8892436465861083E-2</v>
       </c>
       <c r="C80">
         <f t="shared" si="1"/>
         <v>28500</v>
       </c>
     </row>
-    <row r="81" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="81" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B81">
         <f t="shared" si="0"/>
-        <v>6.1066012424913607E-2</v>
+        <v>5.0888343687428006E-2</v>
       </c>
       <c r="C81">
         <f t="shared" si="1"/>
         <v>29000</v>
       </c>
     </row>
-    <row r="82" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="82" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B82">
         <f t="shared" si="0"/>
-        <v>6.3478996311107899E-2</v>
+        <v>5.2899163592589921E-2</v>
       </c>
       <c r="C82">
         <f t="shared" si="1"/>
         <v>29500</v>
       </c>
     </row>
-    <row r="83" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="83" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B83">
         <f t="shared" si="0"/>
-        <v>6.5906305294534395E-2</v>
+        <v>5.4921921078778663E-2</v>
       </c>
       <c r="C83">
         <f t="shared" si="1"/>
         <v>30000</v>
       </c>
     </row>
-    <row r="84" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="84" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B84">
         <f t="shared" si="0"/>
-        <v>6.8344312591966452E-2</v>
+        <v>5.6953593826638713E-2</v>
       </c>
       <c r="C84">
         <f t="shared" si="1"/>
         <v>30500</v>
       </c>
     </row>
-    <row r="85" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="85" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B85">
         <f t="shared" si="0"/>
-        <v>7.0789348833315488E-2</v>
+        <v>5.8991124027762909E-2</v>
       </c>
       <c r="C85">
         <f t="shared" si="1"/>
         <v>31000</v>
       </c>
     </row>
-    <row r="86" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="86" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B86">
         <f t="shared" si="0"/>
-        <v>7.3237716512875015E-2</v>
+        <v>6.1031430427395852E-2</v>
       </c>
       <c r="C86">
         <f t="shared" si="1"/>
         <v>31500</v>
       </c>
     </row>
-    <row r="87" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="87" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B87">
         <f t="shared" si="0"/>
-        <v>7.5685704732924589E-2</v>
+        <v>6.3071420610770493E-2</v>
       </c>
       <c r="C87">
         <f t="shared" si="1"/>
         <v>32000</v>
       </c>
     </row>
-    <row r="88" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="88" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B88">
         <f t="shared" ref="B88:B124" si="2">(1-EXP(-((C88/$B$19-($B$18-0.5))/$B$16)^$B$17))*$B$15</f>
-        <v>7.8129604149794987E-2</v>
+        <v>6.5108003458162492E-2</v>
       </c>
       <c r="C88">
         <f t="shared" si="1"/>
         <v>32500</v>
       </c>
     </row>
-    <row r="89" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="89" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B89">
         <f t="shared" si="2"/>
-        <v>8.0565722028919276E-2</v>
+        <v>6.7138101690766061E-2</v>
       </c>
       <c r="C89">
         <f t="shared" si="1"/>
         <v>33000</v>
       </c>
     </row>
-    <row r="90" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="90" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B90">
         <f t="shared" si="2"/>
-        <v>8.2990397312597802E-2</v>
+        <v>6.915866442716484E-2</v>
       </c>
       <c r="C90">
         <f t="shared" si="1"/>
         <v>33500</v>
       </c>
     </row>
-    <row r="91" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="91" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B91">
         <f t="shared" si="2"/>
-        <v>8.5400015602243903E-2</v>
+        <v>7.1166679668536584E-2</v>
       </c>
       <c r="C91">
         <f t="shared" ref="C91:C124" si="3">C90+500</f>
         <v>34000</v>
       </c>
     </row>
-    <row r="92" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="92" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B92">
         <f t="shared" si="2"/>
-        <v>8.7791023955795813E-2</v>
+        <v>7.3159186629829842E-2</v>
       </c>
       <c r="C92">
         <f t="shared" si="3"/>
         <v>34500</v>
       </c>
     </row>
-    <row r="93" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="93" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B93">
         <f t="shared" si="2"/>
-        <v>9.015994540081855E-2</v>
+        <v>7.5133287834015461E-2</v>
       </c>
       <c r="C93">
         <f t="shared" si="3"/>
         <v>35000</v>
       </c>
     </row>
-    <row r="94" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="94" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B94">
         <f t="shared" si="2"/>
-        <v>9.2503393064599676E-2</v>
+        <v>7.7086160887166397E-2</v>
       </c>
       <c r="C94">
         <f t="shared" si="3"/>
         <v>35500</v>
       </c>
     </row>
-    <row r="95" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="95" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B95">
         <f t="shared" si="2"/>
-        <v>9.4818083824283653E-2</v>
+        <v>7.9015069853569708E-2</v>
       </c>
       <c r="C95">
         <f t="shared" si="3"/>
         <v>36000</v>
       </c>
     </row>
-    <row r="96" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="96" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B96">
         <f t="shared" si="2"/>
-        <v>9.7100851382792161E-2</v>
+        <v>8.0917376152326803E-2</v>
       </c>
       <c r="C96">
         <f t="shared" si="3"/>
         <v>36500</v>
       </c>
     </row>
-    <row r="97" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="97" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B97">
         <f t="shared" si="2"/>
-        <v>9.9348658679935559E-2</v>
+        <v>8.2790548899946304E-2</v>
       </c>
       <c r="C97">
         <f t="shared" si="3"/>
         <v>37000</v>
       </c>
     </row>
-    <row r="98" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="98" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B98">
         <f t="shared" si="2"/>
-        <v>0.10155860955271043</v>
+        <v>8.4632174627258694E-2</v>
       </c>
       <c r="C98">
         <f t="shared" si="3"/>
         <v>37500</v>
       </c>
     </row>
-    <row r="99" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="99" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B99">
         <f t="shared" si="2"/>
-        <v>0.10372795956427108</v>
+        <v>8.643996630355924E-2</v>
       </c>
       <c r="C99">
         <f t="shared" si="3"/>
         <v>38000</v>
       </c>
     </row>
-    <row r="100" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="100" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B100">
         <f t="shared" si="2"/>
-        <v>0.10585412592740542</v>
+        <v>8.8211771606171191E-2</v>
       </c>
       <c r="C100">
         <f t="shared" si="3"/>
         <v>38500</v>
       </c>
     </row>
-    <row r="101" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="101" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B101">
         <f t="shared" si="2"/>
-        <v>0.10793469645549059</v>
+        <v>8.9945580379575493E-2</v>
       </c>
       <c r="C101">
         <f t="shared" si="3"/>
         <v>39000</v>
       </c>
     </row>
-    <row r="102" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="102" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B102">
         <f t="shared" si="2"/>
-        <v>0.10996743748177233</v>
+        <v>9.1639531234810279E-2</v>
       </c>
       <c r="C102">
         <f t="shared" si="3"/>
         <v>39500</v>
       </c>
     </row>
-    <row r="103" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="103" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B103">
         <f t="shared" si="2"/>
-        <v>0.11195030069632968</v>
+        <v>9.32919172469414E-2</v>
       </c>
       <c r="C103">
         <f t="shared" si="3"/>
         <v>40000</v>
       </c>
     </row>
-    <row r="104" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="104" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B104">
         <f t="shared" si="2"/>
-        <v>0.11388142885916275</v>
+        <v>9.4901190715968961E-2</v>
       </c>
       <c r="C104">
         <f t="shared" si="3"/>
         <v>40500</v>
       </c>
     </row>
-    <row r="105" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="105" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B105">
         <f t="shared" si="2"/>
-        <v>0.11575916035737591</v>
+        <v>9.6465966964479927E-2</v>
       </c>
       <c r="C105">
         <f t="shared" si="3"/>
         <v>41000</v>
       </c>
     </row>
-    <row r="106" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="106" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B106">
         <f t="shared" si="2"/>
-        <v>0.11758203258431722</v>
+        <v>9.7985027153597692E-2</v>
       </c>
       <c r="C106">
         <f t="shared" si="3"/>
         <v>41500</v>
       </c>
     </row>
-    <row r="107" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="107" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B107">
         <f t="shared" si="2"/>
-        <v>0.11934878412866376</v>
+        <v>9.9457320107219804E-2</v>
       </c>
       <c r="C107">
         <f t="shared" si="3"/>
         <v>42000</v>
       </c>
     </row>
-    <row r="108" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="108" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B108">
         <f t="shared" si="2"/>
-        <v>0.12105835577169748</v>
+        <v>0.10088196314308123</v>
       </c>
       <c r="C108">
         <f t="shared" si="3"/>
         <v>42500</v>
       </c>
     </row>
-    <row r="109" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="109" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B109">
         <f t="shared" si="2"/>
-        <v>0.12270989030127519</v>
+        <v>0.10225824191772932</v>
       </c>
       <c r="C109">
         <f t="shared" si="3"/>
         <v>43000</v>
       </c>
     </row>
-    <row r="110" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="110" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B110">
         <f t="shared" si="2"/>
-        <v>0.12430273116113988</v>
+        <v>0.1035856093009499</v>
       </c>
       <c r="C110">
         <f t="shared" si="3"/>
         <v>43500</v>
       </c>
     </row>
-    <row r="111" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="111" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B111">
         <f t="shared" si="2"/>
-        <v>0.12583641996413128</v>
+        <v>0.10486368330344273</v>
       </c>
       <c r="C111">
         <f t="shared" si="3"/>
         <v>44000</v>
       </c>
     </row>
-    <row r="112" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="112" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B112">
         <f t="shared" si="2"/>
-        <v>0.12731069290740946</v>
+        <v>0.10609224408950788</v>
       </c>
       <c r="C112">
         <f t="shared" si="3"/>
         <v>44500</v>
       </c>
     </row>
-    <row r="113" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="113" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B113">
         <f t="shared" si="2"/>
-        <v>0.12872547613689861</v>
+        <v>0.10727123011408218</v>
       </c>
       <c r="C113">
         <f t="shared" si="3"/>
         <v>45000</v>
       </c>
     </row>
-    <row r="114" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="114" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B114">
         <f t="shared" si="2"/>
-        <v>0.1300808801166794</v>
+        <v>0.10840073343056618</v>
       </c>
       <c r="C114">
         <f t="shared" si="3"/>
         <v>45500</v>
       </c>
     </row>
-    <row r="115" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="115" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B115">
         <f t="shared" si="2"/>
-        <v>0.13137719306690807</v>
+        <v>0.10948099422242338</v>
       </c>
       <c r="C115">
         <f t="shared" si="3"/>
         <v>46000</v>
       </c>
     </row>
-    <row r="116" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="116" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B116">
         <f t="shared" si="2"/>
-        <v>0.13261487354093182</v>
+        <v>0.11051239461744319</v>
       </c>
       <c r="C116">
         <f t="shared" si="3"/>
         <v>46500</v>
       </c>
     </row>
-    <row r="117" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="117" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B117">
         <f t="shared" si="2"/>
-        <v>0.13379454221852241</v>
+        <v>0.11149545184876868</v>
       </c>
       <c r="C117">
         <f t="shared" si="3"/>
         <v>47000</v>
       </c>
     </row>
-    <row r="118" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="118" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B118">
         <f t="shared" si="2"/>
-        <v>0.1349169729974935</v>
+        <v>0.11243081083124459</v>
       </c>
       <c r="C118">
         <f t="shared" si="3"/>
         <v>47500</v>
       </c>
     </row>
-    <row r="119" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="119" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B119">
         <f t="shared" si="2"/>
-        <v>0.1359830834703562</v>
+        <v>0.11331923622529684</v>
       </c>
       <c r="C119">
         <f t="shared" si="3"/>
         <v>48000</v>
       </c>
     </row>
-    <row r="120" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="120" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B120">
         <f t="shared" si="2"/>
-        <v>0.13699392487605058</v>
+        <v>0.11416160406337549</v>
       </c>
       <c r="C120">
         <f t="shared" si="3"/>
         <v>48500</v>
       </c>
     </row>
-    <row r="121" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="121" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B121">
         <f t="shared" si="2"/>
-        <v>0.13795067161915198</v>
+        <v>0.11495889301595999</v>
       </c>
       <c r="C121">
         <f t="shared" si="3"/>
         <v>49000</v>
       </c>
     </row>
-    <row r="122" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="122" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B122">
         <f t="shared" si="2"/>
-        <v>0.13885461045027209</v>
+        <v>0.11571217537522674</v>
       </c>
       <c r="C122">
         <f t="shared" si="3"/>
         <v>49500</v>
       </c>
     </row>
-    <row r="123" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="123" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B123">
         <f t="shared" si="2"/>
-        <v>0.13970712940166313</v>
+        <v>0.11642260783471928</v>
       </c>
       <c r="C123">
         <f t="shared" si="3"/>
         <v>50000</v>
       </c>
     </row>
-    <row r="124" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="124" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B124">
         <f t="shared" si="2"/>
-        <v>0.14050970657130474</v>
+        <v>0.11709142214275396</v>
       </c>
       <c r="C124">
         <f t="shared" si="3"/>
@@ -5405,13 +5405,13 @@
     <tabColor rgb="FF002060"/>
   </sheetPr>
   <dimension ref="A1:CF2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="23.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:84" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:84" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -5421,334 +5421,334 @@
       </c>
       <c r="C1">
         <f>(1-EXP(-((C2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>1.3563306734076795E-6</v>
+        <v>1.1302755611730664E-6</v>
       </c>
       <c r="D1">
         <f>(1-EXP(-((D2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>1.0850301995346534E-5</v>
+        <v>9.041918329455445E-6</v>
       </c>
       <c r="E1">
         <f>(1-EXP(-((E2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>3.6616623765417522E-5</v>
+        <v>3.0513853137847935E-5</v>
       </c>
       <c r="F1">
         <f>(1-EXP(-((F2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>8.6780443051764905E-5</v>
+        <v>7.2317035876470759E-5</v>
       </c>
       <c r="G1">
         <f>(1-EXP(-((G2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>1.6944632170386997E-4</v>
+        <v>1.4120526808655831E-4</v>
       </c>
       <c r="H1">
         <f>(1-EXP(-((H2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>2.926828338786713E-4</v>
+        <v>2.4390236156555944E-4</v>
       </c>
       <c r="I1">
         <f>(1-EXP(-((I2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>4.6450282648525794E-4</v>
+        <v>3.8708568873771498E-4</v>
       </c>
       <c r="J1">
         <f>(1-EXP(-((J2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>6.9283941201358503E-4</v>
+        <v>5.7736617667798751E-4</v>
       </c>
       <c r="K1">
         <f>(1-EXP(-((K2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>9.8551779614576844E-4</v>
+        <v>8.2126483012147367E-4</v>
       </c>
       <c r="L1">
         <f>(1-EXP(-((L2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>1.3502230815962135E-3</v>
+        <v>1.1251859013301779E-3</v>
       </c>
       <c r="M1">
         <f>(1-EXP(-((M2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>1.7944642344303095E-3</v>
+        <v>1.4953868620252581E-3</v>
       </c>
       <c r="N1">
         <f>(1-EXP(-((N2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>2.325534449188732E-3</v>
+        <v>1.9379453743239433E-3</v>
       </c>
       <c r="O1">
         <f>(1-EXP(-((O2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>2.9504682038741957E-3</v>
+        <v>2.4587235032284965E-3</v>
       </c>
       <c r="P1">
         <f>(1-EXP(-((P2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>3.6759953544767184E-3</v>
+        <v>3.0633294620639323E-3</v>
       </c>
       <c r="Q1">
         <f>(1-EXP(-((Q2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>4.5084926802983977E-3</v>
+        <v>3.7570772335819985E-3</v>
       </c>
       <c r="R1">
         <f>(1-EXP(-((R2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>5.4539333548070607E-3</v>
+        <v>4.5449444623392177E-3</v>
       </c>
       <c r="S1">
         <f>(1-EXP(-((S2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>6.5178348808602399E-3</v>
+        <v>5.4315290673835337E-3</v>
       </c>
       <c r="T1">
         <f>(1-EXP(-((T2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>7.7052060925004657E-3</v>
+        <v>6.4210050770837218E-3</v>
       </c>
       <c r="U1">
         <f>(1-EXP(-((U2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>9.0204938865930274E-3</v>
+        <v>7.5170782388275237E-3</v>
       </c>
       <c r="V1">
         <f>(1-EXP(-((V2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>1.0467530404697972E-2</v>
+        <v>8.7229420039149769E-3</v>
       </c>
       <c r="W1">
         <f>(1-EXP(-((W2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>1.2049481436979681E-2</v>
+        <v>1.0041234530816401E-2</v>
       </c>
       <c r="X1">
         <f>(1-EXP(-((X2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>1.3768796863832604E-2</v>
+        <v>1.1473997386527171E-2</v>
       </c>
       <c r="Y1">
         <f>(1-EXP(-((Y2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>1.5627163985386609E-2</v>
+        <v>1.3022636654488842E-2</v>
       </c>
       <c r="Z1">
         <f>(1-EXP(-((Z2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>1.7625464612310682E-2</v>
+        <v>1.4687887176925568E-2</v>
       </c>
       <c r="AA1">
         <f>(1-EXP(-((AA2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>1.9763736801589746E-2</v>
+        <v>1.6469780667991457E-2</v>
       </c>
       <c r="AB1">
         <f>(1-EXP(-((AB2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>2.2041142116558832E-2</v>
+        <v>1.8367618430465693E-2</v>
       </c>
       <c r="AC1">
         <f>(1-EXP(-((AC2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>2.4455939269979066E-2</v>
+        <v>2.0379949391649221E-2</v>
       </c>
       <c r="AD1">
         <f>(1-EXP(-((AD2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>2.7005464971113717E-2</v>
+        <v>2.2504554142594765E-2</v>
       </c>
       <c r="AE1">
         <f>(1-EXP(-((AE2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>2.9686122741700537E-2</v>
+        <v>2.4738435618083782E-2</v>
       </c>
       <c r="AF1">
         <f>(1-EXP(-((AF2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>3.249338039087727E-2</v>
+        <v>2.7077816992397724E-2</v>
       </c>
       <c r="AG1">
         <f>(1-EXP(-((AG2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>3.5421776745385977E-2</v>
+        <v>2.951814728782165E-2</v>
       </c>
       <c r="AH1">
         <f>(1-EXP(-((AH2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>3.8464938119114063E-2</v>
+        <v>3.2054115099261718E-2</v>
       </c>
       <c r="AI1">
         <f>(1-EXP(-((AI2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>4.1615604876098174E-2</v>
+        <v>3.467967073008181E-2</v>
       </c>
       <c r="AJ1">
         <f>(1-EXP(-((AJ2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>4.4865668294935525E-2</v>
+        <v>3.7388056912446274E-2</v>
       </c>
       <c r="AK1">
         <f>(1-EXP(-((AK2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>4.820621778208041E-2</v>
+        <v>4.0171848151733677E-2</v>
       </c>
       <c r="AL1">
         <f>(1-EXP(-((AL2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>5.1627598309274762E-2</v>
+        <v>4.3022998591062303E-2</v>
       </c>
       <c r="AM1">
         <f>(1-EXP(-((AM2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>5.5119477769415316E-2</v>
+        <v>4.5932898141179429E-2</v>
       </c>
       <c r="AN1">
         <f>(1-EXP(-((AN2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>5.8670923759033294E-2</v>
+        <v>4.8892436465861083E-2</v>
       </c>
       <c r="AO1">
         <f>(1-EXP(-((AO2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>6.2270489108216164E-2</v>
+        <v>5.1892074256846804E-2</v>
       </c>
       <c r="AP1">
         <f>(1-EXP(-((AP2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>6.5906305294534395E-2</v>
+        <v>5.4921921078778663E-2</v>
       </c>
       <c r="AQ1">
         <f>(1-EXP(-((AQ2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>6.9566182700893778E-2</v>
+        <v>5.7971818917411488E-2</v>
       </c>
       <c r="AR1">
         <f>(1-EXP(-((AR2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>7.3237716512875015E-2</v>
+        <v>6.1031430427395852E-2</v>
       </c>
       <c r="AS1">
         <f>(1-EXP(-((AS2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>7.6908396903694956E-2</v>
+        <v>6.4090330753079128E-2</v>
       </c>
       <c r="AT1">
         <f>(1-EXP(-((AT2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>8.0565722028919276E-2</v>
+        <v>6.7138101690766061E-2</v>
       </c>
       <c r="AU1">
         <f>(1-EXP(-((AU2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>8.4197312252647025E-2</v>
+        <v>7.0164426877205852E-2</v>
       </c>
       <c r="AV1">
         <f>(1-EXP(-((AV2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>8.7791023955795813E-2</v>
+        <v>7.3159186629829842E-2</v>
       </c>
       <c r="AW1">
         <f>(1-EXP(-((AW2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>9.1335061238442886E-2</v>
+        <v>7.6112551032035736E-2</v>
       </c>
       <c r="AX1">
         <f>(1-EXP(-((AX2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>9.4818083824283653E-2</v>
+        <v>7.9015069853569708E-2</v>
       </c>
       <c r="AY1">
         <f>(1-EXP(-((AY2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>9.8229309507649534E-2</v>
+        <v>8.1857757923041286E-2</v>
       </c>
       <c r="AZ1">
         <f>(1-EXP(-((AZ2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.10155860955271043</v>
+        <v>8.4632174627258694E-2</v>
       </c>
       <c r="BA1">
         <f>(1-EXP(-((BA2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.10479659555998135</v>
+        <v>8.7330496299984461E-2</v>
       </c>
       <c r="BB1">
         <f>(1-EXP(-((BB2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.10793469645549059</v>
+        <v>8.9945580379575493E-2</v>
       </c>
       <c r="BC1">
         <f>(1-EXP(-((BC2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.11096522443033115</v>
+        <v>9.2471020358609296E-2</v>
       </c>
       <c r="BD1">
         <f>(1-EXP(-((BD2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.11388142885916275</v>
+        <v>9.4901190715968961E-2</v>
       </c>
       <c r="BE1">
         <f>(1-EXP(-((BE2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.11667753745097514</v>
+        <v>9.7231281209145953E-2</v>
       </c>
       <c r="BF1">
         <f>(1-EXP(-((BF2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.11934878412866376</v>
+        <v>9.9457320107219804E-2</v>
       </c>
       <c r="BG1">
         <f>(1-EXP(-((BG2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.12189142338962897</v>
+        <v>0.10157618615802415</v>
       </c>
       <c r="BH1">
         <f>(1-EXP(-((BH2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.12430273116113988</v>
+        <v>0.1035856093009499</v>
       </c>
       <c r="BI1">
         <f>(1-EXP(-((BI2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.12658099242476617</v>
+        <v>0.10548416035397182</v>
       </c>
       <c r="BJ1">
         <f>(1-EXP(-((BJ2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.12872547613689861</v>
+        <v>0.10727123011408218</v>
       </c>
       <c r="BK1">
         <f>(1-EXP(-((BK2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.13073639821054656</v>
+        <v>0.10894699850878881</v>
       </c>
       <c r="BL1">
         <f>(1-EXP(-((BL2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.13261487354093182</v>
+        <v>0.11051239461744319</v>
       </c>
       <c r="BM1">
         <f>(1-EXP(-((BM2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.13436285824823427</v>
+        <v>0.11196904854019522</v>
       </c>
       <c r="BN1">
         <f>(1-EXP(-((BN2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.1359830834703562</v>
+        <v>0.11331923622529684</v>
       </c>
       <c r="BO1">
         <f>(1-EXP(-((BO2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.13747898216292775</v>
+        <v>0.11456581846910648</v>
       </c>
       <c r="BP1">
         <f>(1-EXP(-((BP2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.13885461045027209</v>
+        <v>0.11571217537522674</v>
       </c>
       <c r="BQ1">
         <f>(1-EXP(-((BQ2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.14011456511819612</v>
+        <v>0.11676213759849677</v>
       </c>
       <c r="BR1">
         <f>(1-EXP(-((BR2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.14126389884704021</v>
+        <v>0.11771991570586685</v>
       </c>
       <c r="BS1">
         <f>(1-EXP(-((BS2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.1423080347524181</v>
+        <v>0.11859002896034841</v>
       </c>
       <c r="BT1">
         <f>(1-EXP(-((BT2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.14325268173371089</v>
+        <v>0.11937723477809242</v>
       </c>
       <c r="BU1">
         <f>(1-EXP(-((BU2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.14410375202992939</v>
+        <v>0.12008646002494117</v>
       </c>
       <c r="BV1">
         <f>(1-EXP(-((BV2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.1448672822532501</v>
+        <v>0.12072273521104175</v>
       </c>
       <c r="BW1">
         <f>(1-EXP(-((BW2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.14554935901734684</v>
+        <v>0.12129113251445571</v>
       </c>
       <c r="BX1">
         <f>(1-EXP(-((BX2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.14615605010611638</v>
+        <v>0.12179670842176366</v>
       </c>
       <c r="BY1">
         <f>(1-EXP(-((BY2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.14669334194440264</v>
+        <v>0.12224445162033554</v>
       </c>
       <c r="BZ1">
         <f>(1-EXP(-((BZ2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.14716708394183772</v>
+        <v>0.12263923661819812</v>
       </c>
       <c r="CA1">
         <f>(1-EXP(-((CA2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.14758294008979489</v>
+        <v>0.12298578340816241</v>
       </c>
       <c r="CB1">
         <f>(1-EXP(-((CB2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.1479463480052261</v>
+        <v>0.12328862333768843</v>
       </c>
       <c r="CC1">
         <f>(1-EXP(-((CC2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.14826248543885948</v>
+        <v>0.12355207119904957</v>
       </c>
       <c r="CD1">
         <f>(1-EXP(-((CD2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.14853624410321731</v>
+        <v>0.12378020341934777</v>
       </c>
       <c r="CE1">
         <f>(1-EXP(-((CE2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.1487722105317654</v>
+        <v>0.1239768421098045</v>
       </c>
       <c r="CF1">
         <f>(1-EXP(-((CF2/About!$B$19-(About!$B$18-0.5))/About!$B$16)^About!$B$17))*About!$B$15</f>
-        <v>0.15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:84" x14ac:dyDescent="0.25">
+        <v>0.125</v>
+      </c>
+    </row>
+    <row r="2" spans="1:84" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>40</v>
       </c>
@@ -6095,17 +6095,17 @@
     <tabColor rgb="FF002060"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>34</v>
       </c>
@@ -6124,12 +6124,12 @@
     <tabColor rgb="FF002060"/>
   </sheetPr>
   <dimension ref="A1:AE25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="33.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -6224,7 +6224,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -6319,7 +6319,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -6414,7 +6414,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -6509,7 +6509,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -6604,7 +6604,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -6699,7 +6699,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -6794,7 +6794,7 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -6889,7 +6889,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -6984,7 +6984,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>13</v>
       </c>
@@ -7079,7 +7079,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -7174,7 +7174,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>15</v>
       </c>
@@ -7269,7 +7269,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>16</v>
       </c>
@@ -7364,7 +7364,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>17</v>
       </c>
@@ -7459,7 +7459,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>18</v>
       </c>
@@ -7554,7 +7554,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>19</v>
       </c>
@@ -7649,7 +7649,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>20</v>
       </c>
@@ -7744,7 +7744,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>21</v>
       </c>
@@ -7839,7 +7839,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>22</v>
       </c>
@@ -7934,7 +7934,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>23</v>
       </c>
@@ -8029,7 +8029,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>24</v>
       </c>
@@ -8124,7 +8124,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>25</v>
       </c>
@@ -8219,7 +8219,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>26</v>
       </c>
@@ -8314,7 +8314,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>27</v>
       </c>
@@ -8409,7 +8409,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>28</v>
       </c>

</xml_diff>

<commit_message>
Updated CSC values, moves wind up to 0.8 in the long run.
</commit_message>
<xml_diff>
--- a/InputData/elec/CSC/Capacity Supply Curve.xlsx
+++ b/InputData/elec/CSC/Capacity Supply Curve.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\elec\CSC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\US\Models\eps-us\InputData\elec\CSC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99C13006-32D2-4CA5-92F3-55276C14F54E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E47F4BE-FD2D-4A4A-B43C-9C66510225FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{F87DB1D1-DC21-4EA7-B1DF-998EE56837F8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="23520" xr2:uid="{F87DB1D1-DC21-4EA7-B1DF-998EE56837F8}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -170,10 +170,10 @@
     <t>which in recent years has faced unique siting constraints that have limited new capacity.</t>
   </si>
   <si>
-    <t>For onshore wind, we use a long-term value of 0.5. In the near-term we limit that to 0.25 based on permitting</t>
+    <t>For onshore wind, we use a long-term value of 0.8, reflecting high permitting, siting, and interconnection challenges</t>
   </si>
   <si>
-    <t>and other challenges in the current administration (through 2029).</t>
+    <t>In the near-term we limit that to 0.2 based on permitting and other challenges in the current administration (through 2029).</t>
   </si>
 </sst>
 </file>
@@ -4277,28 +4277,28 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D3D2DEE-686E-48A0-AC3D-0F54DEA5D0EC}">
   <dimension ref="A1:C125"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="88.7265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="88.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
@@ -4306,45 +4306,45 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>37</v>
       </c>
@@ -4352,7 +4352,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>35</v>
       </c>
@@ -4360,7 +4360,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>36</v>
       </c>
@@ -4368,7 +4368,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>38</v>
       </c>
@@ -4376,7 +4376,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>39</v>
       </c>
@@ -4384,7 +4384,7 @@
         <v>60000</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B24">
         <f>(1-EXP(-((C24/$B$20-($B$19-0.5))/$B$17)^$B$18))*$B$16</f>
         <v>0</v>
@@ -4393,7 +4393,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B25">
         <f t="shared" ref="B25:B88" si="0">(1-EXP(-((C25/$B$20-($B$19-0.5))/$B$17)^$B$18))*$B$16</f>
         <v>5.3583604489038093E-7</v>
@@ -4402,7 +4402,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B26">
         <f t="shared" si="0"/>
         <v>4.286648162477036E-6</v>
@@ -4411,7 +4411,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B27">
         <f t="shared" si="0"/>
         <v>1.4467069327128713E-5</v>
@@ -4421,7 +4421,7 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B28">
         <f t="shared" si="0"/>
         <v>3.4290612860687911E-5</v>
@@ -4431,7 +4431,7 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B29">
         <f t="shared" si="0"/>
         <v>6.6968380922527435E-5</v>
@@ -4441,7 +4441,7 @@
         <v>2500</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B30">
         <f t="shared" si="0"/>
         <v>1.1570725740235322E-4</v>
@@ -4451,7 +4451,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B31">
         <f t="shared" si="0"/>
         <v>1.8370758670760434E-4</v>
@@ -4461,7 +4461,7 @@
         <v>3500</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B32">
         <f t="shared" si="0"/>
         <v>2.7416034086391594E-4</v>
@@ -4471,7 +4471,7 @@
         <v>4000</v>
       </c>
     </row>
-    <row r="33" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B33">
         <f t="shared" si="0"/>
         <v>3.9024377850489512E-4</v>
@@ -4481,7 +4481,7 @@
         <v>4500</v>
       </c>
     </row>
-    <row r="34" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B34">
         <f t="shared" si="0"/>
         <v>5.3511960071055413E-4</v>
@@ -4491,7 +4491,7 @@
         <v>5000</v>
       </c>
     </row>
-    <row r="35" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B35">
         <f t="shared" si="0"/>
         <v>7.1192861025950462E-4</v>
@@ -4501,7 +4501,7 @@
         <v>5500</v>
       </c>
     </row>
-    <row r="36" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B36">
         <f t="shared" si="0"/>
         <v>9.2378588268478008E-4</v>
@@ -4511,7 +4511,7 @@
         <v>6000</v>
       </c>
     </row>
-    <row r="37" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B37">
         <f t="shared" si="0"/>
         <v>1.1737754595568363E-3</v>
@@ -4521,7 +4521,7 @@
         <v>6500</v>
       </c>
     </row>
-    <row r="38" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B38">
         <f t="shared" si="0"/>
         <v>1.4649445766562463E-3</v>
@@ -4531,7 +4531,7 @@
         <v>7000</v>
       </c>
     </row>
-    <row r="39" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B39">
         <f t="shared" si="0"/>
         <v>1.8002974421282847E-3</v>
@@ -4541,7 +4541,7 @@
         <v>7500</v>
       </c>
     </row>
-    <row r="40" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B40">
         <f t="shared" si="0"/>
         <v>2.1827885823227922E-3</v>
@@ -4551,7 +4551,7 @@
         <v>8000</v>
       </c>
     </row>
-    <row r="41" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B41">
         <f t="shared" si="0"/>
         <v>2.6153157758011638E-3</v>
@@ -4561,7 +4561,7 @@
         <v>8500</v>
       </c>
     </row>
-    <row r="42" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B42">
         <f t="shared" si="0"/>
         <v>3.1007125989183093E-3</v>
@@ -4571,7 +4571,7 @@
         <v>9000</v>
       </c>
     </row>
-    <row r="43" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B43">
         <f t="shared" si="0"/>
         <v>3.6417406094471309E-3</v>
@@ -4581,7 +4581,7 @@
         <v>9500</v>
       </c>
     </row>
-    <row r="44" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B44">
         <f t="shared" si="0"/>
         <v>4.2410811978808027E-3</v>
@@ -4591,7 +4591,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="45" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="45" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B45">
         <f t="shared" si="0"/>
         <v>4.9013271393022924E-3</v>
@@ -4601,7 +4601,7 @@
         <v>10500</v>
       </c>
     </row>
-    <row r="46" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B46">
         <f t="shared" si="0"/>
         <v>5.6249738820245872E-3</v>
@@ -4611,7 +4611,7 @@
         <v>11000</v>
       </c>
     </row>
-    <row r="47" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B47">
         <f t="shared" si="0"/>
         <v>6.4144106125502594E-3</v>
@@ -4621,7 +4621,7 @@
         <v>11500</v>
       </c>
     </row>
-    <row r="48" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B48">
         <f t="shared" si="0"/>
         <v>7.2719111397427484E-3</v>
@@ -4631,7 +4631,7 @@
         <v>12000</v>
       </c>
     </row>
-    <row r="49" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="49" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B49">
         <f t="shared" si="0"/>
         <v>8.1996246444144827E-3</v>
@@ -4641,7 +4641,7 @@
         <v>12500</v>
       </c>
     </row>
-    <row r="50" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="50" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B50">
         <f t="shared" si="0"/>
         <v>9.1995663437769003E-3</v>
@@ -4651,7 +4651,7 @@
         <v>13000</v>
       </c>
     </row>
-    <row r="51" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="51" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B51">
         <f t="shared" si="0"/>
         <v>1.0273608123333956E-2</v>
@@ -4661,7 +4661,7 @@
         <v>13500</v>
       </c>
     </row>
-    <row r="52" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="52" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B52">
         <f t="shared" si="0"/>
         <v>1.1423469191788382E-2</v>
@@ -4671,7 +4671,7 @@
         <v>14000</v>
       </c>
     </row>
-    <row r="53" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="53" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B53">
         <f t="shared" si="0"/>
         <v>1.2650706817332047E-2</v>
@@ -4681,7 +4681,7 @@
         <v>14500</v>
       </c>
     </row>
-    <row r="54" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="54" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B54">
         <f t="shared" si="0"/>
         <v>1.3956707206263963E-2</v>
@@ -4691,7 +4691,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="55" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="55" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B55">
         <f t="shared" si="0"/>
         <v>1.5342676587180182E-2</v>
@@ -4701,7 +4701,7 @@
         <v>15500</v>
       </c>
     </row>
-    <row r="56" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="56" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B56">
         <f t="shared" si="0"/>
         <v>1.6809632565965439E-2</v>
@@ -4711,7 +4711,7 @@
         <v>16000</v>
       </c>
     </row>
-    <row r="57" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="57" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B57">
         <f t="shared" si="0"/>
         <v>1.8358395818443476E-2</v>
@@ -4721,7 +4721,7 @@
         <v>16500</v>
       </c>
     </row>
-    <row r="58" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="58" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B58">
         <f t="shared" si="0"/>
         <v>1.9989582188770449E-2</v>
@@ -4731,7 +4731,7 @@
         <v>17000</v>
       </c>
     </row>
-    <row r="59" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="59" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B59">
         <f t="shared" si="0"/>
         <v>2.1703595262441103E-2</v>
@@ -4741,7 +4741,7 @@
         <v>17500</v>
       </c>
     </row>
-    <row r="60" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="60" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B60">
         <f t="shared" si="0"/>
         <v>2.3500619483080909E-2</v>
@@ -4751,7 +4751,7 @@
         <v>18000</v>
       </c>
     </row>
-    <row r="61" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="61" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B61">
         <f t="shared" si="0"/>
         <v>2.538061388198436E-2</v>
@@ -4761,7 +4761,7 @@
         <v>18500</v>
       </c>
     </row>
-    <row r="62" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="62" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B62">
         <f t="shared" si="0"/>
         <v>2.7343306488591249E-2</v>
@@ -4771,7 +4771,7 @@
         <v>19000</v>
       </c>
     </row>
-    <row r="63" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="63" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B63">
         <f t="shared" si="0"/>
         <v>2.9388189488745109E-2</v>
@@ -4781,7 +4781,7 @@
         <v>19500</v>
       </c>
     </row>
-    <row r="64" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="64" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B64">
         <f t="shared" si="0"/>
         <v>3.1514515195616613E-2</v>
@@ -4791,7 +4791,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="65" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="65" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B65">
         <f t="shared" si="0"/>
         <v>3.372129289558741E-2</v>
@@ -4801,7 +4801,7 @@
         <v>20500</v>
       </c>
     </row>
-    <row r="66" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="66" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B66">
         <f t="shared" si="0"/>
         <v>3.6007286628151627E-2</v>
@@ -4811,7 +4811,7 @@
         <v>21000</v>
       </c>
     </row>
-    <row r="67" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="67" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B67">
         <f t="shared" si="0"/>
         <v>3.8371013955001823E-2</v>
@@ -4821,7 +4821,7 @@
         <v>21500</v>
       </c>
     </row>
-    <row r="68" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="68" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B68">
         <f t="shared" si="0"/>
         <v>4.0810745768913415E-2</v>
@@ -4831,7 +4831,7 @@
         <v>22000</v>
       </c>
     </row>
-    <row r="69" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="69" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B69">
         <f t="shared" si="0"/>
         <v>4.3324507187836363E-2</v>
@@ -4841,7 +4841,7 @@
         <v>22500</v>
       </c>
     </row>
-    <row r="70" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="70" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B70">
         <f t="shared" si="0"/>
         <v>4.5910079573753593E-2</v>
@@ -4851,7 +4851,7 @@
         <v>23000</v>
       </c>
     </row>
-    <row r="71" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="71" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B71">
         <f t="shared" si="0"/>
         <v>4.8565003709393588E-2</v>
@@ -4861,7 +4861,7 @@
         <v>23500</v>
       </c>
     </row>
-    <row r="72" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="72" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B72">
         <f t="shared" si="0"/>
         <v>5.1286584158818753E-2</v>
@@ -4871,7 +4871,7 @@
         <v>24000</v>
       </c>
     </row>
-    <row r="73" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="73" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B73">
         <f t="shared" si="0"/>
         <v>5.407189483028596E-2</v>
@@ -4881,7 +4881,7 @@
         <v>24500</v>
       </c>
     </row>
-    <row r="74" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="74" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B74">
         <f t="shared" si="0"/>
         <v>5.6917785751641151E-2</v>
@@ -4891,7 +4891,7 @@
         <v>25000</v>
       </c>
     </row>
-    <row r="75" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="75" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B75">
         <f t="shared" si="0"/>
         <v>5.982089105991404E-2</v>
@@ -4901,7 +4901,7 @@
         <v>25500</v>
       </c>
     </row>
-    <row r="76" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="76" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B76">
         <f t="shared" si="0"/>
         <v>6.2777638197790697E-2</v>
@@ -4911,7 +4911,7 @@
         <v>26000</v>
       </c>
     </row>
-    <row r="77" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="77" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B77">
         <f t="shared" si="0"/>
         <v>6.5784258300326109E-2</v>
@@ -4921,7 +4921,7 @@
         <v>26500</v>
       </c>
     </row>
-    <row r="78" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="78" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B78">
         <f t="shared" si="0"/>
         <v>6.8836797745699688E-2</v>
@@ -4931,7 +4931,7 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="79" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="79" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B79">
         <f t="shared" si="0"/>
         <v>7.1931130834093512E-2</v>
@@ -4941,7 +4941,7 @@
         <v>27500</v>
       </c>
     </row>
-    <row r="80" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="80" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B80">
         <f t="shared" si="0"/>
         <v>7.506297354898428E-2</v>
@@ -4951,7 +4951,7 @@
         <v>28000</v>
       </c>
     </row>
-    <row r="81" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="81" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B81">
         <f t="shared" si="0"/>
         <v>7.8227898345377744E-2</v>
@@ -4961,7 +4961,7 @@
         <v>28500</v>
       </c>
     </row>
-    <row r="82" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="82" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B82">
         <f t="shared" si="0"/>
         <v>8.142134989988481E-2</v>
@@ -4971,7 +4971,7 @@
         <v>29000</v>
       </c>
     </row>
-    <row r="83" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="83" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B83">
         <f t="shared" si="0"/>
         <v>8.4638661748143884E-2</v>
@@ -4981,7 +4981,7 @@
         <v>29500</v>
       </c>
     </row>
-    <row r="84" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="84" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B84">
         <f t="shared" si="0"/>
         <v>8.787507372604586E-2</v>
@@ -4991,7 +4991,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="85" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="85" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B85">
         <f t="shared" si="0"/>
         <v>9.1125750122621946E-2</v>
@@ -5001,7 +5001,7 @@
         <v>30500</v>
       </c>
     </row>
-    <row r="86" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="86" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B86">
         <f t="shared" si="0"/>
         <v>9.438579844442066E-2</v>
@@ -5011,7 +5011,7 @@
         <v>31000</v>
       </c>
     </row>
-    <row r="87" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="87" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B87">
         <f t="shared" si="0"/>
         <v>9.7650288683833367E-2</v>
@@ -5021,7 +5021,7 @@
         <v>31500</v>
       </c>
     </row>
-    <row r="88" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="88" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B88">
         <f t="shared" si="0"/>
         <v>0.10091427297723279</v>
@@ -5031,7 +5031,7 @@
         <v>32000</v>
       </c>
     </row>
-    <row r="89" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="89" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B89">
         <f t="shared" ref="B89:B125" si="2">(1-EXP(-((C89/$B$20-($B$19-0.5))/$B$17)^$B$18))*$B$16</f>
         <v>0.10417280553305999</v>
@@ -5041,7 +5041,7 @@
         <v>32500</v>
       </c>
     </row>
-    <row r="90" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="90" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B90">
         <f t="shared" si="2"/>
         <v>0.10742096270522571</v>
@@ -5051,7 +5051,7 @@
         <v>33000</v>
       </c>
     </row>
-    <row r="91" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="91" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B91">
         <f t="shared" si="2"/>
         <v>0.11065386308346375</v>
@@ -5061,7 +5061,7 @@
         <v>33500</v>
       </c>
     </row>
-    <row r="92" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="92" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B92">
         <f t="shared" si="2"/>
         <v>0.11386668746965854</v>
@@ -5071,7 +5071,7 @@
         <v>34000</v>
       </c>
     </row>
-    <row r="93" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="93" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B93">
         <f t="shared" si="2"/>
         <v>0.11705469860772776</v>
@@ -5081,7 +5081,7 @@
         <v>34500</v>
       </c>
     </row>
-    <row r="94" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="94" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B94">
         <f t="shared" si="2"/>
         <v>0.12021326053442474</v>
@@ -5091,7 +5091,7 @@
         <v>35000</v>
       </c>
     </row>
-    <row r="95" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="95" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B95">
         <f t="shared" si="2"/>
         <v>0.12333785741946623</v>
@@ -5101,7 +5101,7 @@
         <v>35500</v>
       </c>
     </row>
-    <row r="96" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="96" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B96">
         <f t="shared" si="2"/>
         <v>0.12642411176571153</v>
@@ -5111,7 +5111,7 @@
         <v>36000</v>
       </c>
     </row>
-    <row r="97" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="97" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B97">
         <f t="shared" si="2"/>
         <v>0.12946780184372289</v>
@@ -5121,7 +5121,7 @@
         <v>36500</v>
       </c>
     </row>
-    <row r="98" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="98" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B98">
         <f t="shared" si="2"/>
         <v>0.1324648782399141</v>
@@ -5131,7 +5131,7 @@
         <v>37000</v>
       </c>
     </row>
-    <row r="99" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="99" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B99">
         <f t="shared" si="2"/>
         <v>0.13541147940361392</v>
@@ -5141,7 +5141,7 @@
         <v>37500</v>
       </c>
     </row>
-    <row r="100" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="100" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B100">
         <f t="shared" si="2"/>
         <v>0.1383039460856948</v>
@@ -5151,7 +5151,7 @@
         <v>38000</v>
       </c>
     </row>
-    <row r="101" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="101" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B101">
         <f t="shared" si="2"/>
         <v>0.14113883456987392</v>
@@ -5161,7 +5161,7 @@
         <v>38500</v>
       </c>
     </row>
-    <row r="102" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="102" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B102">
         <f t="shared" si="2"/>
         <v>0.1439129286073208</v>
@@ -5171,7 +5171,7 @@
         <v>39000</v>
       </c>
     </row>
-    <row r="103" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="103" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B103">
         <f t="shared" si="2"/>
         <v>0.14662324997569645</v>
@@ -5181,7 +5181,7 @@
         <v>39500</v>
       </c>
     </row>
-    <row r="104" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="104" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B104">
         <f t="shared" si="2"/>
         <v>0.14926706759510625</v>
@@ -5191,7 +5191,7 @@
         <v>40000</v>
       </c>
     </row>
-    <row r="105" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="105" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B105">
         <f t="shared" si="2"/>
         <v>0.15184190514555035</v>
@@ -5201,7 +5201,7 @@
         <v>40500</v>
       </c>
     </row>
-    <row r="106" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="106" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B106">
         <f t="shared" si="2"/>
         <v>0.15434554714316789</v>
@@ -5211,7 +5211,7 @@
         <v>41000</v>
       </c>
     </row>
-    <row r="107" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="107" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B107">
         <f t="shared" si="2"/>
         <v>0.15677604344575632</v>
@@ -5221,7 +5221,7 @@
         <v>41500</v>
       </c>
     </row>
-    <row r="108" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="108" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B108">
         <f t="shared" si="2"/>
         <v>0.1591317121715517</v>
@@ -5231,7 +5231,7 @@
         <v>42000</v>
       </c>
     </row>
-    <row r="109" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="109" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B109">
         <f t="shared" si="2"/>
         <v>0.16141114102892998</v>
@@ -5241,7 +5241,7 @@
         <v>42500</v>
       </c>
     </row>
-    <row r="110" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="110" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B110">
         <f t="shared" si="2"/>
         <v>0.16361318706836692</v>
@@ -5251,7 +5251,7 @@
         <v>43000</v>
       </c>
     </row>
-    <row r="111" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="111" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B111">
         <f t="shared" si="2"/>
         <v>0.16573697488151984</v>
@@ -5261,7 +5261,7 @@
         <v>43500</v>
       </c>
     </row>
-    <row r="112" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="112" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B112">
         <f t="shared" si="2"/>
         <v>0.16778189328550838</v>
@@ -5271,7 +5271,7 @@
         <v>44000</v>
       </c>
     </row>
-    <row r="113" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="113" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B113">
         <f t="shared" si="2"/>
         <v>0.16974759054321262</v>
@@ -5281,7 +5281,7 @@
         <v>44500</v>
       </c>
     </row>
-    <row r="114" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="114" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B114">
         <f t="shared" si="2"/>
         <v>0.17163396818253152</v>
@@ -5291,7 +5291,7 @@
         <v>45000</v>
       </c>
     </row>
-    <row r="115" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="115" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B115">
         <f t="shared" si="2"/>
         <v>0.17344117348890589</v>
@@ -5301,7 +5301,7 @@
         <v>45500</v>
       </c>
     </row>
-    <row r="116" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="116" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B116">
         <f t="shared" si="2"/>
         <v>0.17516959075587743</v>
@@ -5311,7 +5311,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="117" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="117" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B117">
         <f t="shared" si="2"/>
         <v>0.17681983138790913</v>
@@ -5321,7 +5321,7 @@
         <v>46500</v>
       </c>
     </row>
-    <row r="118" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="118" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B118">
         <f t="shared" si="2"/>
         <v>0.17839272295802988</v>
@@ -5331,7 +5331,7 @@
         <v>47000</v>
       </c>
     </row>
-    <row r="119" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="119" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B119">
         <f t="shared" si="2"/>
         <v>0.17988929732999137</v>
@@ -5341,7 +5341,7 @@
         <v>47500</v>
       </c>
     </row>
-    <row r="120" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="120" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B120">
         <f t="shared" si="2"/>
         <v>0.18131077796047496</v>
@@ -5351,7 +5351,7 @@
         <v>48000</v>
       </c>
     </row>
-    <row r="121" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="121" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B121">
         <f t="shared" si="2"/>
         <v>0.18265856650140078</v>
@@ -5361,7 +5361,7 @@
         <v>48500</v>
       </c>
     </row>
-    <row r="122" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="122" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B122">
         <f t="shared" si="2"/>
         <v>0.18393422882553601</v>
@@ -5371,7 +5371,7 @@
         <v>49000</v>
       </c>
     </row>
-    <row r="123" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="123" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B123">
         <f t="shared" si="2"/>
         <v>0.18513948060036278</v>
@@ -5381,7 +5381,7 @@
         <v>49500</v>
       </c>
     </row>
-    <row r="124" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="124" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B124">
         <f t="shared" si="2"/>
         <v>0.18627617253555084</v>
@@ -5391,7 +5391,7 @@
         <v>50000</v>
       </c>
     </row>
-    <row r="125" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="125" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B125">
         <f t="shared" si="2"/>
         <v>0.18734627542840634</v>
@@ -5413,13 +5413,13 @@
     <tabColor rgb="FF002060"/>
   </sheetPr>
   <dimension ref="A1:CF2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:84" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:84" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -5756,7 +5756,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="2" spans="1:84" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:84" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>40</v>
       </c>
@@ -6103,17 +6103,17 @@
     <tabColor rgb="FF002060"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>34</v>
       </c>
@@ -6132,12 +6132,12 @@
     <tabColor rgb="FF002060"/>
   </sheetPr>
   <dimension ref="A1:AB25"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="33.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -6223,7 +6223,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -6309,7 +6309,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -6395,7 +6395,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -6481,7 +6481,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -6567,7 +6567,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -6653,12 +6653,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>10</v>
       </c>
       <c r="B7">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="C7">
         <v>0.2</v>
@@ -6676,70 +6676,70 @@
         <v>0.2</v>
       </c>
       <c r="H7">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="I7">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="J7">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="K7">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="L7">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="M7">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="N7">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="O7">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="P7">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="Q7">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="R7">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="S7">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="T7">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="U7">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="V7">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="W7">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="X7">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="Y7">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="Z7">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="AA7">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="AB7">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.35">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -6825,7 +6825,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -6911,7 +6911,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>13</v>
       </c>
@@ -6997,7 +6997,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -7083,7 +7083,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>15</v>
       </c>
@@ -7169,7 +7169,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>16</v>
       </c>
@@ -7255,7 +7255,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>17</v>
       </c>
@@ -7341,7 +7341,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>18</v>
       </c>
@@ -7427,7 +7427,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>19</v>
       </c>
@@ -7513,7 +7513,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>20</v>
       </c>
@@ -7599,7 +7599,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>21</v>
       </c>
@@ -7685,7 +7685,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>22</v>
       </c>
@@ -7771,7 +7771,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>23</v>
       </c>
@@ -7857,7 +7857,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>24</v>
       </c>
@@ -7943,7 +7943,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>25</v>
       </c>
@@ -8029,7 +8029,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>26</v>
       </c>
@@ -8115,7 +8115,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>27</v>
       </c>
@@ -8201,7 +8201,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>28</v>
       </c>

</xml_diff>

<commit_message>
Updates .mdl with slice/hour/tech specific ELCC values, updates SHELF and SYSHECF values, updates CSC parameters. Note that SHELF/SYSHECF .xlsx files not included here and all new AI generated .xlsx files need review.
</commit_message>
<xml_diff>
--- a/InputData/elec/CSC/Capacity Supply Curve.xlsx
+++ b/InputData/elec/CSC/Capacity Supply Curve.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\US\Models\eps-us\InputData\elec\CSC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E47F4BE-FD2D-4A4A-B43C-9C66510225FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60C77A4A-D056-4C78-9131-855A6A3B2DF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="23520" xr2:uid="{F87DB1D1-DC21-4EA7-B1DF-998EE56837F8}"/>
+    <workbookView xWindow="1524" yWindow="0" windowWidth="21516" windowHeight="13680" xr2:uid="{F87DB1D1-DC21-4EA7-B1DF-998EE56837F8}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -622,307 +622,307 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="101"/>
                 <c:pt idx="0">
-                  <c:v>5.3583604489038093E-7</c:v>
+                  <c:v>1.4467069327128713E-5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.286648162477036E-6</c:v>
+                  <c:v>1.1570725740235322E-4</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.4467069327128713E-5</c:v>
+                  <c:v>3.9024377850489512E-4</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>3.4290612860687911E-5</c:v>
+                  <c:v>9.2378588268478008E-4</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>6.6968380922527435E-5</c:v>
+                  <c:v>1.8002974421282847E-3</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.1570725740235322E-4</c:v>
+                  <c:v>3.1007125989183093E-3</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1.8370758670760434E-4</c:v>
+                  <c:v>4.9013271393022924E-3</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>2.7416034086391594E-4</c:v>
+                  <c:v>7.2719111397427484E-3</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>3.9024377850489512E-4</c:v>
+                  <c:v>1.0273608123333956E-2</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>5.3511960071055413E-4</c:v>
+                  <c:v>1.3956707206263963E-2</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>7.1192861025950462E-4</c:v>
+                  <c:v>1.8358395818443476E-2</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>9.2378588268478008E-4</c:v>
+                  <c:v>2.3500619483080909E-2</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>1.1737754595568363E-3</c:v>
+                  <c:v>2.9388189488745109E-2</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>1.4649445766562463E-3</c:v>
+                  <c:v>3.6007286628151627E-2</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>1.8002974421282847E-3</c:v>
+                  <c:v>4.3324507187836363E-2</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>2.1827885823227922E-3</c:v>
+                  <c:v>5.1286584158818753E-2</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>2.6153157758011638E-3</c:v>
+                  <c:v>5.982089105991404E-2</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>3.1007125989183093E-3</c:v>
+                  <c:v>6.8836797745699688E-2</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>3.6417406094471309E-3</c:v>
+                  <c:v>7.8227898345377744E-2</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>4.2410811978808027E-3</c:v>
+                  <c:v>8.787507372604586E-2</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>4.9013271393022924E-3</c:v>
+                  <c:v>9.7650288683833367E-2</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>5.6249738820245872E-3</c:v>
+                  <c:v>0.10742096270522571</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>6.4144106125502594E-3</c:v>
+                  <c:v>0.11705469860772776</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>7.2719111397427484E-3</c:v>
+                  <c:v>0.12642411176571153</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>8.1996246444144827E-3</c:v>
+                  <c:v>0.13541147940361392</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>9.1995663437769003E-3</c:v>
+                  <c:v>0.1439129286073208</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>1.0273608123333956E-2</c:v>
+                  <c:v>0.15184190514555035</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>1.1423469191788382E-2</c:v>
+                  <c:v>0.1591317121715517</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>1.2650706817332047E-2</c:v>
+                  <c:v>0.16573697488151984</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>1.3956707206263963E-2</c:v>
+                  <c:v>0.17163396818253152</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>1.5342676587180182E-2</c:v>
+                  <c:v>0.17681983138790913</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>1.6809632565965439E-2</c:v>
+                  <c:v>0.18131077796047496</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>1.8358395818443476E-2</c:v>
+                  <c:v>0.18513948060036278</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>1.9989582188770449E-2</c:v>
+                  <c:v>0.18835186512938695</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>2.1703595262441103E-2</c:v>
+                  <c:v>0.19100357564494788</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>2.3500619483080909E-2</c:v>
+                  <c:v>0.1931563763376668</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>2.538061388198436E-2</c:v>
+                  <c:v>0.19487473347482187</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>2.7343306488591249E-2</c:v>
+                  <c:v>0.19622277858911699</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>2.9388189488745109E-2</c:v>
+                  <c:v>0.1972617973403015</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>3.1514515195616613E-2</c:v>
+                  <c:v>0.19804832547095644</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>3.372129289558741E-2</c:v>
+                  <c:v>0.19863287140923547</c:v>
                 </c:pt>
                 <c:pt idx="41">
-                  <c:v>3.6007286628151627E-2</c:v>
+                  <c:v>0.19905923098155251</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>3.8371013955001823E-2</c:v>
+                  <c:v>0.199364318136077</c:v>
                 </c:pt>
                 <c:pt idx="43">
-                  <c:v>4.0810745768913415E-2</c:v>
+                  <c:v>0.19957840901739385</c:v>
                 </c:pt>
                 <c:pt idx="44">
-                  <c:v>4.3324507187836363E-2</c:v>
+                  <c:v>0.1997256853595088</c:v>
                 </c:pt>
                 <c:pt idx="45">
-                  <c:v>4.5910079573753593E-2</c:v>
+                  <c:v>0.19982496522253218</c:v>
                 </c:pt>
                 <c:pt idx="46">
-                  <c:v>4.8565003709393588E-2</c:v>
+                  <c:v>0.19989052148534298</c:v>
                 </c:pt>
                 <c:pt idx="47">
-                  <c:v>5.1286584158818753E-2</c:v>
+                  <c:v>0.1999329074744195</c:v>
                 </c:pt>
                 <c:pt idx="48">
-                  <c:v>5.407189483028596E-2</c:v>
+                  <c:v>0.19995973093159392</c:v>
                 </c:pt>
                 <c:pt idx="49">
-                  <c:v>5.6917785751641151E-2</c:v>
+                  <c:v>0.19997633902006273</c:v>
                 </c:pt>
                 <c:pt idx="50">
-                  <c:v>5.982089105991404E-2</c:v>
+                  <c:v>0.19998639592309114</c:v>
                 </c:pt>
                 <c:pt idx="51">
-                  <c:v>6.2777638197790697E-2</c:v>
+                  <c:v>0.19999234945911523</c:v>
                 </c:pt>
                 <c:pt idx="52">
-                  <c:v>6.5784258300326109E-2</c:v>
+                  <c:v>0.19999579357241226</c:v>
                 </c:pt>
                 <c:pt idx="53">
-                  <c:v>6.8836797745699688E-2</c:v>
+                  <c:v>0.19999773981279137</c:v>
                 </c:pt>
                 <c:pt idx="54">
-                  <c:v>7.1931130834093512E-2</c:v>
+                  <c:v>0.19999881369426081</c:v>
                 </c:pt>
                 <c:pt idx="55">
-                  <c:v>7.506297354898428E-2</c:v>
+                  <c:v>0.19999939203080119</c:v>
                 </c:pt>
                 <c:pt idx="56">
-                  <c:v>7.8227898345377744E-2</c:v>
+                  <c:v>0.19999969590396702</c:v>
                 </c:pt>
                 <c:pt idx="57">
-                  <c:v>8.142134989988481E-2</c:v>
+                  <c:v>0.19999985161306397</c:v>
                 </c:pt>
                 <c:pt idx="58">
-                  <c:v>8.4638661748143884E-2</c:v>
+                  <c:v>0.19999992939299016</c:v>
                 </c:pt>
                 <c:pt idx="59">
-                  <c:v>8.787507372604586E-2</c:v>
+                  <c:v>0.19999996725245739</c:v>
                 </c:pt>
                 <c:pt idx="60">
-                  <c:v>9.1125750122621946E-2</c:v>
+                  <c:v>0.19999998520210779</c:v>
                 </c:pt>
                 <c:pt idx="61">
-                  <c:v>9.438579844442066E-2</c:v>
+                  <c:v>0.19999999348787459</c:v>
                 </c:pt>
                 <c:pt idx="62">
-                  <c:v>9.7650288683833367E-2</c:v>
+                  <c:v>0.19999999721029099</c:v>
                 </c:pt>
                 <c:pt idx="63">
-                  <c:v>0.10091427297723279</c:v>
+                  <c:v>0.19999999883716038</c:v>
                 </c:pt>
                 <c:pt idx="64">
-                  <c:v>0.10417280553305999</c:v>
+                  <c:v>0.19999999952857025</c:v>
                 </c:pt>
                 <c:pt idx="65">
-                  <c:v>0.10742096270522571</c:v>
+                  <c:v>0.19999999981419306</c:v>
                 </c:pt>
                 <c:pt idx="66">
-                  <c:v>0.11065386308346375</c:v>
+                  <c:v>0.19999999992883505</c:v>
                 </c:pt>
                 <c:pt idx="67">
-                  <c:v>0.11386668746965854</c:v>
+                  <c:v>0.19999999997352469</c:v>
                 </c:pt>
                 <c:pt idx="68">
-                  <c:v>0.11705469860772776</c:v>
+                  <c:v>0.19999999999043694</c:v>
                 </c:pt>
                 <c:pt idx="69">
-                  <c:v>0.12021326053442474</c:v>
+                  <c:v>0.19999999999664766</c:v>
                 </c:pt>
                 <c:pt idx="70">
-                  <c:v>0.12333785741946623</c:v>
+                  <c:v>0.19999999999886001</c:v>
                 </c:pt>
                 <c:pt idx="71">
-                  <c:v>0.12642411176571153</c:v>
+                  <c:v>0.19999999999962412</c:v>
                 </c:pt>
                 <c:pt idx="72">
-                  <c:v>0.12946780184372289</c:v>
+                  <c:v>0.19999999999987986</c:v>
                 </c:pt>
                 <c:pt idx="73">
-                  <c:v>0.1324648782399141</c:v>
+                  <c:v>0.19999999999996282</c:v>
                 </c:pt>
                 <c:pt idx="74">
-                  <c:v>0.13541147940361392</c:v>
+                  <c:v>0.19999999999998885</c:v>
                 </c:pt>
                 <c:pt idx="75">
-                  <c:v>0.1383039460856948</c:v>
+                  <c:v>0.19999999999999676</c:v>
                 </c:pt>
                 <c:pt idx="76">
-                  <c:v>0.14113883456987392</c:v>
+                  <c:v>0.1999999999999991</c:v>
                 </c:pt>
                 <c:pt idx="77">
-                  <c:v>0.1439129286073208</c:v>
+                  <c:v>0.19999999999999976</c:v>
                 </c:pt>
                 <c:pt idx="78">
-                  <c:v>0.14662324997569645</c:v>
+                  <c:v>0.19999999999999996</c:v>
                 </c:pt>
                 <c:pt idx="79">
-                  <c:v>0.14926706759510625</c:v>
+                  <c:v>0.19999999999999998</c:v>
                 </c:pt>
                 <c:pt idx="80">
-                  <c:v>0.15184190514555035</c:v>
+                  <c:v>0.2</c:v>
                 </c:pt>
                 <c:pt idx="81">
-                  <c:v>0.15434554714316789</c:v>
+                  <c:v>0.2</c:v>
                 </c:pt>
                 <c:pt idx="82">
-                  <c:v>0.15677604344575632</c:v>
+                  <c:v>0.2</c:v>
                 </c:pt>
                 <c:pt idx="83">
-                  <c:v>0.1591317121715517</c:v>
+                  <c:v>0.2</c:v>
                 </c:pt>
                 <c:pt idx="84">
-                  <c:v>0.16141114102892998</c:v>
+                  <c:v>0.2</c:v>
                 </c:pt>
                 <c:pt idx="85">
-                  <c:v>0.16361318706836692</c:v>
+                  <c:v>0.2</c:v>
                 </c:pt>
                 <c:pt idx="86">
-                  <c:v>0.16573697488151984</c:v>
+                  <c:v>0.2</c:v>
                 </c:pt>
                 <c:pt idx="87">
-                  <c:v>0.16778189328550838</c:v>
+                  <c:v>0.2</c:v>
                 </c:pt>
                 <c:pt idx="88">
-                  <c:v>0.16974759054321262</c:v>
+                  <c:v>0.2</c:v>
                 </c:pt>
                 <c:pt idx="89">
-                  <c:v>0.17163396818253152</c:v>
+                  <c:v>0.2</c:v>
                 </c:pt>
                 <c:pt idx="90">
-                  <c:v>0.17344117348890589</c:v>
+                  <c:v>0.2</c:v>
                 </c:pt>
                 <c:pt idx="91">
-                  <c:v>0.17516959075587743</c:v>
+                  <c:v>0.2</c:v>
                 </c:pt>
                 <c:pt idx="92">
-                  <c:v>0.17681983138790913</c:v>
+                  <c:v>0.2</c:v>
                 </c:pt>
                 <c:pt idx="93">
-                  <c:v>0.17839272295802988</c:v>
+                  <c:v>0.2</c:v>
                 </c:pt>
                 <c:pt idx="94">
-                  <c:v>0.17988929732999137</c:v>
+                  <c:v>0.2</c:v>
                 </c:pt>
                 <c:pt idx="95">
-                  <c:v>0.18131077796047496</c:v>
+                  <c:v>0.2</c:v>
                 </c:pt>
                 <c:pt idx="96">
-                  <c:v>0.18265856650140078</c:v>
+                  <c:v>0.2</c:v>
                 </c:pt>
                 <c:pt idx="97">
-                  <c:v>0.18393422882553601</c:v>
+                  <c:v>0.2</c:v>
                 </c:pt>
                 <c:pt idx="98">
-                  <c:v>0.18513948060036278</c:v>
+                  <c:v>0.2</c:v>
                 </c:pt>
                 <c:pt idx="99">
-                  <c:v>0.18627617253555084</c:v>
+                  <c:v>0.2</c:v>
                 </c:pt>
                 <c:pt idx="100">
-                  <c:v>0.18734627542840634</c:v>
+                  <c:v>0.2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1340,124 +1340,124 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.8084408978769062E-6</c:v>
+                  <c:v>4.8822165020556696E-5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.4467069327128713E-5</c:v>
+                  <c:v>3.9024377850489512E-4</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>4.8822165020556696E-5</c:v>
+                  <c:v>1.314023728194358E-3</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1.1570725740235322E-4</c:v>
+                  <c:v>3.1007125989183093E-3</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>2.2592842893849331E-4</c:v>
+                  <c:v>6.0113235737311978E-3</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>3.9024377850489512E-4</c:v>
+                  <c:v>1.0273608123333956E-2</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>6.1933710198034406E-4</c:v>
+                  <c:v>1.6065975249306242E-2</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>9.2378588268478008E-4</c:v>
+                  <c:v>2.3500619483080909E-2</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1.314023728194358E-3</c:v>
+                  <c:v>3.2607919026638753E-2</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1.8002974421282847E-3</c:v>
+                  <c:v>4.3324507187836363E-2</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>2.3926189792404132E-3</c:v>
+                  <c:v>5.5487473168130901E-2</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>3.1007125989183093E-3</c:v>
+                  <c:v>6.8836797745699688E-2</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>3.9339576051655948E-3</c:v>
+                  <c:v>8.3027318810954889E-2</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>4.9013271393022924E-3</c:v>
+                  <c:v>9.7650288683833367E-2</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>6.0113235737311978E-3</c:v>
+                  <c:v>0.11226308300352937</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>7.2719111397427484E-3</c:v>
+                  <c:v>0.12642411176571153</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>8.6904465078136549E-3</c:v>
+                  <c:v>0.13972879407997515</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>1.0273608123333956E-2</c:v>
+                  <c:v>0.15184190514555035</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>1.2027325182124038E-2</c:v>
+                  <c:v>0.16252189785283866</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>1.3956707206263963E-2</c:v>
+                  <c:v>0.17163396818253152</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>1.6065975249306242E-2</c:v>
+                  <c:v>0.17915047766431236</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>1.8358395818443476E-2</c:v>
+                  <c:v>0.18513948060036278</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>2.0836218647182148E-2</c:v>
+                  <c:v>0.18974404633655748</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>2.3500619483080909E-2</c:v>
+                  <c:v>0.1931563763376668</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>2.6351649068786332E-2</c:v>
+                  <c:v>0.19559112259253686</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>2.9388189488745109E-2</c:v>
+                  <c:v>0.1972617973403015</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>3.2607919026638753E-2</c:v>
+                  <c:v>0.19836294737568722</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>3.6007286628151627E-2</c:v>
+                  <c:v>0.19905923098155251</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>3.9581496988934053E-2</c:v>
+                  <c:v>0.19948109182413087</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>4.3324507187836363E-2</c:v>
+                  <c:v>0.1997256853595088</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>4.7229035660514646E-2</c:v>
+                  <c:v>0.19986122147929203</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>5.1286584158818753E-2</c:v>
+                  <c:v>0.1999329074744195</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>5.5487473168130901E-2</c:v>
+                  <c:v>0.19996904944271626</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>5.982089105991404E-2</c:v>
+                  <c:v>0.19998639592309114</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>6.4274957042773889E-2</c:v>
+                  <c:v>0.19999431094957884</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>6.8836797745699688E-2</c:v>
+                  <c:v>0.19999773981279137</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>7.3492637025887084E-2</c:v>
+                  <c:v>0.19999914818203629</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>7.8227898345377744E-2</c:v>
+                  <c:v>0.19999969590396702</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>8.3027318810954889E-2</c:v>
+                  <c:v>0.19999989731662854</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>8.787507372604586E-2</c:v>
+                  <c:v>0.19999996725245739</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1875,124 +1875,124 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.8084408978769062E-6</c:v>
+                  <c:v>4.8822165020556696E-5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.4467069327128713E-5</c:v>
+                  <c:v>3.9024377850489512E-4</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>4.8822165020556696E-5</c:v>
+                  <c:v>1.314023728194358E-3</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1.1570725740235322E-4</c:v>
+                  <c:v>3.1007125989183093E-3</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>2.2592842893849331E-4</c:v>
+                  <c:v>6.0113235737311978E-3</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>3.9024377850489512E-4</c:v>
+                  <c:v>1.0273608123333956E-2</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>6.1933710198034406E-4</c:v>
+                  <c:v>1.6065975249306242E-2</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>9.2378588268478008E-4</c:v>
+                  <c:v>2.3500619483080909E-2</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1.314023728194358E-3</c:v>
+                  <c:v>3.2607919026638753E-2</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1.8002974421282847E-3</c:v>
+                  <c:v>4.3324507187836363E-2</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>2.3926189792404132E-3</c:v>
+                  <c:v>5.5487473168130901E-2</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>3.1007125989183093E-3</c:v>
+                  <c:v>6.8836797745699688E-2</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>3.9339576051655948E-3</c:v>
+                  <c:v>8.3027318810954889E-2</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>4.9013271393022924E-3</c:v>
+                  <c:v>9.7650288683833367E-2</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>6.0113235737311978E-3</c:v>
+                  <c:v>0.11226308300352937</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>7.2719111397427484E-3</c:v>
+                  <c:v>0.12642411176571153</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>8.6904465078136549E-3</c:v>
+                  <c:v>0.13972879407997515</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>1.0273608123333956E-2</c:v>
+                  <c:v>0.15184190514555035</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>1.2027325182124038E-2</c:v>
+                  <c:v>0.16252189785283866</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>1.3956707206263963E-2</c:v>
+                  <c:v>0.17163396818253152</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>1.6065975249306242E-2</c:v>
+                  <c:v>0.17915047766431236</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>1.8358395818443476E-2</c:v>
+                  <c:v>0.18513948060036278</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>2.0836218647182148E-2</c:v>
+                  <c:v>0.18974404633655748</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>2.3500619483080909E-2</c:v>
+                  <c:v>0.1931563763376668</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>2.6351649068786332E-2</c:v>
+                  <c:v>0.19559112259253686</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>2.9388189488745109E-2</c:v>
+                  <c:v>0.1972617973403015</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>3.2607919026638753E-2</c:v>
+                  <c:v>0.19836294737568722</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>3.6007286628151627E-2</c:v>
+                  <c:v>0.19905923098155251</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>3.9581496988934053E-2</c:v>
+                  <c:v>0.19948109182413087</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>4.3324507187836363E-2</c:v>
+                  <c:v>0.1997256853595088</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>4.7229035660514646E-2</c:v>
+                  <c:v>0.19986122147929203</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>5.1286584158818753E-2</c:v>
+                  <c:v>0.1999329074744195</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>5.5487473168130901E-2</c:v>
+                  <c:v>0.19996904944271626</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>5.982089105991404E-2</c:v>
+                  <c:v>0.19998639592309114</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>6.4274957042773889E-2</c:v>
+                  <c:v>0.19999431094957884</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>6.8836797745699688E-2</c:v>
+                  <c:v>0.19999773981279137</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>7.3492637025887084E-2</c:v>
+                  <c:v>0.19999914818203629</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>7.8227898345377744E-2</c:v>
+                  <c:v>0.19999969590396702</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>8.3027318810954889E-2</c:v>
+                  <c:v>0.19999989731662854</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>8.787507372604586E-2</c:v>
+                  <c:v>0.19999996725245739</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3980,9 +3980,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -4020,7 +4020,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -4126,7 +4126,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -4268,7 +4268,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -4277,28 +4277,28 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D3D2DEE-686E-48A0-AC3D-0F54DEA5D0EC}">
   <dimension ref="A1:C125"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="88.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="88.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
@@ -4306,45 +4306,45 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>37</v>
       </c>
@@ -4352,7 +4352,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>35</v>
       </c>
@@ -4360,7 +4360,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>36</v>
       </c>
@@ -4368,7 +4368,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>38</v>
       </c>
@@ -4376,15 +4376,15 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>39</v>
       </c>
       <c r="B20">
-        <v>60000</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B24">
         <f>(1-EXP(-((C24/$B$20-($B$19-0.5))/$B$17)^$B$18))*$B$16</f>
         <v>0</v>
@@ -4393,1008 +4393,1008 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B25">
         <f t="shared" ref="B25:B88" si="0">(1-EXP(-((C25/$B$20-($B$19-0.5))/$B$17)^$B$18))*$B$16</f>
-        <v>5.3583604489038093E-7</v>
+        <v>1.4467069327128713E-5</v>
       </c>
       <c r="C25">
         <v>500</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B26">
         <f t="shared" si="0"/>
-        <v>4.286648162477036E-6</v>
+        <v>1.1570725740235322E-4</v>
       </c>
       <c r="C26">
         <v>1000</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B27">
         <f t="shared" si="0"/>
-        <v>1.4467069327128713E-5</v>
+        <v>3.9024377850489512E-4</v>
       </c>
       <c r="C27">
         <f>C26+500</f>
         <v>1500</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B28">
         <f t="shared" si="0"/>
-        <v>3.4290612860687911E-5</v>
+        <v>9.2378588268478008E-4</v>
       </c>
       <c r="C28">
         <f t="shared" ref="C28:C91" si="1">C27+500</f>
         <v>2000</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B29">
         <f t="shared" si="0"/>
-        <v>6.6968380922527435E-5</v>
+        <v>1.8002974421282847E-3</v>
       </c>
       <c r="C29">
         <f t="shared" si="1"/>
         <v>2500</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B30">
         <f t="shared" si="0"/>
-        <v>1.1570725740235322E-4</v>
+        <v>3.1007125989183093E-3</v>
       </c>
       <c r="C30">
         <f t="shared" si="1"/>
         <v>3000</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B31">
         <f t="shared" si="0"/>
-        <v>1.8370758670760434E-4</v>
+        <v>4.9013271393022924E-3</v>
       </c>
       <c r="C31">
         <f t="shared" si="1"/>
         <v>3500</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B32">
         <f t="shared" si="0"/>
-        <v>2.7416034086391594E-4</v>
+        <v>7.2719111397427484E-3</v>
       </c>
       <c r="C32">
         <f t="shared" si="1"/>
         <v>4000</v>
       </c>
     </row>
-    <row r="33" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B33">
         <f t="shared" si="0"/>
-        <v>3.9024377850489512E-4</v>
+        <v>1.0273608123333956E-2</v>
       </c>
       <c r="C33">
         <f t="shared" si="1"/>
         <v>4500</v>
       </c>
     </row>
-    <row r="34" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B34">
         <f t="shared" si="0"/>
-        <v>5.3511960071055413E-4</v>
+        <v>1.3956707206263963E-2</v>
       </c>
       <c r="C34">
         <f t="shared" si="1"/>
         <v>5000</v>
       </c>
     </row>
-    <row r="35" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B35">
         <f t="shared" si="0"/>
-        <v>7.1192861025950462E-4</v>
+        <v>1.8358395818443476E-2</v>
       </c>
       <c r="C35">
         <f t="shared" si="1"/>
         <v>5500</v>
       </c>
     </row>
-    <row r="36" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B36">
         <f t="shared" si="0"/>
-        <v>9.2378588268478008E-4</v>
+        <v>2.3500619483080909E-2</v>
       </c>
       <c r="C36">
         <f t="shared" si="1"/>
         <v>6000</v>
       </c>
     </row>
-    <row r="37" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B37">
         <f t="shared" si="0"/>
-        <v>1.1737754595568363E-3</v>
+        <v>2.9388189488745109E-2</v>
       </c>
       <c r="C37">
         <f t="shared" si="1"/>
         <v>6500</v>
       </c>
     </row>
-    <row r="38" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B38">
         <f t="shared" si="0"/>
-        <v>1.4649445766562463E-3</v>
+        <v>3.6007286628151627E-2</v>
       </c>
       <c r="C38">
         <f t="shared" si="1"/>
         <v>7000</v>
       </c>
     </row>
-    <row r="39" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B39">
         <f t="shared" si="0"/>
-        <v>1.8002974421282847E-3</v>
+        <v>4.3324507187836363E-2</v>
       </c>
       <c r="C39">
         <f t="shared" si="1"/>
         <v>7500</v>
       </c>
     </row>
-    <row r="40" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B40">
         <f t="shared" si="0"/>
-        <v>2.1827885823227922E-3</v>
+        <v>5.1286584158818753E-2</v>
       </c>
       <c r="C40">
         <f t="shared" si="1"/>
         <v>8000</v>
       </c>
     </row>
-    <row r="41" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B41">
         <f t="shared" si="0"/>
-        <v>2.6153157758011638E-3</v>
+        <v>5.982089105991404E-2</v>
       </c>
       <c r="C41">
         <f t="shared" si="1"/>
         <v>8500</v>
       </c>
     </row>
-    <row r="42" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B42">
         <f t="shared" si="0"/>
-        <v>3.1007125989183093E-3</v>
+        <v>6.8836797745699688E-2</v>
       </c>
       <c r="C42">
         <f t="shared" si="1"/>
         <v>9000</v>
       </c>
     </row>
-    <row r="43" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B43">
         <f t="shared" si="0"/>
-        <v>3.6417406094471309E-3</v>
+        <v>7.8227898345377744E-2</v>
       </c>
       <c r="C43">
         <f t="shared" si="1"/>
         <v>9500</v>
       </c>
     </row>
-    <row r="44" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B44">
         <f t="shared" si="0"/>
-        <v>4.2410811978808027E-3</v>
+        <v>8.787507372604586E-2</v>
       </c>
       <c r="C44">
         <f t="shared" si="1"/>
         <v>10000</v>
       </c>
     </row>
-    <row r="45" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B45">
         <f t="shared" si="0"/>
-        <v>4.9013271393022924E-3</v>
+        <v>9.7650288683833367E-2</v>
       </c>
       <c r="C45">
         <f t="shared" si="1"/>
         <v>10500</v>
       </c>
     </row>
-    <row r="46" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B46">
         <f t="shared" si="0"/>
-        <v>5.6249738820245872E-3</v>
+        <v>0.10742096270522571</v>
       </c>
       <c r="C46">
         <f t="shared" si="1"/>
         <v>11000</v>
       </c>
     </row>
-    <row r="47" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B47">
         <f t="shared" si="0"/>
-        <v>6.4144106125502594E-3</v>
+        <v>0.11705469860772776</v>
       </c>
       <c r="C47">
         <f t="shared" si="1"/>
         <v>11500</v>
       </c>
     </row>
-    <row r="48" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B48">
         <f t="shared" si="0"/>
-        <v>7.2719111397427484E-3</v>
+        <v>0.12642411176571153</v>
       </c>
       <c r="C48">
         <f t="shared" si="1"/>
         <v>12000</v>
       </c>
     </row>
-    <row r="49" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B49">
         <f t="shared" si="0"/>
-        <v>8.1996246444144827E-3</v>
+        <v>0.13541147940361392</v>
       </c>
       <c r="C49">
         <f t="shared" si="1"/>
         <v>12500</v>
       </c>
     </row>
-    <row r="50" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B50">
         <f t="shared" si="0"/>
-        <v>9.1995663437769003E-3</v>
+        <v>0.1439129286073208</v>
       </c>
       <c r="C50">
         <f t="shared" si="1"/>
         <v>13000</v>
       </c>
     </row>
-    <row r="51" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B51">
         <f t="shared" si="0"/>
-        <v>1.0273608123333956E-2</v>
+        <v>0.15184190514555035</v>
       </c>
       <c r="C51">
         <f t="shared" si="1"/>
         <v>13500</v>
       </c>
     </row>
-    <row r="52" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B52">
         <f t="shared" si="0"/>
-        <v>1.1423469191788382E-2</v>
+        <v>0.1591317121715517</v>
       </c>
       <c r="C52">
         <f t="shared" si="1"/>
         <v>14000</v>
       </c>
     </row>
-    <row r="53" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B53">
         <f t="shared" si="0"/>
-        <v>1.2650706817332047E-2</v>
+        <v>0.16573697488151984</v>
       </c>
       <c r="C53">
         <f t="shared" si="1"/>
         <v>14500</v>
       </c>
     </row>
-    <row r="54" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B54">
         <f t="shared" si="0"/>
-        <v>1.3956707206263963E-2</v>
+        <v>0.17163396818253152</v>
       </c>
       <c r="C54">
         <f t="shared" si="1"/>
         <v>15000</v>
       </c>
     </row>
-    <row r="55" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B55">
         <f t="shared" si="0"/>
-        <v>1.5342676587180182E-2</v>
+        <v>0.17681983138790913</v>
       </c>
       <c r="C55">
         <f t="shared" si="1"/>
         <v>15500</v>
       </c>
     </row>
-    <row r="56" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B56">
         <f t="shared" si="0"/>
-        <v>1.6809632565965439E-2</v>
+        <v>0.18131077796047496</v>
       </c>
       <c r="C56">
         <f t="shared" si="1"/>
         <v>16000</v>
       </c>
     </row>
-    <row r="57" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B57">
         <f t="shared" si="0"/>
-        <v>1.8358395818443476E-2</v>
+        <v>0.18513948060036278</v>
       </c>
       <c r="C57">
         <f t="shared" si="1"/>
         <v>16500</v>
       </c>
     </row>
-    <row r="58" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B58">
         <f t="shared" si="0"/>
-        <v>1.9989582188770449E-2</v>
+        <v>0.18835186512938695</v>
       </c>
       <c r="C58">
         <f t="shared" si="1"/>
         <v>17000</v>
       </c>
     </row>
-    <row r="59" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B59">
         <f t="shared" si="0"/>
-        <v>2.1703595262441103E-2</v>
+        <v>0.19100357564494788</v>
       </c>
       <c r="C59">
         <f t="shared" si="1"/>
         <v>17500</v>
       </c>
     </row>
-    <row r="60" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B60">
         <f t="shared" si="0"/>
-        <v>2.3500619483080909E-2</v>
+        <v>0.1931563763376668</v>
       </c>
       <c r="C60">
         <f t="shared" si="1"/>
         <v>18000</v>
       </c>
     </row>
-    <row r="61" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B61">
         <f t="shared" si="0"/>
-        <v>2.538061388198436E-2</v>
+        <v>0.19487473347482187</v>
       </c>
       <c r="C61">
         <f t="shared" si="1"/>
         <v>18500</v>
       </c>
     </row>
-    <row r="62" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B62">
         <f t="shared" si="0"/>
-        <v>2.7343306488591249E-2</v>
+        <v>0.19622277858911699</v>
       </c>
       <c r="C62">
         <f t="shared" si="1"/>
         <v>19000</v>
       </c>
     </row>
-    <row r="63" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B63">
         <f t="shared" si="0"/>
-        <v>2.9388189488745109E-2</v>
+        <v>0.1972617973403015</v>
       </c>
       <c r="C63">
         <f t="shared" si="1"/>
         <v>19500</v>
       </c>
     </row>
-    <row r="64" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B64">
         <f t="shared" si="0"/>
-        <v>3.1514515195616613E-2</v>
+        <v>0.19804832547095644</v>
       </c>
       <c r="C64">
         <f t="shared" si="1"/>
         <v>20000</v>
       </c>
     </row>
-    <row r="65" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B65">
         <f t="shared" si="0"/>
-        <v>3.372129289558741E-2</v>
+        <v>0.19863287140923547</v>
       </c>
       <c r="C65">
         <f t="shared" si="1"/>
         <v>20500</v>
       </c>
     </row>
-    <row r="66" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B66">
         <f t="shared" si="0"/>
-        <v>3.6007286628151627E-2</v>
+        <v>0.19905923098155251</v>
       </c>
       <c r="C66">
         <f t="shared" si="1"/>
         <v>21000</v>
       </c>
     </row>
-    <row r="67" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B67">
         <f t="shared" si="0"/>
-        <v>3.8371013955001823E-2</v>
+        <v>0.199364318136077</v>
       </c>
       <c r="C67">
         <f t="shared" si="1"/>
         <v>21500</v>
       </c>
     </row>
-    <row r="68" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B68">
         <f t="shared" si="0"/>
-        <v>4.0810745768913415E-2</v>
+        <v>0.19957840901739385</v>
       </c>
       <c r="C68">
         <f t="shared" si="1"/>
         <v>22000</v>
       </c>
     </row>
-    <row r="69" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B69">
         <f t="shared" si="0"/>
-        <v>4.3324507187836363E-2</v>
+        <v>0.1997256853595088</v>
       </c>
       <c r="C69">
         <f t="shared" si="1"/>
         <v>22500</v>
       </c>
     </row>
-    <row r="70" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B70">
         <f t="shared" si="0"/>
-        <v>4.5910079573753593E-2</v>
+        <v>0.19982496522253218</v>
       </c>
       <c r="C70">
         <f t="shared" si="1"/>
         <v>23000</v>
       </c>
     </row>
-    <row r="71" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B71">
         <f t="shared" si="0"/>
-        <v>4.8565003709393588E-2</v>
+        <v>0.19989052148534298</v>
       </c>
       <c r="C71">
         <f t="shared" si="1"/>
         <v>23500</v>
       </c>
     </row>
-    <row r="72" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B72">
         <f t="shared" si="0"/>
-        <v>5.1286584158818753E-2</v>
+        <v>0.1999329074744195</v>
       </c>
       <c r="C72">
         <f t="shared" si="1"/>
         <v>24000</v>
       </c>
     </row>
-    <row r="73" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="73" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B73">
         <f t="shared" si="0"/>
-        <v>5.407189483028596E-2</v>
+        <v>0.19995973093159392</v>
       </c>
       <c r="C73">
         <f t="shared" si="1"/>
         <v>24500</v>
       </c>
     </row>
-    <row r="74" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="74" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B74">
         <f t="shared" si="0"/>
-        <v>5.6917785751641151E-2</v>
+        <v>0.19997633902006273</v>
       </c>
       <c r="C74">
         <f t="shared" si="1"/>
         <v>25000</v>
       </c>
     </row>
-    <row r="75" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="75" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B75">
         <f t="shared" si="0"/>
-        <v>5.982089105991404E-2</v>
+        <v>0.19998639592309114</v>
       </c>
       <c r="C75">
         <f t="shared" si="1"/>
         <v>25500</v>
       </c>
     </row>
-    <row r="76" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="76" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B76">
         <f t="shared" si="0"/>
-        <v>6.2777638197790697E-2</v>
+        <v>0.19999234945911523</v>
       </c>
       <c r="C76">
         <f t="shared" si="1"/>
         <v>26000</v>
       </c>
     </row>
-    <row r="77" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="77" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B77">
         <f t="shared" si="0"/>
-        <v>6.5784258300326109E-2</v>
+        <v>0.19999579357241226</v>
       </c>
       <c r="C77">
         <f t="shared" si="1"/>
         <v>26500</v>
       </c>
     </row>
-    <row r="78" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="78" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B78">
         <f t="shared" si="0"/>
-        <v>6.8836797745699688E-2</v>
+        <v>0.19999773981279137</v>
       </c>
       <c r="C78">
         <f t="shared" si="1"/>
         <v>27000</v>
       </c>
     </row>
-    <row r="79" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="79" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B79">
         <f t="shared" si="0"/>
-        <v>7.1931130834093512E-2</v>
+        <v>0.19999881369426081</v>
       </c>
       <c r="C79">
         <f t="shared" si="1"/>
         <v>27500</v>
       </c>
     </row>
-    <row r="80" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="80" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B80">
         <f t="shared" si="0"/>
-        <v>7.506297354898428E-2</v>
+        <v>0.19999939203080119</v>
       </c>
       <c r="C80">
         <f t="shared" si="1"/>
         <v>28000</v>
       </c>
     </row>
-    <row r="81" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="81" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B81">
         <f t="shared" si="0"/>
-        <v>7.8227898345377744E-2</v>
+        <v>0.19999969590396702</v>
       </c>
       <c r="C81">
         <f t="shared" si="1"/>
         <v>28500</v>
       </c>
     </row>
-    <row r="82" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="82" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B82">
         <f t="shared" si="0"/>
-        <v>8.142134989988481E-2</v>
+        <v>0.19999985161306397</v>
       </c>
       <c r="C82">
         <f t="shared" si="1"/>
         <v>29000</v>
       </c>
     </row>
-    <row r="83" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="83" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B83">
         <f t="shared" si="0"/>
-        <v>8.4638661748143884E-2</v>
+        <v>0.19999992939299016</v>
       </c>
       <c r="C83">
         <f t="shared" si="1"/>
         <v>29500</v>
       </c>
     </row>
-    <row r="84" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="84" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B84">
         <f t="shared" si="0"/>
-        <v>8.787507372604586E-2</v>
+        <v>0.19999996725245739</v>
       </c>
       <c r="C84">
         <f t="shared" si="1"/>
         <v>30000</v>
       </c>
     </row>
-    <row r="85" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="85" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B85">
         <f t="shared" si="0"/>
-        <v>9.1125750122621946E-2</v>
+        <v>0.19999998520210779</v>
       </c>
       <c r="C85">
         <f t="shared" si="1"/>
         <v>30500</v>
       </c>
     </row>
-    <row r="86" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="86" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B86">
         <f t="shared" si="0"/>
-        <v>9.438579844442066E-2</v>
+        <v>0.19999999348787459</v>
       </c>
       <c r="C86">
         <f t="shared" si="1"/>
         <v>31000</v>
       </c>
     </row>
-    <row r="87" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="87" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B87">
         <f t="shared" si="0"/>
-        <v>9.7650288683833367E-2</v>
+        <v>0.19999999721029099</v>
       </c>
       <c r="C87">
         <f t="shared" si="1"/>
         <v>31500</v>
       </c>
     </row>
-    <row r="88" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="88" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B88">
         <f t="shared" si="0"/>
-        <v>0.10091427297723279</v>
+        <v>0.19999999883716038</v>
       </c>
       <c r="C88">
         <f t="shared" si="1"/>
         <v>32000</v>
       </c>
     </row>
-    <row r="89" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="89" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B89">
         <f t="shared" ref="B89:B125" si="2">(1-EXP(-((C89/$B$20-($B$19-0.5))/$B$17)^$B$18))*$B$16</f>
-        <v>0.10417280553305999</v>
+        <v>0.19999999952857025</v>
       </c>
       <c r="C89">
         <f t="shared" si="1"/>
         <v>32500</v>
       </c>
     </row>
-    <row r="90" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="90" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B90">
         <f t="shared" si="2"/>
-        <v>0.10742096270522571</v>
+        <v>0.19999999981419306</v>
       </c>
       <c r="C90">
         <f t="shared" si="1"/>
         <v>33000</v>
       </c>
     </row>
-    <row r="91" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="91" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B91">
         <f t="shared" si="2"/>
-        <v>0.11065386308346375</v>
+        <v>0.19999999992883505</v>
       </c>
       <c r="C91">
         <f t="shared" si="1"/>
         <v>33500</v>
       </c>
     </row>
-    <row r="92" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="92" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B92">
         <f t="shared" si="2"/>
-        <v>0.11386668746965854</v>
+        <v>0.19999999997352469</v>
       </c>
       <c r="C92">
         <f t="shared" ref="C92:C125" si="3">C91+500</f>
         <v>34000</v>
       </c>
     </row>
-    <row r="93" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="93" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B93">
         <f t="shared" si="2"/>
-        <v>0.11705469860772776</v>
+        <v>0.19999999999043694</v>
       </c>
       <c r="C93">
         <f t="shared" si="3"/>
         <v>34500</v>
       </c>
     </row>
-    <row r="94" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="94" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B94">
         <f t="shared" si="2"/>
-        <v>0.12021326053442474</v>
+        <v>0.19999999999664766</v>
       </c>
       <c r="C94">
         <f t="shared" si="3"/>
         <v>35000</v>
       </c>
     </row>
-    <row r="95" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="95" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B95">
         <f t="shared" si="2"/>
-        <v>0.12333785741946623</v>
+        <v>0.19999999999886001</v>
       </c>
       <c r="C95">
         <f t="shared" si="3"/>
         <v>35500</v>
       </c>
     </row>
-    <row r="96" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="96" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B96">
         <f t="shared" si="2"/>
-        <v>0.12642411176571153</v>
+        <v>0.19999999999962412</v>
       </c>
       <c r="C96">
         <f t="shared" si="3"/>
         <v>36000</v>
       </c>
     </row>
-    <row r="97" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="97" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B97">
         <f t="shared" si="2"/>
-        <v>0.12946780184372289</v>
+        <v>0.19999999999987986</v>
       </c>
       <c r="C97">
         <f t="shared" si="3"/>
         <v>36500</v>
       </c>
     </row>
-    <row r="98" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="98" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B98">
         <f t="shared" si="2"/>
-        <v>0.1324648782399141</v>
+        <v>0.19999999999996282</v>
       </c>
       <c r="C98">
         <f t="shared" si="3"/>
         <v>37000</v>
       </c>
     </row>
-    <row r="99" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="99" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B99">
         <f t="shared" si="2"/>
-        <v>0.13541147940361392</v>
+        <v>0.19999999999998885</v>
       </c>
       <c r="C99">
         <f t="shared" si="3"/>
         <v>37500</v>
       </c>
     </row>
-    <row r="100" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="100" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B100">
         <f t="shared" si="2"/>
-        <v>0.1383039460856948</v>
+        <v>0.19999999999999676</v>
       </c>
       <c r="C100">
         <f t="shared" si="3"/>
         <v>38000</v>
       </c>
     </row>
-    <row r="101" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="101" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B101">
         <f t="shared" si="2"/>
-        <v>0.14113883456987392</v>
+        <v>0.1999999999999991</v>
       </c>
       <c r="C101">
         <f t="shared" si="3"/>
         <v>38500</v>
       </c>
     </row>
-    <row r="102" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="102" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B102">
         <f t="shared" si="2"/>
-        <v>0.1439129286073208</v>
+        <v>0.19999999999999976</v>
       </c>
       <c r="C102">
         <f t="shared" si="3"/>
         <v>39000</v>
       </c>
     </row>
-    <row r="103" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="103" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B103">
         <f t="shared" si="2"/>
-        <v>0.14662324997569645</v>
+        <v>0.19999999999999996</v>
       </c>
       <c r="C103">
         <f t="shared" si="3"/>
         <v>39500</v>
       </c>
     </row>
-    <row r="104" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="104" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B104">
         <f t="shared" si="2"/>
-        <v>0.14926706759510625</v>
+        <v>0.19999999999999998</v>
       </c>
       <c r="C104">
         <f t="shared" si="3"/>
         <v>40000</v>
       </c>
     </row>
-    <row r="105" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="105" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B105">
         <f t="shared" si="2"/>
-        <v>0.15184190514555035</v>
+        <v>0.2</v>
       </c>
       <c r="C105">
         <f t="shared" si="3"/>
         <v>40500</v>
       </c>
     </row>
-    <row r="106" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="106" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B106">
         <f t="shared" si="2"/>
-        <v>0.15434554714316789</v>
+        <v>0.2</v>
       </c>
       <c r="C106">
         <f t="shared" si="3"/>
         <v>41000</v>
       </c>
     </row>
-    <row r="107" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="107" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B107">
         <f t="shared" si="2"/>
-        <v>0.15677604344575632</v>
+        <v>0.2</v>
       </c>
       <c r="C107">
         <f t="shared" si="3"/>
         <v>41500</v>
       </c>
     </row>
-    <row r="108" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="108" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B108">
         <f t="shared" si="2"/>
-        <v>0.1591317121715517</v>
+        <v>0.2</v>
       </c>
       <c r="C108">
         <f t="shared" si="3"/>
         <v>42000</v>
       </c>
     </row>
-    <row r="109" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="109" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B109">
         <f t="shared" si="2"/>
-        <v>0.16141114102892998</v>
+        <v>0.2</v>
       </c>
       <c r="C109">
         <f t="shared" si="3"/>
         <v>42500</v>
       </c>
     </row>
-    <row r="110" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="110" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B110">
         <f t="shared" si="2"/>
-        <v>0.16361318706836692</v>
+        <v>0.2</v>
       </c>
       <c r="C110">
         <f t="shared" si="3"/>
         <v>43000</v>
       </c>
     </row>
-    <row r="111" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="111" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B111">
         <f t="shared" si="2"/>
-        <v>0.16573697488151984</v>
+        <v>0.2</v>
       </c>
       <c r="C111">
         <f t="shared" si="3"/>
         <v>43500</v>
       </c>
     </row>
-    <row r="112" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="112" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B112">
         <f t="shared" si="2"/>
-        <v>0.16778189328550838</v>
+        <v>0.2</v>
       </c>
       <c r="C112">
         <f t="shared" si="3"/>
         <v>44000</v>
       </c>
     </row>
-    <row r="113" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="113" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B113">
         <f t="shared" si="2"/>
-        <v>0.16974759054321262</v>
+        <v>0.2</v>
       </c>
       <c r="C113">
         <f t="shared" si="3"/>
         <v>44500</v>
       </c>
     </row>
-    <row r="114" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="114" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B114">
         <f t="shared" si="2"/>
-        <v>0.17163396818253152</v>
+        <v>0.2</v>
       </c>
       <c r="C114">
         <f t="shared" si="3"/>
         <v>45000</v>
       </c>
     </row>
-    <row r="115" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="115" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B115">
         <f t="shared" si="2"/>
-        <v>0.17344117348890589</v>
+        <v>0.2</v>
       </c>
       <c r="C115">
         <f t="shared" si="3"/>
         <v>45500</v>
       </c>
     </row>
-    <row r="116" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="116" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B116">
         <f t="shared" si="2"/>
-        <v>0.17516959075587743</v>
+        <v>0.2</v>
       </c>
       <c r="C116">
         <f t="shared" si="3"/>
         <v>46000</v>
       </c>
     </row>
-    <row r="117" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="117" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B117">
         <f t="shared" si="2"/>
-        <v>0.17681983138790913</v>
+        <v>0.2</v>
       </c>
       <c r="C117">
         <f t="shared" si="3"/>
         <v>46500</v>
       </c>
     </row>
-    <row r="118" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="118" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B118">
         <f t="shared" si="2"/>
-        <v>0.17839272295802988</v>
+        <v>0.2</v>
       </c>
       <c r="C118">
         <f t="shared" si="3"/>
         <v>47000</v>
       </c>
     </row>
-    <row r="119" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="119" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B119">
         <f t="shared" si="2"/>
-        <v>0.17988929732999137</v>
+        <v>0.2</v>
       </c>
       <c r="C119">
         <f t="shared" si="3"/>
         <v>47500</v>
       </c>
     </row>
-    <row r="120" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="120" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B120">
         <f t="shared" si="2"/>
-        <v>0.18131077796047496</v>
+        <v>0.2</v>
       </c>
       <c r="C120">
         <f t="shared" si="3"/>
         <v>48000</v>
       </c>
     </row>
-    <row r="121" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="121" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B121">
         <f t="shared" si="2"/>
-        <v>0.18265856650140078</v>
+        <v>0.2</v>
       </c>
       <c r="C121">
         <f t="shared" si="3"/>
         <v>48500</v>
       </c>
     </row>
-    <row r="122" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="122" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B122">
         <f t="shared" si="2"/>
-        <v>0.18393422882553601</v>
+        <v>0.2</v>
       </c>
       <c r="C122">
         <f t="shared" si="3"/>
         <v>49000</v>
       </c>
     </row>
-    <row r="123" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="123" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B123">
         <f t="shared" si="2"/>
-        <v>0.18513948060036278</v>
+        <v>0.2</v>
       </c>
       <c r="C123">
         <f t="shared" si="3"/>
         <v>49500</v>
       </c>
     </row>
-    <row r="124" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="124" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B124">
         <f t="shared" si="2"/>
-        <v>0.18627617253555084</v>
+        <v>0.2</v>
       </c>
       <c r="C124">
         <f t="shared" si="3"/>
         <v>50000</v>
       </c>
     </row>
-    <row r="125" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="125" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B125">
         <f t="shared" si="2"/>
-        <v>0.18734627542840634</v>
+        <v>0.2</v>
       </c>
       <c r="C125">
         <f t="shared" si="3"/>
@@ -5413,13 +5413,13 @@
     <tabColor rgb="FF002060"/>
   </sheetPr>
   <dimension ref="A1:CF2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:84" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:84" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -5429,334 +5429,334 @@
       </c>
       <c r="C1">
         <f>(1-EXP(-((C2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>1.8084408978769062E-6</v>
+        <v>4.8822165020556696E-5</v>
       </c>
       <c r="D1">
         <f>(1-EXP(-((D2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>1.4467069327128713E-5</v>
+        <v>3.9024377850489512E-4</v>
       </c>
       <c r="E1">
         <f>(1-EXP(-((E2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>4.8822165020556696E-5</v>
+        <v>1.314023728194358E-3</v>
       </c>
       <c r="F1">
         <f>(1-EXP(-((F2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>1.1570725740235322E-4</v>
+        <v>3.1007125989183093E-3</v>
       </c>
       <c r="G1">
         <f>(1-EXP(-((G2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>2.2592842893849331E-4</v>
+        <v>6.0113235737311978E-3</v>
       </c>
       <c r="H1">
         <f>(1-EXP(-((H2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>3.9024377850489512E-4</v>
+        <v>1.0273608123333956E-2</v>
       </c>
       <c r="I1">
         <f>(1-EXP(-((I2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>6.1933710198034406E-4</v>
+        <v>1.6065975249306242E-2</v>
       </c>
       <c r="J1">
         <f>(1-EXP(-((J2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>9.2378588268478008E-4</v>
+        <v>2.3500619483080909E-2</v>
       </c>
       <c r="K1">
         <f>(1-EXP(-((K2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>1.314023728194358E-3</v>
+        <v>3.2607919026638753E-2</v>
       </c>
       <c r="L1">
         <f>(1-EXP(-((L2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>1.8002974421282847E-3</v>
+        <v>4.3324507187836363E-2</v>
       </c>
       <c r="M1">
         <f>(1-EXP(-((M2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>2.3926189792404132E-3</v>
+        <v>5.5487473168130901E-2</v>
       </c>
       <c r="N1">
         <f>(1-EXP(-((N2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>3.1007125989183093E-3</v>
+        <v>6.8836797745699688E-2</v>
       </c>
       <c r="O1">
         <f>(1-EXP(-((O2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>3.9339576051655948E-3</v>
+        <v>8.3027318810954889E-2</v>
       </c>
       <c r="P1">
         <f>(1-EXP(-((P2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>4.9013271393022924E-3</v>
+        <v>9.7650288683833367E-2</v>
       </c>
       <c r="Q1">
         <f>(1-EXP(-((Q2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>6.0113235737311978E-3</v>
+        <v>0.11226308300352937</v>
       </c>
       <c r="R1">
         <f>(1-EXP(-((R2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>7.2719111397427484E-3</v>
+        <v>0.12642411176571153</v>
       </c>
       <c r="S1">
         <f>(1-EXP(-((S2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>8.6904465078136549E-3</v>
+        <v>0.13972879407997515</v>
       </c>
       <c r="T1">
         <f>(1-EXP(-((T2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>1.0273608123333956E-2</v>
+        <v>0.15184190514555035</v>
       </c>
       <c r="U1">
         <f>(1-EXP(-((U2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>1.2027325182124038E-2</v>
+        <v>0.16252189785283866</v>
       </c>
       <c r="V1">
         <f>(1-EXP(-((V2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>1.3956707206263963E-2</v>
+        <v>0.17163396818253152</v>
       </c>
       <c r="W1">
         <f>(1-EXP(-((W2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>1.6065975249306242E-2</v>
+        <v>0.17915047766431236</v>
       </c>
       <c r="X1">
         <f>(1-EXP(-((X2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>1.8358395818443476E-2</v>
+        <v>0.18513948060036278</v>
       </c>
       <c r="Y1">
         <f>(1-EXP(-((Y2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>2.0836218647182148E-2</v>
+        <v>0.18974404633655748</v>
       </c>
       <c r="Z1">
         <f>(1-EXP(-((Z2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>2.3500619483080909E-2</v>
+        <v>0.1931563763376668</v>
       </c>
       <c r="AA1">
         <f>(1-EXP(-((AA2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>2.6351649068786332E-2</v>
+        <v>0.19559112259253686</v>
       </c>
       <c r="AB1">
         <f>(1-EXP(-((AB2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>2.9388189488745109E-2</v>
+        <v>0.1972617973403015</v>
       </c>
       <c r="AC1">
         <f>(1-EXP(-((AC2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>3.2607919026638753E-2</v>
+        <v>0.19836294737568722</v>
       </c>
       <c r="AD1">
         <f>(1-EXP(-((AD2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>3.6007286628151627E-2</v>
+        <v>0.19905923098155251</v>
       </c>
       <c r="AE1">
         <f>(1-EXP(-((AE2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>3.9581496988934053E-2</v>
+        <v>0.19948109182413087</v>
       </c>
       <c r="AF1">
         <f>(1-EXP(-((AF2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>4.3324507187836363E-2</v>
+        <v>0.1997256853595088</v>
       </c>
       <c r="AG1">
         <f>(1-EXP(-((AG2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>4.7229035660514646E-2</v>
+        <v>0.19986122147929203</v>
       </c>
       <c r="AH1">
         <f>(1-EXP(-((AH2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>5.1286584158818753E-2</v>
+        <v>0.1999329074744195</v>
       </c>
       <c r="AI1">
         <f>(1-EXP(-((AI2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>5.5487473168130901E-2</v>
+        <v>0.19996904944271626</v>
       </c>
       <c r="AJ1">
         <f>(1-EXP(-((AJ2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>5.982089105991404E-2</v>
+        <v>0.19998639592309114</v>
       </c>
       <c r="AK1">
         <f>(1-EXP(-((AK2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>6.4274957042773889E-2</v>
+        <v>0.19999431094957884</v>
       </c>
       <c r="AL1">
         <f>(1-EXP(-((AL2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>6.8836797745699688E-2</v>
+        <v>0.19999773981279137</v>
       </c>
       <c r="AM1">
         <f>(1-EXP(-((AM2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>7.3492637025887084E-2</v>
+        <v>0.19999914818203629</v>
       </c>
       <c r="AN1">
         <f>(1-EXP(-((AN2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>7.8227898345377744E-2</v>
+        <v>0.19999969590396702</v>
       </c>
       <c r="AO1">
         <f>(1-EXP(-((AO2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>8.3027318810954889E-2</v>
+        <v>0.19999989731662854</v>
       </c>
       <c r="AP1">
         <f>(1-EXP(-((AP2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>8.787507372604586E-2</v>
+        <v>0.19999996725245739</v>
       </c>
       <c r="AQ1">
         <f>(1-EXP(-((AQ2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>9.2754910267858384E-2</v>
+        <v>0.19999999015058653</v>
       </c>
       <c r="AR1">
         <f>(1-EXP(-((AR2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>9.7650288683833367E-2</v>
+        <v>0.19999999721029099</v>
       </c>
       <c r="AS1">
         <f>(1-EXP(-((AS2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.10254452920492661</v>
+        <v>0.19999999925700113</v>
       </c>
       <c r="AT1">
         <f>(1-EXP(-((AT2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.10742096270522571</v>
+        <v>0.19999999981419306</v>
       </c>
       <c r="AU1">
         <f>(1-EXP(-((AU2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.11226308300352937</v>
+        <v>0.19999999995643436</v>
       </c>
       <c r="AV1">
         <f>(1-EXP(-((AV2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.11705469860772776</v>
+        <v>0.19999999999043694</v>
       </c>
       <c r="AW1">
         <f>(1-EXP(-((AW2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.12178008165125719</v>
+        <v>0.19999999999803761</v>
       </c>
       <c r="AX1">
         <f>(1-EXP(-((AX2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.12642411176571153</v>
+        <v>0.19999999999962412</v>
       </c>
       <c r="AY1">
         <f>(1-EXP(-((AY2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.13097241267686607</v>
+        <v>0.1999999999999329</v>
       </c>
       <c r="AZ1">
         <f>(1-EXP(-((AZ2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.13541147940361392</v>
+        <v>0.19999999999998885</v>
       </c>
       <c r="BA1">
         <f>(1-EXP(-((BA2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.13972879407997515</v>
+        <v>0.19999999999999829</v>
       </c>
       <c r="BB1">
         <f>(1-EXP(-((BB2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.1439129286073208</v>
+        <v>0.19999999999999976</v>
       </c>
       <c r="BC1">
         <f>(1-EXP(-((BC2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.14795363257377489</v>
+        <v>0.19999999999999998</v>
       </c>
       <c r="BD1">
         <f>(1-EXP(-((BD2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.15184190514555035</v>
+        <v>0.2</v>
       </c>
       <c r="BE1">
         <f>(1-EXP(-((BE2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.15557004993463353</v>
+        <v>0.2</v>
       </c>
       <c r="BF1">
         <f>(1-EXP(-((BF2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.1591317121715517</v>
+        <v>0.2</v>
       </c>
       <c r="BG1">
         <f>(1-EXP(-((BG2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.16252189785283866</v>
+        <v>0.2</v>
       </c>
       <c r="BH1">
         <f>(1-EXP(-((BH2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.16573697488151984</v>
+        <v>0.2</v>
       </c>
       <c r="BI1">
         <f>(1-EXP(-((BI2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.16877465656635493</v>
+        <v>0.2</v>
       </c>
       <c r="BJ1">
         <f>(1-EXP(-((BJ2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.17163396818253152</v>
+        <v>0.2</v>
       </c>
       <c r="BK1">
         <f>(1-EXP(-((BK2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.17431519761406211</v>
+        <v>0.2</v>
       </c>
       <c r="BL1">
         <f>(1-EXP(-((BL2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.17681983138790913</v>
+        <v>0.2</v>
       </c>
       <c r="BM1">
         <f>(1-EXP(-((BM2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.17915047766431236</v>
+        <v>0.2</v>
       </c>
       <c r="BN1">
         <f>(1-EXP(-((BN2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.18131077796047496</v>
+        <v>0.2</v>
       </c>
       <c r="BO1">
         <f>(1-EXP(-((BO2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.18330530955057037</v>
+        <v>0.2</v>
       </c>
       <c r="BP1">
         <f>(1-EXP(-((BP2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.18513948060036278</v>
+        <v>0.2</v>
       </c>
       <c r="BQ1">
         <f>(1-EXP(-((BQ2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.18681942015759484</v>
+        <v>0.2</v>
       </c>
       <c r="BR1">
         <f>(1-EXP(-((BR2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.18835186512938695</v>
+        <v>0.2</v>
       </c>
       <c r="BS1">
         <f>(1-EXP(-((BS2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.18974404633655748</v>
+        <v>0.2</v>
       </c>
       <c r="BT1">
         <f>(1-EXP(-((BT2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19100357564494788</v>
+        <v>0.2</v>
       </c>
       <c r="BU1">
         <f>(1-EXP(-((BU2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19213833603990588</v>
+        <v>0.2</v>
       </c>
       <c r="BV1">
         <f>(1-EXP(-((BV2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.1931563763376668</v>
+        <v>0.2</v>
       </c>
       <c r="BW1">
         <f>(1-EXP(-((BW2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19406581202312914</v>
+        <v>0.2</v>
       </c>
       <c r="BX1">
         <f>(1-EXP(-((BX2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19487473347482187</v>
+        <v>0.2</v>
       </c>
       <c r="BY1">
         <f>(1-EXP(-((BY2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19559112259253686</v>
+        <v>0.2</v>
       </c>
       <c r="BZ1">
         <f>(1-EXP(-((BZ2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19622277858911699</v>
+        <v>0.2</v>
       </c>
       <c r="CA1">
         <f>(1-EXP(-((CA2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19677725345305985</v>
+        <v>0.2</v>
       </c>
       <c r="CB1">
         <f>(1-EXP(-((CB2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.1972617973403015</v>
+        <v>0.2</v>
       </c>
       <c r="CC1">
         <f>(1-EXP(-((CC2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19768331391847932</v>
+        <v>0.2</v>
       </c>
       <c r="CD1">
         <f>(1-EXP(-((CD2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19804832547095644</v>
+        <v>0.2</v>
       </c>
       <c r="CE1">
         <f>(1-EXP(-((CE2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19836294737568722</v>
+        <v>0.2</v>
       </c>
       <c r="CF1">
         <f>(1-EXP(-((CF2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
         <v>0.2</v>
       </c>
     </row>
-    <row r="2" spans="1:84" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:84" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>40</v>
       </c>
@@ -6103,17 +6103,17 @@
     <tabColor rgb="FF002060"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>34</v>
       </c>
@@ -6132,12 +6132,12 @@
     <tabColor rgb="FF002060"/>
   </sheetPr>
   <dimension ref="A1:AB25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="33.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -6223,7 +6223,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -6309,7 +6309,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -6395,7 +6395,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -6481,7 +6481,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -6567,7 +6567,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -6653,7 +6653,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -6739,7 +6739,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -6825,7 +6825,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -6911,7 +6911,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>13</v>
       </c>
@@ -6997,7 +6997,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -7083,7 +7083,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>15</v>
       </c>
@@ -7169,7 +7169,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>16</v>
       </c>
@@ -7255,7 +7255,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>17</v>
       </c>
@@ -7341,7 +7341,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>18</v>
       </c>
@@ -7427,7 +7427,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>19</v>
       </c>
@@ -7513,7 +7513,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>20</v>
       </c>
@@ -7599,7 +7599,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>21</v>
       </c>
@@ -7685,7 +7685,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>22</v>
       </c>
@@ -7771,7 +7771,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>23</v>
       </c>
@@ -7857,7 +7857,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>24</v>
       </c>
@@ -7943,7 +7943,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>25</v>
       </c>
@@ -8029,7 +8029,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>26</v>
       </c>
@@ -8115,7 +8115,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>27</v>
       </c>
@@ -8201,7 +8201,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>28</v>
       </c>

</xml_diff>

<commit_message>
extend CSC incremental revenue
</commit_message>
<xml_diff>
--- a/InputData/elec/CSC/Capacity Supply Curve.xlsx
+++ b/InputData/elec/CSC/Capacity Supply Curve.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\US\Models\eps-us\InputData\elec\CSC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\elec\CSC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{B2750E72-BF47-44D8-B01F-CAC44956A28F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F883EF7-FBF2-4D5F-B877-C19338E42041}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="23520" xr2:uid="{F87DB1D1-DC21-4EA7-B1DF-998EE56837F8}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{F87DB1D1-DC21-4EA7-B1DF-998EE56837F8}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -3980,9 +3980,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -4020,7 +4020,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -4126,7 +4126,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -4268,7 +4268,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -6088,7 +6088,7 @@
         <v>60750</v>
       </c>
       <c r="CF2" s="2">
-        <v>1000000</v>
+        <v>1000000000000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ties the NEC value to the value used for the CSC max. This ensures in the model that when share of installed capacity built is multiplied by existing capacity, the total possible remains a the minimum (previously it was the defined minimum muliptlied by the shared of installed).
</commit_message>
<xml_diff>
--- a/InputData/elec/CSC/Capacity Supply Curve.xlsx
+++ b/InputData/elec/CSC/Capacity Supply Curve.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\elec\CSC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\US\Models\eps-us\InputData\elec\CSC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F883EF7-FBF2-4D5F-B877-C19338E42041}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{116E205E-B3EA-4C63-A8DD-B0BB7518DD68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{F87DB1D1-DC21-4EA7-B1DF-998EE56837F8}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{F87DB1D1-DC21-4EA7-B1DF-998EE56837F8}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
   <si>
     <t xml:space="preserve">Source: </t>
   </si>
@@ -137,9 +137,6 @@
     <t>Supply Curve Parameters</t>
   </si>
   <si>
-    <t>% of total installed capacity</t>
-  </si>
-  <si>
     <t>Share</t>
   </si>
   <si>
@@ -175,6 +172,12 @@
   <si>
     <t>In the near-term we limit that to 0.2 based on permitting and other challenges in the current administration (through 2029).</t>
   </si>
+  <si>
+    <t>Minimum capacity buildable for plants types with no existing capacity (share if installed)</t>
+  </si>
+  <si>
+    <t>% of total installed capacity (tied to CSC)</t>
+  </si>
 </sst>
 </file>
 
@@ -197,12 +200,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -217,10 +226,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3980,9 +3990,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -4020,7 +4030,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -4126,7 +4136,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -4268,7 +4278,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -4308,27 +4318,27 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -4346,7 +4356,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B16">
         <v>0.2</v>
@@ -4354,7 +4364,7 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B17">
         <v>0.6</v>
@@ -4362,7 +4372,7 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B18">
         <v>3</v>
@@ -4370,7 +4380,7 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B19">
         <v>0.5</v>
@@ -4378,10 +4388,18 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B20">
         <v>40000</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>45</v>
+      </c>
+      <c r="B21">
+        <v>0.02</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -5758,7 +5776,7 @@
     </row>
     <row r="2" spans="1:84" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -6110,15 +6128,16 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="B2">
-        <v>0.02</v>
+        <v>33</v>
+      </c>
+      <c r="B2" s="3">
+        <f>About!B21/About!B16</f>
+        <v>9.9999999999999992E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Revert CSCMBCfPTwNEC to 0.02
</commit_message>
<xml_diff>
--- a/InputData/elec/CSC/Capacity Supply Curve.xlsx
+++ b/InputData/elec/CSC/Capacity Supply Curve.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\US\Models\eps-us\InputData\elec\CSC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\elec\CSC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{116E205E-B3EA-4C63-A8DD-B0BB7518DD68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8A2D900-C6F2-43D6-B67D-94B6FEACA471}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{F87DB1D1-DC21-4EA7-B1DF-998EE56837F8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{F87DB1D1-DC21-4EA7-B1DF-998EE56837F8}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -3990,9 +3990,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -4030,7 +4030,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -4136,7 +4136,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -4278,7 +4278,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -4399,7 +4399,7 @@
         <v>45</v>
       </c>
       <c r="B21">
-        <v>0.02</v>
+        <v>4.0000000000000001E-3</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -6137,7 +6137,7 @@
       </c>
       <c r="B2" s="3">
         <f>About!B21/About!B16</f>
-        <v>9.9999999999999992E-2</v>
+        <v>0.02</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update max probability cutoff to 30k
</commit_message>
<xml_diff>
--- a/InputData/elec/CSC/Capacity Supply Curve.xlsx
+++ b/InputData/elec/CSC/Capacity Supply Curve.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\elec\CSC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{485A19BF-0A7C-4844-998B-EB22EFC7DA61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3121D63-400A-431A-800C-74C80046487D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{F87DB1D1-DC21-4EA7-B1DF-998EE56837F8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{F87DB1D1-DC21-4EA7-B1DF-998EE56837F8}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -632,307 +632,307 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="101"/>
                 <c:pt idx="0">
-                  <c:v>9.259237825798295E-7</c:v>
+                  <c:v>4.286648162477036E-6</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>7.4072702348937371E-6</c:v>
+                  <c:v>3.4290612860687911E-5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2.4998437565093568E-5</c:v>
+                  <c:v>1.1570725740235322E-4</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5.9250480976746905E-5</c:v>
+                  <c:v>2.7416034086391594E-4</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1.1570725740235322E-4</c:v>
+                  <c:v>5.3511960071055413E-4</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.9990003332499563E-4</c:v>
+                  <c:v>9.2378588268478008E-4</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>3.173405633774218E-4</c:v>
+                  <c:v>1.4649445766562463E-3</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>4.7351265218500418E-4</c:v>
+                  <c:v>2.1827885823227922E-3</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>6.7386221786482905E-4</c:v>
+                  <c:v>3.1007125989183093E-3</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>9.2378588268478008E-4</c:v>
+                  <c:v>4.2410811978808027E-3</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1.2286181245915852E-3</c:v>
+                  <c:v>5.6249738820245872E-3</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>1.5936170325878685E-3</c:v>
+                  <c:v>7.2719111397427484E-3</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>2.0239487192203367E-3</c:v>
+                  <c:v>9.1995663437769003E-3</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>2.5246704546594725E-3</c:v>
+                  <c:v>1.1423469191788382E-2</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>3.1007125989183093E-3</c:v>
+                  <c:v>1.3956707206263963E-2</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>3.756859421568759E-3</c:v>
+                  <c:v>1.6809632565965439E-2</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>4.4977289117446254E-3</c:v>
+                  <c:v>1.9989582188770449E-2</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>5.3277516951326436E-3</c:v>
+                  <c:v>2.3500619483080909E-2</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>6.2511491888826987E-3</c:v>
+                  <c:v>2.7343306488591249E-2</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>7.2719111397427484E-3</c:v>
+                  <c:v>3.1514515195616613E-2</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>8.3937727050432676E-3</c:v>
+                  <c:v>3.6007286628151627E-2</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>9.6201912502106527E-3</c:v>
+                  <c:v>4.0810745768913415E-2</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>1.0954323050048865E-2</c:v>
+                  <c:v>4.5910079573753593E-2</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>1.2399000093854107E-2</c:v>
+                  <c:v>5.1286584158818753E-2</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>1.3956707206263963E-2</c:v>
+                  <c:v>5.6917785751641151E-2</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>1.5629559706331463E-2</c:v>
+                  <c:v>6.2777638197790697E-2</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>1.7419281836388589E-2</c:v>
+                  <c:v>6.8836797745699688E-2</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>1.9327186199557179E-2</c:v>
+                  <c:v>7.506297354898428E-2</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>2.1354154450015608E-2</c:v>
+                  <c:v>8.142134989988481E-2</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>2.3500619483080909E-2</c:v>
+                  <c:v>8.787507372604586E-2</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>2.5766549372577496E-2</c:v>
+                  <c:v>9.438579844442066E-2</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>2.8151433300614783E-2</c:v>
+                  <c:v>0.10091427297723279</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>3.0654269719585427E-2</c:v>
+                  <c:v>0.10742096270522571</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>3.3273556977759113E-2</c:v>
+                  <c:v>0.11386668746965854</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>3.6007286628151627E-2</c:v>
+                  <c:v>0.12021326053442474</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>3.8852939625304075E-2</c:v>
+                  <c:v>0.12642411176571153</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>4.1807485596171513E-2</c:v>
+                  <c:v>0.1324648782399141</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>4.4867385349501548E-2</c:v>
+                  <c:v>0.1383039460856948</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>4.8028596762946157E-2</c:v>
+                  <c:v>0.1439129286073208</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>5.1286584158818753E-2</c:v>
+                  <c:v>0.14926706759510625</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>5.4636331248070019E-2</c:v>
+                  <c:v>0.15434554714316789</c:v>
                 </c:pt>
                 <c:pt idx="41">
-                  <c:v>5.8072357687958265E-2</c:v>
+                  <c:v>0.1591317121715517</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>6.1588739262348917E-2</c:v>
+                  <c:v>0.16361318706836692</c:v>
                 </c:pt>
                 <c:pt idx="43">
-                  <c:v>6.5179131654968622E-2</c:v>
+                  <c:v>0.16778189328550838</c:v>
                 </c:pt>
                 <c:pt idx="44">
-                  <c:v>6.8836797745699688E-2</c:v>
+                  <c:v>0.17163396818253152</c:v>
                 </c:pt>
                 <c:pt idx="45">
-                  <c:v>7.2554638318625034E-2</c:v>
+                  <c:v>0.17516959075587743</c:v>
                 </c:pt>
                 <c:pt idx="46">
-                  <c:v>7.6325226028566354E-2</c:v>
+                  <c:v>0.17839272295802988</c:v>
                 </c:pt>
                 <c:pt idx="47">
-                  <c:v>8.0140842430892326E-2</c:v>
+                  <c:v>0.18131077796047496</c:v>
                 </c:pt>
                 <c:pt idx="48">
-                  <c:v>8.3993517838029275E-2</c:v>
+                  <c:v>0.18393422882553601</c:v>
                 </c:pt>
                 <c:pt idx="49">
-                  <c:v>8.787507372604586E-2</c:v>
+                  <c:v>0.18627617253555084</c:v>
                 </c:pt>
                 <c:pt idx="50">
-                  <c:v>9.1777167376563482E-2</c:v>
+                  <c:v>0.18835186512938695</c:v>
                 </c:pt>
                 <c:pt idx="51">
-                  <c:v>9.5691338403747092E-2</c:v>
+                  <c:v>0.19017824380056211</c:v>
                 </c:pt>
                 <c:pt idx="52">
-                  <c:v>9.9609056783910993E-2</c:v>
+                  <c:v>0.19177345124178691</c:v>
                 </c:pt>
                 <c:pt idx="53">
-                  <c:v>0.10352177197697486</c:v>
+                  <c:v>0.1931563763376668</c:v>
                 </c:pt>
                 <c:pt idx="54">
-                  <c:v>0.10742096270522571</c:v>
+                  <c:v>0.19434622360232301</c:v>
                 </c:pt>
                 <c:pt idx="55">
-                  <c:v>0.11129818693613261</c:v>
+                  <c:v>0.19536212164822028</c:v>
                 </c:pt>
                 <c:pt idx="56">
-                  <c:v>0.11514513160280658</c:v>
+                  <c:v>0.19622277858911699</c:v>
                 </c:pt>
                 <c:pt idx="57">
-                  <c:v>0.1189536615885099</c:v>
+                  <c:v>0.19694618976330103</c:v>
                 </c:pt>
                 <c:pt idx="58">
-                  <c:v>0.1227158675007039</c:v>
+                  <c:v>0.19754940065027685</c:v>
                 </c:pt>
                 <c:pt idx="59">
-                  <c:v>0.12642411176571153</c:v>
+                  <c:v>0.19804832547095644</c:v>
                 </c:pt>
                 <c:pt idx="60">
-                  <c:v>0.1300710725872542</c:v>
+                  <c:v>0.19845761981600954</c:v>
                 </c:pt>
                 <c:pt idx="61">
-                  <c:v>0.13364978533089925</c:v>
+                  <c:v>0.19879060382342864</c:v>
                 </c:pt>
                 <c:pt idx="62">
-                  <c:v>0.13715368092169056</c:v>
+                  <c:v>0.19905923098155251</c:v>
                 </c:pt>
                 <c:pt idx="63">
-                  <c:v>0.1405766208736767</c:v>
+                  <c:v>0.19927409659660289</c:v>
                 </c:pt>
                 <c:pt idx="64">
-                  <c:v>0.1439129286073208</c:v>
+                  <c:v>0.19944447933595111</c:v>
                 </c:pt>
                 <c:pt idx="65">
-                  <c:v>0.14715741675338276</c:v>
+                  <c:v>0.19957840901739385</c:v>
                 </c:pt>
                 <c:pt idx="66">
-                  <c:v>0.15030541018919724</c:v>
+                  <c:v>0.19968275391843365</c:v>
                 </c:pt>
                 <c:pt idx="67">
-                  <c:v>0.15335276460462463</c:v>
+                  <c:v>0.19976332127118276</c:v>
                 </c:pt>
                 <c:pt idx="68">
-                  <c:v>0.15629588044952777</c:v>
+                  <c:v>0.19982496522253218</c:v>
                 </c:pt>
                 <c:pt idx="69">
-                  <c:v>0.1591317121715517</c:v>
+                  <c:v>0.19987169730697774</c:v>
                 </c:pt>
                 <c:pt idx="70">
-                  <c:v>0.16185777271132257</c:v>
+                  <c:v>0.19990679533419684</c:v>
                 </c:pt>
                 <c:pt idx="71">
-                  <c:v>0.16447213328097302</c:v>
+                  <c:v>0.1999329074744195</c:v>
                 </c:pt>
                 <c:pt idx="72">
-                  <c:v>0.16697341851014097</c:v>
+                  <c:v>0.19995214918026516</c:v>
                 </c:pt>
                 <c:pt idx="73">
-                  <c:v>0.16936079710030458</c:v>
+                  <c:v>0.19996619137347427</c:v>
                 </c:pt>
                 <c:pt idx="74">
-                  <c:v>0.17163396818253152</c:v>
+                  <c:v>0.19997633902006273</c:v>
                 </c:pt>
                 <c:pt idx="75">
-                  <c:v>0.17379314362452247</c:v>
+                  <c:v>0.19998359980055544</c:v>
                 </c:pt>
                 <c:pt idx="76">
-                  <c:v>0.17583902657936101</c:v>
+                  <c:v>0.19998874304618811</c:v>
                 </c:pt>
                 <c:pt idx="77">
-                  <c:v>0.17777278660987564</c:v>
+                  <c:v>0.19999234945911523</c:v>
                 </c:pt>
                 <c:pt idx="78">
-                  <c:v>0.1795960317583036</c:v>
+                  <c:v>0.19999485237326678</c:v>
                 </c:pt>
                 <c:pt idx="79">
-                  <c:v>0.18131077796047496</c:v>
+                  <c:v>0.1999965714557792</c:v>
                 </c:pt>
                 <c:pt idx="80">
-                  <c:v>0.18291941622657948</c:v>
+                  <c:v>0.19999773981279137</c:v>
                 </c:pt>
                 <c:pt idx="81">
-                  <c:v>0.1844246780264579</c:v>
+                  <c:v>0.19999852546471561</c:v>
                 </c:pt>
                 <c:pt idx="82">
-                  <c:v>0.18582959932613019</c:v>
+                  <c:v>0.19999904811129313</c:v>
                 </c:pt>
                 <c:pt idx="83">
-                  <c:v>0.18713748372393824</c:v>
+                  <c:v>0.19999939203080119</c:v>
                 </c:pt>
                 <c:pt idx="84">
-                  <c:v>0.18835186512938695</c:v>
+                  <c:v>0.19999961586354192</c:v>
                 </c:pt>
                 <c:pt idx="85">
-                  <c:v>0.18947647041579807</c:v>
+                  <c:v>0.19999975992763294</c:v>
                 </c:pt>
                 <c:pt idx="86">
-                  <c:v>0.19051518245966237</c:v>
+                  <c:v>0.19999985161306397</c:v>
                 </c:pt>
                 <c:pt idx="87">
-                  <c:v>0.19147200395561312</c:v>
+                  <c:v>0.19999990930357772</c:v>
                 </c:pt>
                 <c:pt idx="88">
-                  <c:v>0.19235102236688295</c:v>
+                  <c:v>0.19999994518873965</c:v>
                 </c:pt>
                 <c:pt idx="89">
-                  <c:v>0.1931563763376668</c:v>
+                  <c:v>0.19999996725245739</c:v>
                 </c:pt>
                 <c:pt idx="90">
-                  <c:v>0.19389222385677296</c:v>
+                  <c:v>0.19999998065979441</c:v>
                 </c:pt>
                 <c:pt idx="91">
-                  <c:v>0.19456271242214007</c:v>
+                  <c:v>0.19999998871085503</c:v>
                 </c:pt>
                 <c:pt idx="92">
-                  <c:v>0.19517195141408158</c:v>
+                  <c:v>0.19999999348787459</c:v>
                 </c:pt>
                 <c:pt idx="93">
-                  <c:v>0.19572398684234746</c:v>
+                  <c:v>0.19999999628815057</c:v>
                 </c:pt>
                 <c:pt idx="94">
-                  <c:v>0.19622277858911699</c:v>
+                  <c:v>0.19999999790970302</c:v>
                 </c:pt>
                 <c:pt idx="95">
-                  <c:v>0.19667218022765529</c:v>
+                  <c:v>0.19999999883716038</c:v>
                 </c:pt>
                 <c:pt idx="96">
-                  <c:v>0.19707592145534147</c:v>
+                  <c:v>0.19999999936104543</c:v>
                 </c:pt>
                 <c:pt idx="97">
-                  <c:v>0.19743759314079234</c:v>
+                  <c:v>0.19999999965326104</c:v>
                 </c:pt>
                 <c:pt idx="98">
-                  <c:v>0.19776063494846641</c:v>
+                  <c:v>0.19999999981419306</c:v>
                 </c:pt>
                 <c:pt idx="99">
-                  <c:v>0.19804832547095644</c:v>
+                  <c:v>0.19999999990169129</c:v>
                 </c:pt>
                 <c:pt idx="100">
-                  <c:v>0.19830377476957428</c:v>
+                  <c:v>0.19999999994865042</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1350,124 +1350,124 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3.124975586055179E-6</c:v>
+                  <c:v>1.4467069327128713E-5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2.4998437565093568E-5</c:v>
+                  <c:v>1.1570725740235322E-4</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>8.435720465098662E-5</c:v>
+                  <c:v>3.9024377850489512E-4</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1.9990003332499563E-4</c:v>
+                  <c:v>9.2378588268478008E-4</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>3.9024377850489512E-4</c:v>
+                  <c:v>1.8002974421282847E-3</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>6.7386221786482905E-4</c:v>
+                  <c:v>3.1007125989183093E-3</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1.0690078343197351E-3</c:v>
+                  <c:v>4.9013271393022924E-3</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1.5936170325878685E-3</c:v>
+                  <c:v>7.2719111397427484E-3</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>2.2651994893083229E-3</c:v>
+                  <c:v>1.0273608123333956E-2</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>3.1007125989183093E-3</c:v>
+                  <c:v>1.3956707206263963E-2</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>4.1164222751643781E-3</c:v>
+                  <c:v>1.8358395818443476E-2</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>5.3277516951326436E-3</c:v>
+                  <c:v>2.3500619483080909E-2</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>6.7491199219383846E-3</c:v>
+                  <c:v>2.9388189488745109E-2</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>8.3937727050432676E-3</c:v>
+                  <c:v>3.6007286628151627E-2</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>1.0273608123333956E-2</c:v>
+                  <c:v>4.3324507187836363E-2</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>1.2399000093854107E-2</c:v>
+                  <c:v>5.1286584158818753E-2</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>1.4778623105350875E-2</c:v>
+                  <c:v>5.982089105991404E-2</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>1.7419281836388589E-2</c:v>
+                  <c:v>6.8836797745699688E-2</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>2.0325749567763896E-2</c:v>
+                  <c:v>7.8227898345377744E-2</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>2.3500619483080909E-2</c:v>
+                  <c:v>8.787507372604586E-2</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>2.6944173054590095E-2</c:v>
+                  <c:v>9.7650288683833367E-2</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>3.0654269719585427E-2</c:v>
+                  <c:v>0.10742096270522571</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>3.4626261953136429E-2</c:v>
+                  <c:v>0.11705469860772776</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>3.8852939625304075E-2</c:v>
+                  <c:v>0.12642411176571153</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>4.3324507187836363E-2</c:v>
+                  <c:v>0.13541147940361392</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>4.8028596762946157E-2</c:v>
+                  <c:v>0.1439129286073208</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>5.295031960576449E-2</c:v>
+                  <c:v>0.15184190514555035</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>5.8072357687958265E-2</c:v>
+                  <c:v>0.1591317121715517</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>6.3375096313577545E-2</c:v>
+                  <c:v>0.16573697488151984</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>6.8836797745699688E-2</c:v>
+                  <c:v>0.17163396818253152</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>7.4433814815514393E-2</c:v>
+                  <c:v>0.17681983138790913</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>8.0140842430892326E-2</c:v>
+                  <c:v>0.18131077796047496</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>8.5931203830453898E-2</c:v>
+                  <c:v>0.18513948060036278</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>9.1777167376563482E-2</c:v>
+                  <c:v>0.18835186512938695</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>9.7650288683833367E-2</c:v>
+                  <c:v>0.19100357564494788</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>0.10352177197697486</c:v>
+                  <c:v>0.1931563763376668</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>0.10936284380095161</c:v>
+                  <c:v>0.19487473347482187</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>0.11514513160280658</c:v>
+                  <c:v>0.19622277858911699</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>0.12084103929956716</c:v>
+                  <c:v>0.1972617973403015</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>0.12642411176571153</c:v>
+                  <c:v>0.19804832547095644</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1885,124 +1885,124 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3.124975586055179E-6</c:v>
+                  <c:v>1.4467069327128713E-5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2.4998437565093568E-5</c:v>
+                  <c:v>1.1570725740235322E-4</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>8.435720465098662E-5</c:v>
+                  <c:v>3.9024377850489512E-4</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1.9990003332499563E-4</c:v>
+                  <c:v>9.2378588268478008E-4</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>3.9024377850489512E-4</c:v>
+                  <c:v>1.8002974421282847E-3</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>6.7386221786482905E-4</c:v>
+                  <c:v>3.1007125989183093E-3</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1.0690078343197351E-3</c:v>
+                  <c:v>4.9013271393022924E-3</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1.5936170325878685E-3</c:v>
+                  <c:v>7.2719111397427484E-3</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>2.2651994893083229E-3</c:v>
+                  <c:v>1.0273608123333956E-2</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>3.1007125989183093E-3</c:v>
+                  <c:v>1.3956707206263963E-2</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>4.1164222751643781E-3</c:v>
+                  <c:v>1.8358395818443476E-2</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>5.3277516951326436E-3</c:v>
+                  <c:v>2.3500619483080909E-2</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>6.7491199219383846E-3</c:v>
+                  <c:v>2.9388189488745109E-2</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>8.3937727050432676E-3</c:v>
+                  <c:v>3.6007286628151627E-2</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>1.0273608123333956E-2</c:v>
+                  <c:v>4.3324507187836363E-2</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>1.2399000093854107E-2</c:v>
+                  <c:v>5.1286584158818753E-2</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>1.4778623105350875E-2</c:v>
+                  <c:v>5.982089105991404E-2</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>1.7419281836388589E-2</c:v>
+                  <c:v>6.8836797745699688E-2</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>2.0325749567763896E-2</c:v>
+                  <c:v>7.8227898345377744E-2</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>2.3500619483080909E-2</c:v>
+                  <c:v>8.787507372604586E-2</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>2.6944173054590095E-2</c:v>
+                  <c:v>9.7650288683833367E-2</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>3.0654269719585427E-2</c:v>
+                  <c:v>0.10742096270522571</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>3.4626261953136429E-2</c:v>
+                  <c:v>0.11705469860772776</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>3.8852939625304075E-2</c:v>
+                  <c:v>0.12642411176571153</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>4.3324507187836363E-2</c:v>
+                  <c:v>0.13541147940361392</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>4.8028596762946157E-2</c:v>
+                  <c:v>0.1439129286073208</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>5.295031960576449E-2</c:v>
+                  <c:v>0.15184190514555035</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>5.8072357687958265E-2</c:v>
+                  <c:v>0.1591317121715517</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>6.3375096313577545E-2</c:v>
+                  <c:v>0.16573697488151984</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>6.8836797745699688E-2</c:v>
+                  <c:v>0.17163396818253152</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>7.4433814815514393E-2</c:v>
+                  <c:v>0.17681983138790913</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>8.0140842430892326E-2</c:v>
+                  <c:v>0.18131077796047496</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>8.5931203830453898E-2</c:v>
+                  <c:v>0.18513948060036278</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>9.1777167376563482E-2</c:v>
+                  <c:v>0.18835186512938695</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>9.7650288683833367E-2</c:v>
+                  <c:v>0.19100357564494788</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>0.10352177197697486</c:v>
+                  <c:v>0.1931563763376668</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>0.10936284380095161</c:v>
+                  <c:v>0.19487473347482187</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>0.11514513160280658</c:v>
+                  <c:v>0.19622277858911699</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>0.12084103929956716</c:v>
+                  <c:v>0.1972617973403015</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>0.12642411176571153</c:v>
+                  <c:v>0.19804832547095644</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4287,28 +4287,28 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D3D2DEE-686E-48A0-AC3D-0F54DEA5D0EC}">
   <dimension ref="A1:C125"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="88.7265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="88.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
@@ -4316,45 +4316,45 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>36</v>
       </c>
@@ -4362,7 +4362,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>34</v>
       </c>
@@ -4370,7 +4370,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>35</v>
       </c>
@@ -4378,7 +4378,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>37</v>
       </c>
@@ -4386,15 +4386,15 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>38</v>
       </c>
       <c r="B20">
-        <v>50000</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>45</v>
       </c>
@@ -4402,7 +4402,7 @@
         <v>4.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B24">
         <f>(1-EXP(-((C24/$B$20-($B$19-0.5))/$B$17)^$B$18))*$B$16</f>
         <v>0</v>
@@ -4411,1008 +4411,1008 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B25">
         <f t="shared" ref="B25:B88" si="0">(1-EXP(-((C25/$B$20-($B$19-0.5))/$B$17)^$B$18))*$B$16</f>
-        <v>9.259237825798295E-7</v>
+        <v>4.286648162477036E-6</v>
       </c>
       <c r="C25">
         <v>500</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B26">
         <f t="shared" si="0"/>
-        <v>7.4072702348937371E-6</v>
+        <v>3.4290612860687911E-5</v>
       </c>
       <c r="C26">
         <v>1000</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B27">
         <f t="shared" si="0"/>
-        <v>2.4998437565093568E-5</v>
+        <v>1.1570725740235322E-4</v>
       </c>
       <c r="C27">
         <f>C26+500</f>
         <v>1500</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B28">
         <f t="shared" si="0"/>
-        <v>5.9250480976746905E-5</v>
+        <v>2.7416034086391594E-4</v>
       </c>
       <c r="C28">
         <f t="shared" ref="C28:C91" si="1">C27+500</f>
         <v>2000</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B29">
         <f t="shared" si="0"/>
-        <v>1.1570725740235322E-4</v>
+        <v>5.3511960071055413E-4</v>
       </c>
       <c r="C29">
         <f t="shared" si="1"/>
         <v>2500</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B30">
         <f t="shared" si="0"/>
-        <v>1.9990003332499563E-4</v>
+        <v>9.2378588268478008E-4</v>
       </c>
       <c r="C30">
         <f t="shared" si="1"/>
         <v>3000</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B31">
         <f t="shared" si="0"/>
-        <v>3.173405633774218E-4</v>
+        <v>1.4649445766562463E-3</v>
       </c>
       <c r="C31">
         <f t="shared" si="1"/>
         <v>3500</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B32">
         <f t="shared" si="0"/>
-        <v>4.7351265218500418E-4</v>
+        <v>2.1827885823227922E-3</v>
       </c>
       <c r="C32">
         <f t="shared" si="1"/>
         <v>4000</v>
       </c>
     </row>
-    <row r="33" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B33">
         <f t="shared" si="0"/>
-        <v>6.7386221786482905E-4</v>
+        <v>3.1007125989183093E-3</v>
       </c>
       <c r="C33">
         <f t="shared" si="1"/>
         <v>4500</v>
       </c>
     </row>
-    <row r="34" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B34">
         <f t="shared" si="0"/>
-        <v>9.2378588268478008E-4</v>
+        <v>4.2410811978808027E-3</v>
       </c>
       <c r="C34">
         <f t="shared" si="1"/>
         <v>5000</v>
       </c>
     </row>
-    <row r="35" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B35">
         <f t="shared" si="0"/>
-        <v>1.2286181245915852E-3</v>
+        <v>5.6249738820245872E-3</v>
       </c>
       <c r="C35">
         <f t="shared" si="1"/>
         <v>5500</v>
       </c>
     </row>
-    <row r="36" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B36">
         <f t="shared" si="0"/>
-        <v>1.5936170325878685E-3</v>
+        <v>7.2719111397427484E-3</v>
       </c>
       <c r="C36">
         <f t="shared" si="1"/>
         <v>6000</v>
       </c>
     </row>
-    <row r="37" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B37">
         <f t="shared" si="0"/>
-        <v>2.0239487192203367E-3</v>
+        <v>9.1995663437769003E-3</v>
       </c>
       <c r="C37">
         <f t="shared" si="1"/>
         <v>6500</v>
       </c>
     </row>
-    <row r="38" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B38">
         <f t="shared" si="0"/>
-        <v>2.5246704546594725E-3</v>
+        <v>1.1423469191788382E-2</v>
       </c>
       <c r="C38">
         <f t="shared" si="1"/>
         <v>7000</v>
       </c>
     </row>
-    <row r="39" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B39">
         <f t="shared" si="0"/>
-        <v>3.1007125989183093E-3</v>
+        <v>1.3956707206263963E-2</v>
       </c>
       <c r="C39">
         <f t="shared" si="1"/>
         <v>7500</v>
       </c>
     </row>
-    <row r="40" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B40">
         <f t="shared" si="0"/>
-        <v>3.756859421568759E-3</v>
+        <v>1.6809632565965439E-2</v>
       </c>
       <c r="C40">
         <f t="shared" si="1"/>
         <v>8000</v>
       </c>
     </row>
-    <row r="41" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B41">
         <f t="shared" si="0"/>
-        <v>4.4977289117446254E-3</v>
+        <v>1.9989582188770449E-2</v>
       </c>
       <c r="C41">
         <f t="shared" si="1"/>
         <v>8500</v>
       </c>
     </row>
-    <row r="42" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B42">
         <f t="shared" si="0"/>
-        <v>5.3277516951326436E-3</v>
+        <v>2.3500619483080909E-2</v>
       </c>
       <c r="C42">
         <f t="shared" si="1"/>
         <v>9000</v>
       </c>
     </row>
-    <row r="43" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B43">
         <f t="shared" si="0"/>
-        <v>6.2511491888826987E-3</v>
+        <v>2.7343306488591249E-2</v>
       </c>
       <c r="C43">
         <f t="shared" si="1"/>
         <v>9500</v>
       </c>
     </row>
-    <row r="44" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B44">
         <f t="shared" si="0"/>
-        <v>7.2719111397427484E-3</v>
+        <v>3.1514515195616613E-2</v>
       </c>
       <c r="C44">
         <f t="shared" si="1"/>
         <v>10000</v>
       </c>
     </row>
-    <row r="45" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="45" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B45">
         <f t="shared" si="0"/>
-        <v>8.3937727050432676E-3</v>
+        <v>3.6007286628151627E-2</v>
       </c>
       <c r="C45">
         <f t="shared" si="1"/>
         <v>10500</v>
       </c>
     </row>
-    <row r="46" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B46">
         <f t="shared" si="0"/>
-        <v>9.6201912502106527E-3</v>
+        <v>4.0810745768913415E-2</v>
       </c>
       <c r="C46">
         <f t="shared" si="1"/>
         <v>11000</v>
       </c>
     </row>
-    <row r="47" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B47">
         <f t="shared" si="0"/>
-        <v>1.0954323050048865E-2</v>
+        <v>4.5910079573753593E-2</v>
       </c>
       <c r="C47">
         <f t="shared" si="1"/>
         <v>11500</v>
       </c>
     </row>
-    <row r="48" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B48">
         <f t="shared" si="0"/>
-        <v>1.2399000093854107E-2</v>
+        <v>5.1286584158818753E-2</v>
       </c>
       <c r="C48">
         <f t="shared" si="1"/>
         <v>12000</v>
       </c>
     </row>
-    <row r="49" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="49" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B49">
         <f t="shared" si="0"/>
-        <v>1.3956707206263963E-2</v>
+        <v>5.6917785751641151E-2</v>
       </c>
       <c r="C49">
         <f t="shared" si="1"/>
         <v>12500</v>
       </c>
     </row>
-    <row r="50" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="50" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B50">
         <f t="shared" si="0"/>
-        <v>1.5629559706331463E-2</v>
+        <v>6.2777638197790697E-2</v>
       </c>
       <c r="C50">
         <f t="shared" si="1"/>
         <v>13000</v>
       </c>
     </row>
-    <row r="51" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="51" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B51">
         <f t="shared" si="0"/>
-        <v>1.7419281836388589E-2</v>
+        <v>6.8836797745699688E-2</v>
       </c>
       <c r="C51">
         <f t="shared" si="1"/>
         <v>13500</v>
       </c>
     </row>
-    <row r="52" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="52" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B52">
         <f t="shared" si="0"/>
-        <v>1.9327186199557179E-2</v>
+        <v>7.506297354898428E-2</v>
       </c>
       <c r="C52">
         <f t="shared" si="1"/>
         <v>14000</v>
       </c>
     </row>
-    <row r="53" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="53" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B53">
         <f t="shared" si="0"/>
-        <v>2.1354154450015608E-2</v>
+        <v>8.142134989988481E-2</v>
       </c>
       <c r="C53">
         <f t="shared" si="1"/>
         <v>14500</v>
       </c>
     </row>
-    <row r="54" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="54" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B54">
         <f t="shared" si="0"/>
-        <v>2.3500619483080909E-2</v>
+        <v>8.787507372604586E-2</v>
       </c>
       <c r="C54">
         <f t="shared" si="1"/>
         <v>15000</v>
       </c>
     </row>
-    <row r="55" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="55" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B55">
         <f t="shared" si="0"/>
-        <v>2.5766549372577496E-2</v>
+        <v>9.438579844442066E-2</v>
       </c>
       <c r="C55">
         <f t="shared" si="1"/>
         <v>15500</v>
       </c>
     </row>
-    <row r="56" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="56" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B56">
         <f t="shared" si="0"/>
-        <v>2.8151433300614783E-2</v>
+        <v>0.10091427297723279</v>
       </c>
       <c r="C56">
         <f t="shared" si="1"/>
         <v>16000</v>
       </c>
     </row>
-    <row r="57" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="57" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B57">
         <f t="shared" si="0"/>
-        <v>3.0654269719585427E-2</v>
+        <v>0.10742096270522571</v>
       </c>
       <c r="C57">
         <f t="shared" si="1"/>
         <v>16500</v>
       </c>
     </row>
-    <row r="58" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="58" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B58">
         <f t="shared" si="0"/>
-        <v>3.3273556977759113E-2</v>
+        <v>0.11386668746965854</v>
       </c>
       <c r="C58">
         <f t="shared" si="1"/>
         <v>17000</v>
       </c>
     </row>
-    <row r="59" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="59" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B59">
         <f t="shared" si="0"/>
-        <v>3.6007286628151627E-2</v>
+        <v>0.12021326053442474</v>
       </c>
       <c r="C59">
         <f t="shared" si="1"/>
         <v>17500</v>
       </c>
     </row>
-    <row r="60" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="60" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B60">
         <f t="shared" si="0"/>
-        <v>3.8852939625304075E-2</v>
+        <v>0.12642411176571153</v>
       </c>
       <c r="C60">
         <f t="shared" si="1"/>
         <v>18000</v>
       </c>
     </row>
-    <row r="61" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="61" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B61">
         <f t="shared" si="0"/>
-        <v>4.1807485596171513E-2</v>
+        <v>0.1324648782399141</v>
       </c>
       <c r="C61">
         <f t="shared" si="1"/>
         <v>18500</v>
       </c>
     </row>
-    <row r="62" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="62" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B62">
         <f t="shared" si="0"/>
-        <v>4.4867385349501548E-2</v>
+        <v>0.1383039460856948</v>
       </c>
       <c r="C62">
         <f t="shared" si="1"/>
         <v>19000</v>
       </c>
     </row>
-    <row r="63" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="63" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B63">
         <f t="shared" si="0"/>
-        <v>4.8028596762946157E-2</v>
+        <v>0.1439129286073208</v>
       </c>
       <c r="C63">
         <f t="shared" si="1"/>
         <v>19500</v>
       </c>
     </row>
-    <row r="64" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="64" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B64">
         <f t="shared" si="0"/>
-        <v>5.1286584158818753E-2</v>
+        <v>0.14926706759510625</v>
       </c>
       <c r="C64">
         <f t="shared" si="1"/>
         <v>20000</v>
       </c>
     </row>
-    <row r="65" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="65" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B65">
         <f t="shared" si="0"/>
-        <v>5.4636331248070019E-2</v>
+        <v>0.15434554714316789</v>
       </c>
       <c r="C65">
         <f t="shared" si="1"/>
         <v>20500</v>
       </c>
     </row>
-    <row r="66" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="66" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B66">
         <f t="shared" si="0"/>
-        <v>5.8072357687958265E-2</v>
+        <v>0.1591317121715517</v>
       </c>
       <c r="C66">
         <f t="shared" si="1"/>
         <v>21000</v>
       </c>
     </row>
-    <row r="67" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="67" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B67">
         <f t="shared" si="0"/>
-        <v>6.1588739262348917E-2</v>
+        <v>0.16361318706836692</v>
       </c>
       <c r="C67">
         <f t="shared" si="1"/>
         <v>21500</v>
       </c>
     </row>
-    <row r="68" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="68" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B68">
         <f t="shared" si="0"/>
-        <v>6.5179131654968622E-2</v>
+        <v>0.16778189328550838</v>
       </c>
       <c r="C68">
         <f t="shared" si="1"/>
         <v>22000</v>
       </c>
     </row>
-    <row r="69" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="69" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B69">
         <f t="shared" si="0"/>
-        <v>6.8836797745699688E-2</v>
+        <v>0.17163396818253152</v>
       </c>
       <c r="C69">
         <f t="shared" si="1"/>
         <v>22500</v>
       </c>
     </row>
-    <row r="70" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="70" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B70">
         <f t="shared" si="0"/>
-        <v>7.2554638318625034E-2</v>
+        <v>0.17516959075587743</v>
       </c>
       <c r="C70">
         <f t="shared" si="1"/>
         <v>23000</v>
       </c>
     </row>
-    <row r="71" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="71" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B71">
         <f t="shared" si="0"/>
-        <v>7.6325226028566354E-2</v>
+        <v>0.17839272295802988</v>
       </c>
       <c r="C71">
         <f t="shared" si="1"/>
         <v>23500</v>
       </c>
     </row>
-    <row r="72" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="72" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B72">
         <f t="shared" si="0"/>
-        <v>8.0140842430892326E-2</v>
+        <v>0.18131077796047496</v>
       </c>
       <c r="C72">
         <f t="shared" si="1"/>
         <v>24000</v>
       </c>
     </row>
-    <row r="73" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="73" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B73">
         <f t="shared" si="0"/>
-        <v>8.3993517838029275E-2</v>
+        <v>0.18393422882553601</v>
       </c>
       <c r="C73">
         <f t="shared" si="1"/>
         <v>24500</v>
       </c>
     </row>
-    <row r="74" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="74" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B74">
         <f t="shared" si="0"/>
-        <v>8.787507372604586E-2</v>
+        <v>0.18627617253555084</v>
       </c>
       <c r="C74">
         <f t="shared" si="1"/>
         <v>25000</v>
       </c>
     </row>
-    <row r="75" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="75" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B75">
         <f t="shared" si="0"/>
-        <v>9.1777167376563482E-2</v>
+        <v>0.18835186512938695</v>
       </c>
       <c r="C75">
         <f t="shared" si="1"/>
         <v>25500</v>
       </c>
     </row>
-    <row r="76" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="76" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B76">
         <f t="shared" si="0"/>
-        <v>9.5691338403747092E-2</v>
+        <v>0.19017824380056211</v>
       </c>
       <c r="C76">
         <f t="shared" si="1"/>
         <v>26000</v>
       </c>
     </row>
-    <row r="77" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="77" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B77">
         <f t="shared" si="0"/>
-        <v>9.9609056783910993E-2</v>
+        <v>0.19177345124178691</v>
       </c>
       <c r="C77">
         <f t="shared" si="1"/>
         <v>26500</v>
       </c>
     </row>
-    <row r="78" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="78" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B78">
         <f t="shared" si="0"/>
-        <v>0.10352177197697486</v>
+        <v>0.1931563763376668</v>
       </c>
       <c r="C78">
         <f t="shared" si="1"/>
         <v>27000</v>
       </c>
     </row>
-    <row r="79" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="79" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B79">
         <f t="shared" si="0"/>
-        <v>0.10742096270522571</v>
+        <v>0.19434622360232301</v>
       </c>
       <c r="C79">
         <f t="shared" si="1"/>
         <v>27500</v>
       </c>
     </row>
-    <row r="80" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="80" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B80">
         <f t="shared" si="0"/>
-        <v>0.11129818693613261</v>
+        <v>0.19536212164822028</v>
       </c>
       <c r="C80">
         <f t="shared" si="1"/>
         <v>28000</v>
       </c>
     </row>
-    <row r="81" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="81" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B81">
         <f t="shared" si="0"/>
-        <v>0.11514513160280658</v>
+        <v>0.19622277858911699</v>
       </c>
       <c r="C81">
         <f t="shared" si="1"/>
         <v>28500</v>
       </c>
     </row>
-    <row r="82" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="82" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B82">
         <f t="shared" si="0"/>
-        <v>0.1189536615885099</v>
+        <v>0.19694618976330103</v>
       </c>
       <c r="C82">
         <f t="shared" si="1"/>
         <v>29000</v>
       </c>
     </row>
-    <row r="83" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="83" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B83">
         <f t="shared" si="0"/>
-        <v>0.1227158675007039</v>
+        <v>0.19754940065027685</v>
       </c>
       <c r="C83">
         <f t="shared" si="1"/>
         <v>29500</v>
       </c>
     </row>
-    <row r="84" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="84" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B84">
         <f t="shared" si="0"/>
-        <v>0.12642411176571153</v>
+        <v>0.19804832547095644</v>
       </c>
       <c r="C84">
         <f t="shared" si="1"/>
         <v>30000</v>
       </c>
     </row>
-    <row r="85" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="85" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B85">
         <f t="shared" si="0"/>
-        <v>0.1300710725872542</v>
+        <v>0.19845761981600954</v>
       </c>
       <c r="C85">
         <f t="shared" si="1"/>
         <v>30500</v>
       </c>
     </row>
-    <row r="86" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="86" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B86">
         <f t="shared" si="0"/>
-        <v>0.13364978533089925</v>
+        <v>0.19879060382342864</v>
       </c>
       <c r="C86">
         <f t="shared" si="1"/>
         <v>31000</v>
       </c>
     </row>
-    <row r="87" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="87" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B87">
         <f t="shared" si="0"/>
-        <v>0.13715368092169056</v>
+        <v>0.19905923098155251</v>
       </c>
       <c r="C87">
         <f t="shared" si="1"/>
         <v>31500</v>
       </c>
     </row>
-    <row r="88" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="88" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B88">
         <f t="shared" si="0"/>
-        <v>0.1405766208736767</v>
+        <v>0.19927409659660289</v>
       </c>
       <c r="C88">
         <f t="shared" si="1"/>
         <v>32000</v>
       </c>
     </row>
-    <row r="89" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="89" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B89">
         <f t="shared" ref="B89:B125" si="2">(1-EXP(-((C89/$B$20-($B$19-0.5))/$B$17)^$B$18))*$B$16</f>
-        <v>0.1439129286073208</v>
+        <v>0.19944447933595111</v>
       </c>
       <c r="C89">
         <f t="shared" si="1"/>
         <v>32500</v>
       </c>
     </row>
-    <row r="90" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="90" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B90">
         <f t="shared" si="2"/>
-        <v>0.14715741675338276</v>
+        <v>0.19957840901739385</v>
       </c>
       <c r="C90">
         <f t="shared" si="1"/>
         <v>33000</v>
       </c>
     </row>
-    <row r="91" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="91" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B91">
         <f t="shared" si="2"/>
-        <v>0.15030541018919724</v>
+        <v>0.19968275391843365</v>
       </c>
       <c r="C91">
         <f t="shared" si="1"/>
         <v>33500</v>
       </c>
     </row>
-    <row r="92" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="92" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B92">
         <f t="shared" si="2"/>
-        <v>0.15335276460462463</v>
+        <v>0.19976332127118276</v>
       </c>
       <c r="C92">
         <f t="shared" ref="C92:C125" si="3">C91+500</f>
         <v>34000</v>
       </c>
     </row>
-    <row r="93" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="93" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B93">
         <f t="shared" si="2"/>
-        <v>0.15629588044952777</v>
+        <v>0.19982496522253218</v>
       </c>
       <c r="C93">
         <f t="shared" si="3"/>
         <v>34500</v>
       </c>
     </row>
-    <row r="94" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="94" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B94">
         <f t="shared" si="2"/>
-        <v>0.1591317121715517</v>
+        <v>0.19987169730697774</v>
       </c>
       <c r="C94">
         <f t="shared" si="3"/>
         <v>35000</v>
       </c>
     </row>
-    <row r="95" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="95" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B95">
         <f t="shared" si="2"/>
-        <v>0.16185777271132257</v>
+        <v>0.19990679533419684</v>
       </c>
       <c r="C95">
         <f t="shared" si="3"/>
         <v>35500</v>
       </c>
     </row>
-    <row r="96" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="96" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B96">
         <f t="shared" si="2"/>
-        <v>0.16447213328097302</v>
+        <v>0.1999329074744195</v>
       </c>
       <c r="C96">
         <f t="shared" si="3"/>
         <v>36000</v>
       </c>
     </row>
-    <row r="97" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="97" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B97">
         <f t="shared" si="2"/>
-        <v>0.16697341851014097</v>
+        <v>0.19995214918026516</v>
       </c>
       <c r="C97">
         <f t="shared" si="3"/>
         <v>36500</v>
       </c>
     </row>
-    <row r="98" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="98" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B98">
         <f t="shared" si="2"/>
-        <v>0.16936079710030458</v>
+        <v>0.19996619137347427</v>
       </c>
       <c r="C98">
         <f t="shared" si="3"/>
         <v>37000</v>
       </c>
     </row>
-    <row r="99" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="99" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B99">
         <f t="shared" si="2"/>
-        <v>0.17163396818253152</v>
+        <v>0.19997633902006273</v>
       </c>
       <c r="C99">
         <f t="shared" si="3"/>
         <v>37500</v>
       </c>
     </row>
-    <row r="100" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="100" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B100">
         <f t="shared" si="2"/>
-        <v>0.17379314362452247</v>
+        <v>0.19998359980055544</v>
       </c>
       <c r="C100">
         <f t="shared" si="3"/>
         <v>38000</v>
       </c>
     </row>
-    <row r="101" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="101" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B101">
         <f t="shared" si="2"/>
-        <v>0.17583902657936101</v>
+        <v>0.19998874304618811</v>
       </c>
       <c r="C101">
         <f t="shared" si="3"/>
         <v>38500</v>
       </c>
     </row>
-    <row r="102" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="102" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B102">
         <f t="shared" si="2"/>
-        <v>0.17777278660987564</v>
+        <v>0.19999234945911523</v>
       </c>
       <c r="C102">
         <f t="shared" si="3"/>
         <v>39000</v>
       </c>
     </row>
-    <row r="103" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="103" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B103">
         <f t="shared" si="2"/>
-        <v>0.1795960317583036</v>
+        <v>0.19999485237326678</v>
       </c>
       <c r="C103">
         <f t="shared" si="3"/>
         <v>39500</v>
       </c>
     </row>
-    <row r="104" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="104" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B104">
         <f t="shared" si="2"/>
-        <v>0.18131077796047496</v>
+        <v>0.1999965714557792</v>
       </c>
       <c r="C104">
         <f t="shared" si="3"/>
         <v>40000</v>
       </c>
     </row>
-    <row r="105" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="105" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B105">
         <f t="shared" si="2"/>
-        <v>0.18291941622657948</v>
+        <v>0.19999773981279137</v>
       </c>
       <c r="C105">
         <f t="shared" si="3"/>
         <v>40500</v>
       </c>
     </row>
-    <row r="106" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="106" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B106">
         <f t="shared" si="2"/>
-        <v>0.1844246780264579</v>
+        <v>0.19999852546471561</v>
       </c>
       <c r="C106">
         <f t="shared" si="3"/>
         <v>41000</v>
       </c>
     </row>
-    <row r="107" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="107" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B107">
         <f t="shared" si="2"/>
-        <v>0.18582959932613019</v>
+        <v>0.19999904811129313</v>
       </c>
       <c r="C107">
         <f t="shared" si="3"/>
         <v>41500</v>
       </c>
     </row>
-    <row r="108" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="108" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B108">
         <f t="shared" si="2"/>
-        <v>0.18713748372393824</v>
+        <v>0.19999939203080119</v>
       </c>
       <c r="C108">
         <f t="shared" si="3"/>
         <v>42000</v>
       </c>
     </row>
-    <row r="109" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="109" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B109">
         <f t="shared" si="2"/>
-        <v>0.18835186512938695</v>
+        <v>0.19999961586354192</v>
       </c>
       <c r="C109">
         <f t="shared" si="3"/>
         <v>42500</v>
       </c>
     </row>
-    <row r="110" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="110" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B110">
         <f t="shared" si="2"/>
-        <v>0.18947647041579807</v>
+        <v>0.19999975992763294</v>
       </c>
       <c r="C110">
         <f t="shared" si="3"/>
         <v>43000</v>
       </c>
     </row>
-    <row r="111" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="111" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B111">
         <f t="shared" si="2"/>
-        <v>0.19051518245966237</v>
+        <v>0.19999985161306397</v>
       </c>
       <c r="C111">
         <f t="shared" si="3"/>
         <v>43500</v>
       </c>
     </row>
-    <row r="112" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="112" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B112">
         <f t="shared" si="2"/>
-        <v>0.19147200395561312</v>
+        <v>0.19999990930357772</v>
       </c>
       <c r="C112">
         <f t="shared" si="3"/>
         <v>44000</v>
       </c>
     </row>
-    <row r="113" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="113" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B113">
         <f t="shared" si="2"/>
-        <v>0.19235102236688295</v>
+        <v>0.19999994518873965</v>
       </c>
       <c r="C113">
         <f t="shared" si="3"/>
         <v>44500</v>
       </c>
     </row>
-    <row r="114" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="114" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B114">
         <f t="shared" si="2"/>
-        <v>0.1931563763376668</v>
+        <v>0.19999996725245739</v>
       </c>
       <c r="C114">
         <f t="shared" si="3"/>
         <v>45000</v>
       </c>
     </row>
-    <row r="115" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="115" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B115">
         <f t="shared" si="2"/>
-        <v>0.19389222385677296</v>
+        <v>0.19999998065979441</v>
       </c>
       <c r="C115">
         <f t="shared" si="3"/>
         <v>45500</v>
       </c>
     </row>
-    <row r="116" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="116" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B116">
         <f t="shared" si="2"/>
-        <v>0.19456271242214007</v>
+        <v>0.19999998871085503</v>
       </c>
       <c r="C116">
         <f t="shared" si="3"/>
         <v>46000</v>
       </c>
     </row>
-    <row r="117" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="117" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B117">
         <f t="shared" si="2"/>
-        <v>0.19517195141408158</v>
+        <v>0.19999999348787459</v>
       </c>
       <c r="C117">
         <f t="shared" si="3"/>
         <v>46500</v>
       </c>
     </row>
-    <row r="118" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="118" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B118">
         <f t="shared" si="2"/>
-        <v>0.19572398684234746</v>
+        <v>0.19999999628815057</v>
       </c>
       <c r="C118">
         <f t="shared" si="3"/>
         <v>47000</v>
       </c>
     </row>
-    <row r="119" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="119" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B119">
         <f t="shared" si="2"/>
-        <v>0.19622277858911699</v>
+        <v>0.19999999790970302</v>
       </c>
       <c r="C119">
         <f t="shared" si="3"/>
         <v>47500</v>
       </c>
     </row>
-    <row r="120" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="120" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B120">
         <f t="shared" si="2"/>
-        <v>0.19667218022765529</v>
+        <v>0.19999999883716038</v>
       </c>
       <c r="C120">
         <f t="shared" si="3"/>
         <v>48000</v>
       </c>
     </row>
-    <row r="121" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="121" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B121">
         <f t="shared" si="2"/>
-        <v>0.19707592145534147</v>
+        <v>0.19999999936104543</v>
       </c>
       <c r="C121">
         <f t="shared" si="3"/>
         <v>48500</v>
       </c>
     </row>
-    <row r="122" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="122" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B122">
         <f t="shared" si="2"/>
-        <v>0.19743759314079234</v>
+        <v>0.19999999965326104</v>
       </c>
       <c r="C122">
         <f t="shared" si="3"/>
         <v>49000</v>
       </c>
     </row>
-    <row r="123" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="123" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B123">
         <f t="shared" si="2"/>
-        <v>0.19776063494846641</v>
+        <v>0.19999999981419306</v>
       </c>
       <c r="C123">
         <f t="shared" si="3"/>
         <v>49500</v>
       </c>
     </row>
-    <row r="124" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="124" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B124">
         <f t="shared" si="2"/>
-        <v>0.19804832547095644</v>
+        <v>0.19999999990169129</v>
       </c>
       <c r="C124">
         <f t="shared" si="3"/>
         <v>50000</v>
       </c>
     </row>
-    <row r="125" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="125" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B125">
         <f t="shared" si="2"/>
-        <v>0.19830377476957428</v>
+        <v>0.19999999994865042</v>
       </c>
       <c r="C125">
         <f t="shared" si="3"/>
@@ -5431,13 +5431,13 @@
     <tabColor rgb="FF002060"/>
   </sheetPr>
   <dimension ref="A1:CF2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:84" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:84" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -5447,334 +5447,334 @@
       </c>
       <c r="C1">
         <f>(1-EXP(-((C2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>3.124975586055179E-6</v>
+        <v>1.4467069327128713E-5</v>
       </c>
       <c r="D1">
         <f>(1-EXP(-((D2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>2.4998437565093568E-5</v>
+        <v>1.1570725740235322E-4</v>
       </c>
       <c r="E1">
         <f>(1-EXP(-((E2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>8.435720465098662E-5</v>
+        <v>3.9024377850489512E-4</v>
       </c>
       <c r="F1">
         <f>(1-EXP(-((F2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>1.9990003332499563E-4</v>
+        <v>9.2378588268478008E-4</v>
       </c>
       <c r="G1">
         <f>(1-EXP(-((G2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>3.9024377850489512E-4</v>
+        <v>1.8002974421282847E-3</v>
       </c>
       <c r="H1">
         <f>(1-EXP(-((H2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>6.7386221786482905E-4</v>
+        <v>3.1007125989183093E-3</v>
       </c>
       <c r="I1">
         <f>(1-EXP(-((I2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>1.0690078343197351E-3</v>
+        <v>4.9013271393022924E-3</v>
       </c>
       <c r="J1">
         <f>(1-EXP(-((J2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>1.5936170325878685E-3</v>
+        <v>7.2719111397427484E-3</v>
       </c>
       <c r="K1">
         <f>(1-EXP(-((K2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>2.2651994893083229E-3</v>
+        <v>1.0273608123333956E-2</v>
       </c>
       <c r="L1">
         <f>(1-EXP(-((L2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>3.1007125989183093E-3</v>
+        <v>1.3956707206263963E-2</v>
       </c>
       <c r="M1">
         <f>(1-EXP(-((M2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>4.1164222751643781E-3</v>
+        <v>1.8358395818443476E-2</v>
       </c>
       <c r="N1">
         <f>(1-EXP(-((N2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>5.3277516951326436E-3</v>
+        <v>2.3500619483080909E-2</v>
       </c>
       <c r="O1">
         <f>(1-EXP(-((O2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>6.7491199219383846E-3</v>
+        <v>2.9388189488745109E-2</v>
       </c>
       <c r="P1">
         <f>(1-EXP(-((P2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>8.3937727050432676E-3</v>
+        <v>3.6007286628151627E-2</v>
       </c>
       <c r="Q1">
         <f>(1-EXP(-((Q2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>1.0273608123333956E-2</v>
+        <v>4.3324507187836363E-2</v>
       </c>
       <c r="R1">
         <f>(1-EXP(-((R2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>1.2399000093854107E-2</v>
+        <v>5.1286584158818753E-2</v>
       </c>
       <c r="S1">
         <f>(1-EXP(-((S2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>1.4778623105350875E-2</v>
+        <v>5.982089105991404E-2</v>
       </c>
       <c r="T1">
         <f>(1-EXP(-((T2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>1.7419281836388589E-2</v>
+        <v>6.8836797745699688E-2</v>
       </c>
       <c r="U1">
         <f>(1-EXP(-((U2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>2.0325749567763896E-2</v>
+        <v>7.8227898345377744E-2</v>
       </c>
       <c r="V1">
         <f>(1-EXP(-((V2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>2.3500619483080909E-2</v>
+        <v>8.787507372604586E-2</v>
       </c>
       <c r="W1">
         <f>(1-EXP(-((W2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>2.6944173054590095E-2</v>
+        <v>9.7650288683833367E-2</v>
       </c>
       <c r="X1">
         <f>(1-EXP(-((X2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>3.0654269719585427E-2</v>
+        <v>0.10742096270522571</v>
       </c>
       <c r="Y1">
         <f>(1-EXP(-((Y2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>3.4626261953136429E-2</v>
+        <v>0.11705469860772776</v>
       </c>
       <c r="Z1">
         <f>(1-EXP(-((Z2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>3.8852939625304075E-2</v>
+        <v>0.12642411176571153</v>
       </c>
       <c r="AA1">
         <f>(1-EXP(-((AA2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>4.3324507187836363E-2</v>
+        <v>0.13541147940361392</v>
       </c>
       <c r="AB1">
         <f>(1-EXP(-((AB2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>4.8028596762946157E-2</v>
+        <v>0.1439129286073208</v>
       </c>
       <c r="AC1">
         <f>(1-EXP(-((AC2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>5.295031960576449E-2</v>
+        <v>0.15184190514555035</v>
       </c>
       <c r="AD1">
         <f>(1-EXP(-((AD2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>5.8072357687958265E-2</v>
+        <v>0.1591317121715517</v>
       </c>
       <c r="AE1">
         <f>(1-EXP(-((AE2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>6.3375096313577545E-2</v>
+        <v>0.16573697488151984</v>
       </c>
       <c r="AF1">
         <f>(1-EXP(-((AF2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>6.8836797745699688E-2</v>
+        <v>0.17163396818253152</v>
       </c>
       <c r="AG1">
         <f>(1-EXP(-((AG2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>7.4433814815514393E-2</v>
+        <v>0.17681983138790913</v>
       </c>
       <c r="AH1">
         <f>(1-EXP(-((AH2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>8.0140842430892326E-2</v>
+        <v>0.18131077796047496</v>
       </c>
       <c r="AI1">
         <f>(1-EXP(-((AI2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>8.5931203830453898E-2</v>
+        <v>0.18513948060036278</v>
       </c>
       <c r="AJ1">
         <f>(1-EXP(-((AJ2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>9.1777167376563482E-2</v>
+        <v>0.18835186512938695</v>
       </c>
       <c r="AK1">
         <f>(1-EXP(-((AK2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>9.7650288683833367E-2</v>
+        <v>0.19100357564494788</v>
       </c>
       <c r="AL1">
         <f>(1-EXP(-((AL2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.10352177197697486</v>
+        <v>0.1931563763376668</v>
       </c>
       <c r="AM1">
         <f>(1-EXP(-((AM2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.10936284380095161</v>
+        <v>0.19487473347482187</v>
       </c>
       <c r="AN1">
         <f>(1-EXP(-((AN2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.11514513160280658</v>
+        <v>0.19622277858911699</v>
       </c>
       <c r="AO1">
         <f>(1-EXP(-((AO2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.12084103929956716</v>
+        <v>0.1972617973403015</v>
       </c>
       <c r="AP1">
         <f>(1-EXP(-((AP2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.12642411176571153</v>
+        <v>0.19804832547095644</v>
       </c>
       <c r="AQ1">
         <f>(1-EXP(-((AQ2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.13186938023475472</v>
+        <v>0.19863287140923547</v>
       </c>
       <c r="AR1">
         <f>(1-EXP(-((AR2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.13715368092169056</v>
+        <v>0.19905923098155251</v>
       </c>
       <c r="AS1">
         <f>(1-EXP(-((AS2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.14225593973558134</v>
+        <v>0.199364318136077</v>
       </c>
       <c r="AT1">
         <f>(1-EXP(-((AT2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.14715741675338276</v>
+        <v>0.19957840901739385</v>
       </c>
       <c r="AU1">
         <f>(1-EXP(-((AU2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.15184190514555035</v>
+        <v>0.1997256853595088</v>
       </c>
       <c r="AV1">
         <f>(1-EXP(-((AV2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.15629588044952777</v>
+        <v>0.19982496522253218</v>
       </c>
       <c r="AW1">
         <f>(1-EXP(-((AW2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.1605085974384014</v>
+        <v>0.19989052148534298</v>
       </c>
       <c r="AX1">
         <f>(1-EXP(-((AX2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.16447213328097302</v>
+        <v>0.1999329074744195</v>
       </c>
       <c r="AY1">
         <f>(1-EXP(-((AY2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.16818137718312287</v>
+        <v>0.19995973093159392</v>
       </c>
       <c r="AZ1">
         <f>(1-EXP(-((AZ2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.17163396818253152</v>
+        <v>0.19997633902006273</v>
       </c>
       <c r="BA1">
         <f>(1-EXP(-((BA2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.17483018418329768</v>
+        <v>0.19998639592309114</v>
       </c>
       <c r="BB1">
         <f>(1-EXP(-((BB2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.17777278660987564</v>
+        <v>0.19999234945911523</v>
       </c>
       <c r="BC1">
         <f>(1-EXP(-((BC2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.18046682618238061</v>
+        <v>0.19999579357241226</v>
       </c>
       <c r="BD1">
         <f>(1-EXP(-((BD2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.18291941622657948</v>
+        <v>0.19999773981279137</v>
       </c>
       <c r="BE1">
         <f>(1-EXP(-((BE2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.18513948060036278</v>
+        <v>0.19999881369426081</v>
       </c>
       <c r="BF1">
         <f>(1-EXP(-((BF2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.18713748372393824</v>
+        <v>0.19999939203080119</v>
       </c>
       <c r="BG1">
         <f>(1-EXP(-((BG2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.18892515033527318</v>
+        <v>0.19999969590396702</v>
       </c>
       <c r="BH1">
         <f>(1-EXP(-((BH2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19051518245966237</v>
+        <v>0.19999985161306397</v>
       </c>
       <c r="BI1">
         <f>(1-EXP(-((BI2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19192098069883823</v>
+        <v>0.19999992939299016</v>
       </c>
       <c r="BJ1">
         <f>(1-EXP(-((BJ2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.1931563763376668</v>
+        <v>0.19999996725245739</v>
       </c>
       <c r="BK1">
         <f>(1-EXP(-((BK2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19423537997115478</v>
+        <v>0.19999998520210779</v>
       </c>
       <c r="BL1">
         <f>(1-EXP(-((BL2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19517195141408158</v>
+        <v>0.19999999348787459</v>
       </c>
       <c r="BM1">
         <f>(1-EXP(-((BM2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19597979461730688</v>
+        <v>0.19999999721029099</v>
       </c>
       <c r="BN1">
         <f>(1-EXP(-((BN2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19667218022765529</v>
+        <v>0.19999999883716038</v>
       </c>
       <c r="BO1">
         <f>(1-EXP(-((BO2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.1972617973403015</v>
+        <v>0.19999999952857025</v>
       </c>
       <c r="BP1">
         <f>(1-EXP(-((BP2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19776063494846641</v>
+        <v>0.19999999981419306</v>
       </c>
       <c r="BQ1">
         <f>(1-EXP(-((BQ2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19817989263419727</v>
+        <v>0.19999999992883505</v>
       </c>
       <c r="BR1">
         <f>(1-EXP(-((BR2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19852991919811599</v>
+        <v>0.19999999997352469</v>
       </c>
       <c r="BS1">
         <f>(1-EXP(-((BS2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19882017721906764</v>
+        <v>0.19999999999043694</v>
       </c>
       <c r="BT1">
         <f>(1-EXP(-((BT2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19905923098155251</v>
+        <v>0.19999999999664766</v>
       </c>
       <c r="BU1">
         <f>(1-EXP(-((BU2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19925475481581081</v>
+        <v>0.19999999999886001</v>
       </c>
       <c r="BV1">
         <f>(1-EXP(-((BV2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19941355866029969</v>
+        <v>0.19999999999962412</v>
       </c>
       <c r="BW1">
         <f>(1-EXP(-((BW2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19954162756957949</v>
+        <v>0.19999999999987986</v>
       </c>
       <c r="BX1">
         <f>(1-EXP(-((BX2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19964417193684117</v>
+        <v>0.19999999999996282</v>
       </c>
       <c r="BY1">
         <f>(1-EXP(-((BY2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.1997256853595088</v>
+        <v>0.19999999999998885</v>
       </c>
       <c r="BZ1">
         <f>(1-EXP(-((BZ2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19979000732576158</v>
+        <v>0.19999999999999676</v>
       </c>
       <c r="CA1">
         <f>(1-EXP(-((CA2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19984038821541683</v>
+        <v>0.1999999999999991</v>
       </c>
       <c r="CB1">
         <f>(1-EXP(-((CB2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19987955446662847</v>
+        <v>0.19999999999999976</v>
       </c>
       <c r="CC1">
         <f>(1-EXP(-((CC2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.1999097721380175</v>
+        <v>0.19999999999999996</v>
       </c>
       <c r="CD1">
         <f>(1-EXP(-((CD2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.1999329074744195</v>
+        <v>0.19999999999999998</v>
       </c>
       <c r="CE1">
         <f>(1-EXP(-((CE2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19995048344686059</v>
+        <v>0.2</v>
       </c>
       <c r="CF1">
         <f>(1-EXP(-((CF2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
         <v>0.2</v>
       </c>
     </row>
-    <row r="2" spans="1:84" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:84" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>39</v>
       </c>
@@ -6121,17 +6121,17 @@
     <tabColor rgb="FF002060"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>33</v>
       </c>
@@ -6151,12 +6151,12 @@
     <tabColor rgb="FF002060"/>
   </sheetPr>
   <dimension ref="A1:AB25"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="33.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -6242,7 +6242,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -6328,7 +6328,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -6414,7 +6414,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -6500,7 +6500,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -6586,7 +6586,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -6672,7 +6672,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -6758,7 +6758,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -6844,7 +6844,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -6930,7 +6930,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>13</v>
       </c>
@@ -7016,7 +7016,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -7102,7 +7102,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>15</v>
       </c>
@@ -7188,7 +7188,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>16</v>
       </c>
@@ -7274,7 +7274,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>17</v>
       </c>
@@ -7360,7 +7360,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>18</v>
       </c>
@@ -7446,7 +7446,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>19</v>
       </c>
@@ -7532,7 +7532,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>20</v>
       </c>
@@ -7618,7 +7618,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>21</v>
       </c>
@@ -7704,7 +7704,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>22</v>
       </c>
@@ -7790,7 +7790,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>23</v>
       </c>
@@ -7876,7 +7876,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>24</v>
       </c>
@@ -7962,7 +7962,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>25</v>
       </c>
@@ -8048,7 +8048,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>26</v>
       </c>
@@ -8134,7 +8134,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>27</v>
       </c>
@@ -8220,7 +8220,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>28</v>
       </c>

</xml_diff>

<commit_message>
Updates frozen policies wind CSC
</commit_message>
<xml_diff>
--- a/InputData/elec/CSC/Capacity Supply Curve.xlsx
+++ b/InputData/elec/CSC/Capacity Supply Curve.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\elec\CSC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3121D63-400A-431A-800C-74C80046487D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31E78B7F-F39B-40EF-A502-6BA9439E91FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{F87DB1D1-DC21-4EA7-B1DF-998EE56837F8}"/>
+    <workbookView xWindow="10" yWindow="270" windowWidth="18810" windowHeight="11000" activeTab="3" xr2:uid="{F87DB1D1-DC21-4EA7-B1DF-998EE56837F8}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -4287,28 +4287,28 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D3D2DEE-686E-48A0-AC3D-0F54DEA5D0EC}">
   <dimension ref="A1:C125"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="88.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="88.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
@@ -4316,45 +4316,45 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" s="1"/>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>36</v>
       </c>
@@ -4362,7 +4362,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>34</v>
       </c>
@@ -4370,7 +4370,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>35</v>
       </c>
@@ -4378,7 +4378,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>37</v>
       </c>
@@ -4386,7 +4386,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>38</v>
       </c>
@@ -4394,7 +4394,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>45</v>
       </c>
@@ -4402,7 +4402,7 @@
         <v>4.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B24">
         <f>(1-EXP(-((C24/$B$20-($B$19-0.5))/$B$17)^$B$18))*$B$16</f>
         <v>0</v>
@@ -4411,7 +4411,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B25">
         <f t="shared" ref="B25:B88" si="0">(1-EXP(-((C25/$B$20-($B$19-0.5))/$B$17)^$B$18))*$B$16</f>
         <v>4.286648162477036E-6</v>
@@ -4420,7 +4420,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B26">
         <f t="shared" si="0"/>
         <v>3.4290612860687911E-5</v>
@@ -4429,7 +4429,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B27">
         <f t="shared" si="0"/>
         <v>1.1570725740235322E-4</v>
@@ -4439,7 +4439,7 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B28">
         <f t="shared" si="0"/>
         <v>2.7416034086391594E-4</v>
@@ -4449,7 +4449,7 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B29">
         <f t="shared" si="0"/>
         <v>5.3511960071055413E-4</v>
@@ -4459,7 +4459,7 @@
         <v>2500</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B30">
         <f t="shared" si="0"/>
         <v>9.2378588268478008E-4</v>
@@ -4469,7 +4469,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B31">
         <f t="shared" si="0"/>
         <v>1.4649445766562463E-3</v>
@@ -4479,7 +4479,7 @@
         <v>3500</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B32">
         <f t="shared" si="0"/>
         <v>2.1827885823227922E-3</v>
@@ -4489,7 +4489,7 @@
         <v>4000</v>
       </c>
     </row>
-    <row r="33" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B33">
         <f t="shared" si="0"/>
         <v>3.1007125989183093E-3</v>
@@ -4499,7 +4499,7 @@
         <v>4500</v>
       </c>
     </row>
-    <row r="34" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B34">
         <f t="shared" si="0"/>
         <v>4.2410811978808027E-3</v>
@@ -4509,7 +4509,7 @@
         <v>5000</v>
       </c>
     </row>
-    <row r="35" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B35">
         <f t="shared" si="0"/>
         <v>5.6249738820245872E-3</v>
@@ -4519,7 +4519,7 @@
         <v>5500</v>
       </c>
     </row>
-    <row r="36" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B36">
         <f t="shared" si="0"/>
         <v>7.2719111397427484E-3</v>
@@ -4529,7 +4529,7 @@
         <v>6000</v>
       </c>
     </row>
-    <row r="37" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B37">
         <f t="shared" si="0"/>
         <v>9.1995663437769003E-3</v>
@@ -4539,7 +4539,7 @@
         <v>6500</v>
       </c>
     </row>
-    <row r="38" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B38">
         <f t="shared" si="0"/>
         <v>1.1423469191788382E-2</v>
@@ -4549,7 +4549,7 @@
         <v>7000</v>
       </c>
     </row>
-    <row r="39" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B39">
         <f t="shared" si="0"/>
         <v>1.3956707206263963E-2</v>
@@ -4559,7 +4559,7 @@
         <v>7500</v>
       </c>
     </row>
-    <row r="40" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B40">
         <f t="shared" si="0"/>
         <v>1.6809632565965439E-2</v>
@@ -4569,7 +4569,7 @@
         <v>8000</v>
       </c>
     </row>
-    <row r="41" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B41">
         <f t="shared" si="0"/>
         <v>1.9989582188770449E-2</v>
@@ -4579,7 +4579,7 @@
         <v>8500</v>
       </c>
     </row>
-    <row r="42" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B42">
         <f t="shared" si="0"/>
         <v>2.3500619483080909E-2</v>
@@ -4589,7 +4589,7 @@
         <v>9000</v>
       </c>
     </row>
-    <row r="43" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B43">
         <f t="shared" si="0"/>
         <v>2.7343306488591249E-2</v>
@@ -4599,7 +4599,7 @@
         <v>9500</v>
       </c>
     </row>
-    <row r="44" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B44">
         <f t="shared" si="0"/>
         <v>3.1514515195616613E-2</v>
@@ -4609,7 +4609,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="45" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B45">
         <f t="shared" si="0"/>
         <v>3.6007286628151627E-2</v>
@@ -4619,7 +4619,7 @@
         <v>10500</v>
       </c>
     </row>
-    <row r="46" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B46">
         <f t="shared" si="0"/>
         <v>4.0810745768913415E-2</v>
@@ -4629,7 +4629,7 @@
         <v>11000</v>
       </c>
     </row>
-    <row r="47" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B47">
         <f t="shared" si="0"/>
         <v>4.5910079573753593E-2</v>
@@ -4639,7 +4639,7 @@
         <v>11500</v>
       </c>
     </row>
-    <row r="48" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B48">
         <f t="shared" si="0"/>
         <v>5.1286584158818753E-2</v>
@@ -4649,7 +4649,7 @@
         <v>12000</v>
       </c>
     </row>
-    <row r="49" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B49">
         <f t="shared" si="0"/>
         <v>5.6917785751641151E-2</v>
@@ -4659,7 +4659,7 @@
         <v>12500</v>
       </c>
     </row>
-    <row r="50" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B50">
         <f t="shared" si="0"/>
         <v>6.2777638197790697E-2</v>
@@ -4669,7 +4669,7 @@
         <v>13000</v>
       </c>
     </row>
-    <row r="51" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B51">
         <f t="shared" si="0"/>
         <v>6.8836797745699688E-2</v>
@@ -4679,7 +4679,7 @@
         <v>13500</v>
       </c>
     </row>
-    <row r="52" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B52">
         <f t="shared" si="0"/>
         <v>7.506297354898428E-2</v>
@@ -4689,7 +4689,7 @@
         <v>14000</v>
       </c>
     </row>
-    <row r="53" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B53">
         <f t="shared" si="0"/>
         <v>8.142134989988481E-2</v>
@@ -4699,7 +4699,7 @@
         <v>14500</v>
       </c>
     </row>
-    <row r="54" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B54">
         <f t="shared" si="0"/>
         <v>8.787507372604586E-2</v>
@@ -4709,7 +4709,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="55" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B55">
         <f t="shared" si="0"/>
         <v>9.438579844442066E-2</v>
@@ -4719,7 +4719,7 @@
         <v>15500</v>
       </c>
     </row>
-    <row r="56" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B56">
         <f t="shared" si="0"/>
         <v>0.10091427297723279</v>
@@ -4729,7 +4729,7 @@
         <v>16000</v>
       </c>
     </row>
-    <row r="57" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B57">
         <f t="shared" si="0"/>
         <v>0.10742096270522571</v>
@@ -4739,7 +4739,7 @@
         <v>16500</v>
       </c>
     </row>
-    <row r="58" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B58">
         <f t="shared" si="0"/>
         <v>0.11386668746965854</v>
@@ -4749,7 +4749,7 @@
         <v>17000</v>
       </c>
     </row>
-    <row r="59" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B59">
         <f t="shared" si="0"/>
         <v>0.12021326053442474</v>
@@ -4759,7 +4759,7 @@
         <v>17500</v>
       </c>
     </row>
-    <row r="60" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B60">
         <f t="shared" si="0"/>
         <v>0.12642411176571153</v>
@@ -4769,7 +4769,7 @@
         <v>18000</v>
       </c>
     </row>
-    <row r="61" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B61">
         <f t="shared" si="0"/>
         <v>0.1324648782399141</v>
@@ -4779,7 +4779,7 @@
         <v>18500</v>
       </c>
     </row>
-    <row r="62" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B62">
         <f t="shared" si="0"/>
         <v>0.1383039460856948</v>
@@ -4789,7 +4789,7 @@
         <v>19000</v>
       </c>
     </row>
-    <row r="63" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B63">
         <f t="shared" si="0"/>
         <v>0.1439129286073208</v>
@@ -4799,7 +4799,7 @@
         <v>19500</v>
       </c>
     </row>
-    <row r="64" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B64">
         <f t="shared" si="0"/>
         <v>0.14926706759510625</v>
@@ -4809,7 +4809,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="65" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B65">
         <f t="shared" si="0"/>
         <v>0.15434554714316789</v>
@@ -4819,7 +4819,7 @@
         <v>20500</v>
       </c>
     </row>
-    <row r="66" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B66">
         <f t="shared" si="0"/>
         <v>0.1591317121715517</v>
@@ -4829,7 +4829,7 @@
         <v>21000</v>
       </c>
     </row>
-    <row r="67" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B67">
         <f t="shared" si="0"/>
         <v>0.16361318706836692</v>
@@ -4839,7 +4839,7 @@
         <v>21500</v>
       </c>
     </row>
-    <row r="68" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B68">
         <f t="shared" si="0"/>
         <v>0.16778189328550838</v>
@@ -4849,7 +4849,7 @@
         <v>22000</v>
       </c>
     </row>
-    <row r="69" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B69">
         <f t="shared" si="0"/>
         <v>0.17163396818253152</v>
@@ -4859,7 +4859,7 @@
         <v>22500</v>
       </c>
     </row>
-    <row r="70" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B70">
         <f t="shared" si="0"/>
         <v>0.17516959075587743</v>
@@ -4869,7 +4869,7 @@
         <v>23000</v>
       </c>
     </row>
-    <row r="71" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B71">
         <f t="shared" si="0"/>
         <v>0.17839272295802988</v>
@@ -4879,7 +4879,7 @@
         <v>23500</v>
       </c>
     </row>
-    <row r="72" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B72">
         <f t="shared" si="0"/>
         <v>0.18131077796047496</v>
@@ -4889,7 +4889,7 @@
         <v>24000</v>
       </c>
     </row>
-    <row r="73" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="73" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B73">
         <f t="shared" si="0"/>
         <v>0.18393422882553601</v>
@@ -4899,7 +4899,7 @@
         <v>24500</v>
       </c>
     </row>
-    <row r="74" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="74" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B74">
         <f t="shared" si="0"/>
         <v>0.18627617253555084</v>
@@ -4909,7 +4909,7 @@
         <v>25000</v>
       </c>
     </row>
-    <row r="75" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="75" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B75">
         <f t="shared" si="0"/>
         <v>0.18835186512938695</v>
@@ -4919,7 +4919,7 @@
         <v>25500</v>
       </c>
     </row>
-    <row r="76" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="76" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B76">
         <f t="shared" si="0"/>
         <v>0.19017824380056211</v>
@@ -4929,7 +4929,7 @@
         <v>26000</v>
       </c>
     </row>
-    <row r="77" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="77" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B77">
         <f t="shared" si="0"/>
         <v>0.19177345124178691</v>
@@ -4939,7 +4939,7 @@
         <v>26500</v>
       </c>
     </row>
-    <row r="78" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="78" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B78">
         <f t="shared" si="0"/>
         <v>0.1931563763376668</v>
@@ -4949,7 +4949,7 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="79" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="79" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B79">
         <f t="shared" si="0"/>
         <v>0.19434622360232301</v>
@@ -4959,7 +4959,7 @@
         <v>27500</v>
       </c>
     </row>
-    <row r="80" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="80" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B80">
         <f t="shared" si="0"/>
         <v>0.19536212164822028</v>
@@ -4969,7 +4969,7 @@
         <v>28000</v>
       </c>
     </row>
-    <row r="81" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="81" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B81">
         <f t="shared" si="0"/>
         <v>0.19622277858911699</v>
@@ -4979,7 +4979,7 @@
         <v>28500</v>
       </c>
     </row>
-    <row r="82" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="82" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B82">
         <f t="shared" si="0"/>
         <v>0.19694618976330103</v>
@@ -4989,7 +4989,7 @@
         <v>29000</v>
       </c>
     </row>
-    <row r="83" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="83" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B83">
         <f t="shared" si="0"/>
         <v>0.19754940065027685</v>
@@ -4999,7 +4999,7 @@
         <v>29500</v>
       </c>
     </row>
-    <row r="84" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="84" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B84">
         <f t="shared" si="0"/>
         <v>0.19804832547095644</v>
@@ -5009,7 +5009,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="85" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="85" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B85">
         <f t="shared" si="0"/>
         <v>0.19845761981600954</v>
@@ -5019,7 +5019,7 @@
         <v>30500</v>
       </c>
     </row>
-    <row r="86" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="86" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B86">
         <f t="shared" si="0"/>
         <v>0.19879060382342864</v>
@@ -5029,7 +5029,7 @@
         <v>31000</v>
       </c>
     </row>
-    <row r="87" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="87" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B87">
         <f t="shared" si="0"/>
         <v>0.19905923098155251</v>
@@ -5039,7 +5039,7 @@
         <v>31500</v>
       </c>
     </row>
-    <row r="88" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="88" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B88">
         <f t="shared" si="0"/>
         <v>0.19927409659660289</v>
@@ -5049,7 +5049,7 @@
         <v>32000</v>
       </c>
     </row>
-    <row r="89" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="89" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B89">
         <f t="shared" ref="B89:B125" si="2">(1-EXP(-((C89/$B$20-($B$19-0.5))/$B$17)^$B$18))*$B$16</f>
         <v>0.19944447933595111</v>
@@ -5059,7 +5059,7 @@
         <v>32500</v>
       </c>
     </row>
-    <row r="90" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="90" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B90">
         <f t="shared" si="2"/>
         <v>0.19957840901739385</v>
@@ -5069,7 +5069,7 @@
         <v>33000</v>
       </c>
     </row>
-    <row r="91" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="91" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B91">
         <f t="shared" si="2"/>
         <v>0.19968275391843365</v>
@@ -5079,7 +5079,7 @@
         <v>33500</v>
       </c>
     </row>
-    <row r="92" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="92" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B92">
         <f t="shared" si="2"/>
         <v>0.19976332127118276</v>
@@ -5089,7 +5089,7 @@
         <v>34000</v>
       </c>
     </row>
-    <row r="93" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="93" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B93">
         <f t="shared" si="2"/>
         <v>0.19982496522253218</v>
@@ -5099,7 +5099,7 @@
         <v>34500</v>
       </c>
     </row>
-    <row r="94" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="94" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B94">
         <f t="shared" si="2"/>
         <v>0.19987169730697774</v>
@@ -5109,7 +5109,7 @@
         <v>35000</v>
       </c>
     </row>
-    <row r="95" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="95" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B95">
         <f t="shared" si="2"/>
         <v>0.19990679533419684</v>
@@ -5119,7 +5119,7 @@
         <v>35500</v>
       </c>
     </row>
-    <row r="96" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="96" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B96">
         <f t="shared" si="2"/>
         <v>0.1999329074744195</v>
@@ -5129,7 +5129,7 @@
         <v>36000</v>
       </c>
     </row>
-    <row r="97" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="97" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B97">
         <f t="shared" si="2"/>
         <v>0.19995214918026516</v>
@@ -5139,7 +5139,7 @@
         <v>36500</v>
       </c>
     </row>
-    <row r="98" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="98" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B98">
         <f t="shared" si="2"/>
         <v>0.19996619137347427</v>
@@ -5149,7 +5149,7 @@
         <v>37000</v>
       </c>
     </row>
-    <row r="99" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="99" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B99">
         <f t="shared" si="2"/>
         <v>0.19997633902006273</v>
@@ -5159,7 +5159,7 @@
         <v>37500</v>
       </c>
     </row>
-    <row r="100" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="100" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B100">
         <f t="shared" si="2"/>
         <v>0.19998359980055544</v>
@@ -5169,7 +5169,7 @@
         <v>38000</v>
       </c>
     </row>
-    <row r="101" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="101" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B101">
         <f t="shared" si="2"/>
         <v>0.19998874304618811</v>
@@ -5179,7 +5179,7 @@
         <v>38500</v>
       </c>
     </row>
-    <row r="102" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="102" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B102">
         <f t="shared" si="2"/>
         <v>0.19999234945911523</v>
@@ -5189,7 +5189,7 @@
         <v>39000</v>
       </c>
     </row>
-    <row r="103" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="103" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B103">
         <f t="shared" si="2"/>
         <v>0.19999485237326678</v>
@@ -5199,7 +5199,7 @@
         <v>39500</v>
       </c>
     </row>
-    <row r="104" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="104" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B104">
         <f t="shared" si="2"/>
         <v>0.1999965714557792</v>
@@ -5209,7 +5209,7 @@
         <v>40000</v>
       </c>
     </row>
-    <row r="105" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="105" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B105">
         <f t="shared" si="2"/>
         <v>0.19999773981279137</v>
@@ -5219,7 +5219,7 @@
         <v>40500</v>
       </c>
     </row>
-    <row r="106" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="106" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B106">
         <f t="shared" si="2"/>
         <v>0.19999852546471561</v>
@@ -5229,7 +5229,7 @@
         <v>41000</v>
       </c>
     </row>
-    <row r="107" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="107" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B107">
         <f t="shared" si="2"/>
         <v>0.19999904811129313</v>
@@ -5239,7 +5239,7 @@
         <v>41500</v>
       </c>
     </row>
-    <row r="108" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="108" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B108">
         <f t="shared" si="2"/>
         <v>0.19999939203080119</v>
@@ -5249,7 +5249,7 @@
         <v>42000</v>
       </c>
     </row>
-    <row r="109" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="109" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B109">
         <f t="shared" si="2"/>
         <v>0.19999961586354192</v>
@@ -5259,7 +5259,7 @@
         <v>42500</v>
       </c>
     </row>
-    <row r="110" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="110" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B110">
         <f t="shared" si="2"/>
         <v>0.19999975992763294</v>
@@ -5269,7 +5269,7 @@
         <v>43000</v>
       </c>
     </row>
-    <row r="111" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="111" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B111">
         <f t="shared" si="2"/>
         <v>0.19999985161306397</v>
@@ -5279,7 +5279,7 @@
         <v>43500</v>
       </c>
     </row>
-    <row r="112" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="112" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B112">
         <f t="shared" si="2"/>
         <v>0.19999990930357772</v>
@@ -5289,7 +5289,7 @@
         <v>44000</v>
       </c>
     </row>
-    <row r="113" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="113" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B113">
         <f t="shared" si="2"/>
         <v>0.19999994518873965</v>
@@ -5299,7 +5299,7 @@
         <v>44500</v>
       </c>
     </row>
-    <row r="114" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="114" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B114">
         <f t="shared" si="2"/>
         <v>0.19999996725245739</v>
@@ -5309,7 +5309,7 @@
         <v>45000</v>
       </c>
     </row>
-    <row r="115" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="115" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B115">
         <f t="shared" si="2"/>
         <v>0.19999998065979441</v>
@@ -5319,7 +5319,7 @@
         <v>45500</v>
       </c>
     </row>
-    <row r="116" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="116" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B116">
         <f t="shared" si="2"/>
         <v>0.19999998871085503</v>
@@ -5329,7 +5329,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="117" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="117" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B117">
         <f t="shared" si="2"/>
         <v>0.19999999348787459</v>
@@ -5339,7 +5339,7 @@
         <v>46500</v>
       </c>
     </row>
-    <row r="118" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="118" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B118">
         <f t="shared" si="2"/>
         <v>0.19999999628815057</v>
@@ -5349,7 +5349,7 @@
         <v>47000</v>
       </c>
     </row>
-    <row r="119" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="119" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B119">
         <f t="shared" si="2"/>
         <v>0.19999999790970302</v>
@@ -5359,7 +5359,7 @@
         <v>47500</v>
       </c>
     </row>
-    <row r="120" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="120" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B120">
         <f t="shared" si="2"/>
         <v>0.19999999883716038</v>
@@ -5369,7 +5369,7 @@
         <v>48000</v>
       </c>
     </row>
-    <row r="121" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="121" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B121">
         <f t="shared" si="2"/>
         <v>0.19999999936104543</v>
@@ -5379,7 +5379,7 @@
         <v>48500</v>
       </c>
     </row>
-    <row r="122" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="122" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B122">
         <f t="shared" si="2"/>
         <v>0.19999999965326104</v>
@@ -5389,7 +5389,7 @@
         <v>49000</v>
       </c>
     </row>
-    <row r="123" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="123" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B123">
         <f t="shared" si="2"/>
         <v>0.19999999981419306</v>
@@ -5399,7 +5399,7 @@
         <v>49500</v>
       </c>
     </row>
-    <row r="124" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="124" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B124">
         <f t="shared" si="2"/>
         <v>0.19999999990169129</v>
@@ -5409,7 +5409,7 @@
         <v>50000</v>
       </c>
     </row>
-    <row r="125" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="125" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B125">
         <f t="shared" si="2"/>
         <v>0.19999999994865042</v>
@@ -5431,13 +5431,13 @@
     <tabColor rgb="FF002060"/>
   </sheetPr>
   <dimension ref="A1:CF2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="23.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:84" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:84" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -5774,7 +5774,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="2" spans="1:84" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:84" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>39</v>
       </c>
@@ -6121,17 +6121,17 @@
     <tabColor rgb="FF002060"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>33</v>
       </c>
@@ -6151,12 +6151,12 @@
     <tabColor rgb="FF002060"/>
   </sheetPr>
   <dimension ref="A1:AB25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="33.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -6242,7 +6242,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -6328,7 +6328,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -6414,7 +6414,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -6500,7 +6500,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -6586,7 +6586,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -6672,7 +6672,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -6680,25 +6680,25 @@
         <v>0.8</v>
       </c>
       <c r="C7">
-        <v>0.2</v>
+        <v>0.8</v>
       </c>
       <c r="D7">
-        <v>0.2</v>
+        <v>0.8</v>
       </c>
       <c r="E7">
-        <v>0.2</v>
+        <v>0.8</v>
       </c>
       <c r="F7">
-        <v>0.2</v>
+        <v>0.8</v>
       </c>
       <c r="G7">
-        <v>0.2</v>
+        <v>0.8</v>
       </c>
       <c r="H7">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="I7">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="J7">
         <v>0.8</v>
@@ -6758,7 +6758,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -6844,7 +6844,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -6930,7 +6930,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>13</v>
       </c>
@@ -7016,7 +7016,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -7102,7 +7102,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>15</v>
       </c>
@@ -7188,7 +7188,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>16</v>
       </c>
@@ -7274,7 +7274,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>17</v>
       </c>
@@ -7360,7 +7360,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>18</v>
       </c>
@@ -7446,7 +7446,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>19</v>
       </c>
@@ -7532,7 +7532,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>20</v>
       </c>
@@ -7618,7 +7618,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>21</v>
       </c>
@@ -7704,7 +7704,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>22</v>
       </c>
@@ -7790,7 +7790,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>23</v>
       </c>
@@ -7876,7 +7876,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>24</v>
       </c>
@@ -7962,7 +7962,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>25</v>
       </c>
@@ -8048,7 +8048,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>26</v>
       </c>
@@ -8134,7 +8134,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>27</v>
       </c>
@@ -8220,7 +8220,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>28</v>
       </c>

</xml_diff>

<commit_message>
Revert "Updates frozen policies wind CSC"
This reverts commit 3a900adc60ba28cfac9c80b0aca60e7c4a973cba.
</commit_message>
<xml_diff>
--- a/InputData/elec/CSC/Capacity Supply Curve.xlsx
+++ b/InputData/elec/CSC/Capacity Supply Curve.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\elec\CSC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31E78B7F-F39B-40EF-A502-6BA9439E91FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3121D63-400A-431A-800C-74C80046487D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10" yWindow="270" windowWidth="18810" windowHeight="11000" activeTab="3" xr2:uid="{F87DB1D1-DC21-4EA7-B1DF-998EE56837F8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{F87DB1D1-DC21-4EA7-B1DF-998EE56837F8}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -4287,28 +4287,28 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D3D2DEE-686E-48A0-AC3D-0F54DEA5D0EC}">
   <dimension ref="A1:C125"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="88.7265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="88.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
@@ -4316,45 +4316,45 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>36</v>
       </c>
@@ -4362,7 +4362,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>34</v>
       </c>
@@ -4370,7 +4370,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>35</v>
       </c>
@@ -4378,7 +4378,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>37</v>
       </c>
@@ -4386,7 +4386,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>38</v>
       </c>
@@ -4394,7 +4394,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>45</v>
       </c>
@@ -4402,7 +4402,7 @@
         <v>4.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B24">
         <f>(1-EXP(-((C24/$B$20-($B$19-0.5))/$B$17)^$B$18))*$B$16</f>
         <v>0</v>
@@ -4411,7 +4411,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B25">
         <f t="shared" ref="B25:B88" si="0">(1-EXP(-((C25/$B$20-($B$19-0.5))/$B$17)^$B$18))*$B$16</f>
         <v>4.286648162477036E-6</v>
@@ -4420,7 +4420,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B26">
         <f t="shared" si="0"/>
         <v>3.4290612860687911E-5</v>
@@ -4429,7 +4429,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B27">
         <f t="shared" si="0"/>
         <v>1.1570725740235322E-4</v>
@@ -4439,7 +4439,7 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B28">
         <f t="shared" si="0"/>
         <v>2.7416034086391594E-4</v>
@@ -4449,7 +4449,7 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B29">
         <f t="shared" si="0"/>
         <v>5.3511960071055413E-4</v>
@@ -4459,7 +4459,7 @@
         <v>2500</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B30">
         <f t="shared" si="0"/>
         <v>9.2378588268478008E-4</v>
@@ -4469,7 +4469,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B31">
         <f t="shared" si="0"/>
         <v>1.4649445766562463E-3</v>
@@ -4479,7 +4479,7 @@
         <v>3500</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B32">
         <f t="shared" si="0"/>
         <v>2.1827885823227922E-3</v>
@@ -4489,7 +4489,7 @@
         <v>4000</v>
       </c>
     </row>
-    <row r="33" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B33">
         <f t="shared" si="0"/>
         <v>3.1007125989183093E-3</v>
@@ -4499,7 +4499,7 @@
         <v>4500</v>
       </c>
     </row>
-    <row r="34" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B34">
         <f t="shared" si="0"/>
         <v>4.2410811978808027E-3</v>
@@ -4509,7 +4509,7 @@
         <v>5000</v>
       </c>
     </row>
-    <row r="35" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B35">
         <f t="shared" si="0"/>
         <v>5.6249738820245872E-3</v>
@@ -4519,7 +4519,7 @@
         <v>5500</v>
       </c>
     </row>
-    <row r="36" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B36">
         <f t="shared" si="0"/>
         <v>7.2719111397427484E-3</v>
@@ -4529,7 +4529,7 @@
         <v>6000</v>
       </c>
     </row>
-    <row r="37" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B37">
         <f t="shared" si="0"/>
         <v>9.1995663437769003E-3</v>
@@ -4539,7 +4539,7 @@
         <v>6500</v>
       </c>
     </row>
-    <row r="38" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B38">
         <f t="shared" si="0"/>
         <v>1.1423469191788382E-2</v>
@@ -4549,7 +4549,7 @@
         <v>7000</v>
       </c>
     </row>
-    <row r="39" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B39">
         <f t="shared" si="0"/>
         <v>1.3956707206263963E-2</v>
@@ -4559,7 +4559,7 @@
         <v>7500</v>
       </c>
     </row>
-    <row r="40" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B40">
         <f t="shared" si="0"/>
         <v>1.6809632565965439E-2</v>
@@ -4569,7 +4569,7 @@
         <v>8000</v>
       </c>
     </row>
-    <row r="41" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B41">
         <f t="shared" si="0"/>
         <v>1.9989582188770449E-2</v>
@@ -4579,7 +4579,7 @@
         <v>8500</v>
       </c>
     </row>
-    <row r="42" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B42">
         <f t="shared" si="0"/>
         <v>2.3500619483080909E-2</v>
@@ -4589,7 +4589,7 @@
         <v>9000</v>
       </c>
     </row>
-    <row r="43" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B43">
         <f t="shared" si="0"/>
         <v>2.7343306488591249E-2</v>
@@ -4599,7 +4599,7 @@
         <v>9500</v>
       </c>
     </row>
-    <row r="44" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B44">
         <f t="shared" si="0"/>
         <v>3.1514515195616613E-2</v>
@@ -4609,7 +4609,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="45" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="45" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B45">
         <f t="shared" si="0"/>
         <v>3.6007286628151627E-2</v>
@@ -4619,7 +4619,7 @@
         <v>10500</v>
       </c>
     </row>
-    <row r="46" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B46">
         <f t="shared" si="0"/>
         <v>4.0810745768913415E-2</v>
@@ -4629,7 +4629,7 @@
         <v>11000</v>
       </c>
     </row>
-    <row r="47" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B47">
         <f t="shared" si="0"/>
         <v>4.5910079573753593E-2</v>
@@ -4639,7 +4639,7 @@
         <v>11500</v>
       </c>
     </row>
-    <row r="48" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B48">
         <f t="shared" si="0"/>
         <v>5.1286584158818753E-2</v>
@@ -4649,7 +4649,7 @@
         <v>12000</v>
       </c>
     </row>
-    <row r="49" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="49" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B49">
         <f t="shared" si="0"/>
         <v>5.6917785751641151E-2</v>
@@ -4659,7 +4659,7 @@
         <v>12500</v>
       </c>
     </row>
-    <row r="50" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="50" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B50">
         <f t="shared" si="0"/>
         <v>6.2777638197790697E-2</v>
@@ -4669,7 +4669,7 @@
         <v>13000</v>
       </c>
     </row>
-    <row r="51" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="51" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B51">
         <f t="shared" si="0"/>
         <v>6.8836797745699688E-2</v>
@@ -4679,7 +4679,7 @@
         <v>13500</v>
       </c>
     </row>
-    <row r="52" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="52" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B52">
         <f t="shared" si="0"/>
         <v>7.506297354898428E-2</v>
@@ -4689,7 +4689,7 @@
         <v>14000</v>
       </c>
     </row>
-    <row r="53" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="53" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B53">
         <f t="shared" si="0"/>
         <v>8.142134989988481E-2</v>
@@ -4699,7 +4699,7 @@
         <v>14500</v>
       </c>
     </row>
-    <row r="54" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="54" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B54">
         <f t="shared" si="0"/>
         <v>8.787507372604586E-2</v>
@@ -4709,7 +4709,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="55" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="55" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B55">
         <f t="shared" si="0"/>
         <v>9.438579844442066E-2</v>
@@ -4719,7 +4719,7 @@
         <v>15500</v>
       </c>
     </row>
-    <row r="56" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="56" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B56">
         <f t="shared" si="0"/>
         <v>0.10091427297723279</v>
@@ -4729,7 +4729,7 @@
         <v>16000</v>
       </c>
     </row>
-    <row r="57" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="57" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B57">
         <f t="shared" si="0"/>
         <v>0.10742096270522571</v>
@@ -4739,7 +4739,7 @@
         <v>16500</v>
       </c>
     </row>
-    <row r="58" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="58" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B58">
         <f t="shared" si="0"/>
         <v>0.11386668746965854</v>
@@ -4749,7 +4749,7 @@
         <v>17000</v>
       </c>
     </row>
-    <row r="59" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="59" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B59">
         <f t="shared" si="0"/>
         <v>0.12021326053442474</v>
@@ -4759,7 +4759,7 @@
         <v>17500</v>
       </c>
     </row>
-    <row r="60" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="60" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B60">
         <f t="shared" si="0"/>
         <v>0.12642411176571153</v>
@@ -4769,7 +4769,7 @@
         <v>18000</v>
       </c>
     </row>
-    <row r="61" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="61" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B61">
         <f t="shared" si="0"/>
         <v>0.1324648782399141</v>
@@ -4779,7 +4779,7 @@
         <v>18500</v>
       </c>
     </row>
-    <row r="62" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="62" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B62">
         <f t="shared" si="0"/>
         <v>0.1383039460856948</v>
@@ -4789,7 +4789,7 @@
         <v>19000</v>
       </c>
     </row>
-    <row r="63" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="63" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B63">
         <f t="shared" si="0"/>
         <v>0.1439129286073208</v>
@@ -4799,7 +4799,7 @@
         <v>19500</v>
       </c>
     </row>
-    <row r="64" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="64" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B64">
         <f t="shared" si="0"/>
         <v>0.14926706759510625</v>
@@ -4809,7 +4809,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="65" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="65" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B65">
         <f t="shared" si="0"/>
         <v>0.15434554714316789</v>
@@ -4819,7 +4819,7 @@
         <v>20500</v>
       </c>
     </row>
-    <row r="66" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="66" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B66">
         <f t="shared" si="0"/>
         <v>0.1591317121715517</v>
@@ -4829,7 +4829,7 @@
         <v>21000</v>
       </c>
     </row>
-    <row r="67" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="67" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B67">
         <f t="shared" si="0"/>
         <v>0.16361318706836692</v>
@@ -4839,7 +4839,7 @@
         <v>21500</v>
       </c>
     </row>
-    <row r="68" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="68" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B68">
         <f t="shared" si="0"/>
         <v>0.16778189328550838</v>
@@ -4849,7 +4849,7 @@
         <v>22000</v>
       </c>
     </row>
-    <row r="69" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="69" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B69">
         <f t="shared" si="0"/>
         <v>0.17163396818253152</v>
@@ -4859,7 +4859,7 @@
         <v>22500</v>
       </c>
     </row>
-    <row r="70" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="70" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B70">
         <f t="shared" si="0"/>
         <v>0.17516959075587743</v>
@@ -4869,7 +4869,7 @@
         <v>23000</v>
       </c>
     </row>
-    <row r="71" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="71" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B71">
         <f t="shared" si="0"/>
         <v>0.17839272295802988</v>
@@ -4879,7 +4879,7 @@
         <v>23500</v>
       </c>
     </row>
-    <row r="72" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="72" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B72">
         <f t="shared" si="0"/>
         <v>0.18131077796047496</v>
@@ -4889,7 +4889,7 @@
         <v>24000</v>
       </c>
     </row>
-    <row r="73" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="73" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B73">
         <f t="shared" si="0"/>
         <v>0.18393422882553601</v>
@@ -4899,7 +4899,7 @@
         <v>24500</v>
       </c>
     </row>
-    <row r="74" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="74" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B74">
         <f t="shared" si="0"/>
         <v>0.18627617253555084</v>
@@ -4909,7 +4909,7 @@
         <v>25000</v>
       </c>
     </row>
-    <row r="75" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="75" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B75">
         <f t="shared" si="0"/>
         <v>0.18835186512938695</v>
@@ -4919,7 +4919,7 @@
         <v>25500</v>
       </c>
     </row>
-    <row r="76" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="76" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B76">
         <f t="shared" si="0"/>
         <v>0.19017824380056211</v>
@@ -4929,7 +4929,7 @@
         <v>26000</v>
       </c>
     </row>
-    <row r="77" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="77" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B77">
         <f t="shared" si="0"/>
         <v>0.19177345124178691</v>
@@ -4939,7 +4939,7 @@
         <v>26500</v>
       </c>
     </row>
-    <row r="78" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="78" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B78">
         <f t="shared" si="0"/>
         <v>0.1931563763376668</v>
@@ -4949,7 +4949,7 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="79" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="79" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B79">
         <f t="shared" si="0"/>
         <v>0.19434622360232301</v>
@@ -4959,7 +4959,7 @@
         <v>27500</v>
       </c>
     </row>
-    <row r="80" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="80" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B80">
         <f t="shared" si="0"/>
         <v>0.19536212164822028</v>
@@ -4969,7 +4969,7 @@
         <v>28000</v>
       </c>
     </row>
-    <row r="81" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="81" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B81">
         <f t="shared" si="0"/>
         <v>0.19622277858911699</v>
@@ -4979,7 +4979,7 @@
         <v>28500</v>
       </c>
     </row>
-    <row r="82" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="82" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B82">
         <f t="shared" si="0"/>
         <v>0.19694618976330103</v>
@@ -4989,7 +4989,7 @@
         <v>29000</v>
       </c>
     </row>
-    <row r="83" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="83" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B83">
         <f t="shared" si="0"/>
         <v>0.19754940065027685</v>
@@ -4999,7 +4999,7 @@
         <v>29500</v>
       </c>
     </row>
-    <row r="84" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="84" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B84">
         <f t="shared" si="0"/>
         <v>0.19804832547095644</v>
@@ -5009,7 +5009,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="85" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="85" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B85">
         <f t="shared" si="0"/>
         <v>0.19845761981600954</v>
@@ -5019,7 +5019,7 @@
         <v>30500</v>
       </c>
     </row>
-    <row r="86" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="86" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B86">
         <f t="shared" si="0"/>
         <v>0.19879060382342864</v>
@@ -5029,7 +5029,7 @@
         <v>31000</v>
       </c>
     </row>
-    <row r="87" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="87" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B87">
         <f t="shared" si="0"/>
         <v>0.19905923098155251</v>
@@ -5039,7 +5039,7 @@
         <v>31500</v>
       </c>
     </row>
-    <row r="88" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="88" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B88">
         <f t="shared" si="0"/>
         <v>0.19927409659660289</v>
@@ -5049,7 +5049,7 @@
         <v>32000</v>
       </c>
     </row>
-    <row r="89" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="89" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B89">
         <f t="shared" ref="B89:B125" si="2">(1-EXP(-((C89/$B$20-($B$19-0.5))/$B$17)^$B$18))*$B$16</f>
         <v>0.19944447933595111</v>
@@ -5059,7 +5059,7 @@
         <v>32500</v>
       </c>
     </row>
-    <row r="90" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="90" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B90">
         <f t="shared" si="2"/>
         <v>0.19957840901739385</v>
@@ -5069,7 +5069,7 @@
         <v>33000</v>
       </c>
     </row>
-    <row r="91" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="91" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B91">
         <f t="shared" si="2"/>
         <v>0.19968275391843365</v>
@@ -5079,7 +5079,7 @@
         <v>33500</v>
       </c>
     </row>
-    <row r="92" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="92" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B92">
         <f t="shared" si="2"/>
         <v>0.19976332127118276</v>
@@ -5089,7 +5089,7 @@
         <v>34000</v>
       </c>
     </row>
-    <row r="93" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="93" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B93">
         <f t="shared" si="2"/>
         <v>0.19982496522253218</v>
@@ -5099,7 +5099,7 @@
         <v>34500</v>
       </c>
     </row>
-    <row r="94" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="94" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B94">
         <f t="shared" si="2"/>
         <v>0.19987169730697774</v>
@@ -5109,7 +5109,7 @@
         <v>35000</v>
       </c>
     </row>
-    <row r="95" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="95" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B95">
         <f t="shared" si="2"/>
         <v>0.19990679533419684</v>
@@ -5119,7 +5119,7 @@
         <v>35500</v>
       </c>
     </row>
-    <row r="96" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="96" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B96">
         <f t="shared" si="2"/>
         <v>0.1999329074744195</v>
@@ -5129,7 +5129,7 @@
         <v>36000</v>
       </c>
     </row>
-    <row r="97" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="97" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B97">
         <f t="shared" si="2"/>
         <v>0.19995214918026516</v>
@@ -5139,7 +5139,7 @@
         <v>36500</v>
       </c>
     </row>
-    <row r="98" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="98" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B98">
         <f t="shared" si="2"/>
         <v>0.19996619137347427</v>
@@ -5149,7 +5149,7 @@
         <v>37000</v>
       </c>
     </row>
-    <row r="99" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="99" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B99">
         <f t="shared" si="2"/>
         <v>0.19997633902006273</v>
@@ -5159,7 +5159,7 @@
         <v>37500</v>
       </c>
     </row>
-    <row r="100" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="100" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B100">
         <f t="shared" si="2"/>
         <v>0.19998359980055544</v>
@@ -5169,7 +5169,7 @@
         <v>38000</v>
       </c>
     </row>
-    <row r="101" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="101" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B101">
         <f t="shared" si="2"/>
         <v>0.19998874304618811</v>
@@ -5179,7 +5179,7 @@
         <v>38500</v>
       </c>
     </row>
-    <row r="102" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="102" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B102">
         <f t="shared" si="2"/>
         <v>0.19999234945911523</v>
@@ -5189,7 +5189,7 @@
         <v>39000</v>
       </c>
     </row>
-    <row r="103" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="103" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B103">
         <f t="shared" si="2"/>
         <v>0.19999485237326678</v>
@@ -5199,7 +5199,7 @@
         <v>39500</v>
       </c>
     </row>
-    <row r="104" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="104" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B104">
         <f t="shared" si="2"/>
         <v>0.1999965714557792</v>
@@ -5209,7 +5209,7 @@
         <v>40000</v>
       </c>
     </row>
-    <row r="105" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="105" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B105">
         <f t="shared" si="2"/>
         <v>0.19999773981279137</v>
@@ -5219,7 +5219,7 @@
         <v>40500</v>
       </c>
     </row>
-    <row r="106" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="106" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B106">
         <f t="shared" si="2"/>
         <v>0.19999852546471561</v>
@@ -5229,7 +5229,7 @@
         <v>41000</v>
       </c>
     </row>
-    <row r="107" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="107" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B107">
         <f t="shared" si="2"/>
         <v>0.19999904811129313</v>
@@ -5239,7 +5239,7 @@
         <v>41500</v>
       </c>
     </row>
-    <row r="108" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="108" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B108">
         <f t="shared" si="2"/>
         <v>0.19999939203080119</v>
@@ -5249,7 +5249,7 @@
         <v>42000</v>
       </c>
     </row>
-    <row r="109" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="109" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B109">
         <f t="shared" si="2"/>
         <v>0.19999961586354192</v>
@@ -5259,7 +5259,7 @@
         <v>42500</v>
       </c>
     </row>
-    <row r="110" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="110" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B110">
         <f t="shared" si="2"/>
         <v>0.19999975992763294</v>
@@ -5269,7 +5269,7 @@
         <v>43000</v>
       </c>
     </row>
-    <row r="111" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="111" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B111">
         <f t="shared" si="2"/>
         <v>0.19999985161306397</v>
@@ -5279,7 +5279,7 @@
         <v>43500</v>
       </c>
     </row>
-    <row r="112" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="112" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B112">
         <f t="shared" si="2"/>
         <v>0.19999990930357772</v>
@@ -5289,7 +5289,7 @@
         <v>44000</v>
       </c>
     </row>
-    <row r="113" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="113" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B113">
         <f t="shared" si="2"/>
         <v>0.19999994518873965</v>
@@ -5299,7 +5299,7 @@
         <v>44500</v>
       </c>
     </row>
-    <row r="114" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="114" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B114">
         <f t="shared" si="2"/>
         <v>0.19999996725245739</v>
@@ -5309,7 +5309,7 @@
         <v>45000</v>
       </c>
     </row>
-    <row r="115" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="115" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B115">
         <f t="shared" si="2"/>
         <v>0.19999998065979441</v>
@@ -5319,7 +5319,7 @@
         <v>45500</v>
       </c>
     </row>
-    <row r="116" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="116" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B116">
         <f t="shared" si="2"/>
         <v>0.19999998871085503</v>
@@ -5329,7 +5329,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="117" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="117" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B117">
         <f t="shared" si="2"/>
         <v>0.19999999348787459</v>
@@ -5339,7 +5339,7 @@
         <v>46500</v>
       </c>
     </row>
-    <row r="118" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="118" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B118">
         <f t="shared" si="2"/>
         <v>0.19999999628815057</v>
@@ -5349,7 +5349,7 @@
         <v>47000</v>
       </c>
     </row>
-    <row r="119" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="119" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B119">
         <f t="shared" si="2"/>
         <v>0.19999999790970302</v>
@@ -5359,7 +5359,7 @@
         <v>47500</v>
       </c>
     </row>
-    <row r="120" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="120" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B120">
         <f t="shared" si="2"/>
         <v>0.19999999883716038</v>
@@ -5369,7 +5369,7 @@
         <v>48000</v>
       </c>
     </row>
-    <row r="121" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="121" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B121">
         <f t="shared" si="2"/>
         <v>0.19999999936104543</v>
@@ -5379,7 +5379,7 @@
         <v>48500</v>
       </c>
     </row>
-    <row r="122" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="122" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B122">
         <f t="shared" si="2"/>
         <v>0.19999999965326104</v>
@@ -5389,7 +5389,7 @@
         <v>49000</v>
       </c>
     </row>
-    <row r="123" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="123" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B123">
         <f t="shared" si="2"/>
         <v>0.19999999981419306</v>
@@ -5399,7 +5399,7 @@
         <v>49500</v>
       </c>
     </row>
-    <row r="124" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="124" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B124">
         <f t="shared" si="2"/>
         <v>0.19999999990169129</v>
@@ -5409,7 +5409,7 @@
         <v>50000</v>
       </c>
     </row>
-    <row r="125" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="125" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B125">
         <f t="shared" si="2"/>
         <v>0.19999999994865042</v>
@@ -5431,13 +5431,13 @@
     <tabColor rgb="FF002060"/>
   </sheetPr>
   <dimension ref="A1:CF2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:84" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:84" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -5774,7 +5774,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="2" spans="1:84" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:84" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>39</v>
       </c>
@@ -6121,17 +6121,17 @@
     <tabColor rgb="FF002060"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>33</v>
       </c>
@@ -6151,12 +6151,12 @@
     <tabColor rgb="FF002060"/>
   </sheetPr>
   <dimension ref="A1:AB25"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="33.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -6242,7 +6242,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -6328,7 +6328,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -6414,7 +6414,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -6500,7 +6500,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -6586,7 +6586,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -6672,7 +6672,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -6680,25 +6680,25 @@
         <v>0.8</v>
       </c>
       <c r="C7">
-        <v>0.8</v>
+        <v>0.2</v>
       </c>
       <c r="D7">
-        <v>0.8</v>
+        <v>0.2</v>
       </c>
       <c r="E7">
-        <v>0.8</v>
+        <v>0.2</v>
       </c>
       <c r="F7">
-        <v>0.8</v>
+        <v>0.2</v>
       </c>
       <c r="G7">
-        <v>0.8</v>
+        <v>0.2</v>
       </c>
       <c r="H7">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="I7">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="J7">
         <v>0.8</v>
@@ -6758,7 +6758,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -6844,7 +6844,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -6930,7 +6930,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>13</v>
       </c>
@@ -7016,7 +7016,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -7102,7 +7102,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>15</v>
       </c>
@@ -7188,7 +7188,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>16</v>
       </c>
@@ -7274,7 +7274,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>17</v>
       </c>
@@ -7360,7 +7360,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>18</v>
       </c>
@@ -7446,7 +7446,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>19</v>
       </c>
@@ -7532,7 +7532,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>20</v>
       </c>
@@ -7618,7 +7618,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>21</v>
       </c>
@@ -7704,7 +7704,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>22</v>
       </c>
@@ -7790,7 +7790,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>23</v>
       </c>
@@ -7876,7 +7876,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>24</v>
       </c>
@@ -7962,7 +7962,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>25</v>
       </c>
@@ -8048,7 +8048,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>26</v>
       </c>
@@ -8134,7 +8134,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>27</v>
       </c>
@@ -8220,7 +8220,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>28</v>
       </c>

</xml_diff>

<commit_message>
Updated CSC values for wind to reflect real world builds
</commit_message>
<xml_diff>
--- a/InputData/elec/CSC/Capacity Supply Curve.xlsx
+++ b/InputData/elec/CSC/Capacity Supply Curve.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\elec\CSC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\US\Models\eps-us\InputData\elec\CSC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3121D63-400A-431A-800C-74C80046487D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B7F1BAE-163C-41FA-AB1B-7A3F51AD8EB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{F87DB1D1-DC21-4EA7-B1DF-998EE56837F8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="23520" xr2:uid="{F87DB1D1-DC21-4EA7-B1DF-998EE56837F8}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -6680,25 +6680,27 @@
         <v>0.8</v>
       </c>
       <c r="C7">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="D7">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="E7">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="F7">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="G7">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="H7">
-        <v>0.4</v>
+        <f>0.7/3+G7</f>
+        <v>0.33333333333333331</v>
       </c>
       <c r="I7">
-        <v>0.6</v>
+        <f>0.7/3+H7</f>
+        <v>0.56666666666666665</v>
       </c>
       <c r="J7">
         <v>0.8</v>

</xml_diff>

<commit_message>
Moves the capacity supply curve from a LOOKUP to a formula in Vensim; adjusts the minimum build amounts to address an issue we were having; removes extraneous files
</commit_message>
<xml_diff>
--- a/InputData/elec/CSC/Capacity Supply Curve.xlsx
+++ b/InputData/elec/CSC/Capacity Supply Curve.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\US\Models\eps-us\InputData\elec\CSC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B7F1BAE-163C-41FA-AB1B-7A3F51AD8EB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F2CBEFD-F220-4770-9995-1471E0E2C02B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="23520" xr2:uid="{F87DB1D1-DC21-4EA7-B1DF-998EE56837F8}"/>
+    <workbookView xWindow="31305" yWindow="1245" windowWidth="23505" windowHeight="21225" xr2:uid="{F87DB1D1-DC21-4EA7-B1DF-998EE56837F8}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
-    <sheet name="CSC-CSCCCMvSoECBtY" sheetId="2" r:id="rId2"/>
+    <sheet name="CSC-CSCP" sheetId="5" r:id="rId2"/>
     <sheet name="CSC-CSCMBCfPTwNEC" sheetId="3" r:id="rId3"/>
     <sheet name="CSC-CSCSoCECBiaSY" sheetId="4" r:id="rId4"/>
   </sheets>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="47">
   <si>
     <t xml:space="preserve">Source: </t>
   </si>
@@ -45,9 +45,6 @@
   </si>
   <si>
     <t>These are calibrated variables used in establishing supply curves for resources.</t>
-  </si>
-  <si>
-    <t>Share of existing capacity</t>
   </si>
   <si>
     <t>Time (Year)</t>
@@ -140,24 +137,6 @@
     <t>Share</t>
   </si>
   <si>
-    <t>parameter 1</t>
-  </si>
-  <si>
-    <t>parameter 2</t>
-  </si>
-  <si>
-    <t>max share</t>
-  </si>
-  <si>
-    <t>multiplier cutoff</t>
-  </si>
-  <si>
-    <t>Max profitability cutoff</t>
-  </si>
-  <si>
-    <t>Incremental Revenue</t>
-  </si>
-  <si>
     <t>Notes:</t>
   </si>
   <si>
@@ -178,12 +157,33 @@
   <si>
     <t>% of total installed capacity (tied to CSC)</t>
   </si>
+  <si>
+    <t>cutoff parameter</t>
+  </si>
+  <si>
+    <t>saturation</t>
+  </si>
+  <si>
+    <t>scale parameter</t>
+  </si>
+  <si>
+    <t>shape parameter</t>
+  </si>
+  <si>
+    <t>location parameter</t>
+  </si>
+  <si>
+    <t>parameters</t>
+  </si>
+  <si>
+    <t>value</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -193,6 +193,14 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -229,8 +237,8 @@
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1131,1157 +1139,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
-  <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="102"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="2"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
-  <c:chart>
-    <c:title>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
-    </c:title>
-    <c:autoTitleDeleted val="0"/>
-    <c:plotArea>
-      <c:layout/>
-      <c:scatterChart>
-        <c:scatterStyle val="smoothMarker"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent1"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="5"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent1"/>
-              </a:solidFill>
-              <a:ln w="9525">
-                <a:solidFill>
-                  <a:schemeClr val="accent1"/>
-                </a:solidFill>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>'CSC-CSCCCMvSoECBtY'!$B$2:$AP$2</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="41"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>750</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>1500</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>2250</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>3000</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>3750</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>4500</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>5250</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>6000</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>6750</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>7500</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>8250</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>9000</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>9750</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>10500</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>11250</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>12000</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>12750</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>13500</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>14250</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>15000</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>15750</c:v>
-                </c:pt>
-                <c:pt idx="22">
-                  <c:v>16500</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>17250</c:v>
-                </c:pt>
-                <c:pt idx="24">
-                  <c:v>18000</c:v>
-                </c:pt>
-                <c:pt idx="25">
-                  <c:v>18750</c:v>
-                </c:pt>
-                <c:pt idx="26">
-                  <c:v>19500</c:v>
-                </c:pt>
-                <c:pt idx="27">
-                  <c:v>20250</c:v>
-                </c:pt>
-                <c:pt idx="28">
-                  <c:v>21000</c:v>
-                </c:pt>
-                <c:pt idx="29">
-                  <c:v>21750</c:v>
-                </c:pt>
-                <c:pt idx="30">
-                  <c:v>22500</c:v>
-                </c:pt>
-                <c:pt idx="31">
-                  <c:v>23250</c:v>
-                </c:pt>
-                <c:pt idx="32">
-                  <c:v>24000</c:v>
-                </c:pt>
-                <c:pt idx="33">
-                  <c:v>24750</c:v>
-                </c:pt>
-                <c:pt idx="34">
-                  <c:v>25500</c:v>
-                </c:pt>
-                <c:pt idx="35">
-                  <c:v>26250</c:v>
-                </c:pt>
-                <c:pt idx="36">
-                  <c:v>27000</c:v>
-                </c:pt>
-                <c:pt idx="37">
-                  <c:v>27750</c:v>
-                </c:pt>
-                <c:pt idx="38">
-                  <c:v>28500</c:v>
-                </c:pt>
-                <c:pt idx="39">
-                  <c:v>29250</c:v>
-                </c:pt>
-                <c:pt idx="40">
-                  <c:v>30000</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>'CSC-CSCCCMvSoECBtY'!$B$1:$AP$1</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="41"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>1.4467069327128713E-5</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>1.1570725740235322E-4</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>3.9024377850489512E-4</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>9.2378588268478008E-4</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>1.8002974421282847E-3</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>3.1007125989183093E-3</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>4.9013271393022924E-3</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>7.2719111397427484E-3</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>1.0273608123333956E-2</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>1.3956707206263963E-2</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>1.8358395818443476E-2</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>2.3500619483080909E-2</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>2.9388189488745109E-2</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>3.6007286628151627E-2</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>4.3324507187836363E-2</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>5.1286584158818753E-2</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>5.982089105991404E-2</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>6.8836797745699688E-2</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>7.8227898345377744E-2</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>8.787507372604586E-2</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>9.7650288683833367E-2</c:v>
-                </c:pt>
-                <c:pt idx="22">
-                  <c:v>0.10742096270522571</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>0.11705469860772776</c:v>
-                </c:pt>
-                <c:pt idx="24">
-                  <c:v>0.12642411176571153</c:v>
-                </c:pt>
-                <c:pt idx="25">
-                  <c:v>0.13541147940361392</c:v>
-                </c:pt>
-                <c:pt idx="26">
-                  <c:v>0.1439129286073208</c:v>
-                </c:pt>
-                <c:pt idx="27">
-                  <c:v>0.15184190514555035</c:v>
-                </c:pt>
-                <c:pt idx="28">
-                  <c:v>0.1591317121715517</c:v>
-                </c:pt>
-                <c:pt idx="29">
-                  <c:v>0.16573697488151984</c:v>
-                </c:pt>
-                <c:pt idx="30">
-                  <c:v>0.17163396818253152</c:v>
-                </c:pt>
-                <c:pt idx="31">
-                  <c:v>0.17681983138790913</c:v>
-                </c:pt>
-                <c:pt idx="32">
-                  <c:v>0.18131077796047496</c:v>
-                </c:pt>
-                <c:pt idx="33">
-                  <c:v>0.18513948060036278</c:v>
-                </c:pt>
-                <c:pt idx="34">
-                  <c:v>0.18835186512938695</c:v>
-                </c:pt>
-                <c:pt idx="35">
-                  <c:v>0.19100357564494788</c:v>
-                </c:pt>
-                <c:pt idx="36">
-                  <c:v>0.1931563763376668</c:v>
-                </c:pt>
-                <c:pt idx="37">
-                  <c:v>0.19487473347482187</c:v>
-                </c:pt>
-                <c:pt idx="38">
-                  <c:v>0.19622277858911699</c:v>
-                </c:pt>
-                <c:pt idx="39">
-                  <c:v>0.1972617973403015</c:v>
-                </c:pt>
-                <c:pt idx="40">
-                  <c:v>0.19804832547095644</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="1"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-5E3E-4506-B7FF-2865DFAAB582}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:axId val="1627802751"/>
-        <c:axId val="1627803711"/>
-      </c:scatterChart>
-      <c:valAx>
-        <c:axId val="1627802751"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="25000"/>
-                <a:lumOff val="75000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="1627803711"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:valAx>
-        <c:axId val="1627803711"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="25000"/>
-                <a:lumOff val="75000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="1627802751"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-    </c:plotArea>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
-    <c:extLst>
-      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
-        <c16r3:dataDisplayOptions16>
-          <c16r3:dispNaAsBlank val="1"/>
-        </c16r3:dataDisplayOptions16>
-      </c:ext>
-    </c:extLst>
-  </c:chart>
-  <c:spPr>
-    <a:solidFill>
-      <a:schemeClr val="bg1"/>
-    </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:round/>
-    </a:ln>
-    <a:effectLst/>
-  </c:spPr>
-  <c:txPr>
-    <a:bodyPr/>
-    <a:lstStyle/>
-    <a:p>
-      <a:pPr>
-        <a:defRPr/>
-      </a:pPr>
-      <a:endParaRPr lang="en-US"/>
-    </a:p>
-  </c:txPr>
-  <c:printSettings>
-    <c:headerFooter/>
-    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
-    <c:pageSetup/>
-  </c:printSettings>
-</c:chartSpace>
-</file>
-
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
-  <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="102"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="2"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
-  <c:chart>
-    <c:title>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
-    </c:title>
-    <c:autoTitleDeleted val="0"/>
-    <c:plotArea>
-      <c:layout/>
-      <c:scatterChart>
-        <c:scatterStyle val="smoothMarker"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent1"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="5"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent1"/>
-              </a:solidFill>
-              <a:ln w="9525">
-                <a:solidFill>
-                  <a:schemeClr val="accent1"/>
-                </a:solidFill>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>'CSC-CSCCCMvSoECBtY'!$B$2:$AP$2</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="41"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>750</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>1500</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>2250</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>3000</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>3750</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>4500</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>5250</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>6000</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>6750</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>7500</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>8250</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>9000</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>9750</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>10500</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>11250</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>12000</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>12750</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>13500</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>14250</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>15000</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>15750</c:v>
-                </c:pt>
-                <c:pt idx="22">
-                  <c:v>16500</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>17250</c:v>
-                </c:pt>
-                <c:pt idx="24">
-                  <c:v>18000</c:v>
-                </c:pt>
-                <c:pt idx="25">
-                  <c:v>18750</c:v>
-                </c:pt>
-                <c:pt idx="26">
-                  <c:v>19500</c:v>
-                </c:pt>
-                <c:pt idx="27">
-                  <c:v>20250</c:v>
-                </c:pt>
-                <c:pt idx="28">
-                  <c:v>21000</c:v>
-                </c:pt>
-                <c:pt idx="29">
-                  <c:v>21750</c:v>
-                </c:pt>
-                <c:pt idx="30">
-                  <c:v>22500</c:v>
-                </c:pt>
-                <c:pt idx="31">
-                  <c:v>23250</c:v>
-                </c:pt>
-                <c:pt idx="32">
-                  <c:v>24000</c:v>
-                </c:pt>
-                <c:pt idx="33">
-                  <c:v>24750</c:v>
-                </c:pt>
-                <c:pt idx="34">
-                  <c:v>25500</c:v>
-                </c:pt>
-                <c:pt idx="35">
-                  <c:v>26250</c:v>
-                </c:pt>
-                <c:pt idx="36">
-                  <c:v>27000</c:v>
-                </c:pt>
-                <c:pt idx="37">
-                  <c:v>27750</c:v>
-                </c:pt>
-                <c:pt idx="38">
-                  <c:v>28500</c:v>
-                </c:pt>
-                <c:pt idx="39">
-                  <c:v>29250</c:v>
-                </c:pt>
-                <c:pt idx="40">
-                  <c:v>30000</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>'CSC-CSCCCMvSoECBtY'!$B$1:$AP$1</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="41"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>1.4467069327128713E-5</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>1.1570725740235322E-4</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>3.9024377850489512E-4</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>9.2378588268478008E-4</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>1.8002974421282847E-3</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>3.1007125989183093E-3</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>4.9013271393022924E-3</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>7.2719111397427484E-3</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>1.0273608123333956E-2</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>1.3956707206263963E-2</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>1.8358395818443476E-2</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>2.3500619483080909E-2</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>2.9388189488745109E-2</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>3.6007286628151627E-2</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>4.3324507187836363E-2</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>5.1286584158818753E-2</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>5.982089105991404E-2</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>6.8836797745699688E-2</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>7.8227898345377744E-2</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>8.787507372604586E-2</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>9.7650288683833367E-2</c:v>
-                </c:pt>
-                <c:pt idx="22">
-                  <c:v>0.10742096270522571</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>0.11705469860772776</c:v>
-                </c:pt>
-                <c:pt idx="24">
-                  <c:v>0.12642411176571153</c:v>
-                </c:pt>
-                <c:pt idx="25">
-                  <c:v>0.13541147940361392</c:v>
-                </c:pt>
-                <c:pt idx="26">
-                  <c:v>0.1439129286073208</c:v>
-                </c:pt>
-                <c:pt idx="27">
-                  <c:v>0.15184190514555035</c:v>
-                </c:pt>
-                <c:pt idx="28">
-                  <c:v>0.1591317121715517</c:v>
-                </c:pt>
-                <c:pt idx="29">
-                  <c:v>0.16573697488151984</c:v>
-                </c:pt>
-                <c:pt idx="30">
-                  <c:v>0.17163396818253152</c:v>
-                </c:pt>
-                <c:pt idx="31">
-                  <c:v>0.17681983138790913</c:v>
-                </c:pt>
-                <c:pt idx="32">
-                  <c:v>0.18131077796047496</c:v>
-                </c:pt>
-                <c:pt idx="33">
-                  <c:v>0.18513948060036278</c:v>
-                </c:pt>
-                <c:pt idx="34">
-                  <c:v>0.18835186512938695</c:v>
-                </c:pt>
-                <c:pt idx="35">
-                  <c:v>0.19100357564494788</c:v>
-                </c:pt>
-                <c:pt idx="36">
-                  <c:v>0.1931563763376668</c:v>
-                </c:pt>
-                <c:pt idx="37">
-                  <c:v>0.19487473347482187</c:v>
-                </c:pt>
-                <c:pt idx="38">
-                  <c:v>0.19622277858911699</c:v>
-                </c:pt>
-                <c:pt idx="39">
-                  <c:v>0.1972617973403015</c:v>
-                </c:pt>
-                <c:pt idx="40">
-                  <c:v>0.19804832547095644</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="1"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-D9CD-43DB-BDE0-8A392742F499}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:axId val="1627802751"/>
-        <c:axId val="1627803711"/>
-      </c:scatterChart>
-      <c:valAx>
-        <c:axId val="1627802751"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="25000"/>
-                <a:lumOff val="75000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="1627803711"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:valAx>
-        <c:axId val="1627803711"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="25000"/>
-                <a:lumOff val="75000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="1627802751"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-    </c:plotArea>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
-    <c:extLst>
-      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
-        <c16r3:dataDisplayOptions16>
-          <c16r3:dispNaAsBlank val="1"/>
-        </c16r3:dataDisplayOptions16>
-      </c:ext>
-    </c:extLst>
-  </c:chart>
-  <c:spPr>
-    <a:solidFill>
-      <a:schemeClr val="bg1"/>
-    </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:round/>
-    </a:ln>
-    <a:effectLst/>
-  </c:spPr>
-  <c:txPr>
-    <a:bodyPr/>
-    <a:lstStyle/>
-    <a:p>
-      <a:pPr>
-        <a:defRPr/>
-      </a:pPr>
-      <a:endParaRPr lang="en-US"/>
-    </a:p>
-  </c:txPr>
-  <c:printSettings>
-    <c:headerFooter/>
-    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
-    <c:pageSetup/>
-  </c:printSettings>
-</c:chartSpace>
-</file>
-
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
-  <a:schemeClr val="accent1"/>
-  <a:schemeClr val="accent2"/>
-  <a:schemeClr val="accent3"/>
-  <a:schemeClr val="accent4"/>
-  <a:schemeClr val="accent5"/>
-  <a:schemeClr val="accent6"/>
-  <cs:variation/>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-    <a:lumOff val="20000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-    <a:lumOff val="40000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-    <a:lumOff val="30000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-    <a:lumOff val="50000"/>
-  </cs:variation>
-</cs:colorStyle>
-</file>
-
-<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
-  <a:schemeClr val="accent1"/>
-  <a:schemeClr val="accent2"/>
-  <a:schemeClr val="accent3"/>
-  <a:schemeClr val="accent4"/>
-  <a:schemeClr val="accent5"/>
-  <a:schemeClr val="accent6"/>
-  <cs:variation/>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-    <a:lumOff val="20000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-    <a:lumOff val="40000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-    <a:lumOff val="30000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-    <a:lumOff val="50000"/>
-  </cs:variation>
-</cs:colorStyle>
-</file>
-
-<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -2837,1052 +1695,20 @@
 </cs:chartStyle>
 </file>
 
-<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
-  <cs:axisTitle>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:axisTitle>
-  <cs:categoryAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:categoryAxis>
-  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="bg1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:chartArea>
-  <cs:dataLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataLabel>
-  <cs:dataLabelCallout>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
-      <a:spAutoFit/>
-    </cs:bodyPr>
-  </cs:dataLabelCallout>
-  <cs:dataPoint>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint>
-  <cs:dataPoint3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint3D>
-  <cs:dataPointLine>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointLine>
-  <cs:dataPointMarker>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
-  <cs:dataPointWireframe>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointWireframe>
-  <cs:dataTable>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataTable>
-  <cs:downBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="75000"/>
-          <a:lumOff val="25000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:downBar>
-  <cs:dropLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dropLine>
-  <cs:errorBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:errorBar>
-  <cs:floor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:floor>
-  <cs:gridlineMajor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMajor>
-  <cs:gridlineMinor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="5000"/>
-            <a:lumOff val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:legend>
-  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea>
-  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:seriesLine>
-  <cs:title>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
-  </cs:title>
-  <cs:trendline>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:prstDash val="sysDot"/>
-      </a:ln>
-    </cs:spPr>
-  </cs:trendline>
-  <cs:trendlineLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:trendlineLabel>
-  <cs:upBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:upBar>
-  <cs:valueAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:valueAxis>
-  <cs:wall>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:wall>
-</cs:chartStyle>
-</file>
-
-<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
-  <cs:axisTitle>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:axisTitle>
-  <cs:categoryAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:categoryAxis>
-  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="bg1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:chartArea>
-  <cs:dataLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataLabel>
-  <cs:dataLabelCallout>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
-      <a:spAutoFit/>
-    </cs:bodyPr>
-  </cs:dataLabelCallout>
-  <cs:dataPoint>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint>
-  <cs:dataPoint3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint3D>
-  <cs:dataPointLine>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointLine>
-  <cs:dataPointMarker>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
-  <cs:dataPointWireframe>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointWireframe>
-  <cs:dataTable>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataTable>
-  <cs:downBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="75000"/>
-          <a:lumOff val="25000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:downBar>
-  <cs:dropLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dropLine>
-  <cs:errorBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:errorBar>
-  <cs:floor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:floor>
-  <cs:gridlineMajor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMajor>
-  <cs:gridlineMinor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="5000"/>
-            <a:lumOff val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:legend>
-  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea>
-  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:seriesLine>
-  <cs:title>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
-  </cs:title>
-  <cs:trendline>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:prstDash val="sysDot"/>
-      </a:ln>
-    </cs:spPr>
-  </cs:trendline>
-  <cs:trendlineLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:trendlineLabel>
-  <cs:upBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:upBar>
-  <cs:valueAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:valueAxis>
-  <cs:wall>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:wall>
-</cs:chartStyle>
-</file>
-
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>428625</xdr:colOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>484003</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>151130</xdr:rowOff>
+      <xdr:rowOff>184356</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>123825</xdr:colOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>5052459</xdr:colOff>
       <xdr:row>37</xdr:row>
-      <xdr:rowOff>138430</xdr:rowOff>
+      <xdr:rowOff>171656</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -3890,85 +1716,6 @@
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C1103698-6335-5964-6586-96038B70278E}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr/>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="0" y="0"/>
-        <a:ext cx="0" cy="0"/>
-      </xdr:xfrm>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>638175</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>5210175</xdr:colOff>
-      <xdr:row>37</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="4" name="Chart 3">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{12E5539E-DC92-4633-8C32-ACBC3A592645}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr>
-          <a:graphicFrameLocks/>
-        </xdr:cNvGraphicFramePr>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="0" y="0"/>
-        <a:ext cx="0" cy="0"/>
-      </xdr:xfrm>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>190500</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>100012</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>495300</xdr:colOff>
-      <xdr:row>35</xdr:row>
-      <xdr:rowOff>176212</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Chart 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{19E926C4-5B99-77EC-1DCF-F92850905973}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4295,17 +2042,17 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -4318,27 +2065,27 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -4351,12 +2098,12 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="B16">
         <v>0.2</v>
@@ -4364,7 +2111,7 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="B17">
         <v>0.6</v>
@@ -4372,7 +2119,7 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="B18">
         <v>3</v>
@@ -4380,7 +2127,7 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="B19">
         <v>0.5</v>
@@ -4388,7 +2135,7 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B20">
         <v>30000</v>
@@ -4396,7 +2143,7 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="B21">
         <v>4.0000000000000001E-3</v>
@@ -5426,692 +3173,71 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54A8C2E7-868E-446E-8321-CDDE5386BCAC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19F1B329-5591-420B-9DBA-D539EDB26DE6}">
   <sheetPr>
     <tabColor rgb="FF002060"/>
   </sheetPr>
-  <dimension ref="A1:CF2"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:84" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B2" s="2">
+        <f>About!B16</f>
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B3" s="2">
+        <f>About!B17</f>
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B4" s="2">
+        <f>About!B18</f>
         <v>3</v>
       </c>
-      <c r="B1">
-        <f>(1-EXP(-((B2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0</v>
-      </c>
-      <c r="C1">
-        <f>(1-EXP(-((C2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>1.4467069327128713E-5</v>
-      </c>
-      <c r="D1">
-        <f>(1-EXP(-((D2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>1.1570725740235322E-4</v>
-      </c>
-      <c r="E1">
-        <f>(1-EXP(-((E2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>3.9024377850489512E-4</v>
-      </c>
-      <c r="F1">
-        <f>(1-EXP(-((F2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>9.2378588268478008E-4</v>
-      </c>
-      <c r="G1">
-        <f>(1-EXP(-((G2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>1.8002974421282847E-3</v>
-      </c>
-      <c r="H1">
-        <f>(1-EXP(-((H2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>3.1007125989183093E-3</v>
-      </c>
-      <c r="I1">
-        <f>(1-EXP(-((I2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>4.9013271393022924E-3</v>
-      </c>
-      <c r="J1">
-        <f>(1-EXP(-((J2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>7.2719111397427484E-3</v>
-      </c>
-      <c r="K1">
-        <f>(1-EXP(-((K2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>1.0273608123333956E-2</v>
-      </c>
-      <c r="L1">
-        <f>(1-EXP(-((L2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>1.3956707206263963E-2</v>
-      </c>
-      <c r="M1">
-        <f>(1-EXP(-((M2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>1.8358395818443476E-2</v>
-      </c>
-      <c r="N1">
-        <f>(1-EXP(-((N2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>2.3500619483080909E-2</v>
-      </c>
-      <c r="O1">
-        <f>(1-EXP(-((O2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>2.9388189488745109E-2</v>
-      </c>
-      <c r="P1">
-        <f>(1-EXP(-((P2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>3.6007286628151627E-2</v>
-      </c>
-      <c r="Q1">
-        <f>(1-EXP(-((Q2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>4.3324507187836363E-2</v>
-      </c>
-      <c r="R1">
-        <f>(1-EXP(-((R2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>5.1286584158818753E-2</v>
-      </c>
-      <c r="S1">
-        <f>(1-EXP(-((S2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>5.982089105991404E-2</v>
-      </c>
-      <c r="T1">
-        <f>(1-EXP(-((T2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>6.8836797745699688E-2</v>
-      </c>
-      <c r="U1">
-        <f>(1-EXP(-((U2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>7.8227898345377744E-2</v>
-      </c>
-      <c r="V1">
-        <f>(1-EXP(-((V2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>8.787507372604586E-2</v>
-      </c>
-      <c r="W1">
-        <f>(1-EXP(-((W2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>9.7650288683833367E-2</v>
-      </c>
-      <c r="X1">
-        <f>(1-EXP(-((X2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.10742096270522571</v>
-      </c>
-      <c r="Y1">
-        <f>(1-EXP(-((Y2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.11705469860772776</v>
-      </c>
-      <c r="Z1">
-        <f>(1-EXP(-((Z2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.12642411176571153</v>
-      </c>
-      <c r="AA1">
-        <f>(1-EXP(-((AA2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.13541147940361392</v>
-      </c>
-      <c r="AB1">
-        <f>(1-EXP(-((AB2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.1439129286073208</v>
-      </c>
-      <c r="AC1">
-        <f>(1-EXP(-((AC2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.15184190514555035</v>
-      </c>
-      <c r="AD1">
-        <f>(1-EXP(-((AD2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.1591317121715517</v>
-      </c>
-      <c r="AE1">
-        <f>(1-EXP(-((AE2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.16573697488151984</v>
-      </c>
-      <c r="AF1">
-        <f>(1-EXP(-((AF2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.17163396818253152</v>
-      </c>
-      <c r="AG1">
-        <f>(1-EXP(-((AG2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.17681983138790913</v>
-      </c>
-      <c r="AH1">
-        <f>(1-EXP(-((AH2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.18131077796047496</v>
-      </c>
-      <c r="AI1">
-        <f>(1-EXP(-((AI2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.18513948060036278</v>
-      </c>
-      <c r="AJ1">
-        <f>(1-EXP(-((AJ2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.18835186512938695</v>
-      </c>
-      <c r="AK1">
-        <f>(1-EXP(-((AK2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19100357564494788</v>
-      </c>
-      <c r="AL1">
-        <f>(1-EXP(-((AL2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.1931563763376668</v>
-      </c>
-      <c r="AM1">
-        <f>(1-EXP(-((AM2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19487473347482187</v>
-      </c>
-      <c r="AN1">
-        <f>(1-EXP(-((AN2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19622277858911699</v>
-      </c>
-      <c r="AO1">
-        <f>(1-EXP(-((AO2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.1972617973403015</v>
-      </c>
-      <c r="AP1">
-        <f>(1-EXP(-((AP2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19804832547095644</v>
-      </c>
-      <c r="AQ1">
-        <f>(1-EXP(-((AQ2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19863287140923547</v>
-      </c>
-      <c r="AR1">
-        <f>(1-EXP(-((AR2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19905923098155251</v>
-      </c>
-      <c r="AS1">
-        <f>(1-EXP(-((AS2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.199364318136077</v>
-      </c>
-      <c r="AT1">
-        <f>(1-EXP(-((AT2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19957840901739385</v>
-      </c>
-      <c r="AU1">
-        <f>(1-EXP(-((AU2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.1997256853595088</v>
-      </c>
-      <c r="AV1">
-        <f>(1-EXP(-((AV2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19982496522253218</v>
-      </c>
-      <c r="AW1">
-        <f>(1-EXP(-((AW2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19989052148534298</v>
-      </c>
-      <c r="AX1">
-        <f>(1-EXP(-((AX2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.1999329074744195</v>
-      </c>
-      <c r="AY1">
-        <f>(1-EXP(-((AY2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19995973093159392</v>
-      </c>
-      <c r="AZ1">
-        <f>(1-EXP(-((AZ2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19997633902006273</v>
-      </c>
-      <c r="BA1">
-        <f>(1-EXP(-((BA2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19998639592309114</v>
-      </c>
-      <c r="BB1">
-        <f>(1-EXP(-((BB2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19999234945911523</v>
-      </c>
-      <c r="BC1">
-        <f>(1-EXP(-((BC2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19999579357241226</v>
-      </c>
-      <c r="BD1">
-        <f>(1-EXP(-((BD2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19999773981279137</v>
-      </c>
-      <c r="BE1">
-        <f>(1-EXP(-((BE2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19999881369426081</v>
-      </c>
-      <c r="BF1">
-        <f>(1-EXP(-((BF2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19999939203080119</v>
-      </c>
-      <c r="BG1">
-        <f>(1-EXP(-((BG2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19999969590396702</v>
-      </c>
-      <c r="BH1">
-        <f>(1-EXP(-((BH2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19999985161306397</v>
-      </c>
-      <c r="BI1">
-        <f>(1-EXP(-((BI2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19999992939299016</v>
-      </c>
-      <c r="BJ1">
-        <f>(1-EXP(-((BJ2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19999996725245739</v>
-      </c>
-      <c r="BK1">
-        <f>(1-EXP(-((BK2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19999998520210779</v>
-      </c>
-      <c r="BL1">
-        <f>(1-EXP(-((BL2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19999999348787459</v>
-      </c>
-      <c r="BM1">
-        <f>(1-EXP(-((BM2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19999999721029099</v>
-      </c>
-      <c r="BN1">
-        <f>(1-EXP(-((BN2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19999999883716038</v>
-      </c>
-      <c r="BO1">
-        <f>(1-EXP(-((BO2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19999999952857025</v>
-      </c>
-      <c r="BP1">
-        <f>(1-EXP(-((BP2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19999999981419306</v>
-      </c>
-      <c r="BQ1">
-        <f>(1-EXP(-((BQ2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19999999992883505</v>
-      </c>
-      <c r="BR1">
-        <f>(1-EXP(-((BR2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19999999997352469</v>
-      </c>
-      <c r="BS1">
-        <f>(1-EXP(-((BS2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19999999999043694</v>
-      </c>
-      <c r="BT1">
-        <f>(1-EXP(-((BT2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19999999999664766</v>
-      </c>
-      <c r="BU1">
-        <f>(1-EXP(-((BU2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19999999999886001</v>
-      </c>
-      <c r="BV1">
-        <f>(1-EXP(-((BV2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19999999999962412</v>
-      </c>
-      <c r="BW1">
-        <f>(1-EXP(-((BW2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19999999999987986</v>
-      </c>
-      <c r="BX1">
-        <f>(1-EXP(-((BX2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19999999999996282</v>
-      </c>
-      <c r="BY1">
-        <f>(1-EXP(-((BY2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19999999999998885</v>
-      </c>
-      <c r="BZ1">
-        <f>(1-EXP(-((BZ2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19999999999999676</v>
-      </c>
-      <c r="CA1">
-        <f>(1-EXP(-((CA2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.1999999999999991</v>
-      </c>
-      <c r="CB1">
-        <f>(1-EXP(-((CB2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19999999999999976</v>
-      </c>
-      <c r="CC1">
-        <f>(1-EXP(-((CC2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19999999999999996</v>
-      </c>
-      <c r="CD1">
-        <f>(1-EXP(-((CD2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.19999999999999998</v>
-      </c>
-      <c r="CE1">
-        <f>(1-EXP(-((CE2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.2</v>
-      </c>
-      <c r="CF1">
-        <f>(1-EXP(-((CF2/About!$B$20-(About!$B$19-0.5))/About!$B$17)^About!$B$18))*About!$B$16</f>
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:84" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>39</v>
-      </c>
-      <c r="B2">
-        <v>0</v>
-      </c>
-      <c r="C2">
-        <f>B2+750</f>
-        <v>750</v>
-      </c>
-      <c r="D2">
-        <f t="shared" ref="D2:BO2" si="0">C2+750</f>
-        <v>1500</v>
-      </c>
-      <c r="E2">
-        <f t="shared" si="0"/>
-        <v>2250</v>
-      </c>
-      <c r="F2">
-        <f t="shared" si="0"/>
-        <v>3000</v>
-      </c>
-      <c r="G2">
-        <f t="shared" si="0"/>
-        <v>3750</v>
-      </c>
-      <c r="H2">
-        <f t="shared" si="0"/>
-        <v>4500</v>
-      </c>
-      <c r="I2">
-        <f t="shared" si="0"/>
-        <v>5250</v>
-      </c>
-      <c r="J2">
-        <f t="shared" si="0"/>
-        <v>6000</v>
-      </c>
-      <c r="K2">
-        <f t="shared" si="0"/>
-        <v>6750</v>
-      </c>
-      <c r="L2">
-        <f t="shared" si="0"/>
-        <v>7500</v>
-      </c>
-      <c r="M2">
-        <f t="shared" si="0"/>
-        <v>8250</v>
-      </c>
-      <c r="N2">
-        <f t="shared" si="0"/>
-        <v>9000</v>
-      </c>
-      <c r="O2">
-        <f t="shared" si="0"/>
-        <v>9750</v>
-      </c>
-      <c r="P2">
-        <f t="shared" si="0"/>
-        <v>10500</v>
-      </c>
-      <c r="Q2">
-        <f t="shared" si="0"/>
-        <v>11250</v>
-      </c>
-      <c r="R2">
-        <f t="shared" si="0"/>
-        <v>12000</v>
-      </c>
-      <c r="S2">
-        <f t="shared" si="0"/>
-        <v>12750</v>
-      </c>
-      <c r="T2">
-        <f t="shared" si="0"/>
-        <v>13500</v>
-      </c>
-      <c r="U2">
-        <f t="shared" si="0"/>
-        <v>14250</v>
-      </c>
-      <c r="V2">
-        <f t="shared" si="0"/>
-        <v>15000</v>
-      </c>
-      <c r="W2">
-        <f t="shared" si="0"/>
-        <v>15750</v>
-      </c>
-      <c r="X2">
-        <f t="shared" si="0"/>
-        <v>16500</v>
-      </c>
-      <c r="Y2">
-        <f t="shared" si="0"/>
-        <v>17250</v>
-      </c>
-      <c r="Z2">
-        <f t="shared" si="0"/>
-        <v>18000</v>
-      </c>
-      <c r="AA2">
-        <f t="shared" si="0"/>
-        <v>18750</v>
-      </c>
-      <c r="AB2">
-        <f t="shared" si="0"/>
-        <v>19500</v>
-      </c>
-      <c r="AC2">
-        <f t="shared" si="0"/>
-        <v>20250</v>
-      </c>
-      <c r="AD2">
-        <f t="shared" si="0"/>
-        <v>21000</v>
-      </c>
-      <c r="AE2">
-        <f t="shared" si="0"/>
-        <v>21750</v>
-      </c>
-      <c r="AF2">
-        <f t="shared" si="0"/>
-        <v>22500</v>
-      </c>
-      <c r="AG2">
-        <f t="shared" si="0"/>
-        <v>23250</v>
-      </c>
-      <c r="AH2">
-        <f t="shared" si="0"/>
-        <v>24000</v>
-      </c>
-      <c r="AI2">
-        <f t="shared" si="0"/>
-        <v>24750</v>
-      </c>
-      <c r="AJ2">
-        <f t="shared" si="0"/>
-        <v>25500</v>
-      </c>
-      <c r="AK2">
-        <f t="shared" si="0"/>
-        <v>26250</v>
-      </c>
-      <c r="AL2">
-        <f t="shared" si="0"/>
-        <v>27000</v>
-      </c>
-      <c r="AM2">
-        <f t="shared" si="0"/>
-        <v>27750</v>
-      </c>
-      <c r="AN2">
-        <f t="shared" si="0"/>
-        <v>28500</v>
-      </c>
-      <c r="AO2">
-        <f t="shared" si="0"/>
-        <v>29250</v>
-      </c>
-      <c r="AP2">
-        <f t="shared" si="0"/>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B5" s="2">
+        <f>About!B19</f>
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="2">
+        <f>About!B20</f>
         <v>30000</v>
-      </c>
-      <c r="AQ2">
-        <f t="shared" si="0"/>
-        <v>30750</v>
-      </c>
-      <c r="AR2">
-        <f t="shared" si="0"/>
-        <v>31500</v>
-      </c>
-      <c r="AS2">
-        <f t="shared" si="0"/>
-        <v>32250</v>
-      </c>
-      <c r="AT2">
-        <f t="shared" si="0"/>
-        <v>33000</v>
-      </c>
-      <c r="AU2">
-        <f t="shared" si="0"/>
-        <v>33750</v>
-      </c>
-      <c r="AV2">
-        <f t="shared" si="0"/>
-        <v>34500</v>
-      </c>
-      <c r="AW2">
-        <f t="shared" si="0"/>
-        <v>35250</v>
-      </c>
-      <c r="AX2">
-        <f t="shared" si="0"/>
-        <v>36000</v>
-      </c>
-      <c r="AY2">
-        <f t="shared" si="0"/>
-        <v>36750</v>
-      </c>
-      <c r="AZ2">
-        <f t="shared" si="0"/>
-        <v>37500</v>
-      </c>
-      <c r="BA2">
-        <f t="shared" si="0"/>
-        <v>38250</v>
-      </c>
-      <c r="BB2">
-        <f t="shared" si="0"/>
-        <v>39000</v>
-      </c>
-      <c r="BC2">
-        <f t="shared" si="0"/>
-        <v>39750</v>
-      </c>
-      <c r="BD2">
-        <f t="shared" si="0"/>
-        <v>40500</v>
-      </c>
-      <c r="BE2">
-        <f t="shared" si="0"/>
-        <v>41250</v>
-      </c>
-      <c r="BF2">
-        <f t="shared" si="0"/>
-        <v>42000</v>
-      </c>
-      <c r="BG2">
-        <f t="shared" si="0"/>
-        <v>42750</v>
-      </c>
-      <c r="BH2">
-        <f t="shared" si="0"/>
-        <v>43500</v>
-      </c>
-      <c r="BI2">
-        <f t="shared" si="0"/>
-        <v>44250</v>
-      </c>
-      <c r="BJ2">
-        <f t="shared" si="0"/>
-        <v>45000</v>
-      </c>
-      <c r="BK2">
-        <f t="shared" si="0"/>
-        <v>45750</v>
-      </c>
-      <c r="BL2">
-        <f t="shared" si="0"/>
-        <v>46500</v>
-      </c>
-      <c r="BM2">
-        <f t="shared" si="0"/>
-        <v>47250</v>
-      </c>
-      <c r="BN2">
-        <f t="shared" si="0"/>
-        <v>48000</v>
-      </c>
-      <c r="BO2">
-        <f t="shared" si="0"/>
-        <v>48750</v>
-      </c>
-      <c r="BP2">
-        <f t="shared" ref="BP2:CE2" si="1">BO2+750</f>
-        <v>49500</v>
-      </c>
-      <c r="BQ2">
-        <f t="shared" si="1"/>
-        <v>50250</v>
-      </c>
-      <c r="BR2">
-        <f t="shared" si="1"/>
-        <v>51000</v>
-      </c>
-      <c r="BS2">
-        <f t="shared" si="1"/>
-        <v>51750</v>
-      </c>
-      <c r="BT2">
-        <f t="shared" si="1"/>
-        <v>52500</v>
-      </c>
-      <c r="BU2">
-        <f t="shared" si="1"/>
-        <v>53250</v>
-      </c>
-      <c r="BV2">
-        <f t="shared" si="1"/>
-        <v>54000</v>
-      </c>
-      <c r="BW2">
-        <f t="shared" si="1"/>
-        <v>54750</v>
-      </c>
-      <c r="BX2">
-        <f t="shared" si="1"/>
-        <v>55500</v>
-      </c>
-      <c r="BY2">
-        <f t="shared" si="1"/>
-        <v>56250</v>
-      </c>
-      <c r="BZ2">
-        <f t="shared" si="1"/>
-        <v>57000</v>
-      </c>
-      <c r="CA2">
-        <f t="shared" si="1"/>
-        <v>57750</v>
-      </c>
-      <c r="CB2">
-        <f t="shared" si="1"/>
-        <v>58500</v>
-      </c>
-      <c r="CC2">
-        <f t="shared" si="1"/>
-        <v>59250</v>
-      </c>
-      <c r="CD2">
-        <f t="shared" si="1"/>
-        <v>60000</v>
-      </c>
-      <c r="CE2">
-        <f t="shared" si="1"/>
-        <v>60750</v>
-      </c>
-      <c r="CF2" s="2">
-        <v>1000000000000</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -6128,14 +3254,14 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="B2" s="3">
+        <v>32</v>
+      </c>
+      <c r="B2" s="2">
         <f>About!B21/About!B16</f>
         <v>0.02</v>
       </c>
@@ -6158,7 +3284,7 @@
   <sheetData>
     <row r="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B1">
         <v>2024</v>
@@ -6244,7 +3370,7 @@
     </row>
     <row r="2" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -6330,7 +3456,7 @@
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B3">
         <v>1</v>
@@ -6416,7 +3542,7 @@
     </row>
     <row r="4" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B4">
         <v>1</v>
@@ -6502,7 +3628,7 @@
     </row>
     <row r="5" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B5">
         <v>1</v>
@@ -6588,7 +3714,7 @@
     </row>
     <row r="6" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B6">
         <v>1</v>
@@ -6674,7 +3800,7 @@
     </row>
     <row r="7" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B7">
         <v>0.8</v>
@@ -6762,7 +3888,7 @@
     </row>
     <row r="8" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B8">
         <v>1</v>
@@ -6848,7 +3974,7 @@
     </row>
     <row r="9" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B9">
         <v>1</v>
@@ -6934,7 +4060,7 @@
     </row>
     <row r="10" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B10">
         <v>1</v>
@@ -7020,7 +4146,7 @@
     </row>
     <row r="11" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B11">
         <v>1</v>
@@ -7106,7 +4232,7 @@
     </row>
     <row r="12" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B12">
         <v>1</v>
@@ -7192,7 +4318,7 @@
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B13">
         <v>1</v>
@@ -7278,7 +4404,7 @@
     </row>
     <row r="14" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B14">
         <v>1</v>
@@ -7364,7 +4490,7 @@
     </row>
     <row r="15" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B15">
         <v>1</v>
@@ -7450,7 +4576,7 @@
     </row>
     <row r="16" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B16">
         <v>1</v>
@@ -7536,7 +4662,7 @@
     </row>
     <row r="17" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B17">
         <v>1</v>
@@ -7622,7 +4748,7 @@
     </row>
     <row r="18" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B18">
         <v>1</v>
@@ -7708,7 +4834,7 @@
     </row>
     <row r="19" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B19">
         <v>1</v>
@@ -7794,7 +4920,7 @@
     </row>
     <row r="20" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B20">
         <v>1</v>
@@ -7880,7 +5006,7 @@
     </row>
     <row r="21" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B21">
         <v>1</v>
@@ -7966,7 +5092,7 @@
     </row>
     <row r="22" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B22">
         <v>1</v>
@@ -8052,7 +5178,7 @@
     </row>
     <row r="23" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B23">
         <v>1</v>
@@ -8138,7 +5264,7 @@
     </row>
     <row r="24" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B24">
         <v>1</v>
@@ -8224,7 +5350,7 @@
     </row>
     <row r="25" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B25">
         <v>1</v>

</xml_diff>

<commit_message>
In-progress edit to modify soft cap and supply curve logic, avoiding overly large entries for technologies with zero existing capacity
</commit_message>
<xml_diff>
--- a/InputData/elec/CSC/Capacity Supply Curve.xlsx
+++ b/InputData/elec/CSC/Capacity Supply Curve.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\US\Models\eps-us\InputData\elec\CSC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us-seedtest\InputData\elec\CSC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F2CBEFD-F220-4770-9995-1471E0E2C02B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C6D9FC2-5DEB-4799-871F-1C55C23668A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31305" yWindow="1245" windowWidth="23505" windowHeight="21225" xr2:uid="{F87DB1D1-DC21-4EA7-B1DF-998EE56837F8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="4" xr2:uid="{F87DB1D1-DC21-4EA7-B1DF-998EE56837F8}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
-    <sheet name="CSC-CSCP" sheetId="5" r:id="rId2"/>
-    <sheet name="CSC-CSCMBCfPTwNEC" sheetId="3" r:id="rId3"/>
+    <sheet name="CSC-CSCPH" sheetId="6" r:id="rId2"/>
+    <sheet name="CSC-CSCP" sheetId="5" r:id="rId3"/>
     <sheet name="CSC-CSCSoCECBiaSY" sheetId="4" r:id="rId4"/>
+    <sheet name="CSC-CSCSCbPT" sheetId="7" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="100">
   <si>
     <t xml:space="preserve">Source: </t>
   </si>
@@ -134,9 +135,6 @@
     <t>Supply Curve Parameters</t>
   </si>
   <si>
-    <t>Share</t>
-  </si>
-  <si>
     <t>Notes:</t>
   </si>
   <si>
@@ -155,9 +153,6 @@
     <t>Minimum capacity buildable for plants types with no existing capacity (share if installed)</t>
   </si>
   <si>
-    <t>% of total installed capacity (tied to CSC)</t>
-  </si>
-  <si>
     <t>cutoff parameter</t>
   </si>
   <si>
@@ -177,6 +172,171 @@
   </si>
   <si>
     <t>value</t>
+  </si>
+  <si>
+    <t>Multiple of annual build limit available for procurement</t>
+  </si>
+  <si>
+    <t>Headroom</t>
+  </si>
+  <si>
+    <t>Seed Capacity (MW)</t>
+  </si>
+  <si>
+    <t>hard coal</t>
+  </si>
+  <si>
+    <t>natural gas steam turbine</t>
+  </si>
+  <si>
+    <t>natural gas combined cycle</t>
+  </si>
+  <si>
+    <t>nuclear</t>
+  </si>
+  <si>
+    <t>hydro</t>
+  </si>
+  <si>
+    <t>onshore wind</t>
+  </si>
+  <si>
+    <t>solar PV</t>
+  </si>
+  <si>
+    <t>solar thermal</t>
+  </si>
+  <si>
+    <t>biomass</t>
+  </si>
+  <si>
+    <t>geothermal</t>
+  </si>
+  <si>
+    <t>petroleum</t>
+  </si>
+  <si>
+    <t>natural gas peaker</t>
+  </si>
+  <si>
+    <t>lignite</t>
+  </si>
+  <si>
+    <t>offshore wind</t>
+  </si>
+  <si>
+    <t>crude oil</t>
+  </si>
+  <si>
+    <t>heavy or residual fuel oil</t>
+  </si>
+  <si>
+    <t>municipal solid waste</t>
+  </si>
+  <si>
+    <t>hard coal w CCS</t>
+  </si>
+  <si>
+    <t>natural gas combined cycle w CCS</t>
+  </si>
+  <si>
+    <t>biomass w CCS</t>
+  </si>
+  <si>
+    <t>lignite w CCS</t>
+  </si>
+  <si>
+    <t>small modular reactor</t>
+  </si>
+  <si>
+    <t>hydrogen combustion turbine</t>
+  </si>
+  <si>
+    <t>hydrogen combined cycle</t>
+  </si>
+  <si>
+    <t>Added 2026-08 (seed redesign prototype):</t>
+  </si>
+  <si>
+    <t>CSCSCbPT CSC Seed Capacity by Plant Type - growth basis for the annual build soft cap and entry floor.</t>
+  </si>
+  <si>
+    <t>Semantics: largest recent observed annual addition (incumbent types) or typical first-project size (types never yet built).</t>
+  </si>
+  <si>
+    <t>CSCPH CSC Procurement Headroom Factor - multiple of the annual build limit available for procurement on the supply curve (keeps mandates priced on the curve interior).</t>
+  </si>
+  <si>
+    <t>ALL VALUES BELOW ARE DRAFT ENGINEERING PLACEHOLDERS - to be replaced by EIA-860-derived values per the build-cap-calibration plan.</t>
+  </si>
+  <si>
+    <t>Electricity Source</t>
+  </si>
+  <si>
+    <t>Seed (MW)</t>
+  </si>
+  <si>
+    <t>Basis</t>
+  </si>
+  <si>
+    <t>~2 large units; no recent US additions, legacy EPC capability</t>
+  </si>
+  <si>
+    <t>legacy type; ~2 units</t>
+  </si>
+  <si>
+    <t>recent-era max annual US additions (placeholder pending EIA-860 derivation)</t>
+  </si>
+  <si>
+    <t>one AP1000 pair (Vogtle-style)</t>
+  </si>
+  <si>
+    <t>refurbishment/small-project scale</t>
+  </si>
+  <si>
+    <t>~US record annual additions (2020)</t>
+  </si>
+  <si>
+    <t>recent utility-scale annual additions</t>
+  </si>
+  <si>
+    <t>2-3 Ivanpah-scale projects</t>
+  </si>
+  <si>
+    <t>recent max annual additions</t>
+  </si>
+  <si>
+    <t>legacy type</t>
+  </si>
+  <si>
+    <t>recent annual additions envelope</t>
+  </si>
+  <si>
+    <t>~3 concurrent lease build-outs x ~800 MW</t>
+  </si>
+  <si>
+    <t>2-3 waste-to-energy plants</t>
+  </si>
+  <si>
+    <t>2 x 500 MW first-mover capture projects</t>
+  </si>
+  <si>
+    <t>2-3 first-mover capture projects</t>
+  </si>
+  <si>
+    <t>2 x 500 MW first-mover projects</t>
+  </si>
+  <si>
+    <t>1 x 500 MW first-mover project</t>
+  </si>
+  <si>
+    <t>3-4 first-mover multi-module sites x ~300 MW</t>
+  </si>
+  <si>
+    <t>1-2 projects; shares gas-turbine supply chain</t>
+  </si>
+  <si>
+    <t>2 projects; shares gas-turbine supply chain</t>
   </si>
 </sst>
 </file>
@@ -2033,7 +2193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D3D2DEE-686E-48A0-AC3D-0F54DEA5D0EC}">
-  <dimension ref="A1:C125"/>
+  <dimension ref="A1:C157"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="88.7109375" bestFit="1" customWidth="1"/>
@@ -2065,27 +2225,27 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -2103,7 +2263,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B16">
         <v>0.2</v>
@@ -2111,7 +2271,7 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B17">
         <v>0.6</v>
@@ -2119,7 +2279,7 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B18">
         <v>3</v>
@@ -2127,7 +2287,7 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B19">
         <v>0.5</v>
@@ -2135,7 +2295,7 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B20">
         <v>30000</v>
@@ -2143,7 +2303,7 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B21">
         <v>4.0000000000000001E-3</v>
@@ -3036,7 +3196,7 @@
         <v>44000</v>
       </c>
     </row>
-    <row r="113" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B113">
         <f t="shared" si="2"/>
         <v>0.19999994518873965</v>
@@ -3046,7 +3206,7 @@
         <v>44500</v>
       </c>
     </row>
-    <row r="114" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B114">
         <f t="shared" si="2"/>
         <v>0.19999996725245739</v>
@@ -3056,7 +3216,7 @@
         <v>45000</v>
       </c>
     </row>
-    <row r="115" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B115">
         <f t="shared" si="2"/>
         <v>0.19999998065979441</v>
@@ -3066,7 +3226,7 @@
         <v>45500</v>
       </c>
     </row>
-    <row r="116" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B116">
         <f t="shared" si="2"/>
         <v>0.19999998871085503</v>
@@ -3076,7 +3236,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="117" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B117">
         <f t="shared" si="2"/>
         <v>0.19999999348787459</v>
@@ -3086,7 +3246,7 @@
         <v>46500</v>
       </c>
     </row>
-    <row r="118" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B118">
         <f t="shared" si="2"/>
         <v>0.19999999628815057</v>
@@ -3096,7 +3256,7 @@
         <v>47000</v>
       </c>
     </row>
-    <row r="119" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B119">
         <f t="shared" si="2"/>
         <v>0.19999999790970302</v>
@@ -3106,7 +3266,7 @@
         <v>47500</v>
       </c>
     </row>
-    <row r="120" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B120">
         <f t="shared" si="2"/>
         <v>0.19999999883716038</v>
@@ -3116,7 +3276,7 @@
         <v>48000</v>
       </c>
     </row>
-    <row r="121" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B121">
         <f t="shared" si="2"/>
         <v>0.19999999936104543</v>
@@ -3126,7 +3286,7 @@
         <v>48500</v>
       </c>
     </row>
-    <row r="122" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B122">
         <f t="shared" si="2"/>
         <v>0.19999999965326104</v>
@@ -3136,7 +3296,7 @@
         <v>49000</v>
       </c>
     </row>
-    <row r="123" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B123">
         <f t="shared" si="2"/>
         <v>0.19999999981419306</v>
@@ -3146,7 +3306,7 @@
         <v>49500</v>
       </c>
     </row>
-    <row r="124" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B124">
         <f t="shared" si="2"/>
         <v>0.19999999990169129</v>
@@ -3156,7 +3316,7 @@
         <v>50000</v>
       </c>
     </row>
-    <row r="125" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B125">
         <f t="shared" si="2"/>
         <v>0.19999999994865042</v>
@@ -3164,6 +3324,306 @@
       <c r="C125">
         <f t="shared" si="3"/>
         <v>50500</v>
+      </c>
+    </row>
+    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A127" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A128" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="129" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A129" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A130" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="131" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A131" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="133" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A133" t="s">
+        <v>77</v>
+      </c>
+      <c r="B133" t="s">
+        <v>78</v>
+      </c>
+      <c r="C133" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A134" t="s">
+        <v>48</v>
+      </c>
+      <c r="B134">
+        <v>1300</v>
+      </c>
+      <c r="C134" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="135" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A135" t="s">
+        <v>49</v>
+      </c>
+      <c r="B135">
+        <v>600</v>
+      </c>
+      <c r="C135" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="136" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A136" t="s">
+        <v>50</v>
+      </c>
+      <c r="B136">
+        <v>10000</v>
+      </c>
+      <c r="C136" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="137" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A137" t="s">
+        <v>51</v>
+      </c>
+      <c r="B137">
+        <v>2200</v>
+      </c>
+      <c r="C137" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="138" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A138" t="s">
+        <v>52</v>
+      </c>
+      <c r="B138">
+        <v>500</v>
+      </c>
+      <c r="C138" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="139" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A139" t="s">
+        <v>53</v>
+      </c>
+      <c r="B139">
+        <v>15000</v>
+      </c>
+      <c r="C139" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A140" t="s">
+        <v>54</v>
+      </c>
+      <c r="B140">
+        <v>30000</v>
+      </c>
+      <c r="C140" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="141" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A141" t="s">
+        <v>55</v>
+      </c>
+      <c r="B141">
+        <v>400</v>
+      </c>
+      <c r="C141" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A142" t="s">
+        <v>56</v>
+      </c>
+      <c r="B142">
+        <v>500</v>
+      </c>
+      <c r="C142" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A143" t="s">
+        <v>57</v>
+      </c>
+      <c r="B143">
+        <v>150</v>
+      </c>
+      <c r="C143" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A144" t="s">
+        <v>58</v>
+      </c>
+      <c r="B144">
+        <v>200</v>
+      </c>
+      <c r="C144" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A145" t="s">
+        <v>59</v>
+      </c>
+      <c r="B145">
+        <v>5000</v>
+      </c>
+      <c r="C145" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A146" t="s">
+        <v>60</v>
+      </c>
+      <c r="B146">
+        <v>600</v>
+      </c>
+      <c r="C146" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A147" t="s">
+        <v>61</v>
+      </c>
+      <c r="B147">
+        <v>2400</v>
+      </c>
+      <c r="C147" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A148" t="s">
+        <v>62</v>
+      </c>
+      <c r="B148">
+        <v>200</v>
+      </c>
+      <c r="C148" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A149" t="s">
+        <v>63</v>
+      </c>
+      <c r="B149">
+        <v>200</v>
+      </c>
+      <c r="C149" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A150" t="s">
+        <v>64</v>
+      </c>
+      <c r="B150">
+        <v>100</v>
+      </c>
+      <c r="C150" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="151" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A151" t="s">
+        <v>65</v>
+      </c>
+      <c r="B151">
+        <v>1000</v>
+      </c>
+      <c r="C151" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="152" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A152" t="s">
+        <v>66</v>
+      </c>
+      <c r="B152">
+        <v>1500</v>
+      </c>
+      <c r="C152" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="153" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A153" t="s">
+        <v>67</v>
+      </c>
+      <c r="B153">
+        <v>1000</v>
+      </c>
+      <c r="C153" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="154" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A154" t="s">
+        <v>68</v>
+      </c>
+      <c r="B154">
+        <v>500</v>
+      </c>
+      <c r="C154" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="155" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A155" t="s">
+        <v>69</v>
+      </c>
+      <c r="B155">
+        <v>1200</v>
+      </c>
+      <c r="C155" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="156" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A156" t="s">
+        <v>70</v>
+      </c>
+      <c r="B156">
+        <v>400</v>
+      </c>
+      <c r="C156" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="157" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A157" t="s">
+        <v>71</v>
+      </c>
+      <c r="B157">
+        <v>800</v>
+      </c>
+      <c r="C157" t="s">
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -3173,6 +3633,32 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A11C1E0A-8F45-40E3-8B5E-CEBD35E65C82}">
+  <sheetPr>
+    <tabColor theme="4" tint="-0.499984740745262"/>
+  </sheetPr>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19F1B329-5591-420B-9DBA-D539EDB26DE6}">
   <sheetPr>
     <tabColor rgb="FF002060"/>
@@ -3185,15 +3671,15 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B2" s="2">
         <f>About!B16</f>
@@ -3202,7 +3688,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B3" s="2">
         <f>About!B17</f>
@@ -3211,7 +3697,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B4" s="2">
         <f>About!B18</f>
@@ -3220,7 +3706,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B5" s="2">
         <f>About!B19</f>
@@ -3229,41 +3715,11 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B6" s="2">
         <f>About!B20</f>
         <v>30000</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DCC8EED-C1F0-46D1-887C-CF4C1E6085B7}">
-  <sheetPr>
-    <tabColor rgb="FF002060"/>
-  </sheetPr>
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="17.5703125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B2" s="2">
-        <f>About!B21/About!B16</f>
-        <v>0.02</v>
       </c>
     </row>
   </sheetData>
@@ -5437,4 +5893,211 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{465ADDB1-7904-4401-8251-42AFA6AB8D4E}">
+  <dimension ref="A1:B25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B2">
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B3">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B4">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B5">
+        <v>2200</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B6">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>53</v>
+      </c>
+      <c r="B7">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B8">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B9">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>56</v>
+      </c>
+      <c r="B10">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>57</v>
+      </c>
+      <c r="B11">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>58</v>
+      </c>
+      <c r="B12">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>59</v>
+      </c>
+      <c r="B13">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>60</v>
+      </c>
+      <c r="B14">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>61</v>
+      </c>
+      <c r="B15">
+        <v>2400</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>62</v>
+      </c>
+      <c r="B16">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>63</v>
+      </c>
+      <c r="B17">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>64</v>
+      </c>
+      <c r="B18">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>65</v>
+      </c>
+      <c r="B19">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>66</v>
+      </c>
+      <c r="B20">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>67</v>
+      </c>
+      <c r="B21">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>68</v>
+      </c>
+      <c r="B22">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>69</v>
+      </c>
+      <c r="B23">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>70</v>
+      </c>
+      <c r="B24">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>71</v>
+      </c>
+      <c r="B25">
+        <v>800</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>